<commit_message>
Cảnh cuối Follow Adtek thay thẻ bài blog, bỏ link bài viết khỏi caption
Kênh TikTok độc lập với website. Đổi cảnh cuối 6 video đã dựng.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dpu4oyZ8FYSVLE8FrdnGTC
</commit_message>
<xml_diff>
--- a/video/plan/lich-noi-dung-tiktok.xlsx
+++ b/video/plan/lich-noi-dung-tiktok.xlsx
@@ -70,7 +70,7 @@
     <t xml:space="preserve">6 video đã dựng</t>
   </si>
   <si>
-    <t xml:space="preserve">AIO và khu công nghiệp FDI: đang chờ huấn luyện giọng Eleven v4. Cảnh cuối đang dẫn về blog, cần đổi lời kêu gọi trước khi đăng.</t>
+    <t xml:space="preserve">AIO và khu công nghiệp FDI: đang chờ huấn luyện giọng Eleven v4. Cảnh cuối đã đổi sang Follow Adtek, chỉ chờ tạo lại giọng.</t>
   </si>
   <si>
     <t xml:space="preserve">Cột cần cập nhật</t>
@@ -139,7 +139,7 @@
     <t xml:space="preserve">Đã dùng trong video, số liệu đã đối chiếu</t>
   </si>
   <si>
-    <t xml:space="preserve">Dữ liệu Mỹ. Cảnh cuối đang dẫn về blog, cần đổi lời kêu gọi</t>
+    <t xml:space="preserve">Dữ liệu Mỹ. Đã đổi cảnh cuối sang Follow Adtek, chờ tạo lại giọng</t>
   </si>
   <si>
     <t xml:space="preserve">ai overview là gì; aio là gì</t>
@@ -241,7 +241,7 @@
     <t xml:space="preserve">Đã dùng trong video; chưa có link bài cụ thể</t>
   </si>
   <si>
-    <t xml:space="preserve">Cảnh cuối đang dẫn về blog, cần đổi lời kêu gọi</t>
+    <t xml:space="preserve">Đã đổi cảnh cuối sang Follow Adtek, chờ tạo lại giọng</t>
   </si>
   <si>
     <t xml:space="preserve">marketing khu công nghiệp; thu hút fdi</t>

</xml_diff>

<commit_message>
Chuẩn video 1 phút mở đầu bằng câu hỏi; gộp 3 video khu công nghiệp thành 1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dpu4oyZ8FYSVLE8FrdnGTC
</commit_message>
<xml_diff>
--- a/video/plan/lich-noi-dung-tiktok.xlsx
+++ b/video/plan/lich-noi-dung-tiktok.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Dự phòng" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Lịch đăng'!$A$1:$O$48</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Lịch đăng'!$A$1:$O$46</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="680" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="426">
   <si>
     <t xml:space="preserve">Lịch nội dung TikTok Adtek</t>
   </si>
@@ -34,7 +34,7 @@
     <t xml:space="preserve">Cập nhật</t>
   </si>
   <si>
-    <t xml:space="preserve">07/10/2026. 47 video: 3 video AIO đã đăng, 44 video còn lại đăng 4 video mỗi tuần (thứ Sáu, Chủ nhật, thứ Hai, thứ Tư) từ 09/10/2026 đến 23/12/2026. Kênh: @adtek.growth.marketing.</t>
+    <t xml:space="preserve">07/10/2026. 3 video AIO đã đăng; 42 video còn lại đăng 4 video mỗi tuần (thứ Sáu, Chủ nhật, thứ Hai, thứ Tư) từ 09/10/2026 đến 20/12/2026. Kênh: @adtek.growth.marketing.</t>
   </si>
   <si>
     <t xml:space="preserve">Nguyên tắc</t>
@@ -46,7 +46,7 @@
     <t xml:space="preserve">Thứ tự đăng</t>
   </si>
   <si>
-    <t xml:space="preserve">3 video khu công nghiệp FDI đã dựng đăng trước (09/10 đến 12/10). Sau đó mỗi tuần trộn các dịch vụ khác nhau. Video theo mùa: TikTok Shop đăng đúng 11/11; khách từ AI đăng 22/11 trước Black Friday (27/11); quảng cáo Shopee đăng 09/12 trước 12.12; Tết đăng 16/12 để kịp kế hoạch Tết 2027 (06/02/2027).</t>
+    <t xml:space="preserve">Video khu công nghiệp tổng hợp đăng đầu tiên (09/10). Sau đó mỗi tuần trộn các dịch vụ khác nhau. Video theo mùa: TikTok Shop đăng đúng 11/11; khách từ AI đăng 22/11 trước Black Friday (27/11); quảng cáo Shopee đăng 09/12 trước 12.12; Tết đăng 16/12 để kịp kế hoạch Tết 2027 (06/02/2027).</t>
   </si>
   <si>
     <t xml:space="preserve">Kiểm tra nguồn</t>
@@ -67,10 +67,10 @@
     <t xml:space="preserve">Ước tính theo loại từ khóa và độ nóng chủ đề, chưa đo bằng công cụ. Kiểm tra trên TikTok Search và Google Keyword Planner nếu cần.</t>
   </si>
   <si>
-    <t xml:space="preserve">Video đã dựng</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 video AIO đã đăng. 3 video khu công nghiệp FDI chờ huấn luyện giọng Eleven v4; cảnh cuối đã đổi sang Follow Adtek, chỉ chờ tạo lại giọng.</t>
+    <t xml:space="preserve">Chuẩn video</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khoảng 1 phút (50 đến 65 giây), 6 cảnh. Câu đầu tiên là câu hỏi khơi tò mò. Chỉ giữ ý mạnh, có số liệu ấn tượng; mỗi video 3 đến 4 số liệu có nguồn. Cảnh cuối: Follow Adtek.</t>
   </si>
   <si>
     <t xml:space="preserve">Cột cần cập nhật</t>
@@ -205,25 +205,25 @@
     <t xml:space="preserve">Digital Marketing</t>
   </si>
   <si>
-    <t xml:space="preserve">Nhà đầu tư FDI lọc khu công nghiệp từ trên mạng</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vốn FDI tăng 76%, nhưng nhà đầu tư sẽ không gọi cho bạn đầu tiên.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FDI 9 tháng: 28.5 lên 50.4 tỷ USD; người mua B2B dành 27% thời gian tự nghiên cứu, 17% gặp nhà cung cấp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Biểu đồ cột, thanh ngang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cục Thống kê, 10/2026; Gartner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.gso.gov.vn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đã đổi cảnh cuối sang Follow Adtek, chờ tạo lại giọng</t>
+    <t xml:space="preserve">Vốn FDI tăng 76%, sao nhà đầu tư chưa gọi bạn? (gộp 3 video khu công nghiệp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vốn FDI vào Việt Nam tăng 76%. Vậy tại sao nhà đầu tư vẫn chưa gọi cho khu công nghiệp của bạn?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FDI 9 tháng 28.5 lên 50.4 tỷ USD; người mua B2B dành 27% thời gian tự nghiên cứu, 17% gặp nhà cung cấp; Singapore và Hàn Quốc 61% vốn FDI mới; JETRO: top 3 lợi thế không có giá đất</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cột, thanh ngang, danh sách, Follow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cục Thống kê; Gartner; Cổng Thông tin điện tử Chính phủ; JETRO FY2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.jetro.go.jp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kịch bản đã viết (scripts/khu-cong-nghiep-fdi/4.json), chờ giọng</t>
   </si>
   <si>
     <t xml:space="preserve">marketing khu công nghiệp; thu hút fdi</t>
@@ -232,126 +232,84 @@
     <t xml:space="preserve">Thấp, giá trị cao</t>
   </si>
   <si>
-    <t xml:space="preserve">Đã có video, chờ giọng</t>
+    <t xml:space="preserve">Đã viết kịch bản</t>
   </si>
   <si>
     <t xml:space="preserve">Chủ nhật</t>
   </si>
   <si>
-    <t xml:space="preserve">Website khu công nghiệp song ngữ là chưa đủ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Website song ngữ là chưa đủ.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Singapore 35.1%, Hàn Quốc 26.1% vốn FDI đăng ký mới 8 tháng 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Biểu đồ cột, danh sách</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cổng Thông tin điện tử Chính phủ, 09/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://chinhphu.vn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">marketing fdi; website khu công nghiệp</t>
+    <t xml:space="preserve">Performance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8/10 khách muốn nhắn tin trước khi mua</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cứ 10 khách thì 8 người muốn nhắn tin trước khi mua. Shop của bạn có trả lời kịp không?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">82.8% người Việt chọn nhắn tin để liên lạc doanh nghiệp; 61.2% nhắn tin với doanh nghiệp mỗi ngày; 85% mua sắm dịp Tết, 44% tham gia 12.12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ô vuông 100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meta, nghiên cứu do Kantar và Ipsos thực hiện (khảo sát 11/2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.facebook.com/business/news</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chưa có link bài cụ thể; Chưa mở được trang gốc (mạng chặn), đối chiếu qua Việt Nam News</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chưa có URL trang gốc của Meta, cần tìm trước khi dựng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">quảng cáo tin nhắn facebook; mùa sale 11.11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ý tưởng</t>
   </si>
   <si>
     <t xml:space="preserve">Thứ Hai</t>
   </si>
   <si>
-    <t xml:space="preserve">Đừng quảng cáo khu công nghiệp bằng giá đất</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quảng cáo khu công nghiệp bằng giá thuê đất rẻ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JETRO: 3 lợi thế hàng đầu không có giá đất; 67.5% doanh nghiệp Nhật lo thủ tục hành chính</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thanh ngang, ô vuông 100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JETRO, khảo sát FY2025, 906 doanh nghiệp Nhật tại Việt Nam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.jetro.go.jp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">đầu tư nhật bản việt nam; marketing b2b</t>
+    <t xml:space="preserve">Google AI Mode tiếng Việt tròn 1 năm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đúng một năm trước, Google bật Chế độ AI bằng tiếng Việt. Giờ mỗi tháng hơn 1 tỷ người dùng nó.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI Mode vượt 1 tỷ người dùng hằng tháng; AI Overviews hơn 2.5 tỷ; AI Mode có tiếng Việt từ 07/10/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biểu đồ cột</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google, I/O 2026 (Sundar Pichai), 05/2026; Google Search blog, 07/10/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://blog.google/products/search/ai-mode-expands-languages-locations/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua Engadget</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Số người dùng là toàn cầu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chế độ ai google; ai mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cao, đang tăng</t>
   </si>
   <si>
     <t xml:space="preserve">Thứ Tư</t>
   </si>
   <si>
-    <t xml:space="preserve">Performance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8/10 khách muốn nhắn tin trước khi mua</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cứ 10 khách thì 8 người muốn nhắn tin trước khi mua. Shop của bạn có trả lời kịp không?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">82.8% người Việt chọn nhắn tin để liên lạc doanh nghiệp; 61.2% nhắn tin với doanh nghiệp mỗi ngày; 85% mua sắm dịp Tết, 44% tham gia 12.12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ô vuông 100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Meta, nghiên cứu do Kantar và Ipsos thực hiện (khảo sát 11/2025)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.facebook.com/business/news</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chưa có link bài cụ thể; Chưa mở được trang gốc (mạng chặn), đối chiếu qua Việt Nam News</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chưa có URL trang gốc của Meta, cần tìm trước khi dựng</t>
-  </si>
-  <si>
-    <t xml:space="preserve">quảng cáo tin nhắn facebook; mùa sale 11.11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cao</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ý tưởng</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Google AI Mode tiếng Việt tròn 1 năm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đúng một năm trước, Google bật Chế độ AI bằng tiếng Việt. Giờ mỗi tháng hơn 1 tỷ người dùng nó.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AI Mode vượt 1 tỷ người dùng hằng tháng; AI Overviews hơn 2.5 tỷ; AI Mode có tiếng Việt từ 07/10/2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Biểu đồ cột</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Google, I/O 2026 (Sundar Pichai), 05/2026; Google Search blog, 07/10/2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://blog.google/products/search/ai-mode-expands-languages-locations/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua Engadget</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Số người dùng là toàn cầu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">chế độ ai google; ai mode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cao, đang tăng</t>
-  </si>
-  <si>
     <t xml:space="preserve">Growth Marketing</t>
   </si>
   <si>
@@ -685,6 +643,54 @@
     <t xml:space="preserve">ai overview trích dẫn; geo</t>
   </si>
   <si>
+    <t xml:space="preserve">75 tỷ USD quảng cáo mỗi năm đang để AI của Meta tự chạy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mỗi năm, 75 tỷ USD tiền quảng cáo đang để AI của Meta tự chạy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advantage+ vượt 75 tỷ USD doanh thu quy năm (quý 2/2026), từ 60 tỷ USD (quý 3/2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meta, kết quả kinh doanh Q2 2026, 29/07/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Link trang nhà đầu tư Meta; Chưa mở được trang gốc (mạng chặn), đối chiếu qua MarketBeat, MediaPost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Số toàn cầu, Meta tự công bố</t>
+  </si>
+  <si>
+    <t xml:space="preserve">advantage+; quảng cáo facebook ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Người mua livestream tin tài khoản chính hãng hơn KOL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Người mua qua livestream chi 67% tiền mua online ngay trên livestream, nhưng không mua nhiều nhất từ KOL.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Live commerce chiếm ~67% chi tiêu online của người mua livestream; ~50% thích mua từ tài khoản chính hãng, gần gấp đôi qua KOL; chỉ 13% mua bốc đồng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thanh ngang</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q&amp;Me, Xu hướng Live Commerce và hành vi người mua Việt Nam, 04/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://qandme.net/vi/baibaocao/xu-huong-live-commerce-va-hanh-vi-nguoi-mua-viet-nam.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua VnEconomy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mẫu 245 người ở TP.HCM và Hà Nội, video phải nói rõ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">livestream bán hàng; bán hàng livestream tiktok</t>
+  </si>
+  <si>
     <t xml:space="preserve">TikTok Shop giành 41% thị phần trong năm 2025</t>
   </si>
   <si>
@@ -709,54 +715,6 @@
     <t xml:space="preserve">tiktok shop; shopee hay tiktok shop</t>
   </si>
   <si>
-    <t xml:space="preserve">75 tỷ USD quảng cáo mỗi năm đang để AI của Meta tự chạy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mỗi năm, 75 tỷ USD tiền quảng cáo đang để AI của Meta tự chạy.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Advantage+ vượt 75 tỷ USD doanh thu quy năm (quý 2/2026), từ 60 tỷ USD (quý 3/2025)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Meta, kết quả kinh doanh Q2 2026, 29/07/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Link trang nhà đầu tư Meta; Chưa mở được trang gốc (mạng chặn), đối chiếu qua MarketBeat, MediaPost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Số toàn cầu, Meta tự công bố</t>
-  </si>
-  <si>
-    <t xml:space="preserve">advantage+; quảng cáo facebook ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Người mua livestream tin tài khoản chính hãng hơn KOL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Người mua qua livestream chi 67% tiền mua online ngay trên livestream, nhưng không mua nhiều nhất từ KOL.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Live commerce chiếm ~67% chi tiêu online của người mua livestream; ~50% thích mua từ tài khoản chính hãng, gần gấp đôi qua KOL; chỉ 13% mua bốc đồng</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thanh ngang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q&amp;Me, Xu hướng Live Commerce và hành vi người mua Việt Nam, 04/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://qandme.net/vi/baibaocao/xu-huong-live-commerce-va-hanh-vi-nguoi-mua-viet-nam.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua VnEconomy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mẫu 245 người ở TP.HCM và Hà Nội, video phải nói rõ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">livestream bán hàng; bán hàng livestream tiktok</t>
-  </si>
-  <si>
     <t xml:space="preserve">Người Việt dành 127 tỷ giờ trong app</t>
   </si>
   <si>
@@ -826,6 +784,54 @@
     <t xml:space="preserve">kol bị phạt; luật quảng cáo kol</t>
   </si>
   <si>
+    <t xml:space="preserve">Gartner từng nói SEO giảm 25% vào 2026. Thực tế thì sao?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Năm 2024 Gartner nói đến 2026 lượng tìm kiếm sẽ giảm 25%. Giờ đã là 2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dự đoán giảm 25% (02/2024); khảo sát 2026: chỉ ~1/3 người dùng thấy chatbot ngang công cụ tìm kiếm; hơn 2/3 vẫn đọc tiếp sau AI Overview</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Danh sách đối chiếu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gartner, 19/02/2024 và 20/01/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.gartner.com/en/newsroom/press-releases/2024-02-19-gartner-predicts-search-engine-volume-will-drop-25-percent-by-2026-due-to-ai-chatbots-and-other-virtual-agents</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua Demand Gen Report</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khảo sát 377 người Mỹ, mẫu nhỏ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">seo có còn hiệu quả; seo chết chưa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App tài chính Việt Nam cắt 48% ngân sách tìm khách mới</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Các app ngân hàng, ví điện tử vừa cắt 48% ngân sách tìm khách mới. Họ làm gì với số tiền đó?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2025: app tài chính Việt Nam giảm 22% lượt cài, chi phí kéo người dùng giảm 48%; remarketing Đông Nam Á +193%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AppsFlyer, State of Finance for Marketers APAC 2026, 16/04/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.appsflyer.com/resources/reports/apac-finance-marketing/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua Thị trường Tài chính Tiền tệ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">marketing ngân hàng số; remarketing</t>
+  </si>
+  <si>
     <t xml:space="preserve">AIO, Performance</t>
   </si>
   <si>
@@ -853,52 +859,52 @@
     <t xml:space="preserve">traffic từ chatgpt; bán hàng bằng ai</t>
   </si>
   <si>
-    <t xml:space="preserve">Gartner từng nói SEO giảm 25% vào 2026. Thực tế thì sao?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Năm 2024 Gartner nói đến 2026 lượng tìm kiếm sẽ giảm 25%. Giờ đã là 2026.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dự đoán giảm 25% (02/2024); khảo sát 2026: chỉ ~1/3 người dùng thấy chatbot ngang công cụ tìm kiếm; hơn 2/3 vẫn đọc tiếp sau AI Overview</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Danh sách đối chiếu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gartner, 19/02/2024 và 20/01/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.gartner.com/en/newsroom/press-releases/2024-02-19-gartner-predicts-search-engine-volume-will-drop-25-percent-by-2026-due-to-ai-chatbots-and-other-virtual-agents</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua Demand Gen Report</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Khảo sát 377 người Mỹ, mẫu nhỏ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">seo có còn hiệu quả; seo chết chưa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">App tài chính Việt Nam cắt 48% ngân sách tìm khách mới</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Các app ngân hàng, ví điện tử vừa cắt 48% ngân sách tìm khách mới. Họ làm gì với số tiền đó?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2025: app tài chính Việt Nam giảm 22% lượt cài, chi phí kéo người dùng giảm 48%; remarketing Đông Nam Á +193%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AppsFlyer, State of Finance for Marketers APAC 2026, 16/04/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.appsflyer.com/resources/reports/apac-finance-marketing/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua Thị trường Tài chính Tiền tệ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">marketing ngân hàng số; remarketing</t>
+    <t xml:space="preserve">72% khách tin doanh nghiệp ít hơn năm ngoái</t>
+  </si>
+  <si>
+    <t xml:space="preserve">72% khách hàng đang tin doanh nghiệp ít hơn năm ngoái, và dữ liệu là lý do.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">72% tin công ty ít hơn 1 năm trước; 65% thấy doanh nghiệp bất cẩn với dữ liệu; gần 75% muốn biết đang nói chuyện với AI hay người</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salesforce, State of the AI Connected Customer (bản 7), 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.salesforce.com/resources/research-reports/state-of-the-connected-customer/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua salesforce.com/news</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khảo sát 2024. Hợp đăng cạnh video luật dữ liệu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dữ liệu khách hàng; first-party data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luật Bảo vệ dữ liệu cá nhân: phạt tới 5% doanh thu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua một tệp data khách hàng để chạy quảng cáo, doanh nghiệp có thể bị phạt gấp 10 lần số tiền kiếm được.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luật 91/2025/QH15, hiệu lực 01/01/2026: mua bán dữ liệu phạt tới 10 lần khoản thu; chuyển dữ liệu ra nước ngoài trái quy định tới 5% doanh thu; vi phạm khác tới 3 tỷ đồng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quốc hội, Luật Bảo vệ dữ liệu cá nhân 91/2025/QH15; Nghị định 356/2025/NĐ-CP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://thuvienphapluat.vn/van-ban/Bo-may-hanh-chinh/Luat-Bao-ve-du-lieu-ca-nhan-2025-so-91-2025-QH15-625628.aspx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua VnEconomy, Báo Đầu tư, PwC Việt Nam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nội dung pháp lý, nên nhờ luật sư duyệt kịch bản</t>
+  </si>
+  <si>
+    <t xml:space="preserve">luật bảo vệ dữ liệu cá nhân; nghị định 356</t>
   </si>
   <si>
     <t xml:space="preserve">Khách trả phí làm thành viên lại chi nhiều hơn</t>
@@ -922,54 +928,6 @@
     <t xml:space="preserve">khách hàng thân thiết; membership</t>
   </si>
   <si>
-    <t xml:space="preserve">72% khách tin doanh nghiệp ít hơn năm ngoái</t>
-  </si>
-  <si>
-    <t xml:space="preserve">72% khách hàng đang tin doanh nghiệp ít hơn năm ngoái, và dữ liệu là lý do.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">72% tin công ty ít hơn 1 năm trước; 65% thấy doanh nghiệp bất cẩn với dữ liệu; gần 75% muốn biết đang nói chuyện với AI hay người</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Salesforce, State of the AI Connected Customer (bản 7), 2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.salesforce.com/resources/research-reports/state-of-the-connected-customer/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua salesforce.com/news</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Khảo sát 2024. Hợp đăng cạnh video luật dữ liệu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dữ liệu khách hàng; first-party data</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luật Bảo vệ dữ liệu cá nhân: phạt tới 5% doanh thu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mua một tệp data khách hàng để chạy quảng cáo, doanh nghiệp có thể bị phạt gấp 10 lần số tiền kiếm được.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luật 91/2025/QH15, hiệu lực 01/01/2026: mua bán dữ liệu phạt tới 10 lần khoản thu; chuyển dữ liệu ra nước ngoài trái quy định tới 5% doanh thu; vi phạm khác tới 3 tỷ đồng</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quốc hội, Luật Bảo vệ dữ liệu cá nhân 91/2025/QH15; Nghị định 356/2025/NĐ-CP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://thuvienphapluat.vn/van-ban/Bo-may-hanh-chinh/Luat-Bao-ve-du-lieu-ca-nhan-2025-so-91-2025-QH15-625628.aspx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua VnEconomy, Báo Đầu tư, PwC Việt Nam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nội dung pháp lý, nên nhờ luật sư duyệt kịch bản</t>
-  </si>
-  <si>
-    <t xml:space="preserve">luật bảo vệ dữ liệu cá nhân; nghị định 356</t>
-  </si>
-  <si>
     <t xml:space="preserve">25 tỷ lượt tìm kiếm mỗi tháng không cần gõ chữ</t>
   </si>
   <si>
@@ -1063,6 +1021,45 @@
     <t xml:space="preserve">zalo oa; quảng cáo zalo</t>
   </si>
   <si>
+    <t xml:space="preserve">81% người Việt dùng AI mỗi ngày</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cứ 10 người Việt dùng internet thì 8 người nói chuyện với AI mỗi ngày.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">81% tương tác với AI hằng ngày, cao nhất Đông Nam Á (Indonesia 80%, Thái Lan 74%); 96% sẵn sàng chia sẻ dữ liệu với AI agent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua Việt Nam News, VnEconomy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">người việt dùng ai; ai việt nam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lần đầu người dùng chi cho app nhiều hơn cho game</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lần đầu tiên, người dùng chi tiền cho app nhiều hơn cho game.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.3 nghìn tỷ giờ trong app năm 2025 (~3.6 giờ/ngày); chi tiêu in-app 167 tỷ USD (+10%); app không phải game lần đầu vượt game</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sensor Tower, State of Mobile 2026, 21/01/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://sensortower.com/blog/state-of-mobile-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua PR Newswire, 9to5Mac</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Số toàn cầu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">app ai; thời gian dùng điện thoại mỗi ngày</t>
+  </si>
+  <si>
     <t xml:space="preserve">Doanh thu quảng cáo Shopee tăng hơn 70%</t>
   </si>
   <si>
@@ -1087,45 +1084,6 @@
     <t xml:space="preserve">quảng cáo shopee; phí sàn shopee 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">81% người Việt dùng AI mỗi ngày</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cứ 10 người Việt dùng internet thì 8 người nói chuyện với AI mỗi ngày.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">81% tương tác với AI hằng ngày, cao nhất Đông Nam Á (Indonesia 80%, Thái Lan 74%); 96% sẵn sàng chia sẻ dữ liệu với AI agent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua Việt Nam News, VnEconomy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">người việt dùng ai; ai việt nam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lần đầu người dùng chi cho app nhiều hơn cho game</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lần đầu tiên, người dùng chi tiền cho app nhiều hơn cho game.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.3 nghìn tỷ giờ trong app năm 2025 (~3.6 giờ/ngày); chi tiêu in-app 167 tỷ USD (+10%); app không phải game lần đầu vượt game</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sensor Tower, State of Mobile 2026, 21/01/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://sensortower.com/blog/state-of-mobile-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua PR Newswire, 9to5Mac</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Số toàn cầu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">app ai; thời gian dùng điện thoại mỗi ngày</t>
-  </si>
-  <si>
     <t xml:space="preserve">Google AI Max: bật một nút, thêm 14% chuyển đổi?</t>
   </si>
   <si>
@@ -1150,6 +1108,48 @@
     <t xml:space="preserve">google ads ai max; performance max</t>
   </si>
   <si>
+    <t xml:space="preserve">Một thử nghiệm A/B mang về 100 triệu USD mỗi năm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Một thay đổi nhỏ bị bỏ xó 6 tháng, sau đó mang về hơn 100 triệu USD mỗi năm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bing đổi tiêu đề quảng cáo: doanh thu +12%, hơn 100 triệu USD/năm; chỉ 10-20% thử nghiệm ở Google, Bing cho kết quả tích cực</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kohavi và Thomke, Harvard Business Review, 09/2017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://hbr.org/2017/09/the-surprising-power-of-online-experiments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua sách của Kohavi (Cambridge University Press)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Case năm 2012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a/b testing; thử nghiệm marketing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thấp, hợp định vị Growth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kinh tế số Việt Nam 39 tỷ USD, 2/3 là mua sắm online</t>
+  </si>
+  <si>
+    <t xml:space="preserve">39 tỷ USD: quy mô kinh tế số Việt Nam năm 2025, và 2/3 là mua sắm online.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GMV kinh tế số 39 tỷ USD (+17%), tăng nhanh thứ 2 Đông Nam Á; thương mại điện tử 25 tỷ USD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua Bộ Công Thương (vntr.moit.gov.vn)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kinh tế số việt nam; e-conomy sea</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tết vừa rồi TikTok Shop lần đầu bán nhiều hơn Shopee</t>
   </si>
   <si>
@@ -1172,48 +1172,6 @@
   </si>
   <si>
     <t xml:space="preserve">Cao (theo mùa)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Một thử nghiệm A/B mang về 100 triệu USD mỗi năm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Một thay đổi nhỏ bị bỏ xó 6 tháng, sau đó mang về hơn 100 triệu USD mỗi năm.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bing đổi tiêu đề quảng cáo: doanh thu +12%, hơn 100 triệu USD/năm; chỉ 10-20% thử nghiệm ở Google, Bing cho kết quả tích cực</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kohavi và Thomke, Harvard Business Review, 09/2017</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://hbr.org/2017/09/the-surprising-power-of-online-experiments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua sách của Kohavi (Cambridge University Press)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Case năm 2012</t>
-  </si>
-  <si>
-    <t xml:space="preserve">a/b testing; thử nghiệm marketing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thấp, hợp định vị Growth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kinh tế số Việt Nam 39 tỷ USD, 2/3 là mua sắm online</t>
-  </si>
-  <si>
-    <t xml:space="preserve">39 tỷ USD: quy mô kinh tế số Việt Nam năm 2025, và 2/3 là mua sắm online.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GMV kinh tế số 39 tỷ USD (+17%), tăng nhanh thứ 2 Đông Nam Á; thương mại điện tử 25 tỷ USD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chưa mở được trang gốc (mạng chặn), đối chiếu qua Bộ Công Thương (vntr.moit.gov.vn)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kinh tế số việt nam; e-conomy sea</t>
   </si>
   <si>
     <t xml:space="preserve">Internet Việt Nam chạm trần: 85.6 triệu người dùng</t>
@@ -1989,7 +1947,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O48"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -2190,7 +2148,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="n">
         <v>4</v>
       </c>
@@ -2237,7 +2195,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="n">
         <v>5</v>
       </c>
@@ -2248,87 +2206,87 @@
         <v>46306</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>48</v>
+        <v>77</v>
       </c>
       <c r="L6" s="8" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="N6" s="5" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>46307</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="H7" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="L7" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="O7" s="5" t="s">
         <v>81</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="L7" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="M7" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="N7" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="O7" s="5" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2336,46 +2294,46 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>46309</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="L8" s="8" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="M8" s="5" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="N8" s="5" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="O8" s="5" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2389,40 +2347,40 @@
         <v>46311</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>31</v>
+        <v>103</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="J9" s="11" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="L9" s="12" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="M9" s="9" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="N9" s="9" t="s">
-        <v>107</v>
+        <v>80</v>
       </c>
       <c r="O9" s="9" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2436,40 +2394,40 @@
         <v>46313</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>108</v>
+        <v>70</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="J10" s="11" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="L10" s="12" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="M10" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="N10" s="9" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="O10" s="9" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2477,46 +2435,44 @@
         <v>10</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C11" s="10" t="n">
         <v>46314</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="J11" s="11" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="L11" s="12" t="s">
-        <v>124</v>
-      </c>
+        <v>126</v>
+      </c>
+      <c r="L11" s="9"/>
       <c r="M11" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="N11" s="9" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="O11" s="9" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2524,49 +2480,49 @@
         <v>11</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C12" s="10" t="n">
         <v>46316</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>86</v>
+        <v>58</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="J12" s="11" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="L12" s="12" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="M12" s="9" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="N12" s="9" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="O12" s="9" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="n">
         <v>12</v>
       </c>
@@ -2577,38 +2533,40 @@
         <v>46318</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>134</v>
+        <v>70</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>101</v>
+        <v>74</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="L13" s="5"/>
+        <v>142</v>
+      </c>
+      <c r="L13" s="8" t="s">
+        <v>110</v>
+      </c>
       <c r="M13" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="N13" s="5" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="O13" s="5" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2622,87 +2580,85 @@
         <v>46320</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>58</v>
+        <v>94</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>145</v>
+        <v>74</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L14" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M14" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N14" s="5" t="s">
-        <v>96</v>
+        <v>152</v>
       </c>
       <c r="O14" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C15" s="6" t="n">
         <v>46321</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="L15" s="8" t="s">
-        <v>124</v>
-      </c>
+        <v>158</v>
+      </c>
+      <c r="L15" s="5"/>
       <c r="M15" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="N15" s="5" t="s">
-        <v>96</v>
+        <v>160</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2710,49 +2666,49 @@
         <v>15</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C16" s="6" t="n">
         <v>46323</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>108</v>
+        <v>70</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>162</v>
+        <v>141</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="L16" s="8" t="s">
-        <v>164</v>
+        <v>110</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="N16" s="5" t="s">
-        <v>166</v>
+        <v>80</v>
       </c>
       <c r="O16" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="n">
         <v>16</v>
       </c>
@@ -2763,7 +2719,7 @@
         <v>46325</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>117</v>
+        <v>31</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>167</v>
@@ -2775,7 +2731,7 @@
         <v>169</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="I17" s="9" t="s">
         <v>170</v>
@@ -2791,10 +2747,10 @@
         <v>173</v>
       </c>
       <c r="N17" s="9" t="s">
-        <v>174</v>
+        <v>80</v>
       </c>
       <c r="O17" s="9" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2808,85 +2764,85 @@
         <v>46327</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>86</v>
+        <v>58</v>
       </c>
       <c r="E18" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="F18" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="G18" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="H18" s="9" t="s">
         <v>177</v>
-      </c>
-      <c r="H18" s="9" t="s">
-        <v>101</v>
       </c>
       <c r="I18" s="9" t="s">
         <v>178</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>155</v>
+        <v>179</v>
       </c>
       <c r="K18" s="9" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="L18" s="12" t="s">
-        <v>124</v>
+        <v>181</v>
       </c>
       <c r="M18" s="9" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="N18" s="9" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="O18" s="9" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="n">
         <v>18</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C19" s="10" t="n">
         <v>46328</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>31</v>
+        <v>94</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="I19" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="J19" s="11" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="K19" s="9" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="L19" s="9"/>
       <c r="M19" s="9" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="N19" s="9" t="s">
-        <v>96</v>
+        <v>160</v>
       </c>
       <c r="O19" s="9" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2894,46 +2850,46 @@
         <v>19</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C20" s="10" t="n">
         <v>46330</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>58</v>
+        <v>103</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>191</v>
+        <v>86</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J20" s="11" t="s">
-        <v>193</v>
+        <v>108</v>
       </c>
       <c r="K20" s="9" t="s">
         <v>194</v>
       </c>
       <c r="L20" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="M20" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="M20" s="9" t="s">
-        <v>196</v>
-      </c>
       <c r="N20" s="9" t="s">
-        <v>96</v>
+        <v>160</v>
       </c>
       <c r="O20" s="9" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2947,7 +2903,7 @@
         <v>46332</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>108</v>
+        <v>196</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>197</v>
@@ -2959,7 +2915,7 @@
         <v>199</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="I21" s="5" t="s">
         <v>200</v>
@@ -2970,18 +2926,20 @@
       <c r="K21" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="L21" s="5"/>
+      <c r="L21" s="8" t="s">
+        <v>203</v>
+      </c>
       <c r="M21" s="5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="N21" s="5" t="s">
-        <v>174</v>
+        <v>41</v>
       </c>
       <c r="O21" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="n">
         <v>21</v>
       </c>
@@ -2992,40 +2950,40 @@
         <v>46334</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>117</v>
+        <v>70</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="K22" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="L22" s="8" t="s">
-        <v>124</v>
+        <v>210</v>
       </c>
       <c r="M22" s="5" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="N22" s="5" t="s">
-        <v>174</v>
+        <v>80</v>
       </c>
       <c r="O22" s="5" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3033,46 +2991,46 @@
         <v>22</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C23" s="6" t="n">
         <v>46335</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>210</v>
+        <v>58</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>101</v>
+        <v>215</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="J23" s="7" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="L23" s="8" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="M23" s="5" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="N23" s="5" t="s">
-        <v>41</v>
+        <v>80</v>
       </c>
       <c r="O23" s="5" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3080,49 +3038,49 @@
         <v>23</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C24" s="6" t="n">
         <v>46337</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="L24" s="8" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="N24" s="5" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="O24" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="n">
         <v>24</v>
       </c>
@@ -3133,40 +3091,40 @@
         <v>46339</v>
       </c>
       <c r="D25" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="H25" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="E25" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="G25" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="H25" s="9" t="s">
-        <v>101</v>
-      </c>
       <c r="I25" s="9" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="J25" s="11" t="s">
-        <v>130</v>
+        <v>233</v>
       </c>
       <c r="K25" s="9" t="s">
-        <v>231</v>
+        <v>218</v>
       </c>
       <c r="L25" s="12" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="M25" s="9" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="N25" s="9" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="O25" s="9" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3180,54 +3138,52 @@
         <v>46341</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>237</v>
+        <v>86</v>
       </c>
       <c r="I26" s="9" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="J26" s="11" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>240</v>
-      </c>
-      <c r="L26" s="12" t="s">
         <v>241</v>
       </c>
+      <c r="L26" s="9"/>
       <c r="M26" s="9" t="s">
         <v>242</v>
       </c>
       <c r="N26" s="9" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="O26" s="9" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="n">
         <v>26</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C27" s="10" t="n">
         <v>46342</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>117</v>
+        <v>58</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>243</v>
@@ -3239,28 +3195,28 @@
         <v>245</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>101</v>
+        <v>246</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="J27" s="11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="K27" s="9" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="L27" s="12" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="M27" s="9" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="N27" s="9" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3268,47 +3224,49 @@
         <v>27</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C28" s="10" t="n">
         <v>46344</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>86</v>
+        <v>120</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="G28" s="9" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>101</v>
+        <v>255</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="J28" s="11" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="K28" s="9" t="s">
-        <v>255</v>
-      </c>
-      <c r="L28" s="9"/>
+        <v>258</v>
+      </c>
+      <c r="L28" s="12" t="s">
+        <v>259</v>
+      </c>
       <c r="M28" s="9" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="N28" s="9" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="O28" s="9" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="n">
         <v>28</v>
       </c>
@@ -3319,40 +3277,40 @@
         <v>46346</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>58</v>
+        <v>103</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>260</v>
+        <v>86</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="K29" s="5" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="L29" s="8" t="s">
-        <v>264</v>
+        <v>110</v>
       </c>
       <c r="M29" s="5" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="N29" s="5" t="s">
-        <v>96</v>
+        <v>160</v>
       </c>
       <c r="O29" s="5" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3366,40 +3324,40 @@
         <v>46348</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="L30" s="8" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="M30" s="5" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="N30" s="5" t="s">
         <v>41</v>
       </c>
       <c r="O30" s="5" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3407,93 +3365,93 @@
         <v>30</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C31" s="6" t="n">
         <v>46349</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>134</v>
+        <v>94</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>278</v>
+        <v>74</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="K31" s="5" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="L31" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="M31" s="5" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="N31" s="5" t="s">
-        <v>96</v>
+        <v>160</v>
       </c>
       <c r="O31" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="n">
         <v>31</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C32" s="6" t="n">
         <v>46351</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>117</v>
+        <v>58</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>101</v>
+        <v>246</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K32" s="5" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="L32" s="8" t="s">
-        <v>124</v>
+        <v>291</v>
       </c>
       <c r="M32" s="5" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="N32" s="5" t="s">
-        <v>174</v>
+        <v>80</v>
       </c>
       <c r="O32" s="5" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3507,40 +3465,40 @@
         <v>46353</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="I33" s="9" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="J33" s="11" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="K33" s="9" t="s">
-        <v>163</v>
+        <v>149</v>
       </c>
       <c r="L33" s="12" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="M33" s="9" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="N33" s="9" t="s">
-        <v>174</v>
+        <v>160</v>
       </c>
       <c r="O33" s="9" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3554,69 +3512,67 @@
         <v>46355</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="E34" s="9" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="I34" s="9" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="J34" s="11" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="K34" s="9" t="s">
-        <v>303</v>
-      </c>
-      <c r="L34" s="12" t="s">
-        <v>304</v>
-      </c>
+        <v>305</v>
+      </c>
+      <c r="L34" s="9"/>
       <c r="M34" s="9" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="N34" s="9" t="s">
-        <v>174</v>
+        <v>152</v>
       </c>
       <c r="O34" s="9" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="n">
         <v>34</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C35" s="10" t="n">
         <v>46356</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>58</v>
+        <v>103</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="H35" s="9" t="s">
-        <v>260</v>
+        <v>86</v>
       </c>
       <c r="I35" s="9" t="s">
-        <v>309</v>
+        <v>107</v>
       </c>
       <c r="J35" s="11" t="s">
         <v>310</v>
@@ -3631,10 +3587,10 @@
         <v>313</v>
       </c>
       <c r="N35" s="9" t="s">
-        <v>96</v>
+        <v>160</v>
       </c>
       <c r="O35" s="9" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3642,13 +3598,13 @@
         <v>35</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C36" s="10" t="n">
         <v>46358</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>134</v>
+        <v>94</v>
       </c>
       <c r="E36" s="9" t="s">
         <v>314</v>
@@ -3660,26 +3616,28 @@
         <v>316</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>101</v>
+        <v>317</v>
       </c>
       <c r="I36" s="9" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="J36" s="11" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="K36" s="9" t="s">
-        <v>319</v>
-      </c>
-      <c r="L36" s="9"/>
+        <v>320</v>
+      </c>
+      <c r="L36" s="12" t="s">
+        <v>321</v>
+      </c>
       <c r="M36" s="9" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="N36" s="9" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="O36" s="9" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3693,40 +3651,40 @@
         <v>46360</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>117</v>
+        <v>58</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="I37" s="5" t="s">
-        <v>121</v>
+        <v>326</v>
       </c>
       <c r="J37" s="7" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="L37" s="8" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="M37" s="5" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="N37" s="5" t="s">
-        <v>174</v>
+        <v>80</v>
       </c>
       <c r="O37" s="5" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3740,40 +3698,40 @@
         <v>46362</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>108</v>
+        <v>31</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>331</v>
+        <v>131</v>
       </c>
       <c r="I38" s="5" t="s">
-        <v>332</v>
+        <v>239</v>
       </c>
       <c r="J38" s="7" t="s">
-        <v>333</v>
+        <v>240</v>
       </c>
       <c r="K38" s="5" t="s">
         <v>334</v>
       </c>
       <c r="L38" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="M38" s="5" t="s">
         <v>335</v>
       </c>
-      <c r="M38" s="5" t="s">
-        <v>336</v>
-      </c>
       <c r="N38" s="5" t="s">
-        <v>174</v>
+        <v>80</v>
       </c>
       <c r="O38" s="5" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3781,46 +3739,46 @@
         <v>38</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C39" s="6" t="n">
         <v>46363</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>58</v>
+        <v>103</v>
       </c>
       <c r="E39" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="F39" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="F39" s="5" t="s">
+      <c r="G39" s="5" t="s">
         <v>338</v>
       </c>
-      <c r="G39" s="5" t="s">
+      <c r="H39" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I39" s="5" t="s">
         <v>339</v>
       </c>
-      <c r="H39" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="I39" s="5" t="s">
+      <c r="J39" s="7" t="s">
         <v>340</v>
       </c>
-      <c r="J39" s="7" t="s">
+      <c r="K39" s="5" t="s">
         <v>341</v>
       </c>
-      <c r="K39" s="5" t="s">
+      <c r="L39" s="8" t="s">
         <v>342</v>
       </c>
-      <c r="L39" s="8" t="s">
+      <c r="M39" s="5" t="s">
         <v>343</v>
       </c>
-      <c r="M39" s="5" t="s">
-        <v>344</v>
-      </c>
       <c r="N39" s="5" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="O39" s="5" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3828,49 +3786,49 @@
         <v>39</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C40" s="6" t="n">
         <v>46365</v>
       </c>
       <c r="D40" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>345</v>
+      </c>
+      <c r="G40" s="5" t="s">
+        <v>346</v>
+      </c>
+      <c r="H40" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="E40" s="5" t="s">
-        <v>345</v>
-      </c>
-      <c r="F40" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="G40" s="5" t="s">
+      <c r="I40" s="5" t="s">
         <v>347</v>
       </c>
-      <c r="H40" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="I40" s="5" t="s">
+      <c r="J40" s="7" t="s">
         <v>348</v>
       </c>
-      <c r="J40" s="7" t="s">
+      <c r="K40" s="5" t="s">
         <v>349</v>
       </c>
-      <c r="K40" s="5" t="s">
+      <c r="L40" s="8" t="s">
         <v>350</v>
       </c>
-      <c r="L40" s="8" t="s">
+      <c r="M40" s="5" t="s">
         <v>351</v>
       </c>
-      <c r="M40" s="5" t="s">
-        <v>352</v>
-      </c>
       <c r="N40" s="5" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="O40" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="9" t="n">
         <v>40</v>
       </c>
@@ -3881,43 +3839,43 @@
         <v>46367</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>31</v>
+        <v>70</v>
       </c>
       <c r="E41" s="9" t="s">
+        <v>352</v>
+      </c>
+      <c r="F41" s="9" t="s">
         <v>353</v>
       </c>
-      <c r="F41" s="9" t="s">
+      <c r="G41" s="9" t="s">
         <v>354</v>
       </c>
-      <c r="G41" s="9" t="s">
+      <c r="H41" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="I41" s="9" t="s">
         <v>355</v>
       </c>
-      <c r="H41" s="9" t="s">
-        <v>145</v>
-      </c>
-      <c r="I41" s="9" t="s">
-        <v>253</v>
-      </c>
       <c r="J41" s="11" t="s">
-        <v>254</v>
+        <v>356</v>
       </c>
       <c r="K41" s="9" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="L41" s="12" t="s">
-        <v>124</v>
+        <v>358</v>
       </c>
       <c r="M41" s="9" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="N41" s="9" t="s">
-        <v>96</v>
+        <v>160</v>
       </c>
       <c r="O41" s="9" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="9" t="n">
         <v>41</v>
       </c>
@@ -3928,87 +3886,85 @@
         <v>46369</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>117</v>
+        <v>94</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="I42" s="9" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="J42" s="11" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="K42" s="9" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="L42" s="12" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="M42" s="9" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="N42" s="9" t="s">
-        <v>96</v>
+        <v>368</v>
       </c>
       <c r="O42" s="9" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="9" t="n">
         <v>42</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C43" s="10" t="n">
         <v>46370</v>
       </c>
       <c r="D43" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E43" s="9" t="s">
+        <v>369</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>370</v>
+      </c>
+      <c r="G43" s="9" t="s">
+        <v>371</v>
+      </c>
+      <c r="H43" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="E43" s="9" t="s">
-        <v>366</v>
-      </c>
-      <c r="F43" s="9" t="s">
-        <v>367</v>
-      </c>
-      <c r="G43" s="9" t="s">
-        <v>368</v>
-      </c>
-      <c r="H43" s="9" t="s">
-        <v>101</v>
-      </c>
       <c r="I43" s="9" t="s">
-        <v>369</v>
+        <v>239</v>
       </c>
       <c r="J43" s="11" t="s">
-        <v>370</v>
+        <v>240</v>
       </c>
       <c r="K43" s="9" t="s">
-        <v>371</v>
-      </c>
-      <c r="L43" s="12" t="s">
         <v>372</v>
       </c>
+      <c r="L43" s="9"/>
       <c r="M43" s="9" t="s">
         <v>373</v>
       </c>
       <c r="N43" s="9" t="s">
-        <v>174</v>
+        <v>160</v>
       </c>
       <c r="O43" s="9" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4016,13 +3972,13 @@
         <v>43</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C44" s="10" t="n">
         <v>46372</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="E44" s="9" t="s">
         <v>374</v>
@@ -4034,13 +3990,13 @@
         <v>376</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="I44" s="9" t="s">
         <v>377</v>
       </c>
       <c r="J44" s="11" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="K44" s="9" t="s">
         <v>378</v>
@@ -4055,10 +4011,10 @@
         <v>381</v>
       </c>
       <c r="O44" s="9" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="n">
         <v>44</v>
       </c>
@@ -4069,7 +4025,7 @@
         <v>46374</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>108</v>
+        <v>58</v>
       </c>
       <c r="E45" s="5" t="s">
         <v>382</v>
@@ -4081,7 +4037,7 @@
         <v>384</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>101</v>
+        <v>74</v>
       </c>
       <c r="I45" s="5" t="s">
         <v>385</v>
@@ -4099,10 +4055,10 @@
         <v>389</v>
       </c>
       <c r="N45" s="5" t="s">
-        <v>390</v>
+        <v>381</v>
       </c>
       <c r="O45" s="5" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4116,138 +4072,46 @@
         <v>46376</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>58</v>
+        <v>103</v>
       </c>
       <c r="E46" s="5" t="s">
+        <v>390</v>
+      </c>
+      <c r="F46" s="5" t="s">
         <v>391</v>
       </c>
-      <c r="F46" s="5" t="s">
+      <c r="G46" s="5" t="s">
         <v>392</v>
       </c>
-      <c r="G46" s="5" t="s">
+      <c r="H46" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I46" s="5" t="s">
         <v>393</v>
       </c>
-      <c r="H46" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="I46" s="5" t="s">
-        <v>253</v>
-      </c>
       <c r="J46" s="7" t="s">
-        <v>254</v>
+        <v>394</v>
       </c>
       <c r="K46" s="5" t="s">
-        <v>394</v>
-      </c>
-      <c r="L46" s="5"/>
+        <v>395</v>
+      </c>
+      <c r="L46" s="8" t="s">
+        <v>396</v>
+      </c>
       <c r="M46" s="5" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="N46" s="5" t="s">
-        <v>174</v>
+        <v>160</v>
       </c>
       <c r="O46" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="5" t="n">
-        <v>46</v>
-      </c>
-      <c r="B47" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="C47" s="6" t="n">
-        <v>46377</v>
-      </c>
-      <c r="D47" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="E47" s="5" t="s">
-        <v>396</v>
-      </c>
-      <c r="F47" s="5" t="s">
-        <v>397</v>
-      </c>
-      <c r="G47" s="5" t="s">
-        <v>398</v>
-      </c>
-      <c r="H47" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="I47" s="5" t="s">
-        <v>399</v>
-      </c>
-      <c r="J47" s="7" t="s">
-        <v>400</v>
-      </c>
-      <c r="K47" s="5" t="s">
-        <v>401</v>
-      </c>
-      <c r="L47" s="8" t="s">
-        <v>402</v>
-      </c>
-      <c r="M47" s="5" t="s">
-        <v>403</v>
-      </c>
-      <c r="N47" s="5" t="s">
-        <v>381</v>
-      </c>
-      <c r="O47" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="5" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="C48" s="6" t="n">
-        <v>46379</v>
-      </c>
-      <c r="D48" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="E48" s="5" t="s">
-        <v>404</v>
-      </c>
-      <c r="F48" s="5" t="s">
-        <v>405</v>
-      </c>
-      <c r="G48" s="5" t="s">
-        <v>406</v>
-      </c>
-      <c r="H48" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="I48" s="5" t="s">
-        <v>407</v>
-      </c>
-      <c r="J48" s="7" t="s">
-        <v>408</v>
-      </c>
-      <c r="K48" s="5" t="s">
-        <v>409</v>
-      </c>
-      <c r="L48" s="8" t="s">
-        <v>410</v>
-      </c>
-      <c r="M48" s="5" t="s">
-        <v>411</v>
-      </c>
-      <c r="N48" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="O48" s="5" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O48"/>
+  <autoFilter ref="A1:O46"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="O2:O48" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="O2:O46" type="list">
       <formula1>"Ý tưởng,Đã kiểm tra nguồn,Đã viết kịch bản,Đã có video,chờ giọng,Đã có video,Đã đăng"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4256,50 +4120,48 @@
     <hyperlink ref="J2" r:id="rId1" display="https://www.pewresearch.org/short-reads/2025/07/22/google-users-are-less-likely-to-click-on-links-when-an-ai-summary-appears-in-the-results/"/>
     <hyperlink ref="J3" r:id="rId2" display="https://ahrefs.com/blog/"/>
     <hyperlink ref="J4" r:id="rId3" display="https://sparktoro.com/blog/"/>
-    <hyperlink ref="J5" r:id="rId4" display="https://www.gso.gov.vn"/>
-    <hyperlink ref="J6" r:id="rId5" display="https://chinhphu.vn"/>
-    <hyperlink ref="J7" r:id="rId6" display="https://www.jetro.go.jp"/>
-    <hyperlink ref="J8" r:id="rId7" display="https://www.facebook.com/business/news"/>
-    <hyperlink ref="J9" r:id="rId8" display="https://blog.google/products/search/ai-mode-expands-languages-locations/"/>
-    <hyperlink ref="J10" r:id="rId9" display="https://baymard.com/lists/cart-abandonment-rate"/>
-    <hyperlink ref="J11" r:id="rId10" display="https://www.appsflyer.com/resources/reports/app-marketing-vietnam/"/>
-    <hyperlink ref="J12" r:id="rId11" display="https://investor.atmeta.com"/>
-    <hyperlink ref="J13" r:id="rId12" display="https://ahrefs.com/blog/ai-overviews-reduce-clicks-update/"/>
-    <hyperlink ref="J14" r:id="rId13" display="https://newsroom.tiktok.com/tiktok-surpasses-460-million-users-in-southeast-asia-inks-partnership-with-vietnams-ministry-of-culture-sports-and-tourism"/>
-    <hyperlink ref="J15" r:id="rId14" display="https://metric.vn"/>
-    <hyperlink ref="J16" r:id="rId15" display="https://www.mckinsey.com/capabilities/growth-marketing-and-sales/our-insights/the-value-of-getting-personalization-right-or-wrong-is-multiplying"/>
-    <hyperlink ref="J17" r:id="rId16" display="https://www.appsflyer.com/resources/reports/state-fraud-marketers/"/>
-    <hyperlink ref="J18" r:id="rId17" display="https://metric.vn"/>
-    <hyperlink ref="J19" r:id="rId18" display="https://openai.com/index/scaling-ai-for-everyone/"/>
-    <hyperlink ref="J20" r:id="rId19" display="https://thuvienphapluat.vn/van-ban/Thuong-mai/Luat-Thuong-mai-dien-tu-2025-so-122-2025-QH15-662035.aspx"/>
-    <hyperlink ref="J21" r:id="rId20" display="https://www.twilio.com/en-us/press/releases/socer-2025"/>
-    <hyperlink ref="J22" r:id="rId21" display="https://www.appsflyer.com/resources/reports/app-marketing-vietnam/"/>
-    <hyperlink ref="J23" r:id="rId22" display="https://ahrefs.com/blog/ai-overview-citations-top-10/"/>
+    <hyperlink ref="J5" r:id="rId4" display="https://www.jetro.go.jp"/>
+    <hyperlink ref="J6" r:id="rId5" display="https://www.facebook.com/business/news"/>
+    <hyperlink ref="J7" r:id="rId6" display="https://blog.google/products/search/ai-mode-expands-languages-locations/"/>
+    <hyperlink ref="J8" r:id="rId7" display="https://baymard.com/lists/cart-abandonment-rate"/>
+    <hyperlink ref="J9" r:id="rId8" display="https://www.appsflyer.com/resources/reports/app-marketing-vietnam/"/>
+    <hyperlink ref="J10" r:id="rId9" display="https://investor.atmeta.com"/>
+    <hyperlink ref="J11" r:id="rId10" display="https://ahrefs.com/blog/ai-overviews-reduce-clicks-update/"/>
+    <hyperlink ref="J12" r:id="rId11" display="https://newsroom.tiktok.com/tiktok-surpasses-460-million-users-in-southeast-asia-inks-partnership-with-vietnams-ministry-of-culture-sports-and-tourism"/>
+    <hyperlink ref="J13" r:id="rId12" display="https://metric.vn"/>
+    <hyperlink ref="J14" r:id="rId13" display="https://www.mckinsey.com/capabilities/growth-marketing-and-sales/our-insights/the-value-of-getting-personalization-right-or-wrong-is-multiplying"/>
+    <hyperlink ref="J15" r:id="rId14" display="https://www.appsflyer.com/resources/reports/state-fraud-marketers/"/>
+    <hyperlink ref="J16" r:id="rId15" display="https://metric.vn"/>
+    <hyperlink ref="J17" r:id="rId16" display="https://openai.com/index/scaling-ai-for-everyone/"/>
+    <hyperlink ref="J18" r:id="rId17" display="https://thuvienphapluat.vn/van-ban/Thuong-mai/Luat-Thuong-mai-dien-tu-2025-so-122-2025-QH15-662035.aspx"/>
+    <hyperlink ref="J19" r:id="rId18" display="https://www.twilio.com/en-us/press/releases/socer-2025"/>
+    <hyperlink ref="J20" r:id="rId19" display="https://www.appsflyer.com/resources/reports/app-marketing-vietnam/"/>
+    <hyperlink ref="J21" r:id="rId20" display="https://ahrefs.com/blog/ai-overview-citations-top-10/"/>
+    <hyperlink ref="J22" r:id="rId21" display="https://investor.atmeta.com"/>
+    <hyperlink ref="J23" r:id="rId22" display="https://qandme.net/vi/baibaocao/xu-huong-live-commerce-va-hanh-vi-nguoi-mua-viet-nam.html"/>
     <hyperlink ref="J24" r:id="rId23" display="https://metric.vn"/>
-    <hyperlink ref="J25" r:id="rId24" display="https://investor.atmeta.com"/>
-    <hyperlink ref="J26" r:id="rId25" display="https://qandme.net/vi/baibaocao/xu-huong-live-commerce-va-hanh-vi-nguoi-mua-viet-nam.html"/>
-    <hyperlink ref="J27" r:id="rId26" display="https://www.adjust.com/blog/vietnam-app-trends-2026/"/>
-    <hyperlink ref="J28" r:id="rId27" display="https://economysea.withgoogle.com/"/>
-    <hyperlink ref="J29" r:id="rId28" display="https://vbpl.vn"/>
+    <hyperlink ref="J25" r:id="rId24" display="https://www.adjust.com/blog/vietnam-app-trends-2026/"/>
+    <hyperlink ref="J26" r:id="rId25" display="https://economysea.withgoogle.com/"/>
+    <hyperlink ref="J27" r:id="rId26" display="https://vbpl.vn"/>
+    <hyperlink ref="J28" r:id="rId27" display="https://www.gartner.com/en/newsroom/press-releases/2024-02-19-gartner-predicts-search-engine-volume-will-drop-25-percent-by-2026-due-to-ai-chatbots-and-other-virtual-agents"/>
+    <hyperlink ref="J29" r:id="rId28" display="https://www.appsflyer.com/resources/reports/apac-finance-marketing/"/>
     <hyperlink ref="J30" r:id="rId29" display="https://business.adobe.com/blog/ai-traffic-surge-retail-sites-not-machine-readable"/>
-    <hyperlink ref="J31" r:id="rId30" display="https://www.gartner.com/en/newsroom/press-releases/2024-02-19-gartner-predicts-search-engine-volume-will-drop-25-percent-by-2026-due-to-ai-chatbots-and-other-virtual-agents"/>
-    <hyperlink ref="J32" r:id="rId31" display="https://www.appsflyer.com/resources/reports/apac-finance-marketing/"/>
+    <hyperlink ref="J31" r:id="rId30" display="https://www.salesforce.com/resources/research-reports/state-of-the-connected-customer/"/>
+    <hyperlink ref="J32" r:id="rId31" display="https://thuvienphapluat.vn/van-ban/Bo-may-hanh-chinh/Luat-Bao-ve-du-lieu-ca-nhan-2025-so-91-2025-QH15-625628.aspx"/>
     <hyperlink ref="J33" r:id="rId32" display="https://www.mckinsey.com/capabilities/growth-marketing-and-sales/our-insights/coping-with-the-big-switch-how-paid-loyalty-programs-can-help-bring-consumers-back-to-your-brand"/>
-    <hyperlink ref="J34" r:id="rId33" display="https://www.salesforce.com/resources/research-reports/state-of-the-connected-customer/"/>
-    <hyperlink ref="J35" r:id="rId34" display="https://thuvienphapluat.vn/van-ban/Bo-may-hanh-chinh/Luat-Bao-ve-du-lieu-ca-nhan-2025-so-91-2025-QH15-625628.aspx"/>
-    <hyperlink ref="J36" r:id="rId35" display="https://vietnamese.googleblog.com/2026/03/ai-ang-thay-oi-cach-nguoi-tieu-dung-tim.html"/>
-    <hyperlink ref="J37" r:id="rId36" display="https://www.appsflyer.com/resources/reports/app-marketing-vietnam-report/"/>
-    <hyperlink ref="J38" r:id="rId37" display="https://hbr.org/1990/09/zero-defections-quality-comes-to-services"/>
-    <hyperlink ref="J39" r:id="rId38" display="https://vng.com.vn"/>
+    <hyperlink ref="J34" r:id="rId33" display="https://vietnamese.googleblog.com/2026/03/ai-ang-thay-oi-cach-nguoi-tieu-dung-tim.html"/>
+    <hyperlink ref="J35" r:id="rId34" display="https://www.appsflyer.com/resources/reports/app-marketing-vietnam-report/"/>
+    <hyperlink ref="J36" r:id="rId35" display="https://hbr.org/1990/09/zero-defections-quality-comes-to-services"/>
+    <hyperlink ref="J37" r:id="rId36" display="https://vng.com.vn"/>
+    <hyperlink ref="J38" r:id="rId37" display="https://economysea.withgoogle.com/"/>
+    <hyperlink ref="J39" r:id="rId38" display="https://sensortower.com/blog/state-of-mobile-2026"/>
     <hyperlink ref="J40" r:id="rId39" display="https://www.businesswire.com/news/home/20260810021050/en/Sea-Limited-Reports-Second-Quarter-2026-Results"/>
-    <hyperlink ref="J41" r:id="rId40" display="https://economysea.withgoogle.com/"/>
-    <hyperlink ref="J42" r:id="rId41" display="https://sensortower.com/blog/state-of-mobile-2026"/>
-    <hyperlink ref="J43" r:id="rId42" display="https://blog.google/products/ads-commerce/"/>
+    <hyperlink ref="J41" r:id="rId40" display="https://blog.google/products/ads-commerce/"/>
+    <hyperlink ref="J42" r:id="rId41" display="https://hbr.org/2017/09/the-surprising-power-of-online-experiments"/>
+    <hyperlink ref="J43" r:id="rId42" display="https://economysea.withgoogle.com/"/>
     <hyperlink ref="J44" r:id="rId43" display="https://metric.vn"/>
-    <hyperlink ref="J45" r:id="rId44" display="https://hbr.org/2017/09/the-surprising-power-of-online-experiments"/>
-    <hyperlink ref="J46" r:id="rId45" display="https://economysea.withgoogle.com/"/>
-    <hyperlink ref="J47" r:id="rId46" display="https://datareportal.com/reports/digital-2026-vietnam"/>
-    <hyperlink ref="J48" r:id="rId47" display="https://www.adjust.com/resources/ebooks/mobile-app-trends-2026/"/>
+    <hyperlink ref="J45" r:id="rId44" display="https://datareportal.com/reports/digital-2026-vietnam"/>
+    <hyperlink ref="J46" r:id="rId45" display="https://www.adjust.com/resources/ebooks/mobile-app-trends-2026/"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4308,7 +4170,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId48"/>
+  <drawing r:id="rId46"/>
 </worksheet>
 </file>
 
@@ -4329,25 +4191,25 @@
         <v>20</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>412</v>
+        <v>398</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>30</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>413</v>
+        <v>399</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="14" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
       <c r="B2" s="14" t="n">
-        <f aca="false">COUNTIF('Lịch đăng'!$D$2:$D$48,"*SEO*")</f>
+        <f aca="false">COUNTIF('Lịch đăng'!$D$2:$D$46,"*SEO*")</f>
         <v>4</v>
       </c>
       <c r="C2" s="14" t="n">
-        <f aca="false">COUNTIFS('Lịch đăng'!$D$2:$D$48,"*SEO*",'Lịch đăng'!$O$2:$O$48,"Đã đăng")</f>
+        <f aca="false">COUNTIFS('Lịch đăng'!$D$2:$D$46,"*SEO*",'Lịch đăng'!$O$2:$O$46,"Đã đăng")</f>
         <v>0</v>
       </c>
       <c r="D2" s="14" t="n">
@@ -4360,11 +4222,11 @@
         <v>31</v>
       </c>
       <c r="B3" s="14" t="n">
-        <f aca="false">COUNTIF('Lịch đăng'!$D$2:$D$48,"*AIO*")</f>
+        <f aca="false">COUNTIF('Lịch đăng'!$D$2:$D$46,"*AIO*")</f>
         <v>8</v>
       </c>
       <c r="C3" s="14" t="n">
-        <f aca="false">COUNTIFS('Lịch đăng'!$D$2:$D$48,"*AIO*",'Lịch đăng'!$O$2:$O$48,"Đã đăng")</f>
+        <f aca="false">COUNTIFS('Lịch đăng'!$D$2:$D$46,"*AIO*",'Lịch đăng'!$O$2:$O$46,"Đã đăng")</f>
         <v>3</v>
       </c>
       <c r="D3" s="14" t="n">
@@ -4374,14 +4236,14 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="B4" s="14" t="n">
-        <f aca="false">COUNTIF('Lịch đăng'!$D$2:$D$48,"*Performance*")</f>
+        <f aca="false">COUNTIF('Lịch đăng'!$D$2:$D$46,"*Performance*")</f>
         <v>11</v>
       </c>
       <c r="C4" s="14" t="n">
-        <f aca="false">COUNTIFS('Lịch đăng'!$D$2:$D$48,"*Performance*",'Lịch đăng'!$O$2:$O$48,"Đã đăng")</f>
+        <f aca="false">COUNTIFS('Lịch đăng'!$D$2:$D$46,"*Performance*",'Lịch đăng'!$O$2:$O$46,"Đã đăng")</f>
         <v>0</v>
       </c>
       <c r="D4" s="14" t="n">
@@ -4391,14 +4253,14 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>117</v>
+        <v>103</v>
       </c>
       <c r="B5" s="14" t="n">
-        <f aca="false">COUNTIF('Lịch đăng'!$D$2:$D$48,"*App Marketing*")</f>
+        <f aca="false">COUNTIF('Lịch đăng'!$D$2:$D$46,"*App Marketing*")</f>
         <v>8</v>
       </c>
       <c r="C5" s="14" t="n">
-        <f aca="false">COUNTIFS('Lịch đăng'!$D$2:$D$48,"*App Marketing*",'Lịch đăng'!$O$2:$O$48,"Đã đăng")</f>
+        <f aca="false">COUNTIFS('Lịch đăng'!$D$2:$D$46,"*App Marketing*",'Lịch đăng'!$O$2:$O$46,"Đã đăng")</f>
         <v>0</v>
       </c>
       <c r="D5" s="14" t="n">
@@ -4408,14 +4270,14 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="B6" s="14" t="n">
-        <f aca="false">COUNTIF('Lịch đăng'!$D$2:$D$48,"*Growth Marketing*")</f>
+        <f aca="false">COUNTIF('Lịch đăng'!$D$2:$D$46,"*Growth Marketing*")</f>
         <v>7</v>
       </c>
       <c r="C6" s="14" t="n">
-        <f aca="false">COUNTIFS('Lịch đăng'!$D$2:$D$48,"*Growth Marketing*",'Lịch đăng'!$O$2:$O$48,"Đã đăng")</f>
+        <f aca="false">COUNTIFS('Lịch đăng'!$D$2:$D$46,"*Growth Marketing*",'Lịch đăng'!$O$2:$O$46,"Đã đăng")</f>
         <v>0</v>
       </c>
       <c r="D6" s="14" t="n">
@@ -4428,38 +4290,38 @@
         <v>58</v>
       </c>
       <c r="B7" s="14" t="n">
-        <f aca="false">COUNTIF('Lịch đăng'!$D$2:$D$48,"*Digital Marketing*")</f>
-        <v>11</v>
+        <f aca="false">COUNTIF('Lịch đăng'!$D$2:$D$46,"*Digital Marketing*")</f>
+        <v>9</v>
       </c>
       <c r="C7" s="14" t="n">
-        <f aca="false">COUNTIFS('Lịch đăng'!$D$2:$D$48,"*Digital Marketing*",'Lịch đăng'!$O$2:$O$48,"Đã đăng")</f>
+        <f aca="false">COUNTIFS('Lịch đăng'!$D$2:$D$46,"*Digital Marketing*",'Lịch đăng'!$O$2:$O$46,"Đã đăng")</f>
         <v>0</v>
       </c>
       <c r="D7" s="14" t="n">
         <f aca="false">B7-C7</f>
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>414</v>
+        <v>400</v>
       </c>
       <c r="B8" s="15" t="n">
-        <f aca="false">COUNTA('Lịch đăng'!$A$2:$A$48)</f>
-        <v>47</v>
+        <f aca="false">COUNTA('Lịch đăng'!$A$2:$A$46)</f>
+        <v>45</v>
       </c>
       <c r="C8" s="15" t="n">
-        <f aca="false">COUNTIF('Lịch đăng'!$O$2:$O$48,"Đã đăng")</f>
+        <f aca="false">COUNTIF('Lịch đăng'!$O$2:$O$46,"Đã đăng")</f>
         <v>3</v>
       </c>
       <c r="D8" s="15" t="n">
         <f aca="false">B8-C8</f>
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>415</v>
+        <v>401</v>
       </c>
     </row>
   </sheetData>
@@ -4492,13 +4354,13 @@
         <v>20</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>416</v>
+        <v>402</v>
       </c>
       <c r="C1" s="17" t="s">
         <v>25</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>417</v>
+        <v>403</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4506,27 +4368,27 @@
         <v>31</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>418</v>
+        <v>404</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>419</v>
+        <v>405</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>420</v>
+        <v>406</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="18" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>421</v>
+        <v>407</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>422</v>
+        <v>408</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>423</v>
+        <v>409</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4534,69 +4396,69 @@
         <v>31</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>424</v>
+        <v>410</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>425</v>
+        <v>411</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>426</v>
+        <v>412</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>427</v>
+        <v>413</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>428</v>
+        <v>414</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>429</v>
+        <v>415</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>117</v>
+        <v>103</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>430</v>
+        <v>416</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>431</v>
+        <v>417</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>432</v>
+        <v>418</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>117</v>
+        <v>103</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>433</v>
+        <v>419</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>434</v>
+        <v>420</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>435</v>
+        <v>421</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>436</v>
+        <v>422</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>437</v>
+        <v>423</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>438</v>
+        <v>424</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>439</v>
+        <v>425</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Viết lại video khu công nghiệp cho tự nhiên, thêm quy tắc viết tiếng Việt không dịch thẳng
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dpu4oyZ8FYSVLE8FrdnGTC
</commit_message>
<xml_diff>
--- a/video/plan/lich-noi-dung-tiktok.xlsx
+++ b/video/plan/lich-noi-dung-tiktok.xlsx
@@ -39,7 +39,7 @@
     <t xml:space="preserve">Chuẩn video</t>
   </si>
   <si>
-    <t xml:space="preserve">Khoảng 1 phút, 6 cảnh. Câu đầu tiên là câu hỏi khơi tò mò. Mỗi video gộp 2 đến 4 số liệu mạnh về cùng một chủ đề. Cảnh cuối: Follow Adtek.</t>
+    <t xml:space="preserve">Khoảng 1 phút, 6 cảnh. Câu đầu tiên là câu hỏi khơi tò mò. Mỗi video gộp 2 đến 4 số liệu mạnh về cùng một chủ đề. Cảnh cuối: Follow Adtek. Viết tiếng Việt tự nhiên như người Việt nói, không dịch thẳng từ tiếng Anh. Cột số liệu là ghi chú nội bộ, khi viết kịch bản phải viết lại cho tự nhiên.</t>
   </si>
   <si>
     <t xml:space="preserve">Nguyên tắc nguồn</t>
@@ -206,7 +206,7 @@
     <t xml:space="preserve">Khách hàng của bạn đang hỏi AI</t>
   </si>
   <si>
-    <t xml:space="preserve">Mỗi tuần 900 triệu người hỏi ChatGPT. Họ có nghe thấy tên thương hiệu của bạn không?</t>
+    <t xml:space="preserve">Mỗi tuần 900 triệu người hỏi ChatGPT. Có ai được nó gợi ý tên thương hiệu của bạn chưa?</t>
   </si>
   <si>
     <t xml:space="preserve">• 900 triệu người dùng hằng tuần (từ 800 triệu, 10/2025); hơn 50 triệu người trả phí
@@ -357,7 +357,7 @@
     <t xml:space="preserve">quảng cáo facebook 2026; advantage+; ai max</t>
   </si>
   <si>
-    <t xml:space="preserve">Livestream bán hàng: ai đang thắng?</t>
+    <t xml:space="preserve">Livestream bán hàng: người mua tin ai?</t>
   </si>
   <si>
     <t xml:space="preserve">650,000 nhà bán đang livestream. Người mua thật sự tin ai?</t>
@@ -508,7 +508,7 @@
     <t xml:space="preserve">Digital, Growth</t>
   </si>
   <si>
-    <t xml:space="preserve">Dữ liệu khách hàng: tài sản hay rủi ro?</t>
+    <t xml:space="preserve">Mua data khách hàng để chạy quảng cáo: rủi ro tới đâu?</t>
   </si>
   <si>
     <t xml:space="preserve">Mua một tệp data khách hàng để chạy quảng cáo, rủi ro lớn nhất là gì?</t>
@@ -537,7 +537,7 @@
     <t xml:space="preserve">luật bảo vệ dữ liệu cá nhân; data khách hàng</t>
   </si>
   <si>
-    <t xml:space="preserve">Kinh tế số 39 tỷ USD, internet đã chạm trần</t>
+    <t xml:space="preserve">Kinh tế số 39 tỷ USD, nhưng người dùng mới gần như không tăng</t>
   </si>
   <si>
     <t xml:space="preserve">Kinh tế số Việt Nam 39 tỷ USD. Vì sao tìm khách mới online ngày càng khó?</t>
@@ -1281,7 +1281,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
Trang hub video TikTok, video khu công nghiệp tổng hợp (giọng v4), cập nhật quy trình
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dpu4oyZ8FYSVLE8FrdnGTC
</commit_message>
<xml_diff>
--- a/video/plan/lich-noi-dung-tiktok.xlsx
+++ b/video/plan/lich-noi-dung-tiktok.xlsx
@@ -57,7 +57,7 @@
     <t xml:space="preserve">Slot trống (màu cam nhạt)</t>
   </si>
   <si>
-    <t xml:space="preserve">Dành cho chủ đề trend lấy từ TikTok Creator Search Insights. Mỗi chủ đề trend vẫn phải gắn với dịch vụ Adtek và có số liệu từ nguồn gốc.</t>
+    <t xml:space="preserve">Claude tự chọn chủ đề đang được quan tâm khi viết kịch bản mỗi thứ Bảy. Mỗi chủ đề vẫn phải gắn với dịch vụ Adtek và có số liệu từ nguồn gốc.</t>
   </si>
   <si>
     <t xml:space="preserve">Lưu ý khi dùng</t>
@@ -147,7 +147,8 @@
     <t xml:space="preserve">• Đã dùng trong video; chưa có link bài cụ thể</t>
   </si>
   <si>
-    <t xml:space="preserve">• Kịch bản đã viết (scripts/khu-cong-nghiep-fdi/4.json), chờ giọng</t>
+    <t xml:space="preserve">• Kịch bản đã viết (scripts/khu-cong-nghiep-fdi/4.json), chờ giọng
+• Giọng v4 chưa huấn luyện; video trên trang hub</t>
   </si>
   <si>
     <t xml:space="preserve">marketing khu công nghiệp; thu hút fdi</t>
@@ -156,7 +157,7 @@
     <t xml:space="preserve">Thấp, giá trị cao</t>
   </si>
   <si>
-    <t xml:space="preserve">Đã viết kịch bản</t>
+    <t xml:space="preserve">Đã có video</t>
   </si>
   <si>
     <t xml:space="preserve">Chủ nhật</t>
@@ -565,7 +566,7 @@
     <t xml:space="preserve">kinh tế số việt nam; digital 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Slot trống: chủ đề trend từ Creator Search Insights</t>
+    <t xml:space="preserve">Slot trống: chủ đề trend Claude tự chọn khi viết kịch bản thứ Bảy</t>
   </si>
   <si>
     <t xml:space="preserve">Cần chủ đề</t>
@@ -894,8 +895,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -947,11 +952,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1263,61 +1268,61 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="95"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="B1" s="3"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+    <row r="3" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1340,1544 +1345,1544 @@
   <dimension ref="A1:N46"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="n">
+    <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5" t="s">
+      <c r="B2" s="6"/>
+      <c r="C2" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5" t="s">
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5" t="s">
+      <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="n">
+    <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5" t="s">
+      <c r="B3" s="6"/>
+      <c r="C3" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5" t="s">
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5" t="s">
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="n">
+    <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5" t="s">
+      <c r="B4" s="6"/>
+      <c r="C4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5" t="s">
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5" t="s">
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="n">
+    <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="7" t="n">
         <v>46304</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="J5" s="5" t="s">
+      <c r="J5" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="K5" s="7" t="s">
+      <c r="K5" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="L5" s="5" t="s">
+      <c r="L5" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="M5" s="5" t="s">
+      <c r="M5" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="N5" s="5" t="s">
+      <c r="N5" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="n">
+    <row r="6" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="7" t="n">
         <v>46306</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="J6" s="5" t="s">
+      <c r="J6" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="K6" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="L6" s="5" t="s">
+      <c r="L6" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="M6" s="5" t="s">
+      <c r="M6" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="N6" s="5" t="s">
+      <c r="N6" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="n">
+    <row r="7" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="7" t="n">
         <v>46307</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="J7" s="5" t="s">
+      <c r="J7" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="K7" s="7" t="s">
+      <c r="K7" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="L7" s="5" t="s">
+      <c r="L7" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="M7" s="5" t="s">
+      <c r="M7" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="N7" s="5" t="s">
+      <c r="N7" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="n">
+    <row r="8" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="7" t="n">
         <v>46309</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="J8" s="5" t="s">
+      <c r="J8" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="K8" s="7" t="s">
+      <c r="K8" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="L8" s="5" t="s">
+      <c r="L8" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="M8" s="5" t="s">
+      <c r="M8" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="N8" s="5" t="s">
+      <c r="N8" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="n">
+    <row r="9" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C9" s="10" t="n">
         <v>46311</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="H9" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="I9" s="8" t="s">
+      <c r="I9" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="J9" s="8" t="s">
+      <c r="J9" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="K9" s="10" t="s">
+      <c r="K9" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="L9" s="8" t="s">
+      <c r="L9" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="M9" s="8" t="s">
+      <c r="M9" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="N9" s="8" t="s">
+      <c r="N9" s="9" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="n">
+    <row r="10" customFormat="false" ht="135.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="9" t="n">
+      <c r="C10" s="10" t="n">
         <v>46313</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="H10" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="I10" s="8" t="s">
+      <c r="I10" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="J10" s="8" t="s">
+      <c r="J10" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="K10" s="10" t="s">
+      <c r="K10" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="L10" s="8" t="s">
+      <c r="L10" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="M10" s="8" t="s">
+      <c r="M10" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="N10" s="8" t="s">
+      <c r="N10" s="9" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="n">
+    <row r="11" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C11" s="9" t="n">
+      <c r="C11" s="10" t="n">
         <v>46314</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="G11" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="H11" s="8" t="s">
+      <c r="H11" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="I11" s="8" t="s">
+      <c r="I11" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="J11" s="8" t="s">
+      <c r="J11" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="K11" s="10" t="s">
+      <c r="K11" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="L11" s="8" t="s">
+      <c r="L11" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="M11" s="8" t="s">
+      <c r="M11" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="N11" s="8" t="s">
+      <c r="N11" s="9" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="n">
+    <row r="12" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="C12" s="9" t="n">
+      <c r="C12" s="10" t="n">
         <v>46316</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="H12" s="8" t="s">
+      <c r="H12" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="I12" s="8" t="s">
+      <c r="I12" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="J12" s="8" t="s">
+      <c r="J12" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="K12" s="10" t="s">
+      <c r="K12" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="L12" s="8" t="s">
+      <c r="L12" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="M12" s="8" t="s">
+      <c r="M12" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="N12" s="8" t="s">
+      <c r="N12" s="9" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="n">
+    <row r="13" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C13" s="7" t="n">
         <v>46318</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="G13" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="H13" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="I13" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="J13" s="5" t="s">
+      <c r="J13" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="K13" s="7" t="s">
+      <c r="K13" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="L13" s="5" t="s">
+      <c r="L13" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="M13" s="5" t="s">
+      <c r="M13" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="N13" s="5" t="s">
+      <c r="N13" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="n">
+    <row r="14" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C14" s="7" t="n">
         <v>46320</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="G14" s="5" t="s">
+      <c r="G14" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="H14" s="5" t="s">
+      <c r="H14" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="I14" s="5" t="s">
+      <c r="I14" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="J14" s="5" t="s">
+      <c r="J14" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="K14" s="7" t="s">
+      <c r="K14" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="L14" s="5" t="s">
+      <c r="L14" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="M14" s="5" t="s">
+      <c r="M14" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="N14" s="5" t="s">
+      <c r="N14" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="n">
+    <row r="15" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="C15" s="7" t="n">
         <v>46321</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="E15" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="F15" s="5" t="s">
+      <c r="F15" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="G15" s="5" t="s">
+      <c r="G15" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="H15" s="5" t="s">
+      <c r="H15" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="I15" s="5" t="s">
+      <c r="I15" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="J15" s="5" t="s">
+      <c r="J15" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="K15" s="7" t="s">
+      <c r="K15" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="L15" s="5" t="s">
+      <c r="L15" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="M15" s="5" t="s">
+      <c r="M15" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="N15" s="5" t="s">
+      <c r="N15" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="n">
+    <row r="16" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C16" s="7" t="n">
         <v>46323</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="E16" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="F16" s="5" t="s">
+      <c r="F16" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="G16" s="5" t="s">
+      <c r="G16" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="H16" s="5" t="s">
+      <c r="H16" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="I16" s="5" t="s">
+      <c r="I16" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="J16" s="5" t="s">
+      <c r="J16" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="K16" s="7" t="s">
+      <c r="K16" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="L16" s="5" t="s">
+      <c r="L16" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="M16" s="5" t="s">
+      <c r="M16" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="N16" s="5" t="s">
+      <c r="N16" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="n">
+    <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="12" t="n">
+      <c r="C17" s="13" t="n">
         <v>46325</v>
       </c>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11" t="s">
+      <c r="D17" s="12"/>
+      <c r="E17" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11"/>
-      <c r="K17" s="11"/>
-      <c r="L17" s="11"/>
-      <c r="M17" s="11"/>
-      <c r="N17" s="11" t="s">
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="12"/>
+      <c r="L17" s="12"/>
+      <c r="M17" s="12"/>
+      <c r="N17" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="n">
+    <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="C18" s="12" t="n">
+      <c r="C18" s="13" t="n">
         <v>46327</v>
       </c>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11" t="s">
+      <c r="D18" s="12"/>
+      <c r="E18" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="11"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="11"/>
-      <c r="N18" s="11" t="s">
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="12"/>
+      <c r="L18" s="12"/>
+      <c r="M18" s="12"/>
+      <c r="N18" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="n">
+    <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C19" s="12" t="n">
+      <c r="C19" s="13" t="n">
         <v>46328</v>
       </c>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11" t="s">
+      <c r="D19" s="12"/>
+      <c r="E19" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="11"/>
-      <c r="K19" s="11"/>
-      <c r="L19" s="11"/>
-      <c r="M19" s="11"/>
-      <c r="N19" s="11" t="s">
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="12"/>
+      <c r="M19" s="12"/>
+      <c r="N19" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="n">
+    <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="12" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="C20" s="12" t="n">
+      <c r="C20" s="13" t="n">
         <v>46330</v>
       </c>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11" t="s">
+      <c r="D20" s="12"/>
+      <c r="E20" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="11"/>
-      <c r="K20" s="11"/>
-      <c r="L20" s="11"/>
-      <c r="M20" s="11"/>
-      <c r="N20" s="11" t="s">
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="12"/>
+      <c r="L20" s="12"/>
+      <c r="M20" s="12"/>
+      <c r="N20" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="n">
+    <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="12" t="n">
+      <c r="C21" s="13" t="n">
         <v>46332</v>
       </c>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11" t="s">
+      <c r="D21" s="12"/>
+      <c r="E21" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="11"/>
-      <c r="L21" s="11"/>
-      <c r="M21" s="11"/>
-      <c r="N21" s="11" t="s">
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="12"/>
+      <c r="L21" s="12"/>
+      <c r="M21" s="12"/>
+      <c r="N21" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="n">
+    <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="12" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="C22" s="12" t="n">
+      <c r="C22" s="13" t="n">
         <v>46334</v>
       </c>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11" t="s">
+      <c r="D22" s="12"/>
+      <c r="E22" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="11"/>
-      <c r="J22" s="11"/>
-      <c r="K22" s="11"/>
-      <c r="L22" s="11"/>
-      <c r="M22" s="11"/>
-      <c r="N22" s="11" t="s">
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="12"/>
+      <c r="L22" s="12"/>
+      <c r="M22" s="12"/>
+      <c r="N22" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="n">
+    <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="12" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C23" s="12" t="n">
+      <c r="C23" s="13" t="n">
         <v>46335</v>
       </c>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11" t="s">
+      <c r="D23" s="12"/>
+      <c r="E23" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="11"/>
-      <c r="K23" s="11"/>
-      <c r="L23" s="11"/>
-      <c r="M23" s="11"/>
-      <c r="N23" s="11" t="s">
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="12"/>
+      <c r="L23" s="12"/>
+      <c r="M23" s="12"/>
+      <c r="N23" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="n">
+    <row r="24" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C24" s="6" t="n">
+      <c r="C24" s="7" t="n">
         <v>46337</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="E24" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="F24" s="5" t="s">
+      <c r="F24" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="G24" s="5" t="s">
+      <c r="G24" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="H24" s="5" t="s">
+      <c r="H24" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="I24" s="5" t="s">
+      <c r="I24" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="J24" s="5" t="s">
+      <c r="J24" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="K24" s="7" t="s">
+      <c r="K24" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="L24" s="5" t="s">
+      <c r="L24" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="M24" s="5" t="s">
+      <c r="M24" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="N24" s="5" t="s">
+      <c r="N24" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="n">
+    <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="12" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C25" s="12" t="n">
+      <c r="C25" s="13" t="n">
         <v>46339</v>
       </c>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11" t="s">
+      <c r="D25" s="12"/>
+      <c r="E25" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="11"/>
-      <c r="J25" s="11"/>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11"/>
-      <c r="M25" s="11"/>
-      <c r="N25" s="11" t="s">
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
+      <c r="I25" s="12"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="12"/>
+      <c r="L25" s="12"/>
+      <c r="M25" s="12"/>
+      <c r="N25" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11" t="n">
+    <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="12" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="C26" s="12" t="n">
+      <c r="C26" s="13" t="n">
         <v>46341</v>
       </c>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11" t="s">
+      <c r="D26" s="12"/>
+      <c r="E26" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F26" s="11"/>
-      <c r="G26" s="11"/>
-      <c r="H26" s="11"/>
-      <c r="I26" s="11"/>
-      <c r="J26" s="11"/>
-      <c r="K26" s="11"/>
-      <c r="L26" s="11"/>
-      <c r="M26" s="11"/>
-      <c r="N26" s="11" t="s">
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="12"/>
+      <c r="J26" s="12"/>
+      <c r="K26" s="12"/>
+      <c r="L26" s="12"/>
+      <c r="M26" s="12"/>
+      <c r="N26" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="n">
+    <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="12" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C27" s="12" t="n">
+      <c r="C27" s="13" t="n">
         <v>46342</v>
       </c>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11" t="s">
+      <c r="D27" s="12"/>
+      <c r="E27" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F27" s="11"/>
-      <c r="G27" s="11"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="11"/>
-      <c r="J27" s="11"/>
-      <c r="K27" s="11"/>
-      <c r="L27" s="11"/>
-      <c r="M27" s="11"/>
-      <c r="N27" s="11" t="s">
+      <c r="F27" s="12"/>
+      <c r="G27" s="12"/>
+      <c r="H27" s="12"/>
+      <c r="I27" s="12"/>
+      <c r="J27" s="12"/>
+      <c r="K27" s="12"/>
+      <c r="L27" s="12"/>
+      <c r="M27" s="12"/>
+      <c r="N27" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="11" t="n">
+    <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="12" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="11" t="s">
+      <c r="B28" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="C28" s="12" t="n">
+      <c r="C28" s="13" t="n">
         <v>46344</v>
       </c>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11" t="s">
+      <c r="D28" s="12"/>
+      <c r="E28" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F28" s="11"/>
-      <c r="G28" s="11"/>
-      <c r="H28" s="11"/>
-      <c r="I28" s="11"/>
-      <c r="J28" s="11"/>
-      <c r="K28" s="11"/>
-      <c r="L28" s="11"/>
-      <c r="M28" s="11"/>
-      <c r="N28" s="11" t="s">
+      <c r="F28" s="12"/>
+      <c r="G28" s="12"/>
+      <c r="H28" s="12"/>
+      <c r="I28" s="12"/>
+      <c r="J28" s="12"/>
+      <c r="K28" s="12"/>
+      <c r="L28" s="12"/>
+      <c r="M28" s="12"/>
+      <c r="N28" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="11" t="n">
+    <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="12" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="11" t="s">
+      <c r="B29" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C29" s="12" t="n">
+      <c r="C29" s="13" t="n">
         <v>46346</v>
       </c>
-      <c r="D29" s="11"/>
-      <c r="E29" s="11" t="s">
+      <c r="D29" s="12"/>
+      <c r="E29" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F29" s="11"/>
-      <c r="G29" s="11"/>
-      <c r="H29" s="11"/>
-      <c r="I29" s="11"/>
-      <c r="J29" s="11"/>
-      <c r="K29" s="11"/>
-      <c r="L29" s="11"/>
-      <c r="M29" s="11"/>
-      <c r="N29" s="11" t="s">
+      <c r="F29" s="12"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
+      <c r="I29" s="12"/>
+      <c r="J29" s="12"/>
+      <c r="K29" s="12"/>
+      <c r="L29" s="12"/>
+      <c r="M29" s="12"/>
+      <c r="N29" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5" t="n">
+    <row r="30" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="C30" s="6" t="n">
+      <c r="C30" s="7" t="n">
         <v>46348</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="D30" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="E30" s="5" t="s">
+      <c r="E30" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="F30" s="5" t="s">
+      <c r="F30" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="G30" s="5" t="s">
+      <c r="G30" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="H30" s="5" t="s">
+      <c r="H30" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="I30" s="5" t="s">
+      <c r="I30" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="J30" s="5" t="s">
+      <c r="J30" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="K30" s="7" t="s">
+      <c r="K30" s="8" t="s">
         <v>162</v>
       </c>
-      <c r="L30" s="5" t="s">
+      <c r="L30" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="M30" s="5" t="s">
+      <c r="M30" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="N30" s="5" t="s">
+      <c r="N30" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11" t="n">
+    <row r="31" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="12" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C31" s="12" t="n">
+      <c r="C31" s="13" t="n">
         <v>46349</v>
       </c>
-      <c r="D31" s="11"/>
-      <c r="E31" s="11" t="s">
+      <c r="D31" s="12"/>
+      <c r="E31" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F31" s="11"/>
-      <c r="G31" s="11"/>
-      <c r="H31" s="11"/>
-      <c r="I31" s="11"/>
-      <c r="J31" s="11"/>
-      <c r="K31" s="11"/>
-      <c r="L31" s="11"/>
-      <c r="M31" s="11"/>
-      <c r="N31" s="11" t="s">
+      <c r="F31" s="12"/>
+      <c r="G31" s="12"/>
+      <c r="H31" s="12"/>
+      <c r="I31" s="12"/>
+      <c r="J31" s="12"/>
+      <c r="K31" s="12"/>
+      <c r="L31" s="12"/>
+      <c r="M31" s="12"/>
+      <c r="N31" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="11" t="n">
+    <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="12" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="C32" s="12" t="n">
+      <c r="C32" s="13" t="n">
         <v>46351</v>
       </c>
-      <c r="D32" s="11"/>
-      <c r="E32" s="11" t="s">
+      <c r="D32" s="12"/>
+      <c r="E32" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F32" s="11"/>
-      <c r="G32" s="11"/>
-      <c r="H32" s="11"/>
-      <c r="I32" s="11"/>
-      <c r="J32" s="11"/>
-      <c r="K32" s="11"/>
-      <c r="L32" s="11"/>
-      <c r="M32" s="11"/>
-      <c r="N32" s="11" t="s">
+      <c r="F32" s="12"/>
+      <c r="G32" s="12"/>
+      <c r="H32" s="12"/>
+      <c r="I32" s="12"/>
+      <c r="J32" s="12"/>
+      <c r="K32" s="12"/>
+      <c r="L32" s="12"/>
+      <c r="M32" s="12"/>
+      <c r="N32" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="8" t="n">
+    <row r="33" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="9" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="8" t="s">
+      <c r="B33" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="C33" s="9" t="n">
+      <c r="C33" s="10" t="n">
         <v>46353</v>
       </c>
-      <c r="D33" s="8" t="s">
+      <c r="D33" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="E33" s="8" t="s">
+      <c r="E33" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="F33" s="8" t="s">
+      <c r="F33" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="G33" s="8" t="s">
+      <c r="G33" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="H33" s="8" t="s">
+      <c r="H33" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="I33" s="8" t="s">
+      <c r="I33" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="J33" s="8" t="s">
+      <c r="J33" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="K33" s="10" t="s">
+      <c r="K33" s="11" t="s">
         <v>171</v>
       </c>
-      <c r="L33" s="8" t="s">
+      <c r="L33" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="M33" s="8" t="s">
+      <c r="M33" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="N33" s="8" t="s">
+      <c r="N33" s="9" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="11" t="n">
+    <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="12" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="11" t="s">
+      <c r="B34" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="C34" s="12" t="n">
+      <c r="C34" s="13" t="n">
         <v>46355</v>
       </c>
-      <c r="D34" s="11"/>
-      <c r="E34" s="11" t="s">
+      <c r="D34" s="12"/>
+      <c r="E34" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F34" s="11"/>
-      <c r="G34" s="11"/>
-      <c r="H34" s="11"/>
-      <c r="I34" s="11"/>
-      <c r="J34" s="11"/>
-      <c r="K34" s="11"/>
-      <c r="L34" s="11"/>
-      <c r="M34" s="11"/>
-      <c r="N34" s="11" t="s">
+      <c r="F34" s="12"/>
+      <c r="G34" s="12"/>
+      <c r="H34" s="12"/>
+      <c r="I34" s="12"/>
+      <c r="J34" s="12"/>
+      <c r="K34" s="12"/>
+      <c r="L34" s="12"/>
+      <c r="M34" s="12"/>
+      <c r="N34" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="11" t="n">
+    <row r="35" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="12" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="11" t="s">
+      <c r="B35" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C35" s="12" t="n">
+      <c r="C35" s="13" t="n">
         <v>46356</v>
       </c>
-      <c r="D35" s="11"/>
-      <c r="E35" s="11" t="s">
+      <c r="D35" s="12"/>
+      <c r="E35" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F35" s="11"/>
-      <c r="G35" s="11"/>
-      <c r="H35" s="11"/>
-      <c r="I35" s="11"/>
-      <c r="J35" s="11"/>
-      <c r="K35" s="11"/>
-      <c r="L35" s="11"/>
-      <c r="M35" s="11"/>
-      <c r="N35" s="11" t="s">
+      <c r="F35" s="12"/>
+      <c r="G35" s="12"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="12"/>
+      <c r="J35" s="12"/>
+      <c r="K35" s="12"/>
+      <c r="L35" s="12"/>
+      <c r="M35" s="12"/>
+      <c r="N35" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="11" t="n">
+    <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="12" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="11" t="s">
+      <c r="B36" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="C36" s="12" t="n">
+      <c r="C36" s="13" t="n">
         <v>46358</v>
       </c>
-      <c r="D36" s="11"/>
-      <c r="E36" s="11" t="s">
+      <c r="D36" s="12"/>
+      <c r="E36" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F36" s="11"/>
-      <c r="G36" s="11"/>
-      <c r="H36" s="11"/>
-      <c r="I36" s="11"/>
-      <c r="J36" s="11"/>
-      <c r="K36" s="11"/>
-      <c r="L36" s="11"/>
-      <c r="M36" s="11"/>
-      <c r="N36" s="11" t="s">
+      <c r="F36" s="12"/>
+      <c r="G36" s="12"/>
+      <c r="H36" s="12"/>
+      <c r="I36" s="12"/>
+      <c r="J36" s="12"/>
+      <c r="K36" s="12"/>
+      <c r="L36" s="12"/>
+      <c r="M36" s="12"/>
+      <c r="N36" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="11" t="n">
+    <row r="37" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="12" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="11" t="s">
+      <c r="B37" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C37" s="12" t="n">
+      <c r="C37" s="13" t="n">
         <v>46360</v>
       </c>
-      <c r="D37" s="11"/>
-      <c r="E37" s="11" t="s">
+      <c r="D37" s="12"/>
+      <c r="E37" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F37" s="11"/>
-      <c r="G37" s="11"/>
-      <c r="H37" s="11"/>
-      <c r="I37" s="11"/>
-      <c r="J37" s="11"/>
-      <c r="K37" s="11"/>
-      <c r="L37" s="11"/>
-      <c r="M37" s="11"/>
-      <c r="N37" s="11" t="s">
+      <c r="F37" s="12"/>
+      <c r="G37" s="12"/>
+      <c r="H37" s="12"/>
+      <c r="I37" s="12"/>
+      <c r="J37" s="12"/>
+      <c r="K37" s="12"/>
+      <c r="L37" s="12"/>
+      <c r="M37" s="12"/>
+      <c r="N37" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="11" t="n">
+    <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="12" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="11" t="s">
+      <c r="B38" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="C38" s="12" t="n">
+      <c r="C38" s="13" t="n">
         <v>46362</v>
       </c>
-      <c r="D38" s="11"/>
-      <c r="E38" s="11" t="s">
+      <c r="D38" s="12"/>
+      <c r="E38" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F38" s="11"/>
-      <c r="G38" s="11"/>
-      <c r="H38" s="11"/>
-      <c r="I38" s="11"/>
-      <c r="J38" s="11"/>
-      <c r="K38" s="11"/>
-      <c r="L38" s="11"/>
-      <c r="M38" s="11"/>
-      <c r="N38" s="11" t="s">
+      <c r="F38" s="12"/>
+      <c r="G38" s="12"/>
+      <c r="H38" s="12"/>
+      <c r="I38" s="12"/>
+      <c r="J38" s="12"/>
+      <c r="K38" s="12"/>
+      <c r="L38" s="12"/>
+      <c r="M38" s="12"/>
+      <c r="N38" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="11" t="n">
+    <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="12" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="11" t="s">
+      <c r="B39" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C39" s="12" t="n">
+      <c r="C39" s="13" t="n">
         <v>46363</v>
       </c>
-      <c r="D39" s="11"/>
-      <c r="E39" s="11" t="s">
+      <c r="D39" s="12"/>
+      <c r="E39" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F39" s="11"/>
-      <c r="G39" s="11"/>
-      <c r="H39" s="11"/>
-      <c r="I39" s="11"/>
-      <c r="J39" s="11"/>
-      <c r="K39" s="11"/>
-      <c r="L39" s="11"/>
-      <c r="M39" s="11"/>
-      <c r="N39" s="11" t="s">
+      <c r="F39" s="12"/>
+      <c r="G39" s="12"/>
+      <c r="H39" s="12"/>
+      <c r="I39" s="12"/>
+      <c r="J39" s="12"/>
+      <c r="K39" s="12"/>
+      <c r="L39" s="12"/>
+      <c r="M39" s="12"/>
+      <c r="N39" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5" t="n">
+    <row r="40" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="6" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="B40" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C40" s="6" t="n">
+      <c r="C40" s="7" t="n">
         <v>46365</v>
       </c>
-      <c r="D40" s="5" t="s">
+      <c r="D40" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="E40" s="5" t="s">
+      <c r="E40" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="F40" s="5" t="s">
+      <c r="F40" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="G40" s="5" t="s">
+      <c r="G40" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="H40" s="5" t="s">
+      <c r="H40" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="I40" s="5" t="s">
+      <c r="I40" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="J40" s="5" t="s">
+      <c r="J40" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="K40" s="7" t="s">
+      <c r="K40" s="8" t="s">
         <v>179</v>
       </c>
-      <c r="L40" s="5" t="s">
+      <c r="L40" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="M40" s="5" t="s">
+      <c r="M40" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="N40" s="5" t="s">
+      <c r="N40" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="11" t="n">
+    <row r="41" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="12" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="11" t="s">
+      <c r="B41" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C41" s="12" t="n">
+      <c r="C41" s="13" t="n">
         <v>46367</v>
       </c>
-      <c r="D41" s="11"/>
-      <c r="E41" s="11" t="s">
+      <c r="D41" s="12"/>
+      <c r="E41" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F41" s="11"/>
-      <c r="G41" s="11"/>
-      <c r="H41" s="11"/>
-      <c r="I41" s="11"/>
-      <c r="J41" s="11"/>
-      <c r="K41" s="11"/>
-      <c r="L41" s="11"/>
-      <c r="M41" s="11"/>
-      <c r="N41" s="11" t="s">
+      <c r="F41" s="12"/>
+      <c r="G41" s="12"/>
+      <c r="H41" s="12"/>
+      <c r="I41" s="12"/>
+      <c r="J41" s="12"/>
+      <c r="K41" s="12"/>
+      <c r="L41" s="12"/>
+      <c r="M41" s="12"/>
+      <c r="N41" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="11" t="n">
+    <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="12" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="11" t="s">
+      <c r="B42" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="C42" s="12" t="n">
+      <c r="C42" s="13" t="n">
         <v>46369</v>
       </c>
-      <c r="D42" s="11"/>
-      <c r="E42" s="11" t="s">
+      <c r="D42" s="12"/>
+      <c r="E42" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F42" s="11"/>
-      <c r="G42" s="11"/>
-      <c r="H42" s="11"/>
-      <c r="I42" s="11"/>
-      <c r="J42" s="11"/>
-      <c r="K42" s="11"/>
-      <c r="L42" s="11"/>
-      <c r="M42" s="11"/>
-      <c r="N42" s="11" t="s">
+      <c r="F42" s="12"/>
+      <c r="G42" s="12"/>
+      <c r="H42" s="12"/>
+      <c r="I42" s="12"/>
+      <c r="J42" s="12"/>
+      <c r="K42" s="12"/>
+      <c r="L42" s="12"/>
+      <c r="M42" s="12"/>
+      <c r="N42" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="11" t="n">
+    <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="12" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="11" t="s">
+      <c r="B43" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C43" s="12" t="n">
+      <c r="C43" s="13" t="n">
         <v>46370</v>
       </c>
-      <c r="D43" s="11"/>
-      <c r="E43" s="11" t="s">
+      <c r="D43" s="12"/>
+      <c r="E43" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F43" s="11"/>
-      <c r="G43" s="11"/>
-      <c r="H43" s="11"/>
-      <c r="I43" s="11"/>
-      <c r="J43" s="11"/>
-      <c r="K43" s="11"/>
-      <c r="L43" s="11"/>
-      <c r="M43" s="11"/>
-      <c r="N43" s="11" t="s">
+      <c r="F43" s="12"/>
+      <c r="G43" s="12"/>
+      <c r="H43" s="12"/>
+      <c r="I43" s="12"/>
+      <c r="J43" s="12"/>
+      <c r="K43" s="12"/>
+      <c r="L43" s="12"/>
+      <c r="M43" s="12"/>
+      <c r="N43" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="8" t="n">
+    <row r="44" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="9" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="8" t="s">
+      <c r="B44" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="C44" s="9" t="n">
+      <c r="C44" s="10" t="n">
         <v>46372</v>
       </c>
-      <c r="D44" s="8" t="s">
+      <c r="D44" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="E44" s="8" t="s">
+      <c r="E44" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="F44" s="8" t="s">
+      <c r="F44" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="G44" s="8" t="s">
+      <c r="G44" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="H44" s="8" t="s">
+      <c r="H44" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="I44" s="8" t="s">
+      <c r="I44" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="J44" s="8" t="s">
+      <c r="J44" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="K44" s="10" t="s">
+      <c r="K44" s="11" t="s">
         <v>187</v>
       </c>
-      <c r="L44" s="8" t="s">
+      <c r="L44" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="M44" s="8" t="s">
+      <c r="M44" s="9" t="s">
         <v>189</v>
       </c>
-      <c r="N44" s="8" t="s">
+      <c r="N44" s="9" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="11" t="n">
+    <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="12" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="11" t="s">
+      <c r="B45" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C45" s="12" t="n">
+      <c r="C45" s="13" t="n">
         <v>46374</v>
       </c>
-      <c r="D45" s="11"/>
-      <c r="E45" s="11" t="s">
+      <c r="D45" s="12"/>
+      <c r="E45" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F45" s="11"/>
-      <c r="G45" s="11"/>
-      <c r="H45" s="11"/>
-      <c r="I45" s="11"/>
-      <c r="J45" s="11"/>
-      <c r="K45" s="11"/>
-      <c r="L45" s="11"/>
-      <c r="M45" s="11"/>
-      <c r="N45" s="11" t="s">
+      <c r="F45" s="12"/>
+      <c r="G45" s="12"/>
+      <c r="H45" s="12"/>
+      <c r="I45" s="12"/>
+      <c r="J45" s="12"/>
+      <c r="K45" s="12"/>
+      <c r="L45" s="12"/>
+      <c r="M45" s="12"/>
+      <c r="N45" s="12" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="11" t="n">
+    <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="12" t="n">
         <v>45</v>
       </c>
-      <c r="B46" s="11" t="s">
+      <c r="B46" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="C46" s="12" t="n">
+      <c r="C46" s="13" t="n">
         <v>46376</v>
       </c>
-      <c r="D46" s="11"/>
-      <c r="E46" s="11" t="s">
+      <c r="D46" s="12"/>
+      <c r="E46" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="F46" s="11"/>
-      <c r="G46" s="11"/>
-      <c r="H46" s="11"/>
-      <c r="I46" s="11"/>
-      <c r="J46" s="11"/>
-      <c r="K46" s="11"/>
-      <c r="L46" s="11"/>
-      <c r="M46" s="11"/>
-      <c r="N46" s="11" t="s">
+      <c r="F46" s="12"/>
+      <c r="G46" s="12"/>
+      <c r="H46" s="12"/>
+      <c r="I46" s="12"/>
+      <c r="J46" s="12"/>
+      <c r="K46" s="12"/>
+      <c r="L46" s="12"/>
+      <c r="M46" s="12"/>
+      <c r="N46" s="12" t="s">
         <v>146</v>
       </c>
     </row>
@@ -2908,50 +2913,50 @@
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="14" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="14" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="15" t="s">
         <v>192</v>
       </c>
-      <c r="B2" s="14" t="n">
+      <c r="B2" s="15" t="n">
         <f aca="false">COUNTA('Lịch đăng'!$A$2:$A$46)</f>
         <v>45</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="14" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="14" t="n">
+      <c r="B3" s="15" t="n">
         <f aca="false">COUNTIF('Lịch đăng'!$N$2:$N$46,"Đã đăng")</f>
         <v>3</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="15" t="s">
         <v>193</v>
       </c>
-      <c r="B4" s="14" t="n">
+      <c r="B4" s="15" t="n">
         <f aca="false">COUNTIF('Lịch đăng'!$N$2:$N$46,"Cần chủ đề")</f>
         <v>25</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="15" t="s">
         <v>194</v>
       </c>
-      <c r="B5" s="14" t="n">
+      <c r="B5" s="15" t="n">
         <f aca="false">B2-B3-B4</f>
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
Bỏ video SEO vì trùng ý video AIO đã đăng, thêm video bỏ giỏ hàng 10/10
Lịch mới: 08/10 nhắn tin trước khi mua, 09/10 khách hỏi AI, 10/10 khách
bỏ giỏ hàng. Thêm quy tắc không trùng góc nhìn và số liệu với video đã đăng.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dpu4oyZ8FYSVLE8FrdnGTC
</commit_message>
<xml_diff>
--- a/video/plan/lich-noi-dung-tiktok.xlsx
+++ b/video/plan/lich-noi-dung-tiktok.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="189">
   <si>
     <t xml:space="preserve">Lịch nội dung TikTok Adtek</t>
   </si>
@@ -158,53 +158,6 @@
   </si>
   <si>
     <t xml:space="preserve">Thứ Năm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đứng top 1 Google vẫn mất khách</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đứng top 1 Google, vì sao vẫn mất hơn nửa lượt bấm?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• CTR trang top 1 thấp hơn 58% khi có AI Overview (300,000 từ khóa, 12/2023 so với 12/2025); lần đo 04/2025 là 34.5%
-• 37.9% URL được trích nằm trong top 10, giảm từ 76.1% (07/2025); 31% nằm ngoài top 100
-• Dự đoán giảm 25% (02/2024); khảo sát 2026: chỉ ~1/3 người dùng thấy chatbot ngang công cụ tìm kiếm; hơn 2/3 vẫn đọc tiếp sau AI Overview</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Ahrefs, "AI Overviews Reduce Clicks by 58%", 05/2026
-• Ahrefs, "38% of AI Overview Citations Pull From The Top 10", 02/03/2026
-• Gartner, 19/02/2024 và 20/01/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://ahrefs.com/blog/ai-overviews-reduce-clicks-update/
-https://ahrefs.com/blog/ai-overview-citations-top-10/
-https://www.gartner.com/en/newsroom/press-releases/2024-02-19-gartner-predicts-search-engine-volume-will-drop-25-percent-by-2026-due-to-ai-chatbots-and-other-virtual-agents</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Chưa mở được trang gốc (mạng chặn), đối chiếu qua Business Wire
-• Chưa mở được trang gốc (mạng chặn), đối chiếu qua đoạn trích ahrefs.com
-• Chưa mở được trang gốc (mạng chặn), đối chiếu qua Demand Gen Report</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Ahrefs lưu ý một phần chênh lệch do công cụ đo tốt hơn, nên nói rõ
-• Khảo sát 377 người Mỹ, mẫu nhỏ
-• Kịch bản scripts/top-1-google-van-mat-khach/1.json; số liệu Pew là của Mỹ, Ahrefs là số quốc tế
-• Giọng v4 chưa huấn luyện; video trên trang hub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">seo 2026; ai overview; seo có còn hiệu quả</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cao</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đã có video</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Sáu</t>
   </si>
   <si>
     <t xml:space="preserve">Performance, Digital</t>
@@ -240,7 +193,13 @@
     <t xml:space="preserve">quảng cáo tin nhắn; zalo oa; chốt đơn inbox</t>
   </si>
   <si>
-    <t xml:space="preserve">Thứ Bảy</t>
+    <t xml:space="preserve">Cao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đã có video</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Sáu</t>
   </si>
   <si>
     <t xml:space="preserve">Khách hàng của bạn đang hỏi AI</t>
@@ -281,19 +240,7 @@
     <t xml:space="preserve">chatgpt; ai mode; người việt dùng ai</t>
   </si>
   <si>
-    <t xml:space="preserve">Chủ nhật</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Slot trống: chủ đề trend Claude tự chọn khi viết kịch bản thứ Bảy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cần chủ đề</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Hai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Ba</t>
+    <t xml:space="preserve">Thứ Bảy</t>
   </si>
   <si>
     <t xml:space="preserve">Growth Marketing</t>
@@ -326,13 +273,27 @@
   </si>
   <si>
     <t xml:space="preserve">• Tỷ lệ từng nguyên nhân khác nhau theo năm, dùng 70.22% làm số chính
-• Dữ liệu 2021, ghi rõ năm</t>
+• Dữ liệu 2021, ghi rõ năm
+• Kịch bản scripts/khach-bo-gio-hang/1.json; dùng thêm số liệu Việt Nam của Milieu Insight (09/2025), chưa mở được trang gốc (mạng chặn), đối chiếu qua PR Newswire, Marketech APAC
+• Giọng v4 chưa huấn luyện; video trên trang hub</t>
   </si>
   <si>
     <t xml:space="preserve">bỏ giỏ hàng; tăng tỷ lệ chuyển đổi; cá nhân hóa</t>
   </si>
   <si>
-    <t xml:space="preserve">Ý tưởng</t>
+    <t xml:space="preserve">Chủ nhật</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slot trống: chủ đề trend Claude tự chọn khi viết kịch bản thứ Bảy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cần chủ đề</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Hai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Ba</t>
   </si>
   <si>
     <t xml:space="preserve">Performance</t>
@@ -375,6 +336,9 @@
   </si>
   <si>
     <t xml:space="preserve">quảng cáo facebook 2026; advantage+; ai max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ý tưởng</t>
   </si>
   <si>
     <t xml:space="preserve">Livestream bán hàng: người mua tin ai?</t>
@@ -1545,7 +1509,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="n">
         <v>5</v>
       </c>
@@ -1589,7 +1553,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="n">
         <v>6</v>
       </c>
@@ -1600,31 +1564,31 @@
         <v>46304</v>
       </c>
       <c r="D7" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="F7" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="G7" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="H7" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="I7" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="J7" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="J7" s="6" t="s">
+      <c r="K7" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="K7" s="8" t="s">
+      <c r="L7" s="6" t="s">
         <v>63</v>
-      </c>
-      <c r="L7" s="6" t="s">
-        <v>64</v>
       </c>
       <c r="M7" s="6" t="s">
         <v>53</v>
@@ -1638,13 +1602,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C8" s="7" t="n">
         <v>46305</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>27</v>
+        <v>65</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>66</v>
@@ -1729,48 +1693,30 @@
         <v>76</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="n">
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="10" t="n">
         <v>46308</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="J11" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="K11" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="L11" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="M11" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="N11" s="6" t="s">
-        <v>88</v>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="9"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="9" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="135.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1784,31 +1730,31 @@
         <v>46309</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="K12" s="8" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="M12" s="6" t="s">
         <v>53</v>
@@ -1828,31 +1774,31 @@
         <v>46310</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="K13" s="8" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="M13" s="6" t="s">
         <v>53</v>
@@ -1872,34 +1818,34 @@
         <v>46311</v>
       </c>
       <c r="D14" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="H14" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="I14" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="J14" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="K14" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="L14" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="M14" s="11" t="s">
         <v>106</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="G14" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="H14" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="I14" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="J14" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="K14" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="L14" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="M14" s="11" t="s">
-        <v>115</v>
       </c>
       <c r="N14" s="11" t="s">
         <v>88</v>
@@ -1910,40 +1856,40 @@
         <v>14</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C15" s="12" t="n">
         <v>46312</v>
       </c>
       <c r="D15" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="H15" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="J15" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="K15" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="L15" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="M15" s="11" t="s">
         <v>106</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="F15" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="G15" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="H15" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="I15" s="11" t="s">
-        <v>120</v>
-      </c>
-      <c r="J15" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="K15" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="L15" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="M15" s="11" t="s">
-        <v>115</v>
       </c>
       <c r="N15" s="11" t="s">
         <v>88</v>
@@ -1960,31 +1906,31 @@
         <v>46313</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="K16" s="13" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="L16" s="11" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="M16" s="11" t="s">
         <v>53</v>
@@ -2004,31 +1950,31 @@
         <v>46314</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="J17" s="11" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="K17" s="13" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="L17" s="11" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="M17" s="11" t="s">
         <v>53</v>
@@ -2051,31 +1997,31 @@
         <v>33</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="K18" s="13" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="L18" s="11" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="M18" s="11" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="N18" s="11" t="s">
         <v>88</v>
@@ -2164,7 +2110,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C22" s="10" t="n">
         <v>46319</v>
@@ -2346,7 +2292,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C29" s="10" t="n">
         <v>46326</v>
@@ -2528,7 +2474,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C36" s="10" t="n">
         <v>46333</v>
@@ -2638,31 +2584,31 @@
         <v>46337</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="I40" s="6" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="J40" s="6" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="K40" s="8" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="L40" s="6" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="M40" s="6" t="s">
         <v>53</v>
@@ -2728,7 +2674,7 @@
         <v>42</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C43" s="10" t="n">
         <v>46340</v>
@@ -2910,7 +2856,7 @@
         <v>49</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C50" s="10" t="n">
         <v>46347</v>
@@ -2942,34 +2888,34 @@
         <v>46348</v>
       </c>
       <c r="D51" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="E51" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="F51" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="G51" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="H51" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="I51" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="J51" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="K51" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="L51" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="M51" s="6" t="s">
         <v>158</v>
-      </c>
-      <c r="E51" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="F51" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="G51" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="H51" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="I51" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="J51" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="K51" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="L51" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="M51" s="6" t="s">
-        <v>167</v>
       </c>
       <c r="N51" s="6" t="s">
         <v>88</v>
@@ -3090,34 +3036,34 @@
         <v>46353</v>
       </c>
       <c r="D56" s="11" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="E56" s="11" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="G56" s="11" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H56" s="11" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="J56" s="11" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="K56" s="13" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="L56" s="11" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="M56" s="11" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="N56" s="11" t="s">
         <v>88</v>
@@ -3128,7 +3074,7 @@
         <v>56</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C57" s="10" t="n">
         <v>46354</v>
@@ -3310,7 +3256,7 @@
         <v>63</v>
       </c>
       <c r="B64" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C64" s="10" t="n">
         <v>46361</v>
@@ -3420,31 +3366,31 @@
         <v>46365</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="I68" s="6" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="J68" s="6" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="K68" s="8" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="L68" s="6" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="M68" s="6" t="s">
         <v>53</v>
@@ -3510,7 +3456,7 @@
         <v>70</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C71" s="10" t="n">
         <v>46368</v>
@@ -3620,34 +3566,34 @@
         <v>46372</v>
       </c>
       <c r="D75" s="11" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="E75" s="11" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="F75" s="11" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="G75" s="11" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="H75" s="11" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="I75" s="11" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="J75" s="11" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="K75" s="13" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="L75" s="11" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="M75" s="11" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="N75" s="11" t="s">
         <v>88</v>
@@ -3710,7 +3656,7 @@
         <v>77</v>
       </c>
       <c r="B78" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C78" s="10" t="n">
         <v>46375</v>
@@ -3790,15 +3736,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="B2" s="15" t="n">
         <f aca="false">COUNTA('Lịch đăng'!$A$2:$A$79)</f>
@@ -3816,20 +3762,20 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="B4" s="15" t="n">
         <f aca="false">COUNTIF('Lịch đăng'!$N$2:$N$79,"Cần chủ đề")</f>
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="B5" s="15" t="n">
         <f aca="false">B2-B3-B4</f>
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ưu tiên số liệu Việt Nam: viết lại video 09/10 và 10/10
Thay số toàn cầu bằng số Việt Nam đã kiểm tra trên trang gốc (Vietnam Report
08/2026, e-Conomy SEA 2025 trang 143, Milieu Insight). Sửa Thái Lan 76% (trước
ghi 74%) và ghi chú 1/3 người mua ngừng mua theo đúng nguyên văn. Thêm quy tắc
thứ tự ưu tiên Việt Nam, Đông Nam Á, rồi mới đến toàn cầu.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dpu4oyZ8FYSVLE8FrdnGTC
</commit_message>
<xml_diff>
--- a/video/plan/lich-noi-dung-tiktok.xlsx
+++ b/video/plan/lich-noi-dung-tiktok.xlsx
@@ -206,31 +206,23 @@
     <t xml:space="preserve">Khách hàng của bạn đang hỏi AI</t>
   </si>
   <si>
-    <t xml:space="preserve">Mỗi tuần 900 triệu người hỏi ChatGPT. Có ai được nó gợi ý tên thương hiệu của bạn chưa?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• 900 triệu người dùng hằng tuần (từ 800 triệu, 10/2025); hơn 50 triệu người trả phí
-• AI Mode vượt 1 tỷ người dùng hằng tháng; AI Overviews hơn 2.5 tỷ; AI Mode có tiếng Việt từ 07/10/2025
-• 81% tương tác với AI hằng ngày, cao nhất Đông Nam Á (Indonesia 80%, Thái Lan 74%); 96% sẵn sàng chia sẻ dữ liệu với AI agent
-• Google Lens hơn 25 tỷ lượt tìm mỗi tháng (2024: ~20 tỷ, 1/4 có ý định mua hàng)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• OpenAI, "Scaling AI for everyone", 27/02/2026
-• Google, I/O 2026 (Sundar Pichai), 05/2026; Google Search blog, 07/10/2025
-• Google, Temasek, Bain &amp; Company, e-Conomy SEA 2025, 11/2025
-• Google Việt Nam Blog, 03/2026; Google, 10/2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://openai.com/index/scaling-ai-for-everyone/
-https://blog.google/products/search/ai-mode-expands-languages-locations/
-https://economysea.withgoogle.com/
-https://vietnamese.googleblog.com/2026/03/ai-ang-thay-oi-cach-nguoi-tieu-dung-tim.html</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Chưa mở được trang gốc (mạng chặn), đối chiếu qua TechCrunch
-• Chưa mở được trang gốc (mạng chặn), đối chiếu qua Engadget
-• Chưa mở được trang gốc (mạng chặn), đối chiếu qua Việt Nam News, VnEconomy
-• Chưa mở được trang gốc (mạng chặn), đối chiếu qua Advertising Vietnam</t>
+    <t xml:space="preserve">Khi khách hỏi AI nên mua gì, thương hiệu của bạn có được nhắc tên không?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• 78.4% người tiêu dùng Gen Y, Gen Z đã dùng AI khi mua sắm; dùng để tìm hiểu sản phẩm 44.4%, gợi ý 23.5%, so sánh 19.8%
+• 81% người Việt tương tác với AI mỗi ngày (Indonesia 80%, Thái Lan 76%, Singapore 65%); 42% lo bảo mật khi để AI làm thay (Đông Nam Á 50%); 96% sẵn sàng chia sẻ dữ liệu với AI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Vietnam Report, khảo sát người tiêu dùng ngành bán lẻ, 08/2026
+• Google, Temasek, Bain &amp; Company, e-Conomy SEA 2025, trang 143 (khảo sát Google và Milieu, 09/2025, 7,200 người)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://vietnamreport.net.vn/Top-10-Cong-ty-uy-tin-nganh-Ban-le-nam-2026-12576-1006.html
+https://services.google.com/fh/files/misc/e_conomy_sea_2025_report_combined.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Đã mở trang gốc, khớp số liệu (08/10/2026)
+• Đã mở báo cáo gốc; Thái Lan là 76% (bản trước ghi 74% là sai)</t>
   </si>
   <si>
     <t xml:space="preserve">• Số người dùng là toàn cầu
@@ -250,27 +242,24 @@
     <t xml:space="preserve">Khách bỏ đi ở phút cuối</t>
   </si>
   <si>
-    <t xml:space="preserve">Cứ 10 người bỏ hàng vào giỏ, bao nhiêu người thật sự thanh toán?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Tỷ lệ bỏ giỏ trung bình 70.22% (50 nghiên cứu); lý do số 1 là phí phát sinh; tối ưu bước thanh toán tăng chuyển đổi tới 35.26%
-• 71% kỳ vọng được cá nhân hóa; 76% bực khi không được; doanh nghiệp tăng trưởng nhanh có doanh thu từ cá nhân hóa cao hơn 40%
-• 88% người tiêu dùng có xu hướng mua hơn khi được cá nhân hóa theo thời gian thực; chỉ 44% thương hiệu làm được; khảo sát 7,600 người, 18 quốc gia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Baymard Institute, Cart Abandonment Rate Statistics, cập nhật 09/2025
-• McKinsey &amp; Company, Next in Personalization, 11/2021
-• Twilio, State of Customer Engagement Report 2025, 03/06/2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://baymard.com/lists/cart-abandonment-rate
-https://www.mckinsey.com/capabilities/growth-marketing-and-sales/our-insights/the-value-of-getting-personalization-right-or-wrong-is-multiplying
-https://www.twilio.com/en-us/press/releases/socer-2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Chưa mở được trang gốc (mạng chặn), đối chiếu qua eMarketer
-• Chưa mở được trang gốc (mạng chặn), đối chiếu qua đoạn trích mckinsey.com
-• Chưa mở được trang gốc (mạng chặn), đối chiếu qua investors.twilio.com</t>
+    <t xml:space="preserve">Vì sao khách bỏ hàng vào giỏ rồi lại không thanh toán?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• 89.5% so giá nhiều nơi trước khi mua; 39.5% hoãn mua chờ khuyến mãi
+• 1/2 bỏ giỏ khi gặp phí phát sinh; 49% bỏ nếu shop chưa có đánh giá; 46% nếu đổi trả không rõ; 53% coi trọng giao đúng hẹn hơn phí ship rẻ (45%); 7/10 sẵn sàng chi nhiều hơn cho shop dịch vụ đáng tin; 1/3 ngừng mua sau trải nghiệm tệ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Vietnam Report, khảo sát người tiêu dùng ngành bán lẻ, 08/2026
+• Milieu Insight, Vietnam's online shoppers demand speed and reliability in 2025, 09/2025
+• Baymard Institute (số Mỹ, chỉ trong phần Làm gì ngay); Klaviyo 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://vietnamreport.net.vn/Top-10-Cong-ty-uy-tin-nganh-Ban-le-nam-2026-12576-1006.html
+https://www.mili.eu/vn/insights/vietnams-online-shoppers-demand-speed-and-reliability-in-2025
+https://baymard.com/lists/cart-abandonment-rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Đã mở trang gốc, khớp số liệu (08/10/2026)</t>
   </si>
   <si>
     <t xml:space="preserve">• Tỷ lệ từng nguyên nhân khác nhau theo năm, dùng 70.22% làm số chính

</xml_diff>

<commit_message>
Mở đầu hiện sẵn hook, ảnh bìa, âm thanh, cảnh đố số liệu và phá hiểu lầm
- Cảnh đầu hiện ở trạng thái cuối của hiệu ứng, khung đầu đã có con số.
- Ảnh bìa riêng (trường cover, out/<id>-cover.png), âm thanh chuyển cảnh và
  khi số hiện (public/sfx).
- Cảnh mới quiz (đố số liệu, lật đáp án) và myth (đóng dấu SAI); follow có
  câu hỏi kêu gọi bình luận.
- Video mẫu kiểu đố số liệu cho 10/10. Cập nhật lịch: 2 video bản cũ đã đăng
  08/10, video nhắn tin dời sang 09/10.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dpu4oyZ8FYSVLE8FrdnGTC
</commit_message>
<xml_diff>
--- a/video/plan/lich-noi-dung-tiktok.xlsx
+++ b/video/plan/lich-noi-dung-tiktok.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Tổng quan" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Lịch đăng'!$A$1:$N$79</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Lịch đăng'!$A$1:$N$80</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="197">
   <si>
     <t xml:space="preserve">Lịch nội dung TikTok Adtek</t>
   </si>
@@ -158,6 +158,72 @@
   </si>
   <si>
     <t xml:space="preserve">Thứ Năm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khách hàng của bạn đang hỏi AI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khi khách hỏi AI nên mua gì, thương hiệu của bạn có được nhắc tên không?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• 78.4% người tiêu dùng Gen Y, Gen Z đã dùng AI khi mua sắm; dùng để tìm hiểu sản phẩm 44.4%, gợi ý 23.5%, so sánh 19.8%
+• 81% người Việt tương tác với AI mỗi ngày (Indonesia 80%, Thái Lan 76%, Singapore 65%); 42% lo bảo mật khi để AI làm thay (Đông Nam Á 50%); 96% sẵn sàng chia sẻ dữ liệu với AI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Vietnam Report, khảo sát người tiêu dùng ngành bán lẻ, 08/2026
+• Google, Temasek, Bain &amp; Company, e-Conomy SEA 2025, trang 143 (khảo sát Google và Milieu, 09/2025, 7,200 người)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://vietnamreport.net.vn/Top-10-Cong-ty-uy-tin-nganh-Ban-le-nam-2026-12576-1006.html
+https://services.google.com/fh/files/misc/e_conomy_sea_2025_report_combined.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Đã mở trang gốc, khớp số liệu (08/10/2026)
+• Đã mở báo cáo gốc; Thái Lan là 76% (bản trước ghi 74% là sai)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Đã đăng ngày 08/10/2026, bản cũ (900 triệu người dùng ChatGPT). Bản viết lại bằng số liệu Việt Nam không dùng vì trùng chủ đề</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chatgpt; ai mode; người việt dùng ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growth Marketing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khách bỏ đi ở phút cuối</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vì sao khách bỏ hàng vào giỏ rồi lại không thanh toán?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• 89.5% so giá nhiều nơi trước khi mua; 39.5% hoãn mua chờ khuyến mãi
+• 1/2 bỏ giỏ khi gặp phí phát sinh; 49% bỏ nếu shop chưa có đánh giá; 46% nếu đổi trả không rõ; 53% coi trọng giao đúng hẹn hơn phí ship rẻ (45%); 7/10 sẵn sàng chi nhiều hơn cho shop dịch vụ đáng tin; 1/3 ngừng mua sau trải nghiệm tệ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Vietnam Report, khảo sát người tiêu dùng ngành bán lẻ, 08/2026
+• Milieu Insight, Vietnam's online shoppers demand speed and reliability in 2025, 09/2025
+• Baymard Institute (số Mỹ, chỉ trong phần Làm gì ngay); Klaviyo 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://vietnamreport.net.vn/Top-10-Cong-ty-uy-tin-nganh-Ban-le-nam-2026-12576-1006.html
+https://www.mili.eu/vn/insights/vietnams-online-shoppers-demand-speed-and-reliability-in-2025
+https://baymard.com/lists/cart-abandonment-rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Đã mở trang gốc, khớp số liệu (08/10/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Đã đăng ngày 08/10/2026, bản cũ (7/10 giỏ hàng, số Baymard). Bản viết lại bằng số liệu Việt Nam không dùng vì trùng chủ đề</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bỏ giỏ hàng; tăng tỷ lệ chuyển đổi; cá nhân hóa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Sáu</t>
   </si>
   <si>
     <t xml:space="preserve">Performance, Digital</t>
@@ -188,87 +254,44 @@
     <t xml:space="preserve">• Chưa có URL trang gốc của Meta, cần tìm trước khi dựng
 • Doanh nghiệp tự công bố
 • Giọng v4 chưa huấn luyện; video trên trang hub
-• Đã nhắc</t>
+• Nằm trong Drafts của TikTok, dời sang 09/10</t>
   </si>
   <si>
     <t xml:space="preserve">quảng cáo tin nhắn; zalo oa; chốt đơn inbox</t>
   </si>
   <si>
-    <t xml:space="preserve">Cao</t>
-  </si>
-  <si>
     <t xml:space="preserve">Đã có video</t>
   </si>
   <si>
-    <t xml:space="preserve">Thứ Sáu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Khách hàng của bạn đang hỏi AI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Khi khách hỏi AI nên mua gì, thương hiệu của bạn có được nhắc tên không?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• 78.4% người tiêu dùng Gen Y, Gen Z đã dùng AI khi mua sắm; dùng để tìm hiểu sản phẩm 44.4%, gợi ý 23.5%, so sánh 19.8%
-• 81% người Việt tương tác với AI mỗi ngày (Indonesia 80%, Thái Lan 76%, Singapore 65%); 42% lo bảo mật khi để AI làm thay (Đông Nam Á 50%); 96% sẵn sàng chia sẻ dữ liệu với AI</t>
+    <t xml:space="preserve">Thứ Bảy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growth, Performance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khách so giá, chờ sale (đố số liệu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đoán thử: bao nhiêu % người Việt so giá ở nhiều nơi trước khi mua?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• 89.5% so giá nhiều nơi trước khi mua; 39.5% hoãn mua chờ khuyến mãi
+• 65% mua online mỗi tuần (Đông Nam Á 50%); lý do mua: giảm giá 64%, ship rẻ 55%, nhiều lựa chọn 52% (khu vực 47%)</t>
   </si>
   <si>
     <t xml:space="preserve">• Vietnam Report, khảo sát người tiêu dùng ngành bán lẻ, 08/2026
-• Google, Temasek, Bain &amp; Company, e-Conomy SEA 2025, trang 143 (khảo sát Google và Milieu, 09/2025, 7,200 người)</t>
+• Milieu Insight, 09/2025</t>
   </si>
   <si>
     <t xml:space="preserve">https://vietnamreport.net.vn/Top-10-Cong-ty-uy-tin-nganh-Ban-le-nam-2026-12576-1006.html
-https://services.google.com/fh/files/misc/e_conomy_sea_2025_report_combined.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Đã mở trang gốc, khớp số liệu (08/10/2026)
-• Đã mở báo cáo gốc; Thái Lan là 76% (bản trước ghi 74% là sai)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Số người dùng là toàn cầu
-• Dữ liệu Việt Nam
+https://www.mili.eu/vn/insights/vietnams-online-shoppers-demand-speed-and-reliability-in-2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Video mẫu kiểu đố số liệu (scripts/khach-so-gia-cho-sale/1.json)
 • Giọng v4 chưa huấn luyện; video trên trang hub</t>
   </si>
   <si>
-    <t xml:space="preserve">chatgpt; ai mode; người việt dùng ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Bảy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Growth Marketing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Khách bỏ đi ở phút cuối</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vì sao khách bỏ hàng vào giỏ rồi lại không thanh toán?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• 89.5% so giá nhiều nơi trước khi mua; 39.5% hoãn mua chờ khuyến mãi
-• 1/2 bỏ giỏ khi gặp phí phát sinh; 49% bỏ nếu shop chưa có đánh giá; 46% nếu đổi trả không rõ; 53% coi trọng giao đúng hẹn hơn phí ship rẻ (45%); 7/10 sẵn sàng chi nhiều hơn cho shop dịch vụ đáng tin; 1/3 ngừng mua sau trải nghiệm tệ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Vietnam Report, khảo sát người tiêu dùng ngành bán lẻ, 08/2026
-• Milieu Insight, Vietnam's online shoppers demand speed and reliability in 2025, 09/2025
-• Baymard Institute (số Mỹ, chỉ trong phần Làm gì ngay); Klaviyo 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://vietnamreport.net.vn/Top-10-Cong-ty-uy-tin-nganh-Ban-le-nam-2026-12576-1006.html
-https://www.mili.eu/vn/insights/vietnams-online-shoppers-demand-speed-and-reliability-in-2025
-https://baymard.com/lists/cart-abandonment-rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Đã mở trang gốc, khớp số liệu (08/10/2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Tỷ lệ từng nguyên nhân khác nhau theo năm, dùng 70.22% làm số chính
-• Dữ liệu 2021, ghi rõ năm
-• Kịch bản scripts/khach-bo-gio-hang/1.json; dùng thêm số liệu Việt Nam của Milieu Insight (09/2025), chưa mở được trang gốc (mạng chặn), đối chiếu qua PR Newswire, Marketech APAC
-• Giọng v4 chưa huấn luyện; video trên trang hub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bỏ giỏ hàng; tăng tỷ lệ chuyển đổi; cá nhân hóa</t>
+    <t xml:space="preserve">so sánh giá; săn sale; khuyến mãi</t>
   </si>
   <si>
     <t xml:space="preserve">Chủ nhật</t>
@@ -1309,7 +1332,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N79"/>
+  <dimension ref="A1:N80"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
@@ -1499,7 +1522,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="n">
         <v>5</v>
       </c>
@@ -1510,37 +1533,37 @@
         <v>46303</v>
       </c>
       <c r="D6" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="H6" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="I6" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="J6" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="J6" s="6" t="s">
+      <c r="K6" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="K6" s="8" t="s">
+      <c r="L6" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="L6" s="6" t="s">
+      <c r="M6" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="M6" s="6" t="s">
-        <v>53</v>
-      </c>
       <c r="N6" s="6" t="s">
-        <v>54</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1548,113 +1571,131 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>46303</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F7" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C7" s="7" t="n">
-        <v>46304</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="6" t="s">
+      <c r="G7" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="H7" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="I7" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="J7" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="K7" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="J7" s="6" t="s">
+      <c r="L7" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="K7" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="L7" s="6" t="s">
-        <v>63</v>
-      </c>
       <c r="M7" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N7" s="6" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>46304</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="F8" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="L8" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="M8" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="N8" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="7" t="n">
         <v>46305</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="K8" s="8" t="s">
+      <c r="D9" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="K9" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="M9" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="N9" s="6" t="s">
         <v>72</v>
-      </c>
-      <c r="L8" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="M8" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="N8" s="6" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="C9" s="10" t="n">
-        <v>46306</v>
-      </c>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="9" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1662,14 +1703,14 @@
         <v>9</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C10" s="10" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F10" s="9"/>
       <c r="G10" s="9"/>
@@ -1680,7 +1721,7 @@
       <c r="L10" s="9"/>
       <c r="M10" s="9"/>
       <c r="N10" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1688,14 +1729,14 @@
         <v>10</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F11" s="9"/>
       <c r="G11" s="9"/>
@@ -1706,285 +1747,267 @@
       <c r="L11" s="9"/>
       <c r="M11" s="9"/>
       <c r="N11" s="9" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="135.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>46309</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="J12" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="K12" s="8" t="s">
+      <c r="B12" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="L12" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="M12" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="N12" s="6" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C12" s="10" t="n">
+        <v>46308</v>
+      </c>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="9"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="9" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="135.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>46309</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="K13" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="L13" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="M13" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="N13" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C14" s="7" t="n">
         <v>46310</v>
       </c>
-      <c r="D13" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="J13" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="K13" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="L13" s="6" t="s">
+      <c r="D14" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="K14" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="L14" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="M14" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="N14" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="M13" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="N13" s="6" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" s="12" t="n">
-        <v>46311</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>97</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="G14" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="H14" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="I14" s="11" t="s">
-        <v>102</v>
-      </c>
-      <c r="J14" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="K14" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="L14" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="M14" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="N14" s="11" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="15" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C15" s="12" t="n">
-        <v>46312</v>
+        <v>46311</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="E15" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="F15" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="G15" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="G15" s="11" t="s">
+      <c r="H15" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="H15" s="11" t="s">
+      <c r="I15" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="I15" s="11" t="s">
+      <c r="J15" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="J15" s="11" t="s">
+      <c r="K15" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="K15" s="13" t="s">
+      <c r="L15" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="L15" s="11" t="s">
+      <c r="M15" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="M15" s="11" t="s">
-        <v>106</v>
-      </c>
       <c r="N15" s="11" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="n">
         <v>15</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C16" s="12" t="n">
-        <v>46313</v>
+        <v>46312</v>
       </c>
       <c r="D16" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="E16" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="F16" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="G16" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="H16" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="H16" s="11" t="s">
+      <c r="I16" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="I16" s="11" t="s">
+      <c r="J16" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="J16" s="11" t="s">
+      <c r="K16" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="K16" s="13" t="s">
+      <c r="L16" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="L16" s="11" t="s">
-        <v>123</v>
-      </c>
       <c r="M16" s="11" t="s">
-        <v>53</v>
+        <v>114</v>
       </c>
       <c r="N16" s="11" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="n">
         <v>16</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C17" s="12" t="n">
-        <v>46314</v>
+        <v>46313</v>
       </c>
       <c r="D17" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="E17" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="F17" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="G17" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="G17" s="11" t="s">
+      <c r="H17" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="H17" s="11" t="s">
+      <c r="I17" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="I17" s="11" t="s">
+      <c r="J17" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="J17" s="11" t="s">
+      <c r="K17" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="K17" s="13" t="s">
+      <c r="L17" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="L17" s="11" t="s">
-        <v>132</v>
-      </c>
       <c r="M17" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N17" s="11" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="n">
         <v>17</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="C18" s="12" t="n">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>33</v>
+        <v>132</v>
       </c>
       <c r="E18" s="11" t="s">
         <v>133</v>
@@ -2011,36 +2034,54 @@
         <v>140</v>
       </c>
       <c r="M18" s="11" t="s">
-        <v>106</v>
+        <v>52</v>
       </c>
       <c r="N18" s="11" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C19" s="10" t="n">
-        <v>46316</v>
-      </c>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="9"/>
-      <c r="K19" s="9"/>
-      <c r="L19" s="9"/>
-      <c r="M19" s="9"/>
-      <c r="N19" s="9" t="s">
-        <v>76</v>
+      <c r="B19" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="C19" s="12" t="n">
+        <v>46315</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="G19" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="H19" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="I19" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="J19" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="K19" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="L19" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="M19" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="N19" s="11" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2048,14 +2089,14 @@
         <v>19</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="C20" s="10" t="n">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="D20" s="9"/>
       <c r="E20" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F20" s="9"/>
       <c r="G20" s="9"/>
@@ -2066,7 +2107,7 @@
       <c r="L20" s="9"/>
       <c r="M20" s="9"/>
       <c r="N20" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2074,14 +2115,14 @@
         <v>20</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="C21" s="10" t="n">
-        <v>46318</v>
+        <v>46317</v>
       </c>
       <c r="D21" s="9"/>
       <c r="E21" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F21" s="9"/>
       <c r="G21" s="9"/>
@@ -2092,7 +2133,7 @@
       <c r="L21" s="9"/>
       <c r="M21" s="9"/>
       <c r="N21" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2100,14 +2141,14 @@
         <v>21</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C22" s="10" t="n">
-        <v>46319</v>
+        <v>46318</v>
       </c>
       <c r="D22" s="9"/>
       <c r="E22" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F22" s="9"/>
       <c r="G22" s="9"/>
@@ -2118,7 +2159,7 @@
       <c r="L22" s="9"/>
       <c r="M22" s="9"/>
       <c r="N22" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2126,14 +2167,14 @@
         <v>22</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C23" s="10" t="n">
-        <v>46320</v>
+        <v>46319</v>
       </c>
       <c r="D23" s="9"/>
       <c r="E23" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F23" s="9"/>
       <c r="G23" s="9"/>
@@ -2144,7 +2185,7 @@
       <c r="L23" s="9"/>
       <c r="M23" s="9"/>
       <c r="N23" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2152,14 +2193,14 @@
         <v>23</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C24" s="10" t="n">
-        <v>46321</v>
+        <v>46320</v>
       </c>
       <c r="D24" s="9"/>
       <c r="E24" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F24" s="9"/>
       <c r="G24" s="9"/>
@@ -2170,7 +2211,7 @@
       <c r="L24" s="9"/>
       <c r="M24" s="9"/>
       <c r="N24" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2178,14 +2219,14 @@
         <v>24</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="C25" s="10" t="n">
-        <v>46322</v>
+        <v>46321</v>
       </c>
       <c r="D25" s="9"/>
       <c r="E25" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
@@ -2196,7 +2237,7 @@
       <c r="L25" s="9"/>
       <c r="M25" s="9"/>
       <c r="N25" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2204,14 +2245,14 @@
         <v>25</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>32</v>
+        <v>86</v>
       </c>
       <c r="C26" s="10" t="n">
-        <v>46323</v>
+        <v>46322</v>
       </c>
       <c r="D26" s="9"/>
       <c r="E26" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F26" s="9"/>
       <c r="G26" s="9"/>
@@ -2222,7 +2263,7 @@
       <c r="L26" s="9"/>
       <c r="M26" s="9"/>
       <c r="N26" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2230,14 +2271,14 @@
         <v>26</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="C27" s="10" t="n">
-        <v>46324</v>
+        <v>46323</v>
       </c>
       <c r="D27" s="9"/>
       <c r="E27" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F27" s="9"/>
       <c r="G27" s="9"/>
@@ -2248,7 +2289,7 @@
       <c r="L27" s="9"/>
       <c r="M27" s="9"/>
       <c r="N27" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2256,14 +2297,14 @@
         <v>27</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="C28" s="10" t="n">
-        <v>46325</v>
+        <v>46324</v>
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -2274,7 +2315,7 @@
       <c r="L28" s="9"/>
       <c r="M28" s="9"/>
       <c r="N28" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2282,14 +2323,14 @@
         <v>28</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C29" s="10" t="n">
-        <v>46326</v>
+        <v>46325</v>
       </c>
       <c r="D29" s="9"/>
       <c r="E29" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F29" s="9"/>
       <c r="G29" s="9"/>
@@ -2300,7 +2341,7 @@
       <c r="L29" s="9"/>
       <c r="M29" s="9"/>
       <c r="N29" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2308,14 +2349,14 @@
         <v>29</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C30" s="10" t="n">
-        <v>46327</v>
+        <v>46326</v>
       </c>
       <c r="D30" s="9"/>
       <c r="E30" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F30" s="9"/>
       <c r="G30" s="9"/>
@@ -2326,7 +2367,7 @@
       <c r="L30" s="9"/>
       <c r="M30" s="9"/>
       <c r="N30" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2334,14 +2375,14 @@
         <v>30</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C31" s="10" t="n">
-        <v>46328</v>
+        <v>46327</v>
       </c>
       <c r="D31" s="9"/>
       <c r="E31" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F31" s="9"/>
       <c r="G31" s="9"/>
@@ -2352,7 +2393,7 @@
       <c r="L31" s="9"/>
       <c r="M31" s="9"/>
       <c r="N31" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2360,14 +2401,14 @@
         <v>31</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="C32" s="10" t="n">
-        <v>46329</v>
+        <v>46328</v>
       </c>
       <c r="D32" s="9"/>
       <c r="E32" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F32" s="9"/>
       <c r="G32" s="9"/>
@@ -2378,7 +2419,7 @@
       <c r="L32" s="9"/>
       <c r="M32" s="9"/>
       <c r="N32" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2386,14 +2427,14 @@
         <v>32</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>32</v>
+        <v>86</v>
       </c>
       <c r="C33" s="10" t="n">
-        <v>46330</v>
+        <v>46329</v>
       </c>
       <c r="D33" s="9"/>
       <c r="E33" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -2404,7 +2445,7 @@
       <c r="L33" s="9"/>
       <c r="M33" s="9"/>
       <c r="N33" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2412,14 +2453,14 @@
         <v>33</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="C34" s="10" t="n">
-        <v>46331</v>
+        <v>46330</v>
       </c>
       <c r="D34" s="9"/>
       <c r="E34" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -2430,7 +2471,7 @@
       <c r="L34" s="9"/>
       <c r="M34" s="9"/>
       <c r="N34" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2438,14 +2479,14 @@
         <v>34</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="C35" s="10" t="n">
-        <v>46332</v>
+        <v>46331</v>
       </c>
       <c r="D35" s="9"/>
       <c r="E35" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -2456,7 +2497,7 @@
       <c r="L35" s="9"/>
       <c r="M35" s="9"/>
       <c r="N35" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2464,14 +2505,14 @@
         <v>35</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C36" s="10" t="n">
-        <v>46333</v>
+        <v>46332</v>
       </c>
       <c r="D36" s="9"/>
       <c r="E36" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -2482,7 +2523,7 @@
       <c r="L36" s="9"/>
       <c r="M36" s="9"/>
       <c r="N36" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2490,14 +2531,14 @@
         <v>36</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C37" s="10" t="n">
-        <v>46334</v>
+        <v>46333</v>
       </c>
       <c r="D37" s="9"/>
       <c r="E37" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
@@ -2508,7 +2549,7 @@
       <c r="L37" s="9"/>
       <c r="M37" s="9"/>
       <c r="N37" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2516,14 +2557,14 @@
         <v>37</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C38" s="10" t="n">
-        <v>46335</v>
+        <v>46334</v>
       </c>
       <c r="D38" s="9"/>
       <c r="E38" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F38" s="9"/>
       <c r="G38" s="9"/>
@@ -2534,7 +2575,7 @@
       <c r="L38" s="9"/>
       <c r="M38" s="9"/>
       <c r="N38" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2542,14 +2583,14 @@
         <v>38</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="C39" s="10" t="n">
-        <v>46336</v>
+        <v>46335</v>
       </c>
       <c r="D39" s="9"/>
       <c r="E39" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F39" s="9"/>
       <c r="G39" s="9"/>
@@ -2560,77 +2601,77 @@
       <c r="L39" s="9"/>
       <c r="M39" s="9"/>
       <c r="N39" s="9" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="6" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="9" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C40" s="10" t="n">
+        <v>46336</v>
+      </c>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="F40" s="9"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9"/>
+      <c r="I40" s="9"/>
+      <c r="J40" s="9"/>
+      <c r="K40" s="9"/>
+      <c r="L40" s="9"/>
+      <c r="M40" s="9"/>
+      <c r="N40" s="9" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C40" s="7" t="n">
+      <c r="C41" s="7" t="n">
         <v>46337</v>
       </c>
-      <c r="D40" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="F40" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="G40" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="H40" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="I40" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="J40" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="K40" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="L40" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="M40" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="N40" s="6" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="9" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C41" s="10" t="n">
-        <v>46338</v>
-      </c>
-      <c r="D41" s="9"/>
-      <c r="E41" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="F41" s="9"/>
-      <c r="G41" s="9"/>
-      <c r="H41" s="9"/>
-      <c r="I41" s="9"/>
-      <c r="J41" s="9"/>
-      <c r="K41" s="9"/>
-      <c r="L41" s="9"/>
-      <c r="M41" s="9"/>
-      <c r="N41" s="9" t="s">
-        <v>76</v>
+      <c r="D41" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="I41" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="J41" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="K41" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="L41" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="M41" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="N41" s="6" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2638,14 +2679,14 @@
         <v>41</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="C42" s="10" t="n">
-        <v>46339</v>
+        <v>46338</v>
       </c>
       <c r="D42" s="9"/>
       <c r="E42" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F42" s="9"/>
       <c r="G42" s="9"/>
@@ -2656,7 +2697,7 @@
       <c r="L42" s="9"/>
       <c r="M42" s="9"/>
       <c r="N42" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2664,14 +2705,14 @@
         <v>42</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C43" s="10" t="n">
-        <v>46340</v>
+        <v>46339</v>
       </c>
       <c r="D43" s="9"/>
       <c r="E43" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F43" s="9"/>
       <c r="G43" s="9"/>
@@ -2682,7 +2723,7 @@
       <c r="L43" s="9"/>
       <c r="M43" s="9"/>
       <c r="N43" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2690,14 +2731,14 @@
         <v>43</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C44" s="10" t="n">
-        <v>46341</v>
+        <v>46340</v>
       </c>
       <c r="D44" s="9"/>
       <c r="E44" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F44" s="9"/>
       <c r="G44" s="9"/>
@@ -2708,7 +2749,7 @@
       <c r="L44" s="9"/>
       <c r="M44" s="9"/>
       <c r="N44" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2716,14 +2757,14 @@
         <v>44</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C45" s="10" t="n">
-        <v>46342</v>
+        <v>46341</v>
       </c>
       <c r="D45" s="9"/>
       <c r="E45" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F45" s="9"/>
       <c r="G45" s="9"/>
@@ -2734,7 +2775,7 @@
       <c r="L45" s="9"/>
       <c r="M45" s="9"/>
       <c r="N45" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2742,14 +2783,14 @@
         <v>45</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="C46" s="10" t="n">
-        <v>46343</v>
+        <v>46342</v>
       </c>
       <c r="D46" s="9"/>
       <c r="E46" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F46" s="9"/>
       <c r="G46" s="9"/>
@@ -2760,7 +2801,7 @@
       <c r="L46" s="9"/>
       <c r="M46" s="9"/>
       <c r="N46" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2768,14 +2809,14 @@
         <v>46</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>32</v>
+        <v>86</v>
       </c>
       <c r="C47" s="10" t="n">
-        <v>46344</v>
+        <v>46343</v>
       </c>
       <c r="D47" s="9"/>
       <c r="E47" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F47" s="9"/>
       <c r="G47" s="9"/>
@@ -2786,7 +2827,7 @@
       <c r="L47" s="9"/>
       <c r="M47" s="9"/>
       <c r="N47" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2794,14 +2835,14 @@
         <v>47</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="C48" s="10" t="n">
-        <v>46345</v>
+        <v>46344</v>
       </c>
       <c r="D48" s="9"/>
       <c r="E48" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F48" s="9"/>
       <c r="G48" s="9"/>
@@ -2812,7 +2853,7 @@
       <c r="L48" s="9"/>
       <c r="M48" s="9"/>
       <c r="N48" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2820,14 +2861,14 @@
         <v>48</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="C49" s="10" t="n">
-        <v>46346</v>
+        <v>46345</v>
       </c>
       <c r="D49" s="9"/>
       <c r="E49" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F49" s="9"/>
       <c r="G49" s="9"/>
@@ -2838,7 +2879,7 @@
       <c r="L49" s="9"/>
       <c r="M49" s="9"/>
       <c r="N49" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2846,14 +2887,14 @@
         <v>49</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C50" s="10" t="n">
-        <v>46347</v>
+        <v>46346</v>
       </c>
       <c r="D50" s="9"/>
       <c r="E50" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F50" s="9"/>
       <c r="G50" s="9"/>
@@ -2864,77 +2905,77 @@
       <c r="L50" s="9"/>
       <c r="M50" s="9"/>
       <c r="N50" s="9" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="6" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="B51" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="C51" s="7" t="n">
+      <c r="B51" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C51" s="10" t="n">
+        <v>46347</v>
+      </c>
+      <c r="D51" s="9"/>
+      <c r="E51" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="F51" s="9"/>
+      <c r="G51" s="9"/>
+      <c r="H51" s="9"/>
+      <c r="I51" s="9"/>
+      <c r="J51" s="9"/>
+      <c r="K51" s="9"/>
+      <c r="L51" s="9"/>
+      <c r="M51" s="9"/>
+      <c r="N51" s="9" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C52" s="7" t="n">
         <v>46348</v>
       </c>
-      <c r="D51" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="E51" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="F51" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="G51" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="H51" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="I51" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="J51" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="K51" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="L51" s="6" t="s">
+      <c r="D52" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="M51" s="6" t="s">
+      <c r="E52" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="N51" s="6" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="9" t="n">
-        <v>51</v>
-      </c>
-      <c r="B52" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="C52" s="10" t="n">
-        <v>46349</v>
-      </c>
-      <c r="D52" s="9"/>
-      <c r="E52" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="F52" s="9"/>
-      <c r="G52" s="9"/>
-      <c r="H52" s="9"/>
-      <c r="I52" s="9"/>
-      <c r="J52" s="9"/>
-      <c r="K52" s="9"/>
-      <c r="L52" s="9"/>
-      <c r="M52" s="9"/>
-      <c r="N52" s="9" t="s">
-        <v>76</v>
+      <c r="F52" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="G52" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="H52" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="I52" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="J52" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="K52" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="L52" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="M52" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="N52" s="6" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2942,14 +2983,14 @@
         <v>52</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="C53" s="10" t="n">
-        <v>46350</v>
+        <v>46349</v>
       </c>
       <c r="D53" s="9"/>
       <c r="E53" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F53" s="9"/>
       <c r="G53" s="9"/>
@@ -2960,7 +3001,7 @@
       <c r="L53" s="9"/>
       <c r="M53" s="9"/>
       <c r="N53" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2968,14 +3009,14 @@
         <v>53</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>32</v>
+        <v>86</v>
       </c>
       <c r="C54" s="10" t="n">
-        <v>46351</v>
+        <v>46350</v>
       </c>
       <c r="D54" s="9"/>
       <c r="E54" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F54" s="9"/>
       <c r="G54" s="9"/>
@@ -2986,7 +3027,7 @@
       <c r="L54" s="9"/>
       <c r="M54" s="9"/>
       <c r="N54" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2994,14 +3035,14 @@
         <v>54</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="C55" s="10" t="n">
-        <v>46352</v>
+        <v>46351</v>
       </c>
       <c r="D55" s="9"/>
       <c r="E55" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F55" s="9"/>
       <c r="G55" s="9"/>
@@ -3012,77 +3053,77 @@
       <c r="L55" s="9"/>
       <c r="M55" s="9"/>
       <c r="N55" s="9" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="11" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="9" t="n">
         <v>55</v>
       </c>
-      <c r="B56" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="C56" s="12" t="n">
+      <c r="B56" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C56" s="10" t="n">
+        <v>46352</v>
+      </c>
+      <c r="D56" s="9"/>
+      <c r="E56" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="F56" s="9"/>
+      <c r="G56" s="9"/>
+      <c r="H56" s="9"/>
+      <c r="I56" s="9"/>
+      <c r="J56" s="9"/>
+      <c r="K56" s="9"/>
+      <c r="L56" s="9"/>
+      <c r="M56" s="9"/>
+      <c r="N56" s="9" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="11" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="C57" s="12" t="n">
         <v>46353</v>
       </c>
-      <c r="D56" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="E56" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="F56" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="G56" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="H56" s="11" t="s">
-        <v>162</v>
-      </c>
-      <c r="I56" s="11" t="s">
-        <v>163</v>
-      </c>
-      <c r="J56" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="K56" s="13" t="s">
-        <v>165</v>
-      </c>
-      <c r="L56" s="11" t="s">
-        <v>166</v>
-      </c>
-      <c r="M56" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="N56" s="11" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="9" t="n">
-        <v>56</v>
-      </c>
-      <c r="B57" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="C57" s="10" t="n">
-        <v>46354</v>
-      </c>
-      <c r="D57" s="9"/>
-      <c r="E57" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="F57" s="9"/>
-      <c r="G57" s="9"/>
-      <c r="H57" s="9"/>
-      <c r="I57" s="9"/>
-      <c r="J57" s="9"/>
-      <c r="K57" s="9"/>
-      <c r="L57" s="9"/>
-      <c r="M57" s="9"/>
-      <c r="N57" s="9" t="s">
-        <v>76</v>
+      <c r="D57" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="E57" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="F57" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="G57" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="H57" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="I57" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="J57" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="K57" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="L57" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="M57" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="N57" s="11" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3090,14 +3131,14 @@
         <v>57</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C58" s="10" t="n">
-        <v>46355</v>
+        <v>46354</v>
       </c>
       <c r="D58" s="9"/>
       <c r="E58" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F58" s="9"/>
       <c r="G58" s="9"/>
@@ -3108,7 +3149,7 @@
       <c r="L58" s="9"/>
       <c r="M58" s="9"/>
       <c r="N58" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3116,14 +3157,14 @@
         <v>58</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C59" s="10" t="n">
-        <v>46356</v>
+        <v>46355</v>
       </c>
       <c r="D59" s="9"/>
       <c r="E59" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F59" s="9"/>
       <c r="G59" s="9"/>
@@ -3134,7 +3175,7 @@
       <c r="L59" s="9"/>
       <c r="M59" s="9"/>
       <c r="N59" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3142,14 +3183,14 @@
         <v>59</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="C60" s="10" t="n">
-        <v>46357</v>
+        <v>46356</v>
       </c>
       <c r="D60" s="9"/>
       <c r="E60" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F60" s="9"/>
       <c r="G60" s="9"/>
@@ -3160,7 +3201,7 @@
       <c r="L60" s="9"/>
       <c r="M60" s="9"/>
       <c r="N60" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3168,14 +3209,14 @@
         <v>60</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>32</v>
+        <v>86</v>
       </c>
       <c r="C61" s="10" t="n">
-        <v>46358</v>
+        <v>46357</v>
       </c>
       <c r="D61" s="9"/>
       <c r="E61" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F61" s="9"/>
       <c r="G61" s="9"/>
@@ -3186,7 +3227,7 @@
       <c r="L61" s="9"/>
       <c r="M61" s="9"/>
       <c r="N61" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3194,14 +3235,14 @@
         <v>61</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="C62" s="10" t="n">
-        <v>46359</v>
+        <v>46358</v>
       </c>
       <c r="D62" s="9"/>
       <c r="E62" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F62" s="9"/>
       <c r="G62" s="9"/>
@@ -3212,7 +3253,7 @@
       <c r="L62" s="9"/>
       <c r="M62" s="9"/>
       <c r="N62" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3220,14 +3261,14 @@
         <v>62</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="C63" s="10" t="n">
-        <v>46360</v>
+        <v>46359</v>
       </c>
       <c r="D63" s="9"/>
       <c r="E63" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F63" s="9"/>
       <c r="G63" s="9"/>
@@ -3238,7 +3279,7 @@
       <c r="L63" s="9"/>
       <c r="M63" s="9"/>
       <c r="N63" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3246,14 +3287,14 @@
         <v>63</v>
       </c>
       <c r="B64" s="9" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C64" s="10" t="n">
-        <v>46361</v>
+        <v>46360</v>
       </c>
       <c r="D64" s="9"/>
       <c r="E64" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F64" s="9"/>
       <c r="G64" s="9"/>
@@ -3264,7 +3305,7 @@
       <c r="L64" s="9"/>
       <c r="M64" s="9"/>
       <c r="N64" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3272,14 +3313,14 @@
         <v>64</v>
       </c>
       <c r="B65" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C65" s="10" t="n">
-        <v>46362</v>
+        <v>46361</v>
       </c>
       <c r="D65" s="9"/>
       <c r="E65" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F65" s="9"/>
       <c r="G65" s="9"/>
@@ -3290,7 +3331,7 @@
       <c r="L65" s="9"/>
       <c r="M65" s="9"/>
       <c r="N65" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3298,14 +3339,14 @@
         <v>65</v>
       </c>
       <c r="B66" s="9" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C66" s="10" t="n">
-        <v>46363</v>
+        <v>46362</v>
       </c>
       <c r="D66" s="9"/>
       <c r="E66" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F66" s="9"/>
       <c r="G66" s="9"/>
@@ -3316,7 +3357,7 @@
       <c r="L66" s="9"/>
       <c r="M66" s="9"/>
       <c r="N66" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3324,14 +3365,14 @@
         <v>66</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="C67" s="10" t="n">
-        <v>46364</v>
+        <v>46363</v>
       </c>
       <c r="D67" s="9"/>
       <c r="E67" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F67" s="9"/>
       <c r="G67" s="9"/>
@@ -3342,77 +3383,77 @@
       <c r="L67" s="9"/>
       <c r="M67" s="9"/>
       <c r="N67" s="9" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="6" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="9" t="n">
         <v>67</v>
       </c>
-      <c r="B68" s="6" t="s">
+      <c r="B68" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C68" s="10" t="n">
+        <v>46364</v>
+      </c>
+      <c r="D68" s="9"/>
+      <c r="E68" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="F68" s="9"/>
+      <c r="G68" s="9"/>
+      <c r="H68" s="9"/>
+      <c r="I68" s="9"/>
+      <c r="J68" s="9"/>
+      <c r="K68" s="9"/>
+      <c r="L68" s="9"/>
+      <c r="M68" s="9"/>
+      <c r="N68" s="9" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="6" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C68" s="7" t="n">
+      <c r="C69" s="7" t="n">
         <v>46365</v>
       </c>
-      <c r="D68" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="E68" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="F68" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="G68" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="H68" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="I68" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="J68" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="K68" s="8" t="s">
-        <v>173</v>
-      </c>
-      <c r="L68" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="M68" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="N68" s="6" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="9" t="n">
-        <v>68</v>
-      </c>
-      <c r="B69" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C69" s="10" t="n">
-        <v>46366</v>
-      </c>
-      <c r="D69" s="9"/>
-      <c r="E69" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="F69" s="9"/>
-      <c r="G69" s="9"/>
-      <c r="H69" s="9"/>
-      <c r="I69" s="9"/>
-      <c r="J69" s="9"/>
-      <c r="K69" s="9"/>
-      <c r="L69" s="9"/>
-      <c r="M69" s="9"/>
-      <c r="N69" s="9" t="s">
-        <v>76</v>
+      <c r="D69" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="E69" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="G69" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="H69" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="I69" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J69" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="K69" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="L69" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="M69" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="N69" s="6" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3420,14 +3461,14 @@
         <v>69</v>
       </c>
       <c r="B70" s="9" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="C70" s="10" t="n">
-        <v>46367</v>
+        <v>46366</v>
       </c>
       <c r="D70" s="9"/>
       <c r="E70" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F70" s="9"/>
       <c r="G70" s="9"/>
@@ -3438,7 +3479,7 @@
       <c r="L70" s="9"/>
       <c r="M70" s="9"/>
       <c r="N70" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3446,14 +3487,14 @@
         <v>70</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C71" s="10" t="n">
-        <v>46368</v>
+        <v>46367</v>
       </c>
       <c r="D71" s="9"/>
       <c r="E71" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F71" s="9"/>
       <c r="G71" s="9"/>
@@ -3464,7 +3505,7 @@
       <c r="L71" s="9"/>
       <c r="M71" s="9"/>
       <c r="N71" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3472,14 +3513,14 @@
         <v>71</v>
       </c>
       <c r="B72" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C72" s="10" t="n">
-        <v>46369</v>
+        <v>46368</v>
       </c>
       <c r="D72" s="9"/>
       <c r="E72" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F72" s="9"/>
       <c r="G72" s="9"/>
@@ -3490,7 +3531,7 @@
       <c r="L72" s="9"/>
       <c r="M72" s="9"/>
       <c r="N72" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3498,14 +3539,14 @@
         <v>72</v>
       </c>
       <c r="B73" s="9" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C73" s="10" t="n">
-        <v>46370</v>
+        <v>46369</v>
       </c>
       <c r="D73" s="9"/>
       <c r="E73" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F73" s="9"/>
       <c r="G73" s="9"/>
@@ -3516,7 +3557,7 @@
       <c r="L73" s="9"/>
       <c r="M73" s="9"/>
       <c r="N73" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3524,14 +3565,14 @@
         <v>73</v>
       </c>
       <c r="B74" s="9" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="C74" s="10" t="n">
-        <v>46371</v>
+        <v>46370</v>
       </c>
       <c r="D74" s="9"/>
       <c r="E74" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F74" s="9"/>
       <c r="G74" s="9"/>
@@ -3542,77 +3583,77 @@
       <c r="L74" s="9"/>
       <c r="M74" s="9"/>
       <c r="N74" s="9" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="11" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="9" t="n">
         <v>74</v>
       </c>
-      <c r="B75" s="11" t="s">
+      <c r="B75" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C75" s="10" t="n">
+        <v>46371</v>
+      </c>
+      <c r="D75" s="9"/>
+      <c r="E75" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="F75" s="9"/>
+      <c r="G75" s="9"/>
+      <c r="H75" s="9"/>
+      <c r="I75" s="9"/>
+      <c r="J75" s="9"/>
+      <c r="K75" s="9"/>
+      <c r="L75" s="9"/>
+      <c r="M75" s="9"/>
+      <c r="N75" s="9" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="11" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C75" s="12" t="n">
+      <c r="C76" s="12" t="n">
         <v>46372</v>
       </c>
-      <c r="D75" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="E75" s="11" t="s">
-        <v>175</v>
-      </c>
-      <c r="F75" s="11" t="s">
-        <v>176</v>
-      </c>
-      <c r="G75" s="11" t="s">
-        <v>177</v>
-      </c>
-      <c r="H75" s="11" t="s">
-        <v>178</v>
-      </c>
-      <c r="I75" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="J75" s="11" t="s">
-        <v>180</v>
-      </c>
-      <c r="K75" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="L75" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="M75" s="11" t="s">
+      <c r="D76" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E76" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="N75" s="11" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="9" t="n">
-        <v>75</v>
-      </c>
-      <c r="B76" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C76" s="10" t="n">
-        <v>46373</v>
-      </c>
-      <c r="D76" s="9"/>
-      <c r="E76" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="F76" s="9"/>
-      <c r="G76" s="9"/>
-      <c r="H76" s="9"/>
-      <c r="I76" s="9"/>
-      <c r="J76" s="9"/>
-      <c r="K76" s="9"/>
-      <c r="L76" s="9"/>
-      <c r="M76" s="9"/>
-      <c r="N76" s="9" t="s">
-        <v>76</v>
+      <c r="F76" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="G76" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="H76" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="I76" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="J76" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="K76" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="L76" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="M76" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="N76" s="11" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3620,14 +3661,14 @@
         <v>76</v>
       </c>
       <c r="B77" s="9" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="C77" s="10" t="n">
-        <v>46374</v>
+        <v>46373</v>
       </c>
       <c r="D77" s="9"/>
       <c r="E77" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F77" s="9"/>
       <c r="G77" s="9"/>
@@ -3638,7 +3679,7 @@
       <c r="L77" s="9"/>
       <c r="M77" s="9"/>
       <c r="N77" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3646,14 +3687,14 @@
         <v>77</v>
       </c>
       <c r="B78" s="9" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C78" s="10" t="n">
-        <v>46375</v>
+        <v>46374</v>
       </c>
       <c r="D78" s="9"/>
       <c r="E78" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F78" s="9"/>
       <c r="G78" s="9"/>
@@ -3664,7 +3705,7 @@
       <c r="L78" s="9"/>
       <c r="M78" s="9"/>
       <c r="N78" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3672,14 +3713,14 @@
         <v>78</v>
       </c>
       <c r="B79" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C79" s="10" t="n">
-        <v>46376</v>
+        <v>46375</v>
       </c>
       <c r="D79" s="9"/>
       <c r="E79" s="9" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="F79" s="9"/>
       <c r="G79" s="9"/>
@@ -3690,13 +3731,39 @@
       <c r="L79" s="9"/>
       <c r="M79" s="9"/>
       <c r="N79" s="9" t="s">
-        <v>76</v>
+        <v>84</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="9" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C80" s="10" t="n">
+        <v>46376</v>
+      </c>
+      <c r="D80" s="9"/>
+      <c r="E80" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="F80" s="9"/>
+      <c r="G80" s="9"/>
+      <c r="H80" s="9"/>
+      <c r="I80" s="9"/>
+      <c r="J80" s="9"/>
+      <c r="K80" s="9"/>
+      <c r="L80" s="9"/>
+      <c r="M80" s="9"/>
+      <c r="N80" s="9" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N79"/>
+  <autoFilter ref="A1:N80"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N2:N79" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N2:N80" type="list">
       <formula1>"Cần chủ đề,Ý tưởng,Đã kiểm tra nguồn,Đã viết kịch bản,Đã có video,Đã đăng"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3726,19 +3793,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="B2" s="15" t="n">
-        <f aca="false">COUNTA('Lịch đăng'!$A$2:$A$79)</f>
-        <v>78</v>
+        <f aca="false">COUNTA('Lịch đăng'!$A$2:$A$80)</f>
+        <v>79</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3746,26 +3813,26 @@
         <v>26</v>
       </c>
       <c r="B3" s="15" t="n">
-        <f aca="false">COUNTIF('Lịch đăng'!$N$2:$N$79,"Đã đăng")</f>
-        <v>4</v>
+        <f aca="false">COUNTIF('Lịch đăng'!$N$2:$N$80,"Đã đăng")</f>
+        <v>6</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="B4" s="15" t="n">
-        <f aca="false">COUNTIF('Lịch đăng'!$N$2:$N$79,"Cần chủ đề")</f>
+        <f aca="false">COUNTIF('Lịch đăng'!$N$2:$N$80,"Cần chủ đề")</f>
         <v>59</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B5" s="15" t="n">
         <f aca="false">B2-B3-B4</f>
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Xuất lại video 09/10 theo hướng A và C, thêm nút tải ảnh bìa trên hub, ghi đã nhắc
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dpu4oyZ8FYSVLE8FrdnGTC
</commit_message>
<xml_diff>
--- a/video/plan/lich-noi-dung-tiktok.xlsx
+++ b/video/plan/lich-noi-dung-tiktok.xlsx
@@ -254,7 +254,9 @@
     <t xml:space="preserve">• Chưa có URL trang gốc của Meta, cần tìm trước khi dựng
 • Doanh nghiệp tự công bố
 • Giọng v4 chưa huấn luyện; video trên trang hub
-• Nằm trong Drafts của TikTok, dời sang 09/10</t>
+• Nằm trong Drafts của TikTok, dời sang 09/10
+• Xuất lại 09/10 theo hướng A và C
+• Đã nhắc</t>
   </si>
   <si>
     <t xml:space="preserve">quảng cáo tin nhắn; zalo oa; chốt đơn inbox</t>

</xml_diff>

<commit_message>
Thêm 3 chủ đề 11-13/10 đã kiểm tra nguồn gốc (KOL, shop Mall, tiếp cận quảng cáo)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dpu4oyZ8FYSVLE8FrdnGTC
</commit_message>
<xml_diff>
--- a/video/plan/lich-noi-dung-tiktok.xlsx
+++ b/video/plan/lich-noi-dung-tiktok.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="223">
   <si>
     <t xml:space="preserve">Lịch nội dung TikTok Adtek</t>
   </si>
@@ -299,16 +299,115 @@
     <t xml:space="preserve">Chủ nhật</t>
   </si>
   <si>
-    <t xml:space="preserve">Slot trống: chủ đề trend Claude tự chọn khi viết kịch bản thứ Bảy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cần chủ đề</t>
+    <t xml:space="preserve">Digital, Performance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thuê KOL nổi tiếng là khách sẽ tin? (phá hiểu lầm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Cứ thuê KOL nổi tiếng là khách sẽ tin và chốt đơn." Đúng hay sai?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• 54% tin đánh giá của người dùng thường hơn KOL, chỉ 13% nghiêng về người nổi tiếng
+• 78% bị đánh giá online ảnh hưởng mạnh tới lựa chọn (87% ở tuổi 20)
+• Đánh giá đáng tin: có ảnh/video 69%, nội dung chi tiết 60%, số sao 51%; dưới 3.6 sao bị loại; 74% cần từ 50 đánh giá
+• 67% tự tin nhận ra đánh giá giả</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Q&amp;Me, How Vietnamese consumers trust online reviews, khoảng 09/2026, 200 người 20-49 tuổi tại Hà Nội và TP.HCM
+• Việc làm ngay: Google Business Profile Help (xin đánh giá bằng link/QR, cấm tặng quà đổi đánh giá, trả lời đánh giá); TikTok Ads Help (Spark Ads dùng video của khách, nhà sáng tạo nhỏ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://qandme.net/en/report/how-vietnamese-consumers-trust-online-reviews.html
+https://support.google.com/business/answer/3474122
+https://support.google.com/business/answer/3474050
+https://ads.tiktok.com/help/article/spark-ads</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Đã mở trang gốc, khớp số liệu (09/10/2026). Báo cáo đầy đủ cần đăng ký, chỉ kiểm tra phần tóm tắt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Kiểu phá hiểu lầm, đóng dấu SAI
+• Mẫu nhỏ (200 người, chỉ HN và HCM), phải ghi rõ trên video
+• Ngày phát hành ước tính cuối 09/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kol; review sản phẩm; đánh giá 5 sao; chốt đơn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đã kiểm tra nguồn</t>
   </si>
   <si>
     <t xml:space="preserve">Thứ Hai</t>
   </si>
   <si>
+    <t xml:space="preserve">Performance, Growth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chưa tới 3% gian hàng nắm 1/3 doanh số sàn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trên Shopee, TikTok Shop, Lazada, cứ 100 gian hàng thì chưa tới 3 shop Mall. Họ đang nắm bao nhiêu phần doanh số?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Shop Mall: 2.79% số gian hàng nhưng 34.2% doanh số (Shopee, Lazada, TikTok Shop, 6 tháng 2026); số shop Mall giảm 6%, doanh số tăng 54%
+• 4 sàn đạt 291.6 nghìn tỷ đồng, tăng 44.11%; 613.8 nghìn shop có đơn
+• Thị phần GMV: Shopee 54.5% (+15%), TikTok Shop 43.4% (+27%); TikTok Shop nắm 56.2% ngành thời trang
+• Hàng trên 1 triệu đồng chiếm 18.2% doanh số (+3.1 điểm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Metric, Báo cáo TMĐT Việt Nam 6 tháng đầu năm 2026, 29/07/2026
+• YouNet ECI, Toàn cảnh TMĐT Việt Nam nửa đầu năm 2026, 12/08/2026
+• Việc làm ngay: TikTok Shop Seller University (Mall, lịch 11.11 từ 03-12/11 và 12.12, Cộng tác mở); Shopee Help (tiếp thị liên kết trả theo đơn)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://metric.vn/insights/metric-bao-cao-thuong-mai-dien-tu-viet-nam-6-thang-dau-nam-2026/
+https://www.younetgroup.com/vi/bao-cao-toan-canh-tmdt-viet-nam-nua-dau-nam-2026
+https://seller-vn.tiktok.com/university/essay?knowledge_id=6210902215264001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Đã mở trang gốc, khớp số liệu (09/10/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Metric (doanh số, +44%) và YouNet (GMV, +19%) đo khác nhau: không đặt chung một biểu đồ
+• Tỷ lệ Mall tính trên 3 sàn, không phải 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shopee mall; tiktok shop mall; bán hàng trên sàn 2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">Thứ Ba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quảng cáo nền tảng nào tiếp cận nhiều người Việt nhất? (đố số liệu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đoán thử: quảng cáo trên nền tảng nào tiếp cận nhiều người Việt nhất? A. TikTok, B. Facebook, C. YouTube</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Lượng người quảng cáo có thể tiếp cận: Facebook 79.0 triệu, TikTok 76.1 triệu (18+), YouTube 62.1 triệu, Messenger 57.8 triệu (cuối 2025)
+• Thời gian dùng mỗi ngày (Android, 08/2025): TikTok 1 giờ 56 phút, YouTube 1 giờ 21 phút, Facebook 1 giờ 11 phút
+• 84.9% người dùng internet tìm thông tin thương hiệu trên mạng xã hội
+• Zalo 81.3 triệu người dùng tháng (quý 2/2026, VNG): là số người dùng, không so trực tiếp với số tiếp cận quảng cáo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• DataReportal, Digital 2026: Vietnam (số liệu đến 10/2025)
+• VNG, Snapshot quý 2/2026
+• Việc làm ngay: TikTok Spark Ads; Google Ads Demand Gen (YouTube Shorts, Lookalike); Zalo Business Message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://datareportal.com/reports/digital-2026-vietnam
+https://cms-investor-cdn.vng.com.vn/VNG_Snapshot_Q2_2026_EN_8dc74b151d.pdf
+https://support.google.com/google-ads/answer/13695777
+https://zalo.solutions/business-message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Kiểu đố số liệu, ảnh bìa không lộ đáp án
+• Số tiếp cận quảng cáo không phải số người dùng thật, có thể trùng; ghi rõ
+• Tránh lặp quảng cáo Click-to-Messenger (đã nói trong video nhắn tin 09/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">quảng cáo facebook hay tiktok; chạy quảng cáo youtube; zalo ads</t>
   </si>
   <si>
     <t xml:space="preserve">Performance</t>
@@ -562,6 +661,12 @@
   </si>
   <si>
     <t xml:space="preserve">kinh tế số việt nam; digital 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slot trống: chủ đề trend Claude tự chọn khi viết kịch bản thứ Bảy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cần chủ đề</t>
   </si>
   <si>
     <t xml:space="preserve">TikTok Shop hay Shopee?</t>
@@ -961,7 +1066,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="7">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -997,6 +1102,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1710,20 +1823,38 @@
       <c r="C10" s="10" t="n">
         <v>46306</v>
       </c>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9" t="s">
+      <c r="D10" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="9"/>
-      <c r="L10" s="9"/>
-      <c r="M10" s="9"/>
+      <c r="E10" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="J10" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="K10" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="L10" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="M10" s="9" t="s">
+        <v>52</v>
+      </c>
       <c r="N10" s="9" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1731,25 +1862,43 @@
         <v>10</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C11" s="10" t="n">
         <v>46307</v>
       </c>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="9"/>
-      <c r="M11" s="9"/>
+      <c r="D11" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="I11" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="J11" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="K11" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="L11" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="M11" s="9" t="s">
+        <v>52</v>
+      </c>
       <c r="N11" s="9" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1757,25 +1906,43 @@
         <v>11</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="C12" s="10" t="n">
         <v>46308</v>
       </c>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9" t="s">
+      <c r="D12" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
-      <c r="M12" s="9"/>
+      <c r="E12" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="I12" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="J12" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="K12" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="L12" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="M12" s="9" t="s">
+        <v>52</v>
+      </c>
       <c r="N12" s="9" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="135.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1789,37 +1956,37 @@
         <v>46309</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>88</v>
+        <v>112</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>89</v>
+        <v>113</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>90</v>
+        <v>114</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>91</v>
+        <v>115</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>92</v>
+        <v>116</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>93</v>
+        <v>117</v>
       </c>
       <c r="K13" s="8" t="s">
-        <v>94</v>
+        <v>118</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="M13" s="6" t="s">
         <v>52</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1836,34 +2003,34 @@
         <v>63</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>98</v>
+        <v>122</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>100</v>
+        <v>124</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>101</v>
+        <v>125</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>102</v>
+        <v>126</v>
       </c>
       <c r="K14" s="8" t="s">
-        <v>103</v>
+        <v>127</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>104</v>
+        <v>128</v>
       </c>
       <c r="M14" s="6" t="s">
         <v>52</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1877,37 +2044,37 @@
         <v>46311</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>105</v>
+        <v>129</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>106</v>
+        <v>130</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>107</v>
+        <v>131</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>108</v>
+        <v>132</v>
       </c>
       <c r="H15" s="11" t="s">
-        <v>109</v>
+        <v>133</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>110</v>
+        <v>134</v>
       </c>
       <c r="J15" s="11" t="s">
-        <v>111</v>
+        <v>135</v>
       </c>
       <c r="K15" s="13" t="s">
-        <v>112</v>
+        <v>136</v>
       </c>
       <c r="L15" s="11" t="s">
-        <v>113</v>
+        <v>137</v>
       </c>
       <c r="M15" s="11" t="s">
-        <v>114</v>
+        <v>138</v>
       </c>
       <c r="N15" s="11" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1921,37 +2088,37 @@
         <v>46312</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>105</v>
+        <v>129</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>115</v>
+        <v>139</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>116</v>
+        <v>140</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>119</v>
+        <v>143</v>
       </c>
       <c r="J16" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="K16" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="L16" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="M16" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="N16" s="11" t="s">
         <v>120</v>
-      </c>
-      <c r="K16" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="L16" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="M16" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="N16" s="11" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1965,37 +2132,37 @@
         <v>46313</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>123</v>
+        <v>147</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>124</v>
+        <v>148</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>125</v>
+        <v>149</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>126</v>
+        <v>150</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>127</v>
+        <v>151</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>128</v>
+        <v>152</v>
       </c>
       <c r="J17" s="11" t="s">
-        <v>129</v>
+        <v>153</v>
       </c>
       <c r="K17" s="13" t="s">
-        <v>130</v>
+        <v>154</v>
       </c>
       <c r="L17" s="11" t="s">
-        <v>131</v>
+        <v>155</v>
       </c>
       <c r="M17" s="11" t="s">
         <v>52</v>
       </c>
       <c r="N17" s="11" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2003,43 +2170,43 @@
         <v>17</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C18" s="12" t="n">
         <v>46314</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>133</v>
+        <v>157</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>136</v>
+        <v>160</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>137</v>
+        <v>161</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>138</v>
+        <v>162</v>
       </c>
       <c r="K18" s="13" t="s">
-        <v>139</v>
+        <v>163</v>
       </c>
       <c r="L18" s="11" t="s">
-        <v>140</v>
+        <v>164</v>
       </c>
       <c r="M18" s="11" t="s">
         <v>52</v>
       </c>
       <c r="N18" s="11" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2047,7 +2214,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="C19" s="12" t="n">
         <v>46315</v>
@@ -2056,34 +2223,34 @@
         <v>33</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>141</v>
+        <v>165</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>142</v>
+        <v>166</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>143</v>
+        <v>167</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>145</v>
+        <v>169</v>
       </c>
       <c r="J19" s="11" t="s">
-        <v>146</v>
+        <v>170</v>
       </c>
       <c r="K19" s="13" t="s">
-        <v>147</v>
+        <v>171</v>
       </c>
       <c r="L19" s="11" t="s">
-        <v>148</v>
+        <v>172</v>
       </c>
       <c r="M19" s="11" t="s">
-        <v>114</v>
+        <v>138</v>
       </c>
       <c r="N19" s="11" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2098,7 +2265,7 @@
       </c>
       <c r="D20" s="9"/>
       <c r="E20" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F20" s="9"/>
       <c r="G20" s="9"/>
@@ -2109,7 +2276,7 @@
       <c r="L20" s="9"/>
       <c r="M20" s="9"/>
       <c r="N20" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2124,7 +2291,7 @@
       </c>
       <c r="D21" s="9"/>
       <c r="E21" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F21" s="9"/>
       <c r="G21" s="9"/>
@@ -2135,7 +2302,7 @@
       <c r="L21" s="9"/>
       <c r="M21" s="9"/>
       <c r="N21" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2150,7 +2317,7 @@
       </c>
       <c r="D22" s="9"/>
       <c r="E22" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F22" s="9"/>
       <c r="G22" s="9"/>
@@ -2161,7 +2328,7 @@
       <c r="L22" s="9"/>
       <c r="M22" s="9"/>
       <c r="N22" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2176,7 +2343,7 @@
       </c>
       <c r="D23" s="9"/>
       <c r="E23" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F23" s="9"/>
       <c r="G23" s="9"/>
@@ -2187,7 +2354,7 @@
       <c r="L23" s="9"/>
       <c r="M23" s="9"/>
       <c r="N23" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2202,7 +2369,7 @@
       </c>
       <c r="D24" s="9"/>
       <c r="E24" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F24" s="9"/>
       <c r="G24" s="9"/>
@@ -2213,7 +2380,7 @@
       <c r="L24" s="9"/>
       <c r="M24" s="9"/>
       <c r="N24" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2221,14 +2388,14 @@
         <v>24</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C25" s="10" t="n">
         <v>46321</v>
       </c>
       <c r="D25" s="9"/>
       <c r="E25" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
@@ -2239,7 +2406,7 @@
       <c r="L25" s="9"/>
       <c r="M25" s="9"/>
       <c r="N25" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2247,14 +2414,14 @@
         <v>25</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="C26" s="10" t="n">
         <v>46322</v>
       </c>
       <c r="D26" s="9"/>
       <c r="E26" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F26" s="9"/>
       <c r="G26" s="9"/>
@@ -2265,7 +2432,7 @@
       <c r="L26" s="9"/>
       <c r="M26" s="9"/>
       <c r="N26" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2280,7 +2447,7 @@
       </c>
       <c r="D27" s="9"/>
       <c r="E27" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F27" s="9"/>
       <c r="G27" s="9"/>
@@ -2291,7 +2458,7 @@
       <c r="L27" s="9"/>
       <c r="M27" s="9"/>
       <c r="N27" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2306,7 +2473,7 @@
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -2317,7 +2484,7 @@
       <c r="L28" s="9"/>
       <c r="M28" s="9"/>
       <c r="N28" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2332,7 +2499,7 @@
       </c>
       <c r="D29" s="9"/>
       <c r="E29" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F29" s="9"/>
       <c r="G29" s="9"/>
@@ -2343,7 +2510,7 @@
       <c r="L29" s="9"/>
       <c r="M29" s="9"/>
       <c r="N29" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2358,7 +2525,7 @@
       </c>
       <c r="D30" s="9"/>
       <c r="E30" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F30" s="9"/>
       <c r="G30" s="9"/>
@@ -2369,7 +2536,7 @@
       <c r="L30" s="9"/>
       <c r="M30" s="9"/>
       <c r="N30" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2384,7 +2551,7 @@
       </c>
       <c r="D31" s="9"/>
       <c r="E31" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F31" s="9"/>
       <c r="G31" s="9"/>
@@ -2395,7 +2562,7 @@
       <c r="L31" s="9"/>
       <c r="M31" s="9"/>
       <c r="N31" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2403,14 +2570,14 @@
         <v>31</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C32" s="10" t="n">
         <v>46328</v>
       </c>
       <c r="D32" s="9"/>
       <c r="E32" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F32" s="9"/>
       <c r="G32" s="9"/>
@@ -2421,7 +2588,7 @@
       <c r="L32" s="9"/>
       <c r="M32" s="9"/>
       <c r="N32" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2429,14 +2596,14 @@
         <v>32</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="C33" s="10" t="n">
         <v>46329</v>
       </c>
       <c r="D33" s="9"/>
       <c r="E33" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -2447,7 +2614,7 @@
       <c r="L33" s="9"/>
       <c r="M33" s="9"/>
       <c r="N33" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2462,7 +2629,7 @@
       </c>
       <c r="D34" s="9"/>
       <c r="E34" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -2473,7 +2640,7 @@
       <c r="L34" s="9"/>
       <c r="M34" s="9"/>
       <c r="N34" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2488,7 +2655,7 @@
       </c>
       <c r="D35" s="9"/>
       <c r="E35" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -2499,7 +2666,7 @@
       <c r="L35" s="9"/>
       <c r="M35" s="9"/>
       <c r="N35" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2514,7 +2681,7 @@
       </c>
       <c r="D36" s="9"/>
       <c r="E36" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -2525,7 +2692,7 @@
       <c r="L36" s="9"/>
       <c r="M36" s="9"/>
       <c r="N36" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2540,7 +2707,7 @@
       </c>
       <c r="D37" s="9"/>
       <c r="E37" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
@@ -2551,7 +2718,7 @@
       <c r="L37" s="9"/>
       <c r="M37" s="9"/>
       <c r="N37" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2566,7 +2733,7 @@
       </c>
       <c r="D38" s="9"/>
       <c r="E38" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F38" s="9"/>
       <c r="G38" s="9"/>
@@ -2577,7 +2744,7 @@
       <c r="L38" s="9"/>
       <c r="M38" s="9"/>
       <c r="N38" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2585,14 +2752,14 @@
         <v>38</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C39" s="10" t="n">
         <v>46335</v>
       </c>
       <c r="D39" s="9"/>
       <c r="E39" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F39" s="9"/>
       <c r="G39" s="9"/>
@@ -2603,7 +2770,7 @@
       <c r="L39" s="9"/>
       <c r="M39" s="9"/>
       <c r="N39" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2611,14 +2778,14 @@
         <v>39</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="C40" s="10" t="n">
         <v>46336</v>
       </c>
       <c r="D40" s="9"/>
       <c r="E40" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F40" s="9"/>
       <c r="G40" s="9"/>
@@ -2629,7 +2796,7 @@
       <c r="L40" s="9"/>
       <c r="M40" s="9"/>
       <c r="N40" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2643,37 +2810,37 @@
         <v>46337</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>149</v>
+        <v>175</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>150</v>
+        <v>176</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>151</v>
+        <v>177</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>152</v>
+        <v>178</v>
       </c>
       <c r="I41" s="6" t="s">
-        <v>153</v>
+        <v>179</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>154</v>
+        <v>180</v>
       </c>
       <c r="K41" s="8" t="s">
-        <v>155</v>
+        <v>181</v>
       </c>
       <c r="L41" s="6" t="s">
-        <v>156</v>
+        <v>182</v>
       </c>
       <c r="M41" s="6" t="s">
         <v>52</v>
       </c>
       <c r="N41" s="6" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2688,7 +2855,7 @@
       </c>
       <c r="D42" s="9"/>
       <c r="E42" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F42" s="9"/>
       <c r="G42" s="9"/>
@@ -2699,7 +2866,7 @@
       <c r="L42" s="9"/>
       <c r="M42" s="9"/>
       <c r="N42" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2714,7 +2881,7 @@
       </c>
       <c r="D43" s="9"/>
       <c r="E43" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F43" s="9"/>
       <c r="G43" s="9"/>
@@ -2725,7 +2892,7 @@
       <c r="L43" s="9"/>
       <c r="M43" s="9"/>
       <c r="N43" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2740,7 +2907,7 @@
       </c>
       <c r="D44" s="9"/>
       <c r="E44" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F44" s="9"/>
       <c r="G44" s="9"/>
@@ -2751,7 +2918,7 @@
       <c r="L44" s="9"/>
       <c r="M44" s="9"/>
       <c r="N44" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2766,7 +2933,7 @@
       </c>
       <c r="D45" s="9"/>
       <c r="E45" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F45" s="9"/>
       <c r="G45" s="9"/>
@@ -2777,7 +2944,7 @@
       <c r="L45" s="9"/>
       <c r="M45" s="9"/>
       <c r="N45" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2785,14 +2952,14 @@
         <v>45</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C46" s="10" t="n">
         <v>46342</v>
       </c>
       <c r="D46" s="9"/>
       <c r="E46" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F46" s="9"/>
       <c r="G46" s="9"/>
@@ -2803,7 +2970,7 @@
       <c r="L46" s="9"/>
       <c r="M46" s="9"/>
       <c r="N46" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2811,14 +2978,14 @@
         <v>46</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="C47" s="10" t="n">
         <v>46343</v>
       </c>
       <c r="D47" s="9"/>
       <c r="E47" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F47" s="9"/>
       <c r="G47" s="9"/>
@@ -2829,7 +2996,7 @@
       <c r="L47" s="9"/>
       <c r="M47" s="9"/>
       <c r="N47" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2844,7 +3011,7 @@
       </c>
       <c r="D48" s="9"/>
       <c r="E48" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F48" s="9"/>
       <c r="G48" s="9"/>
@@ -2855,7 +3022,7 @@
       <c r="L48" s="9"/>
       <c r="M48" s="9"/>
       <c r="N48" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2870,7 +3037,7 @@
       </c>
       <c r="D49" s="9"/>
       <c r="E49" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F49" s="9"/>
       <c r="G49" s="9"/>
@@ -2881,7 +3048,7 @@
       <c r="L49" s="9"/>
       <c r="M49" s="9"/>
       <c r="N49" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2896,7 +3063,7 @@
       </c>
       <c r="D50" s="9"/>
       <c r="E50" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F50" s="9"/>
       <c r="G50" s="9"/>
@@ -2907,7 +3074,7 @@
       <c r="L50" s="9"/>
       <c r="M50" s="9"/>
       <c r="N50" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2922,7 +3089,7 @@
       </c>
       <c r="D51" s="9"/>
       <c r="E51" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F51" s="9"/>
       <c r="G51" s="9"/>
@@ -2933,7 +3100,7 @@
       <c r="L51" s="9"/>
       <c r="M51" s="9"/>
       <c r="N51" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2947,37 +3114,37 @@
         <v>46348</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>157</v>
+        <v>183</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>158</v>
+        <v>184</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>159</v>
+        <v>185</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>160</v>
+        <v>186</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>161</v>
+        <v>187</v>
       </c>
       <c r="I52" s="6" t="s">
-        <v>162</v>
+        <v>188</v>
       </c>
       <c r="J52" s="6" t="s">
-        <v>163</v>
+        <v>189</v>
       </c>
       <c r="K52" s="8" t="s">
-        <v>164</v>
+        <v>190</v>
       </c>
       <c r="L52" s="6" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="M52" s="6" t="s">
-        <v>166</v>
+        <v>192</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2985,14 +3152,14 @@
         <v>52</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C53" s="10" t="n">
         <v>46349</v>
       </c>
       <c r="D53" s="9"/>
       <c r="E53" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F53" s="9"/>
       <c r="G53" s="9"/>
@@ -3003,7 +3170,7 @@
       <c r="L53" s="9"/>
       <c r="M53" s="9"/>
       <c r="N53" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3011,14 +3178,14 @@
         <v>53</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="C54" s="10" t="n">
         <v>46350</v>
       </c>
       <c r="D54" s="9"/>
       <c r="E54" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F54" s="9"/>
       <c r="G54" s="9"/>
@@ -3029,7 +3196,7 @@
       <c r="L54" s="9"/>
       <c r="M54" s="9"/>
       <c r="N54" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3044,7 +3211,7 @@
       </c>
       <c r="D55" s="9"/>
       <c r="E55" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F55" s="9"/>
       <c r="G55" s="9"/>
@@ -3055,7 +3222,7 @@
       <c r="L55" s="9"/>
       <c r="M55" s="9"/>
       <c r="N55" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3070,7 +3237,7 @@
       </c>
       <c r="D56" s="9"/>
       <c r="E56" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F56" s="9"/>
       <c r="G56" s="9"/>
@@ -3081,7 +3248,7 @@
       <c r="L56" s="9"/>
       <c r="M56" s="9"/>
       <c r="N56" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3098,34 +3265,34 @@
         <v>53</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>167</v>
+        <v>193</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>168</v>
+        <v>194</v>
       </c>
       <c r="G57" s="11" t="s">
-        <v>169</v>
+        <v>195</v>
       </c>
       <c r="H57" s="11" t="s">
-        <v>170</v>
+        <v>196</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>172</v>
+        <v>198</v>
       </c>
       <c r="K57" s="13" t="s">
-        <v>173</v>
+        <v>199</v>
       </c>
       <c r="L57" s="11" t="s">
-        <v>174</v>
+        <v>200</v>
       </c>
       <c r="M57" s="11" t="s">
-        <v>114</v>
+        <v>138</v>
       </c>
       <c r="N57" s="11" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3140,7 +3307,7 @@
       </c>
       <c r="D58" s="9"/>
       <c r="E58" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F58" s="9"/>
       <c r="G58" s="9"/>
@@ -3151,7 +3318,7 @@
       <c r="L58" s="9"/>
       <c r="M58" s="9"/>
       <c r="N58" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3166,7 +3333,7 @@
       </c>
       <c r="D59" s="9"/>
       <c r="E59" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F59" s="9"/>
       <c r="G59" s="9"/>
@@ -3177,7 +3344,7 @@
       <c r="L59" s="9"/>
       <c r="M59" s="9"/>
       <c r="N59" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3185,14 +3352,14 @@
         <v>59</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C60" s="10" t="n">
         <v>46356</v>
       </c>
       <c r="D60" s="9"/>
       <c r="E60" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F60" s="9"/>
       <c r="G60" s="9"/>
@@ -3203,7 +3370,7 @@
       <c r="L60" s="9"/>
       <c r="M60" s="9"/>
       <c r="N60" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3211,14 +3378,14 @@
         <v>60</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="C61" s="10" t="n">
         <v>46357</v>
       </c>
       <c r="D61" s="9"/>
       <c r="E61" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F61" s="9"/>
       <c r="G61" s="9"/>
@@ -3229,7 +3396,7 @@
       <c r="L61" s="9"/>
       <c r="M61" s="9"/>
       <c r="N61" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3244,7 +3411,7 @@
       </c>
       <c r="D62" s="9"/>
       <c r="E62" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F62" s="9"/>
       <c r="G62" s="9"/>
@@ -3255,7 +3422,7 @@
       <c r="L62" s="9"/>
       <c r="M62" s="9"/>
       <c r="N62" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3270,7 +3437,7 @@
       </c>
       <c r="D63" s="9"/>
       <c r="E63" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F63" s="9"/>
       <c r="G63" s="9"/>
@@ -3281,7 +3448,7 @@
       <c r="L63" s="9"/>
       <c r="M63" s="9"/>
       <c r="N63" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3296,7 +3463,7 @@
       </c>
       <c r="D64" s="9"/>
       <c r="E64" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F64" s="9"/>
       <c r="G64" s="9"/>
@@ -3307,7 +3474,7 @@
       <c r="L64" s="9"/>
       <c r="M64" s="9"/>
       <c r="N64" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3322,7 +3489,7 @@
       </c>
       <c r="D65" s="9"/>
       <c r="E65" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F65" s="9"/>
       <c r="G65" s="9"/>
@@ -3333,7 +3500,7 @@
       <c r="L65" s="9"/>
       <c r="M65" s="9"/>
       <c r="N65" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3348,7 +3515,7 @@
       </c>
       <c r="D66" s="9"/>
       <c r="E66" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F66" s="9"/>
       <c r="G66" s="9"/>
@@ -3359,7 +3526,7 @@
       <c r="L66" s="9"/>
       <c r="M66" s="9"/>
       <c r="N66" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3367,14 +3534,14 @@
         <v>66</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C67" s="10" t="n">
         <v>46363</v>
       </c>
       <c r="D67" s="9"/>
       <c r="E67" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F67" s="9"/>
       <c r="G67" s="9"/>
@@ -3385,7 +3552,7 @@
       <c r="L67" s="9"/>
       <c r="M67" s="9"/>
       <c r="N67" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3393,14 +3560,14 @@
         <v>67</v>
       </c>
       <c r="B68" s="9" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="C68" s="10" t="n">
         <v>46364</v>
       </c>
       <c r="D68" s="9"/>
       <c r="E68" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F68" s="9"/>
       <c r="G68" s="9"/>
@@ -3411,7 +3578,7 @@
       <c r="L68" s="9"/>
       <c r="M68" s="9"/>
       <c r="N68" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3425,37 +3592,37 @@
         <v>46365</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>175</v>
+        <v>201</v>
       </c>
       <c r="F69" s="6" t="s">
-        <v>176</v>
+        <v>202</v>
       </c>
       <c r="G69" s="6" t="s">
-        <v>177</v>
+        <v>203</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>178</v>
+        <v>204</v>
       </c>
       <c r="I69" s="6" t="s">
-        <v>179</v>
+        <v>205</v>
       </c>
       <c r="J69" s="6" t="s">
-        <v>180</v>
+        <v>206</v>
       </c>
       <c r="K69" s="8" t="s">
-        <v>181</v>
+        <v>207</v>
       </c>
       <c r="L69" s="6" t="s">
-        <v>182</v>
+        <v>208</v>
       </c>
       <c r="M69" s="6" t="s">
         <v>52</v>
       </c>
       <c r="N69" s="6" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3470,7 +3637,7 @@
       </c>
       <c r="D70" s="9"/>
       <c r="E70" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F70" s="9"/>
       <c r="G70" s="9"/>
@@ -3481,7 +3648,7 @@
       <c r="L70" s="9"/>
       <c r="M70" s="9"/>
       <c r="N70" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3496,7 +3663,7 @@
       </c>
       <c r="D71" s="9"/>
       <c r="E71" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F71" s="9"/>
       <c r="G71" s="9"/>
@@ -3507,7 +3674,7 @@
       <c r="L71" s="9"/>
       <c r="M71" s="9"/>
       <c r="N71" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3522,7 +3689,7 @@
       </c>
       <c r="D72" s="9"/>
       <c r="E72" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F72" s="9"/>
       <c r="G72" s="9"/>
@@ -3533,7 +3700,7 @@
       <c r="L72" s="9"/>
       <c r="M72" s="9"/>
       <c r="N72" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3548,7 +3715,7 @@
       </c>
       <c r="D73" s="9"/>
       <c r="E73" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F73" s="9"/>
       <c r="G73" s="9"/>
@@ -3559,7 +3726,7 @@
       <c r="L73" s="9"/>
       <c r="M73" s="9"/>
       <c r="N73" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3567,14 +3734,14 @@
         <v>73</v>
       </c>
       <c r="B74" s="9" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C74" s="10" t="n">
         <v>46370</v>
       </c>
       <c r="D74" s="9"/>
       <c r="E74" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F74" s="9"/>
       <c r="G74" s="9"/>
@@ -3585,7 +3752,7 @@
       <c r="L74" s="9"/>
       <c r="M74" s="9"/>
       <c r="N74" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3593,14 +3760,14 @@
         <v>74</v>
       </c>
       <c r="B75" s="9" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="C75" s="10" t="n">
         <v>46371</v>
       </c>
       <c r="D75" s="9"/>
       <c r="E75" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F75" s="9"/>
       <c r="G75" s="9"/>
@@ -3611,7 +3778,7 @@
       <c r="L75" s="9"/>
       <c r="M75" s="9"/>
       <c r="N75" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3625,37 +3792,37 @@
         <v>46372</v>
       </c>
       <c r="D76" s="11" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
       <c r="E76" s="11" t="s">
-        <v>183</v>
+        <v>209</v>
       </c>
       <c r="F76" s="11" t="s">
-        <v>184</v>
+        <v>210</v>
       </c>
       <c r="G76" s="11" t="s">
-        <v>185</v>
+        <v>211</v>
       </c>
       <c r="H76" s="11" t="s">
-        <v>186</v>
+        <v>212</v>
       </c>
       <c r="I76" s="11" t="s">
-        <v>187</v>
+        <v>213</v>
       </c>
       <c r="J76" s="11" t="s">
-        <v>188</v>
+        <v>214</v>
       </c>
       <c r="K76" s="13" t="s">
-        <v>189</v>
+        <v>215</v>
       </c>
       <c r="L76" s="11" t="s">
-        <v>190</v>
+        <v>216</v>
       </c>
       <c r="M76" s="11" t="s">
-        <v>191</v>
+        <v>217</v>
       </c>
       <c r="N76" s="11" t="s">
-        <v>96</v>
+        <v>120</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3670,7 +3837,7 @@
       </c>
       <c r="D77" s="9"/>
       <c r="E77" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F77" s="9"/>
       <c r="G77" s="9"/>
@@ -3681,7 +3848,7 @@
       <c r="L77" s="9"/>
       <c r="M77" s="9"/>
       <c r="N77" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3696,7 +3863,7 @@
       </c>
       <c r="D78" s="9"/>
       <c r="E78" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F78" s="9"/>
       <c r="G78" s="9"/>
@@ -3707,7 +3874,7 @@
       <c r="L78" s="9"/>
       <c r="M78" s="9"/>
       <c r="N78" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3722,7 +3889,7 @@
       </c>
       <c r="D79" s="9"/>
       <c r="E79" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F79" s="9"/>
       <c r="G79" s="9"/>
@@ -3733,7 +3900,7 @@
       <c r="L79" s="9"/>
       <c r="M79" s="9"/>
       <c r="N79" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3748,7 +3915,7 @@
       </c>
       <c r="D80" s="9"/>
       <c r="E80" s="9" t="s">
-        <v>83</v>
+        <v>173</v>
       </c>
       <c r="F80" s="9"/>
       <c r="G80" s="9"/>
@@ -3759,7 +3926,7 @@
       <c r="L80" s="9"/>
       <c r="M80" s="9"/>
       <c r="N80" s="9" t="s">
-        <v>84</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -3795,15 +3962,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>192</v>
+        <v>218</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>193</v>
+        <v>219</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>194</v>
+        <v>220</v>
       </c>
       <c r="B2" s="15" t="n">
         <f aca="false">COUNTA('Lịch đăng'!$A$2:$A$80)</f>
@@ -3821,20 +3988,20 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>195</v>
+        <v>221</v>
       </c>
       <c r="B4" s="15" t="n">
         <f aca="false">COUNTIF('Lịch đăng'!$N$2:$N$80,"Cần chủ đề")</f>
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>196</v>
+        <v>222</v>
       </c>
       <c r="B5" s="15" t="n">
         <f aca="false">B2-B3-B4</f>
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Kịch bản tuần 11-18/10 chờ duyệt, ảnh duyệt trên hub, danh sách tự thu gọn khi chữ dài
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dpu4oyZ8FYSVLE8FrdnGTC
</commit_message>
<xml_diff>
--- a/video/plan/lich-noi-dung-tiktok.xlsx
+++ b/video/plan/lich-noi-dung-tiktok.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="220">
   <si>
     <t xml:space="preserve">Lịch nội dung TikTok Adtek</t>
   </si>
@@ -336,7 +336,7 @@
     <t xml:space="preserve">kol; review sản phẩm; đánh giá 5 sao; chốt đơn</t>
   </si>
   <si>
-    <t xml:space="preserve">Đã kiểm tra nguồn</t>
+    <t xml:space="preserve">Đã viết kịch bản</t>
   </si>
   <si>
     <t xml:space="preserve">Thứ Hai</t>
@@ -414,81 +414,60 @@
     <t xml:space="preserve">Performance</t>
   </si>
   <si>
-    <t xml:space="preserve">Quảng cáo Facebook đắt hơn, có nên giao cho AI?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quảng cáo Facebook đắt hơn 12% so với năm ngoái. Có nên giao hết cho AI chạy?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Quý 2/2026: giá trung bình mỗi quảng cáo +12%, lượt hiển thị +14%, doanh thu Meta 60.8 tỷ USD (+28%)
-• Advantage+ vượt 75 tỷ USD doanh thu quy năm (quý 2/2026), từ 60 tỷ USD (quý 3/2025)
-• Thêm 14% chuyển đổi với CPA/ROAS tương đương; 27% với chiến dịch chủ yếu đối sánh chính xác
-• Bing đổi tiêu đề quảng cáo: doanh thu +12%, hơn 100 triệu USD/năm; chỉ 10-20% thử nghiệm ở Google, Bing cho kết quả tích cực</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Meta, "Meta Reports Second Quarter 2026 Results", 29/07/2026
-• Meta, kết quả kinh doanh Q2 2026, 29/07/2026
-• Google Ads &amp; Commerce Blog, AI Max for Search, 05/2025
-• Kohavi và Thomke, Harvard Business Review, 09/2017</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://investor.atmeta.com
-https://investor.atmeta.com
-https://blog.google/products/ads-commerce/
-https://hbr.org/2017/09/the-surprising-power-of-online-experiments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Link trang nhà đầu tư Meta; Chưa mở được trang gốc (mạng chặn), đối chiếu qua Nasdaq, SEC 10-Q
-• Link trang nhà đầu tư Meta; Chưa mở được trang gốc (mạng chặn), đối chiếu qua MarketBeat, MediaPost
-• Chưa có link bài cụ thể; Chưa mở được trang gốc (mạng chặn), đối chiếu qua MediaPost, Campaign Asia
-• Chưa mở được trang gốc (mạng chặn), đối chiếu qua sách của Kohavi (Cambridge University Press)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Số toàn cầu. Hợp đăng đầu mùa sale cuối năm
-• Số toàn cầu, Meta tự công bố
-• Số liệu Google tự công bố, video nên nói rõ cần tự thử nghiệm
-• Case năm 2012</t>
-  </si>
-  <si>
-    <t xml:space="preserve">quảng cáo facebook 2026; advantage+; ai max</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ý tưởng</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Livestream bán hàng: người mua tin ai?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">650,000 nhà bán đang livestream. Người mua thật sự tin ai?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Việt Nam có 650,000 nhà bán thương mại video (+60%); thương mại video chiếm ~25% GMV TMĐT Đông Nam Á
-• Live commerce chiếm ~67% chi tiêu online của người mua livestream; ~50% thích mua từ tài khoản chính hãng, gần gấp đôi qua KOL; chỉ 13% mua bốc đồng
-• Luật Thương mại điện tử 122/2025/QH15, hiệu lực 01/07/2026: người livestream và affiliate phải xác thực danh tính; nền tảng lưu buổi live tối thiểu 1 năm
-• Nghị định 87/2026/NĐ-CP, hiệu lực 15/05/2026: chưa dùng sản phẩm mà giới thiệu phạt 80-100 triệu đồng; không thông báo việc quảng cáo 60-80 triệu đồng</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Google, Temasek, Bain &amp; Company, e-Conomy SEA 2025, 11/2025
-• Q&amp;Me, Xu hướng Live Commerce và hành vi người mua Việt Nam, 04/2026
-• Quốc hội, Luật Thương mại điện tử 122/2025/QH15
-• Chính phủ, Nghị định 87/2026/NĐ-CP; Luật Quảng cáo sửa đổi 75/2025/QH15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://economysea.withgoogle.com/
-https://qandme.net/vi/baibaocao/xu-huong-live-commerce-va-hanh-vi-nguoi-mua-viet-nam.html
-https://thuvienphapluat.vn/van-ban/Thuong-mai/Luat-Thuong-mai-dien-tu-2025-so-122-2025-QH15-662035.aspx
-https://vbpl.vn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Chưa mở được trang gốc (mạng chặn), đối chiếu qua VnEconomy, Vietstock
-• Chưa mở được trang gốc (mạng chặn), đối chiếu qua VnEconomy
-• Chưa mở được trang gốc (mạng chặn), đối chiếu qua Tiền Phong
-• Chưa có link văn bản cụ thể; Chưa mở được trang gốc (mạng chặn), đối chiếu qua Tạp chí Luật sư Việt Nam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Mẫu 245 người ở TP.HCM và Hà Nội, video phải nói rõ
-• Nội dung pháp lý, nên nhờ luật sư duyệt
-• Cần kiểm tra mức phạt áp cho cá nhân hay tổ chức</t>
+    <t xml:space="preserve">Giá quảng cáo Meta +12%, có nên giao hết cho Advantage+?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quảng cáo Facebook đang đắt lên, có nên giao hết cho AI chạy?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Giá mỗi quảng cáo Meta +12%, lượt hiển thị +14% (quý 2/2026)
+• Advantage+ vượt 75 tỷ USD/năm, từ 60 tỷ (quý 3/2025)
+• Haus, 640 thử nghiệm: 58% thương hiệu hiệu quả hơn khi tự cài chiến dịch; sau khi tắt quảng cáo: tự cài +32%, Advantage+ +17%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Meta, kết quả quý 2/2026 (29/07/2026) và họp công bố quý 3/2025, quý 2/2026
+• Haus, The Meta report: 640 incrementality experiments, 07/2025
+• Việc làm ngay: Trung tâm trợ giúp Meta Business (A/B testing, Audience segments, giới hạn chi khách cũ, Incremental attribution)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://s21.q4cdn.com/399680738/files/doc_news/Meta-Reports-Second-Quarter-2026-Results-2026.pdf
+https://www.haus.io/blog/the-meta-report-lessons-from-640-haus-incrementality-experiments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Đã mở trang gốc (10/10/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Toàn bộ là số liệu toàn cầu (không tìm được số Việt Nam kiểm chứng được), ghi rõ trên video
+• Số Advantage+ do Meta tự công bố; Haus phần lớn là thương hiệu lớn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">quảng cáo facebook 2026; advantage+; meta ads</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Livestream: chỉ 13% khách mua ngẫu hứng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Livestream sống nhờ khách mua ngẫu hứng?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Chỉ 13% mua ngẫu hứng; 47% đang cân nhắc; 40% định mua từ trước
+• 650,000 người bán và cửa hàng bán qua video (+60%), 1.3 tỷ giao dịch
+• 50% chủ yếu mua từ tài khoản chính thức của thương hiệu
+• Luật TMĐT 122/2025 (từ 01/07/2026): xác thực người live, lưu buổi live 1 năm; Nghị định 87/2026: người có ảnh hưởng giới thiệu hàng chưa dùng phạt 80-100 triệu, tổ chức gấp đôi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Q&amp;Me, Live commerce, 04/2026, 245 người (mẫu nhỏ)
+• e-Conomy SEA 2025, trang 144
+• Luật Thương mại điện tử 122/2025/QH15; Nghị định 87/2026/NĐ-CP (vanban.chinhphu.vn)
+• Việc làm ngay: TikTok Shop Seller University</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://qandme.net/vi/baibaocao/xu-huong-live-commerce-va-hanh-vi-nguoi-mua-viet-nam.html
+https://services.google.com/fh/files/misc/e_conomy_sea_2025_report_combined.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Nội dung pháp lý, nên nhờ luật sư duyệt câu chữ
+• Mẫu Q&amp;Me nhỏ, ghi rõ trên video</t>
   </si>
   <si>
     <t xml:space="preserve">livestream bán hàng; luật livestream; kol bị phạt</t>
@@ -497,35 +476,28 @@
     <t xml:space="preserve">App Marketing</t>
   </si>
   <si>
-    <t xml:space="preserve">Thị trường app Việt Nam đã chạm đỉnh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lượt cài app ở Việt Nam vừa lần đầu đi xuống. Tiền quảng cáo app nên đổ vào đâu?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• 2.17 tỷ lượt cài năm 2024, giảm ~2% năm 2025; tăng hơn 136% từ 2018
-• Android 78% xuống 66%, iOS 22% lên 33% (2017 đến 2025); iOS chiếm 55% lượt cài app tài chính
-• 397 triệu USD chi phí kéo người dùng (Q3/2023 đến Q2/2025); 59% studio game Việt dựa vào quảng cáo trong app</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• AppsFlyer, State of App Marketing in Vietnam 2025, 10/2025
-• AppsFlyer, State of App Marketing in Vietnam 2025
-• AppsFlyer, State of App Marketing in Vietnam 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.appsflyer.com/resources/reports/app-marketing-vietnam/
-https://www.appsflyer.com/resources/reports/app-marketing-vietnam/
-https://www.appsflyer.com/resources/reports/app-marketing-vietnam-report/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Chưa mở được trang gốc (mạng chặn), đối chiếu qua Thị trường Tài chính Tiền tệ, Lao Động
-• Chưa mở được trang gốc (mạng chặn), đối chiếu qua Thị trường Tài chính Tiền tệ, Advertising Vietnam
-• Chưa mở được trang gốc, chỉ có đoạn trích của appsflyer.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Dữ liệu Việt Nam
-• Dữ liệu Việt Nam
-• Là tổng 2 năm, không phải 1 năm</t>
+    <t xml:space="preserve">Thị trường app Việt Nam đã chạm đỉnh?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thị trường app Việt Nam đã chạm đỉnh? Tiền quảng cáo app nên đổ vào đâu?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Lượt cài +136% từ 2018, 2.17 tỷ năm 2024, giảm nhẹ 2025
+• iOS 22% lên 33% (2017-2025); app tài chính iOS 54.5%
+• Quý 2/2026 ngân sách kéo người dùng Android: tài chính +153%, giải trí +194%, game -46%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• AppsFlyer, State of App Marketing in Vietnam 2025, 11/2025
+• AppsFlyer, State of Marketing in APAC 2026, 09/2026
+• Việc làm ngay: Apple custom product pages, Play Console custom store listings, Google Ads App campaigns engagement, AppsFlyer Cohort</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.appsflyer.com/resources/reports/app-marketing-vietnam-report/
+https://www.appsflyer.com/resources/reports/state-of-marketing-apac-report/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Biểu đồ xu hướng dùng chỉ số quy đổi của AppsFlyer, đã ghi rõ
+• Số liệu là lượt cài AppsFlyer đo được, không phải toàn thị trường</t>
   </si>
   <si>
     <t xml:space="preserve">thị trường app việt nam; quảng cáo app; iphone hay android</t>
@@ -534,34 +506,28 @@
     <t xml:space="preserve">Trung bình</t>
   </si>
   <si>
-    <t xml:space="preserve">Bao nhiêu lượt cài app là thật?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trả tiền cho 100 lượt cài app, bao nhiêu lượt là người thật?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Tỷ lệ gian lận ở Việt Nam giảm từ 29% (Q1/2025) xuống 20% (Q1/2026); toàn cầu, 52% lượt cài gian lận giả dạng organic
-• 2025: app tài chính Việt Nam giảm 22% lượt cài, chi phí kéo người dùng giảm 48%; remarketing Đông Nam Á +193%
-• CPI game toàn cầu tăng 30% năm 2025, lên 0.56 USD; tỷ lệ paid/organic tăng 61%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• AppsFlyer, State of Fraud for Marketers 2026, 07/2026
-• AppsFlyer, State of Finance for Marketers APAC 2026, 16/04/2026
-• Adjust, Gaming App Insights Report 2026, 10/03/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.appsflyer.com/resources/reports/state-fraud-marketers/
-https://www.appsflyer.com/resources/reports/apac-finance-marketing/
-https://www.adjust.com/resources/ebooks/mobile-app-trends-2026/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Chưa mở được trang gốc (mạng chặn), đối chiếu qua SecurityBrief, CMOtech Asia
-• Chưa mở được trang gốc (mạng chặn), đối chiếu qua Thị trường Tài chính Tiền tệ
-• Số +61% có trong thông cáo Business Wire; số 0.56 USD và +30% cần đối chiếu file PDF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Dữ liệu Việt Nam
-• Phải mở PDF gốc trước khi dựng</t>
+    <t xml:space="preserve">Bao nhiêu lượt cài app là gian lận? (đố số liệu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cứ 100 lượt cài app ở Việt Nam, bao nhiêu lượt là gian lận? A 5, B 20, C 50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Việt Nam 20% (quý 1/2026), từ 29%; Indonesia 17% xuống 13%
+• App tài chính Việt Nam 46% vs 22% châu Á Thái Bình Dương (2025)
+• Toàn cầu: 52% lượt cài gian lận nằm ở nguồn tự nhiên, affiliate gần 40%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• AppsFlyer, State of Fraud for Marketers 2026, 06/2026
+• AppsFlyer, State of Finance for Marketers APAC 2026
+• Việc làm ngay: AppsFlyer Protect360 và Validation Rules, Adjust Fraud Prevention, Apple AdAttributionKit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.appsflyer.com/resources/reports/state-fraud-marketers-report/
+https://www.appsflyer.com/resources/reports/apac-finance-marketing-report/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Kiểu đố số liệu, ảnh bìa không lộ đáp án
+• Tỷ lệ 20% là toàn thị trường, có thể chỉ Android; mức giảm một phần do một đường dây gian lận bị chặn</t>
   </si>
   <si>
     <t xml:space="preserve">gian lận quảng cáo; cpi là gì; marketing app tài chính</t>
@@ -570,35 +536,31 @@
     <t xml:space="preserve">App Marketing, Digital</t>
   </si>
   <si>
-    <t xml:space="preserve">Người Việt sống trong app bao nhiêu giờ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Người Việt dành bao nhiêu giờ trong các ứng dụng mỗi năm?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Việt Nam thứ 11 thế giới về lượt tải; 127 tỷ giờ dùng app; Q1/2026 app giải trí +76% phiên dùng
-• ~70 triệu người dùng hằng tháng tại Việt Nam; hơn 460 triệu toàn Đông Nam Á
-• 5.3 nghìn tỷ giờ trong app năm 2025 (~3.6 giờ/ngày); chi tiêu in-app 167 tỷ USD (+10%); app không phải game lần đầu vượt game</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Adjust, Mobile App Trends Spotlight: Vietnam 2026, 06/2026
-• TikTok Newsroom, 2025
-• Sensor Tower, State of Mobile 2026, 21/01/2026</t>
+    <t xml:space="preserve">Người Việt sống trong app 127 tỷ giờ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Một năm, người Việt dành bao nhiêu giờ trong app?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• 127 tỷ giờ dùng app năm 2025 (thế giới khoảng 3.6 giờ/người/ngày)
+• Mỗi lần mở app giải trí 24.46 phút (quý 1/2026), Đông Nam Á 14.28 phút
+• App giải trí quý 1/2026: lượt cài +32%, số lần mở +76%
+• Chỉ 8% quay lại ngày hôm sau, ngày 30 còn 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Adjust, Mobile app trends spotlight: Vietnam 2026 (PDF 26/05/2026)
+• Sensor Tower, State of Mobile 2026
+• Việc làm ngay: GA4 Cohort exploration, Firebase In-App Messaging, Google Ads App campaigns engagement, Apple In-App Events</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.adjust.com/blog/vietnam-app-trends-2026/
-https://newsroom.tiktok.com/tiktok-surpasses-460-million-users-in-southeast-asia-inks-partnership-with-vietnams-ministry-of-culture-sports-and-tourism
 https://sensortower.com/blog/state-of-mobile-2026</t>
   </si>
   <si>
-    <t xml:space="preserve">• Chưa mở được trang gốc (mạng chặn), đối chiếu qua VnEconomy
-• Chưa mở được trang gốc (mạng chặn), đối chiếu qua Tuổi Trẻ News, Việt Nam News
-• Chưa mở được trang gốc (mạng chặn), đối chiếu qua PR Newswire, 9to5Mac</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Không đặt chung số 2.88 tỷ lượt tải của Adjust với số 2.17 tỷ của AppsFlyer
-• Cần kiểm tra ngày công bố
-• Số toàn cầu</t>
+    <t xml:space="preserve">• adjust.com chặn truy cập tự động (lỗi 429); đã đọc file PDF gốc của Adjust qua bản đăng lại, khớp số liệu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Số liệu chỉ gồm app Adjust đo được</t>
   </si>
   <si>
     <t xml:space="preserve">thời gian dùng điện thoại; tiktok việt nam; app ai</t>
@@ -634,6 +596,9 @@
   </si>
   <si>
     <t xml:space="preserve">luật bảo vệ dữ liệu cá nhân; data khách hàng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ý tưởng</t>
   </si>
   <si>
     <t xml:space="preserve">Kinh tế số 39 tỷ USD, nhưng người dùng mới gần như không tăng</t>
@@ -1987,7 +1952,7 @@
         <v>52</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>120</v>
+        <v>92</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2004,34 +1969,34 @@
         <v>63</v>
       </c>
       <c r="E14" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="F14" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="G14" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="H14" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="H14" s="6" t="s">
+      <c r="I14" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="I14" s="6" t="s">
+      <c r="J14" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="K14" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="J14" s="6" t="s">
+      <c r="L14" s="6" t="s">
         <v>126</v>
-      </c>
-      <c r="K14" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="L14" s="6" t="s">
-        <v>128</v>
       </c>
       <c r="M14" s="6" t="s">
         <v>52</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>120</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2045,37 +2010,37 @@
         <v>46311</v>
       </c>
       <c r="D15" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="F15" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="G15" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="H15" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="G15" s="11" t="s">
+      <c r="I15" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="H15" s="11" t="s">
+      <c r="J15" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="K15" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="I15" s="11" t="s">
+      <c r="L15" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="J15" s="11" t="s">
+      <c r="M15" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="K15" s="13" t="s">
-        <v>136</v>
-      </c>
-      <c r="L15" s="11" t="s">
-        <v>137</v>
-      </c>
-      <c r="M15" s="11" t="s">
-        <v>138</v>
-      </c>
       <c r="N15" s="11" t="s">
-        <v>120</v>
+        <v>92</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2089,37 +2054,37 @@
         <v>46312</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E16" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="G16" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="H16" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="I16" s="11" t="s">
         <v>140</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="J16" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="K16" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="H16" s="11" t="s">
+      <c r="L16" s="11" t="s">
         <v>142</v>
       </c>
-      <c r="I16" s="11" t="s">
-        <v>143</v>
-      </c>
-      <c r="J16" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="K16" s="13" t="s">
-        <v>145</v>
-      </c>
-      <c r="L16" s="11" t="s">
-        <v>146</v>
-      </c>
       <c r="M16" s="11" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="N16" s="11" t="s">
-        <v>120</v>
+        <v>92</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2133,37 +2098,37 @@
         <v>46313</v>
       </c>
       <c r="D17" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="H17" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="I17" s="11" t="s">
         <v>148</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="J17" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="G17" s="11" t="s">
+      <c r="K17" s="13" t="s">
         <v>150</v>
       </c>
-      <c r="H17" s="11" t="s">
+      <c r="L17" s="11" t="s">
         <v>151</v>
-      </c>
-      <c r="I17" s="11" t="s">
-        <v>152</v>
-      </c>
-      <c r="J17" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="K17" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="L17" s="11" t="s">
-        <v>155</v>
       </c>
       <c r="M17" s="11" t="s">
         <v>52</v>
       </c>
       <c r="N17" s="11" t="s">
-        <v>120</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2177,37 +2142,37 @@
         <v>46314</v>
       </c>
       <c r="D18" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="G18" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="H18" s="11" t="s">
         <v>156</v>
       </c>
-      <c r="E18" s="11" t="s">
+      <c r="I18" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="F18" s="11" t="s">
+      <c r="J18" s="11" t="s">
         <v>158</v>
       </c>
-      <c r="G18" s="11" t="s">
+      <c r="K18" s="13" t="s">
         <v>159</v>
       </c>
-      <c r="H18" s="11" t="s">
+      <c r="L18" s="11" t="s">
         <v>160</v>
-      </c>
-      <c r="I18" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="J18" s="11" t="s">
-        <v>162</v>
-      </c>
-      <c r="K18" s="13" t="s">
-        <v>163</v>
-      </c>
-      <c r="L18" s="11" t="s">
-        <v>164</v>
       </c>
       <c r="M18" s="11" t="s">
         <v>52</v>
       </c>
       <c r="N18" s="11" t="s">
-        <v>120</v>
+        <v>161</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2224,34 +2189,34 @@
         <v>33</v>
       </c>
       <c r="E19" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="G19" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="H19" s="11" t="s">
         <v>165</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="I19" s="11" t="s">
         <v>166</v>
       </c>
-      <c r="G19" s="11" t="s">
+      <c r="J19" s="11" t="s">
         <v>167</v>
       </c>
-      <c r="H19" s="11" t="s">
+      <c r="K19" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="I19" s="11" t="s">
+      <c r="L19" s="11" t="s">
         <v>169</v>
       </c>
-      <c r="J19" s="11" t="s">
-        <v>170</v>
-      </c>
-      <c r="K19" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="L19" s="11" t="s">
-        <v>172</v>
-      </c>
       <c r="M19" s="11" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="N19" s="11" t="s">
-        <v>120</v>
+        <v>161</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2266,7 +2231,7 @@
       </c>
       <c r="D20" s="9"/>
       <c r="E20" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F20" s="9"/>
       <c r="G20" s="9"/>
@@ -2277,7 +2242,7 @@
       <c r="L20" s="9"/>
       <c r="M20" s="9"/>
       <c r="N20" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2292,7 +2257,7 @@
       </c>
       <c r="D21" s="9"/>
       <c r="E21" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F21" s="9"/>
       <c r="G21" s="9"/>
@@ -2303,7 +2268,7 @@
       <c r="L21" s="9"/>
       <c r="M21" s="9"/>
       <c r="N21" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2318,7 +2283,7 @@
       </c>
       <c r="D22" s="9"/>
       <c r="E22" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F22" s="9"/>
       <c r="G22" s="9"/>
@@ -2329,7 +2294,7 @@
       <c r="L22" s="9"/>
       <c r="M22" s="9"/>
       <c r="N22" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2344,7 +2309,7 @@
       </c>
       <c r="D23" s="9"/>
       <c r="E23" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F23" s="9"/>
       <c r="G23" s="9"/>
@@ -2355,7 +2320,7 @@
       <c r="L23" s="9"/>
       <c r="M23" s="9"/>
       <c r="N23" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2370,7 +2335,7 @@
       </c>
       <c r="D24" s="9"/>
       <c r="E24" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F24" s="9"/>
       <c r="G24" s="9"/>
@@ -2381,7 +2346,7 @@
       <c r="L24" s="9"/>
       <c r="M24" s="9"/>
       <c r="N24" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2396,7 +2361,7 @@
       </c>
       <c r="D25" s="9"/>
       <c r="E25" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
@@ -2407,7 +2372,7 @@
       <c r="L25" s="9"/>
       <c r="M25" s="9"/>
       <c r="N25" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2422,7 +2387,7 @@
       </c>
       <c r="D26" s="9"/>
       <c r="E26" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F26" s="9"/>
       <c r="G26" s="9"/>
@@ -2433,7 +2398,7 @@
       <c r="L26" s="9"/>
       <c r="M26" s="9"/>
       <c r="N26" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2448,7 +2413,7 @@
       </c>
       <c r="D27" s="9"/>
       <c r="E27" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F27" s="9"/>
       <c r="G27" s="9"/>
@@ -2459,7 +2424,7 @@
       <c r="L27" s="9"/>
       <c r="M27" s="9"/>
       <c r="N27" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2474,7 +2439,7 @@
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -2485,7 +2450,7 @@
       <c r="L28" s="9"/>
       <c r="M28" s="9"/>
       <c r="N28" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2500,7 +2465,7 @@
       </c>
       <c r="D29" s="9"/>
       <c r="E29" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F29" s="9"/>
       <c r="G29" s="9"/>
@@ -2511,7 +2476,7 @@
       <c r="L29" s="9"/>
       <c r="M29" s="9"/>
       <c r="N29" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2526,7 +2491,7 @@
       </c>
       <c r="D30" s="9"/>
       <c r="E30" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F30" s="9"/>
       <c r="G30" s="9"/>
@@ -2537,7 +2502,7 @@
       <c r="L30" s="9"/>
       <c r="M30" s="9"/>
       <c r="N30" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2552,7 +2517,7 @@
       </c>
       <c r="D31" s="9"/>
       <c r="E31" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F31" s="9"/>
       <c r="G31" s="9"/>
@@ -2563,7 +2528,7 @@
       <c r="L31" s="9"/>
       <c r="M31" s="9"/>
       <c r="N31" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2578,7 +2543,7 @@
       </c>
       <c r="D32" s="9"/>
       <c r="E32" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F32" s="9"/>
       <c r="G32" s="9"/>
@@ -2589,7 +2554,7 @@
       <c r="L32" s="9"/>
       <c r="M32" s="9"/>
       <c r="N32" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2604,7 +2569,7 @@
       </c>
       <c r="D33" s="9"/>
       <c r="E33" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -2615,7 +2580,7 @@
       <c r="L33" s="9"/>
       <c r="M33" s="9"/>
       <c r="N33" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2630,7 +2595,7 @@
       </c>
       <c r="D34" s="9"/>
       <c r="E34" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -2641,7 +2606,7 @@
       <c r="L34" s="9"/>
       <c r="M34" s="9"/>
       <c r="N34" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2656,7 +2621,7 @@
       </c>
       <c r="D35" s="9"/>
       <c r="E35" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -2667,7 +2632,7 @@
       <c r="L35" s="9"/>
       <c r="M35" s="9"/>
       <c r="N35" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2682,7 +2647,7 @@
       </c>
       <c r="D36" s="9"/>
       <c r="E36" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -2693,7 +2658,7 @@
       <c r="L36" s="9"/>
       <c r="M36" s="9"/>
       <c r="N36" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2708,7 +2673,7 @@
       </c>
       <c r="D37" s="9"/>
       <c r="E37" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
@@ -2719,7 +2684,7 @@
       <c r="L37" s="9"/>
       <c r="M37" s="9"/>
       <c r="N37" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2734,7 +2699,7 @@
       </c>
       <c r="D38" s="9"/>
       <c r="E38" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F38" s="9"/>
       <c r="G38" s="9"/>
@@ -2745,7 +2710,7 @@
       <c r="L38" s="9"/>
       <c r="M38" s="9"/>
       <c r="N38" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2760,7 +2725,7 @@
       </c>
       <c r="D39" s="9"/>
       <c r="E39" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F39" s="9"/>
       <c r="G39" s="9"/>
@@ -2771,7 +2736,7 @@
       <c r="L39" s="9"/>
       <c r="M39" s="9"/>
       <c r="N39" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2786,7 +2751,7 @@
       </c>
       <c r="D40" s="9"/>
       <c r="E40" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F40" s="9"/>
       <c r="G40" s="9"/>
@@ -2797,7 +2762,7 @@
       <c r="L40" s="9"/>
       <c r="M40" s="9"/>
       <c r="N40" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2814,34 +2779,34 @@
         <v>111</v>
       </c>
       <c r="E41" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="H41" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="F41" s="6" t="s">
+      <c r="I41" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="G41" s="6" t="s">
+      <c r="J41" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="H41" s="6" t="s">
+      <c r="K41" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="I41" s="6" t="s">
+      <c r="L41" s="6" t="s">
         <v>179</v>
-      </c>
-      <c r="J41" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="K41" s="8" t="s">
-        <v>181</v>
-      </c>
-      <c r="L41" s="6" t="s">
-        <v>182</v>
       </c>
       <c r="M41" s="6" t="s">
         <v>52</v>
       </c>
       <c r="N41" s="6" t="s">
-        <v>120</v>
+        <v>161</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2856,7 +2821,7 @@
       </c>
       <c r="D42" s="9"/>
       <c r="E42" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F42" s="9"/>
       <c r="G42" s="9"/>
@@ -2867,7 +2832,7 @@
       <c r="L42" s="9"/>
       <c r="M42" s="9"/>
       <c r="N42" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2882,7 +2847,7 @@
       </c>
       <c r="D43" s="9"/>
       <c r="E43" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F43" s="9"/>
       <c r="G43" s="9"/>
@@ -2893,7 +2858,7 @@
       <c r="L43" s="9"/>
       <c r="M43" s="9"/>
       <c r="N43" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2908,7 +2873,7 @@
       </c>
       <c r="D44" s="9"/>
       <c r="E44" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F44" s="9"/>
       <c r="G44" s="9"/>
@@ -2919,7 +2884,7 @@
       <c r="L44" s="9"/>
       <c r="M44" s="9"/>
       <c r="N44" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2934,7 +2899,7 @@
       </c>
       <c r="D45" s="9"/>
       <c r="E45" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F45" s="9"/>
       <c r="G45" s="9"/>
@@ -2945,7 +2910,7 @@
       <c r="L45" s="9"/>
       <c r="M45" s="9"/>
       <c r="N45" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2960,7 +2925,7 @@
       </c>
       <c r="D46" s="9"/>
       <c r="E46" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F46" s="9"/>
       <c r="G46" s="9"/>
@@ -2971,7 +2936,7 @@
       <c r="L46" s="9"/>
       <c r="M46" s="9"/>
       <c r="N46" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2986,7 +2951,7 @@
       </c>
       <c r="D47" s="9"/>
       <c r="E47" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F47" s="9"/>
       <c r="G47" s="9"/>
@@ -2997,7 +2962,7 @@
       <c r="L47" s="9"/>
       <c r="M47" s="9"/>
       <c r="N47" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3012,7 +2977,7 @@
       </c>
       <c r="D48" s="9"/>
       <c r="E48" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F48" s="9"/>
       <c r="G48" s="9"/>
@@ -3023,7 +2988,7 @@
       <c r="L48" s="9"/>
       <c r="M48" s="9"/>
       <c r="N48" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3038,7 +3003,7 @@
       </c>
       <c r="D49" s="9"/>
       <c r="E49" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F49" s="9"/>
       <c r="G49" s="9"/>
@@ -3049,7 +3014,7 @@
       <c r="L49" s="9"/>
       <c r="M49" s="9"/>
       <c r="N49" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3064,7 +3029,7 @@
       </c>
       <c r="D50" s="9"/>
       <c r="E50" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F50" s="9"/>
       <c r="G50" s="9"/>
@@ -3075,7 +3040,7 @@
       <c r="L50" s="9"/>
       <c r="M50" s="9"/>
       <c r="N50" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3090,7 +3055,7 @@
       </c>
       <c r="D51" s="9"/>
       <c r="E51" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F51" s="9"/>
       <c r="G51" s="9"/>
@@ -3101,7 +3066,7 @@
       <c r="L51" s="9"/>
       <c r="M51" s="9"/>
       <c r="N51" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3115,37 +3080,37 @@
         <v>46348</v>
       </c>
       <c r="D52" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="E52" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="F52" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="G52" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="E52" s="6" t="s">
+      <c r="H52" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="F52" s="6" t="s">
+      <c r="I52" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="G52" s="6" t="s">
+      <c r="J52" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="H52" s="6" t="s">
+      <c r="K52" s="8" t="s">
         <v>187</v>
       </c>
-      <c r="I52" s="6" t="s">
+      <c r="L52" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="J52" s="6" t="s">
+      <c r="M52" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="K52" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="L52" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="M52" s="6" t="s">
-        <v>192</v>
-      </c>
       <c r="N52" s="6" t="s">
-        <v>120</v>
+        <v>161</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3160,7 +3125,7 @@
       </c>
       <c r="D53" s="9"/>
       <c r="E53" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F53" s="9"/>
       <c r="G53" s="9"/>
@@ -3171,7 +3136,7 @@
       <c r="L53" s="9"/>
       <c r="M53" s="9"/>
       <c r="N53" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3186,7 +3151,7 @@
       </c>
       <c r="D54" s="9"/>
       <c r="E54" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F54" s="9"/>
       <c r="G54" s="9"/>
@@ -3197,7 +3162,7 @@
       <c r="L54" s="9"/>
       <c r="M54" s="9"/>
       <c r="N54" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3212,7 +3177,7 @@
       </c>
       <c r="D55" s="9"/>
       <c r="E55" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F55" s="9"/>
       <c r="G55" s="9"/>
@@ -3223,7 +3188,7 @@
       <c r="L55" s="9"/>
       <c r="M55" s="9"/>
       <c r="N55" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3238,7 +3203,7 @@
       </c>
       <c r="D56" s="9"/>
       <c r="E56" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F56" s="9"/>
       <c r="G56" s="9"/>
@@ -3249,7 +3214,7 @@
       <c r="L56" s="9"/>
       <c r="M56" s="9"/>
       <c r="N56" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3266,34 +3231,34 @@
         <v>53</v>
       </c>
       <c r="E57" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="F57" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="G57" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="H57" s="11" t="s">
         <v>193</v>
       </c>
-      <c r="F57" s="11" t="s">
+      <c r="I57" s="11" t="s">
         <v>194</v>
       </c>
-      <c r="G57" s="11" t="s">
+      <c r="J57" s="11" t="s">
         <v>195</v>
       </c>
-      <c r="H57" s="11" t="s">
+      <c r="K57" s="13" t="s">
         <v>196</v>
       </c>
-      <c r="I57" s="11" t="s">
+      <c r="L57" s="11" t="s">
         <v>197</v>
       </c>
-      <c r="J57" s="11" t="s">
-        <v>198</v>
-      </c>
-      <c r="K57" s="13" t="s">
-        <v>199</v>
-      </c>
-      <c r="L57" s="11" t="s">
-        <v>200</v>
-      </c>
       <c r="M57" s="11" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="N57" s="11" t="s">
-        <v>120</v>
+        <v>161</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3308,7 +3273,7 @@
       </c>
       <c r="D58" s="9"/>
       <c r="E58" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F58" s="9"/>
       <c r="G58" s="9"/>
@@ -3319,7 +3284,7 @@
       <c r="L58" s="9"/>
       <c r="M58" s="9"/>
       <c r="N58" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3334,7 +3299,7 @@
       </c>
       <c r="D59" s="9"/>
       <c r="E59" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F59" s="9"/>
       <c r="G59" s="9"/>
@@ -3345,7 +3310,7 @@
       <c r="L59" s="9"/>
       <c r="M59" s="9"/>
       <c r="N59" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3360,7 +3325,7 @@
       </c>
       <c r="D60" s="9"/>
       <c r="E60" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F60" s="9"/>
       <c r="G60" s="9"/>
@@ -3371,7 +3336,7 @@
       <c r="L60" s="9"/>
       <c r="M60" s="9"/>
       <c r="N60" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3386,7 +3351,7 @@
       </c>
       <c r="D61" s="9"/>
       <c r="E61" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F61" s="9"/>
       <c r="G61" s="9"/>
@@ -3397,7 +3362,7 @@
       <c r="L61" s="9"/>
       <c r="M61" s="9"/>
       <c r="N61" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3412,7 +3377,7 @@
       </c>
       <c r="D62" s="9"/>
       <c r="E62" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F62" s="9"/>
       <c r="G62" s="9"/>
@@ -3423,7 +3388,7 @@
       <c r="L62" s="9"/>
       <c r="M62" s="9"/>
       <c r="N62" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3438,7 +3403,7 @@
       </c>
       <c r="D63" s="9"/>
       <c r="E63" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F63" s="9"/>
       <c r="G63" s="9"/>
@@ -3449,7 +3414,7 @@
       <c r="L63" s="9"/>
       <c r="M63" s="9"/>
       <c r="N63" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3464,7 +3429,7 @@
       </c>
       <c r="D64" s="9"/>
       <c r="E64" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F64" s="9"/>
       <c r="G64" s="9"/>
@@ -3475,7 +3440,7 @@
       <c r="L64" s="9"/>
       <c r="M64" s="9"/>
       <c r="N64" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3490,7 +3455,7 @@
       </c>
       <c r="D65" s="9"/>
       <c r="E65" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F65" s="9"/>
       <c r="G65" s="9"/>
@@ -3501,7 +3466,7 @@
       <c r="L65" s="9"/>
       <c r="M65" s="9"/>
       <c r="N65" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3516,7 +3481,7 @@
       </c>
       <c r="D66" s="9"/>
       <c r="E66" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F66" s="9"/>
       <c r="G66" s="9"/>
@@ -3527,7 +3492,7 @@
       <c r="L66" s="9"/>
       <c r="M66" s="9"/>
       <c r="N66" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3542,7 +3507,7 @@
       </c>
       <c r="D67" s="9"/>
       <c r="E67" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F67" s="9"/>
       <c r="G67" s="9"/>
@@ -3553,7 +3518,7 @@
       <c r="L67" s="9"/>
       <c r="M67" s="9"/>
       <c r="N67" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3568,7 +3533,7 @@
       </c>
       <c r="D68" s="9"/>
       <c r="E68" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F68" s="9"/>
       <c r="G68" s="9"/>
@@ -3579,7 +3544,7 @@
       <c r="L68" s="9"/>
       <c r="M68" s="9"/>
       <c r="N68" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3596,34 +3561,34 @@
         <v>111</v>
       </c>
       <c r="E69" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="G69" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="H69" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="F69" s="6" t="s">
+      <c r="I69" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="G69" s="6" t="s">
+      <c r="J69" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="H69" s="6" t="s">
+      <c r="K69" s="8" t="s">
         <v>204</v>
       </c>
-      <c r="I69" s="6" t="s">
+      <c r="L69" s="6" t="s">
         <v>205</v>
-      </c>
-      <c r="J69" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="K69" s="8" t="s">
-        <v>207</v>
-      </c>
-      <c r="L69" s="6" t="s">
-        <v>208</v>
       </c>
       <c r="M69" s="6" t="s">
         <v>52</v>
       </c>
       <c r="N69" s="6" t="s">
-        <v>120</v>
+        <v>161</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3638,7 +3603,7 @@
       </c>
       <c r="D70" s="9"/>
       <c r="E70" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F70" s="9"/>
       <c r="G70" s="9"/>
@@ -3649,7 +3614,7 @@
       <c r="L70" s="9"/>
       <c r="M70" s="9"/>
       <c r="N70" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3664,7 +3629,7 @@
       </c>
       <c r="D71" s="9"/>
       <c r="E71" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F71" s="9"/>
       <c r="G71" s="9"/>
@@ -3675,7 +3640,7 @@
       <c r="L71" s="9"/>
       <c r="M71" s="9"/>
       <c r="N71" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3690,7 +3655,7 @@
       </c>
       <c r="D72" s="9"/>
       <c r="E72" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F72" s="9"/>
       <c r="G72" s="9"/>
@@ -3701,7 +3666,7 @@
       <c r="L72" s="9"/>
       <c r="M72" s="9"/>
       <c r="N72" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3716,7 +3681,7 @@
       </c>
       <c r="D73" s="9"/>
       <c r="E73" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F73" s="9"/>
       <c r="G73" s="9"/>
@@ -3727,7 +3692,7 @@
       <c r="L73" s="9"/>
       <c r="M73" s="9"/>
       <c r="N73" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3742,7 +3707,7 @@
       </c>
       <c r="D74" s="9"/>
       <c r="E74" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F74" s="9"/>
       <c r="G74" s="9"/>
@@ -3753,7 +3718,7 @@
       <c r="L74" s="9"/>
       <c r="M74" s="9"/>
       <c r="N74" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3768,7 +3733,7 @@
       </c>
       <c r="D75" s="9"/>
       <c r="E75" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F75" s="9"/>
       <c r="G75" s="9"/>
@@ -3779,7 +3744,7 @@
       <c r="L75" s="9"/>
       <c r="M75" s="9"/>
       <c r="N75" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3796,34 +3761,34 @@
         <v>111</v>
       </c>
       <c r="E76" s="11" t="s">
+        <v>206</v>
+      </c>
+      <c r="F76" s="11" t="s">
+        <v>207</v>
+      </c>
+      <c r="G76" s="11" t="s">
+        <v>208</v>
+      </c>
+      <c r="H76" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="F76" s="11" t="s">
+      <c r="I76" s="11" t="s">
         <v>210</v>
       </c>
-      <c r="G76" s="11" t="s">
+      <c r="J76" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="H76" s="11" t="s">
+      <c r="K76" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="I76" s="11" t="s">
+      <c r="L76" s="11" t="s">
         <v>213</v>
       </c>
-      <c r="J76" s="11" t="s">
+      <c r="M76" s="11" t="s">
         <v>214</v>
       </c>
-      <c r="K76" s="13" t="s">
-        <v>215</v>
-      </c>
-      <c r="L76" s="11" t="s">
-        <v>216</v>
-      </c>
-      <c r="M76" s="11" t="s">
-        <v>217</v>
-      </c>
       <c r="N76" s="11" t="s">
-        <v>120</v>
+        <v>161</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3838,7 +3803,7 @@
       </c>
       <c r="D77" s="9"/>
       <c r="E77" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F77" s="9"/>
       <c r="G77" s="9"/>
@@ -3849,7 +3814,7 @@
       <c r="L77" s="9"/>
       <c r="M77" s="9"/>
       <c r="N77" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3864,7 +3829,7 @@
       </c>
       <c r="D78" s="9"/>
       <c r="E78" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F78" s="9"/>
       <c r="G78" s="9"/>
@@ -3875,7 +3840,7 @@
       <c r="L78" s="9"/>
       <c r="M78" s="9"/>
       <c r="N78" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3890,7 +3855,7 @@
       </c>
       <c r="D79" s="9"/>
       <c r="E79" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F79" s="9"/>
       <c r="G79" s="9"/>
@@ -3901,7 +3866,7 @@
       <c r="L79" s="9"/>
       <c r="M79" s="9"/>
       <c r="N79" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3916,7 +3881,7 @@
       </c>
       <c r="D80" s="9"/>
       <c r="E80" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="F80" s="9"/>
       <c r="G80" s="9"/>
@@ -3927,7 +3892,7 @@
       <c r="L80" s="9"/>
       <c r="M80" s="9"/>
       <c r="N80" s="9" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -3963,15 +3928,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B2" s="15" t="n">
         <f aca="false">COUNTA('Lịch đăng'!$A$2:$A$80)</f>
@@ -3989,7 +3954,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="B4" s="15" t="n">
         <f aca="false">COUNTIF('Lịch đăng'!$N$2:$N$80,"Cần chủ đề")</f>
@@ -3998,7 +3963,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B5" s="15" t="n">
         <f aca="false">B2-B3-B4</f>

</xml_diff>

<commit_message>
Sản xuất video 11/10: thuê KOL nổi tiếng là khách sẽ tin?
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dpu4oyZ8FYSVLE8FrdnGTC
</commit_message>
<xml_diff>
--- a/video/plan/lich-noi-dung-tiktok.xlsx
+++ b/video/plan/lich-noi-dung-tiktok.xlsx
@@ -336,9 +336,6 @@
     <t xml:space="preserve">kol; review sản phẩm; đánh giá 5 sao; chốt đơn</t>
   </si>
   <si>
-    <t xml:space="preserve">Đã viết kịch bản</t>
-  </si>
-  <si>
     <t xml:space="preserve">Thứ Hai</t>
   </si>
   <si>
@@ -375,6 +372,9 @@
   </si>
   <si>
     <t xml:space="preserve">shopee mall; tiktok shop mall; bán hàng trên sàn 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đã viết kịch bản</t>
   </si>
   <si>
     <t xml:space="preserve">Thứ Ba</t>
@@ -1820,7 +1820,7 @@
         <v>52</v>
       </c>
       <c r="N10" s="9" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1828,43 +1828,43 @@
         <v>10</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C11" s="10" t="n">
         <v>46307</v>
       </c>
       <c r="D11" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="G11" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="H11" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="I11" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="I11" s="9" t="s">
+      <c r="J11" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="J11" s="9" t="s">
+      <c r="K11" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="K11" s="9" t="s">
+      <c r="L11" s="9" t="s">
         <v>101</v>
-      </c>
-      <c r="L11" s="9" t="s">
-        <v>102</v>
       </c>
       <c r="M11" s="9" t="s">
         <v>52</v>
       </c>
       <c r="N11" s="9" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1896,7 +1896,7 @@
         <v>108</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K12" s="9" t="s">
         <v>109</v>
@@ -1908,7 +1908,7 @@
         <v>52</v>
       </c>
       <c r="N12" s="9" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="135.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1952,7 +1952,7 @@
         <v>52</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1996,7 +1996,7 @@
         <v>52</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2040,7 +2040,7 @@
         <v>135</v>
       </c>
       <c r="N15" s="11" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2084,7 +2084,7 @@
         <v>135</v>
       </c>
       <c r="N16" s="11" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2128,7 +2128,7 @@
         <v>52</v>
       </c>
       <c r="N17" s="11" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2136,7 +2136,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C18" s="12" t="n">
         <v>46314</v>
@@ -2354,7 +2354,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C25" s="10" t="n">
         <v>46321</v>
@@ -2536,7 +2536,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C32" s="10" t="n">
         <v>46328</v>
@@ -2718,7 +2718,7 @@
         <v>38</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C39" s="10" t="n">
         <v>46335</v>
@@ -2918,7 +2918,7 @@
         <v>45</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C46" s="10" t="n">
         <v>46342</v>
@@ -3118,7 +3118,7 @@
         <v>52</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C53" s="10" t="n">
         <v>46349</v>
@@ -3318,7 +3318,7 @@
         <v>59</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C60" s="10" t="n">
         <v>46356</v>
@@ -3500,7 +3500,7 @@
         <v>66</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C67" s="10" t="n">
         <v>46363</v>
@@ -3700,7 +3700,7 @@
         <v>73</v>
       </c>
       <c r="B74" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C74" s="10" t="n">
         <v>46370</v>

</xml_diff>

<commit_message>
Quy tắc xoay vòng 7 dạng video mỗi tuần; lên lịch 4 video dạng mới (20, 21, 22, 28/10); hub có nút tải ảnh lướt theo tuần
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dpu4oyZ8FYSVLE8FrdnGTC
</commit_message>
<xml_diff>
--- a/video/plan/lich-noi-dung-tiktok.xlsx
+++ b/video/plan/lich-noi-dung-tiktok.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="242">
   <si>
     <t xml:space="preserve">Lịch nội dung TikTok Adtek</t>
   </si>
@@ -601,38 +601,100 @@
     <t xml:space="preserve">Ý tưởng</t>
   </si>
   <si>
-    <t xml:space="preserve">Kinh tế số 39 tỷ USD, nhưng người dùng mới gần như không tăng</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kinh tế số Việt Nam 39 tỷ USD. Vì sao tìm khách mới online ngày càng khó?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• GMV kinh tế số 39 tỷ USD (+17%), tăng nhanh thứ 2 Đông Nam Á; thương mại điện tử 25 tỷ USD
-• 85.6 triệu người dùng internet (84.2% dân số), chỉ +508 nghìn (+0.6%); 79 triệu tài khoản mạng xã hội; 137 triệu kết nối di động</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Google, Temasek, Bain &amp; Company, e-Conomy SEA 2025, 11/2025
-• DataReportal (Kepios, We Are Social, Meltwater), Digital 2026: Vietnam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://economysea.withgoogle.com/
-https://datareportal.com/reports/digital-2026-vietnam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Chưa mở được trang gốc (mạng chặn), đối chiếu qua Bộ Công Thương (vntr.moit.gov.vn)
-• Chưa mở được trang gốc, có đoạn trích của datareportal.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Digital 2027 ra khoảng tháng 2, cập nhật nếu đã có</t>
+    <t xml:space="preserve">Bản đồ: kinh tế số Việt Nam tăng 17%, nhanh thứ 2 Đông Nam Á</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kinh tế số Việt Nam tăng nhanh hay chậm so với láng giềng? Năm 2025, con số là 17%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tăng trưởng GMV kinh tế số 2025: Malaysia 19%, Việt Nam 17%, Thái Lan 16%, Philippines 16%, Indonesia 14%, Singapore 7%; Việt Nam 39 tỷ USD (2025, ước tính)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google, Temasek, Bain &amp; Company, e-Conomy SEA 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://services.google.com/fh/files/misc/e_conomy_sea_2025_report_combined.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đã mở báo cáo gốc (trang 84 đến 140)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Số 2025 là ước tính, quy đổi từ 6 tháng đầu năm. Dạng bản đồ.</t>
   </si>
   <si>
     <t xml:space="preserve">kinh tế số việt nam; digital 2026</t>
   </si>
   <si>
+    <t xml:space="preserve">Chữ động: đừng chạy sale 11.11 nếu chưa biết 3 điều này</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chỉ còn 3 tuần nữa là 11.11, bạn định chạy sale mà chưa chuẩn bị gì sao?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.10.2025: 4 sàn bán 6,608 tỷ đồng, 376,000 gian hàng; khách thêm vào giỏ sớm 3 đến 5 ngày; Meta cần khoảng 50 kết quả trong 1 tuần; Google Ads điều chỉnh thời vụ cho sale 1 đến 7 ngày</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metric; Meta Business Help Center; Google Ads Help</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://metric.vn/insights/4-nhom-san-pham-ban-chay-nhat-tren-san-sau-ngay-doi-10-10/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đã mở trang gốc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Gấp hơn 5 lần' và 'gần 29%' là phép tính từ số Metric. Dạng chữ động.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đếm ngược: top 5 từ khóa tăng mạnh nhất trên Google năm 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Năm 2025, người Việt tìm gì trên Google tăng mạnh nhất? Đoán thử hạng 1 rồi comment trước nhé.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xu hướng chung 2025: 5 Pixverse AI, 4 Gemini, 3 Phụ nữ trong các ngành STEM, 2 Chat GPT, 1 Deep Seek</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google Year in Search 2025 Việt Nam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://trends.withgoogle.com/year-in-search/2025/vn/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đã mở trang gốc và trang phương pháp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xếp theo mức tăng, không phải lượt tìm. Đăng trước khi có bản 2026 (đầu tháng 12). Dạng đếm ngược.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Slot trống: chủ đề trend Claude tự chọn khi viết kịch bản thứ Bảy</t>
   </si>
   <si>
     <t xml:space="preserve">Cần chủ đề</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biểu đồ đua: Shopee và TikTok Shop, khoảng cách 22 điểm còn 11 điểm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shopee còn giữ ngôi số 1 được bao lâu? Năm 2024, Shopee chiếm 64% doanh số các sàn, TikTok Shop 29%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thị phần doanh số tháng 1 đến 9/2025: Shopee 59% xuống 54%, TikTok Shop 37% lên 43%; năm 2024: Shopee 64%, TikTok Shop 29%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://metric.vn/insights/metric-bao-cao-thi-truong-san-thuong-mai-dien-tu-viet-nam-quy-3-2025/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đã mở báo cáo và biểu đồ gốc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Không có lượt vượt mặt. Cách video shop Mall (12/10) hơn 2 tuần. Dạng biểu đồ đua.</t>
   </si>
   <si>
     <t xml:space="preserve">TikTok Shop hay Shopee?</t>
@@ -2186,7 +2248,7 @@
         <v>46315</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>33</v>
+        <v>152</v>
       </c>
       <c r="E19" s="11" t="s">
         <v>162</v>
@@ -2216,7 +2278,7 @@
         <v>135</v>
       </c>
       <c r="N19" s="11" t="s">
-        <v>161</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2229,20 +2291,34 @@
       <c r="C20" s="10" t="n">
         <v>46316</v>
       </c>
-      <c r="D20" s="9"/>
+      <c r="D20" s="9" t="s">
+        <v>111</v>
+      </c>
       <c r="E20" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
-      <c r="K20" s="9"/>
+      <c r="F20" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="I20" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="J20" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="K20" s="9" t="s">
+        <v>176</v>
+      </c>
       <c r="L20" s="9"/>
       <c r="M20" s="9"/>
       <c r="N20" s="9" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2255,20 +2331,34 @@
       <c r="C21" s="10" t="n">
         <v>46317</v>
       </c>
-      <c r="D21" s="9"/>
+      <c r="D21" s="9" t="s">
+        <v>177</v>
+      </c>
       <c r="E21" s="9" t="s">
-        <v>170</v>
-      </c>
-      <c r="F21" s="9"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
-      <c r="J21" s="9"/>
-      <c r="K21" s="9"/>
+        <v>178</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="I21" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="J21" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="K21" s="9" t="s">
+        <v>184</v>
+      </c>
       <c r="L21" s="9"/>
       <c r="M21" s="9"/>
       <c r="N21" s="9" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2283,7 +2373,7 @@
       </c>
       <c r="D22" s="9"/>
       <c r="E22" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F22" s="9"/>
       <c r="G22" s="9"/>
@@ -2294,7 +2384,7 @@
       <c r="L22" s="9"/>
       <c r="M22" s="9"/>
       <c r="N22" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2309,7 +2399,7 @@
       </c>
       <c r="D23" s="9"/>
       <c r="E23" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F23" s="9"/>
       <c r="G23" s="9"/>
@@ -2320,7 +2410,7 @@
       <c r="L23" s="9"/>
       <c r="M23" s="9"/>
       <c r="N23" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2335,7 +2425,7 @@
       </c>
       <c r="D24" s="9"/>
       <c r="E24" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F24" s="9"/>
       <c r="G24" s="9"/>
@@ -2346,7 +2436,7 @@
       <c r="L24" s="9"/>
       <c r="M24" s="9"/>
       <c r="N24" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2361,7 +2451,7 @@
       </c>
       <c r="D25" s="9"/>
       <c r="E25" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
@@ -2372,7 +2462,7 @@
       <c r="L25" s="9"/>
       <c r="M25" s="9"/>
       <c r="N25" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2387,7 +2477,7 @@
       </c>
       <c r="D26" s="9"/>
       <c r="E26" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F26" s="9"/>
       <c r="G26" s="9"/>
@@ -2398,7 +2488,7 @@
       <c r="L26" s="9"/>
       <c r="M26" s="9"/>
       <c r="N26" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2411,20 +2501,34 @@
       <c r="C27" s="10" t="n">
         <v>46323</v>
       </c>
-      <c r="D27" s="9"/>
+      <c r="D27" s="9" t="s">
+        <v>63</v>
+      </c>
       <c r="E27" s="9" t="s">
-        <v>170</v>
-      </c>
-      <c r="F27" s="9"/>
-      <c r="G27" s="9"/>
-      <c r="H27" s="9"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="9"/>
-      <c r="K27" s="9"/>
+        <v>187</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="G27" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="H27" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="I27" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="J27" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="K27" s="9" t="s">
+        <v>193</v>
+      </c>
       <c r="L27" s="9"/>
       <c r="M27" s="9"/>
       <c r="N27" s="9" t="s">
-        <v>171</v>
+        <v>72</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2439,7 +2543,7 @@
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -2450,7 +2554,7 @@
       <c r="L28" s="9"/>
       <c r="M28" s="9"/>
       <c r="N28" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2465,7 +2569,7 @@
       </c>
       <c r="D29" s="9"/>
       <c r="E29" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F29" s="9"/>
       <c r="G29" s="9"/>
@@ -2476,7 +2580,7 @@
       <c r="L29" s="9"/>
       <c r="M29" s="9"/>
       <c r="N29" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2491,7 +2595,7 @@
       </c>
       <c r="D30" s="9"/>
       <c r="E30" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F30" s="9"/>
       <c r="G30" s="9"/>
@@ -2502,7 +2606,7 @@
       <c r="L30" s="9"/>
       <c r="M30" s="9"/>
       <c r="N30" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2517,7 +2621,7 @@
       </c>
       <c r="D31" s="9"/>
       <c r="E31" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F31" s="9"/>
       <c r="G31" s="9"/>
@@ -2528,7 +2632,7 @@
       <c r="L31" s="9"/>
       <c r="M31" s="9"/>
       <c r="N31" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2543,7 +2647,7 @@
       </c>
       <c r="D32" s="9"/>
       <c r="E32" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F32" s="9"/>
       <c r="G32" s="9"/>
@@ -2554,7 +2658,7 @@
       <c r="L32" s="9"/>
       <c r="M32" s="9"/>
       <c r="N32" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2569,7 +2673,7 @@
       </c>
       <c r="D33" s="9"/>
       <c r="E33" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -2580,7 +2684,7 @@
       <c r="L33" s="9"/>
       <c r="M33" s="9"/>
       <c r="N33" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2595,7 +2699,7 @@
       </c>
       <c r="D34" s="9"/>
       <c r="E34" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -2606,7 +2710,7 @@
       <c r="L34" s="9"/>
       <c r="M34" s="9"/>
       <c r="N34" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2621,7 +2725,7 @@
       </c>
       <c r="D35" s="9"/>
       <c r="E35" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -2632,7 +2736,7 @@
       <c r="L35" s="9"/>
       <c r="M35" s="9"/>
       <c r="N35" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2647,7 +2751,7 @@
       </c>
       <c r="D36" s="9"/>
       <c r="E36" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -2658,7 +2762,7 @@
       <c r="L36" s="9"/>
       <c r="M36" s="9"/>
       <c r="N36" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2673,7 +2777,7 @@
       </c>
       <c r="D37" s="9"/>
       <c r="E37" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
@@ -2684,7 +2788,7 @@
       <c r="L37" s="9"/>
       <c r="M37" s="9"/>
       <c r="N37" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2699,7 +2803,7 @@
       </c>
       <c r="D38" s="9"/>
       <c r="E38" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F38" s="9"/>
       <c r="G38" s="9"/>
@@ -2710,7 +2814,7 @@
       <c r="L38" s="9"/>
       <c r="M38" s="9"/>
       <c r="N38" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2725,7 +2829,7 @@
       </c>
       <c r="D39" s="9"/>
       <c r="E39" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F39" s="9"/>
       <c r="G39" s="9"/>
@@ -2736,7 +2840,7 @@
       <c r="L39" s="9"/>
       <c r="M39" s="9"/>
       <c r="N39" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2751,7 +2855,7 @@
       </c>
       <c r="D40" s="9"/>
       <c r="E40" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F40" s="9"/>
       <c r="G40" s="9"/>
@@ -2762,7 +2866,7 @@
       <c r="L40" s="9"/>
       <c r="M40" s="9"/>
       <c r="N40" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2779,28 +2883,28 @@
         <v>111</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>172</v>
+        <v>194</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>173</v>
+        <v>195</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>174</v>
+        <v>196</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>175</v>
+        <v>197</v>
       </c>
       <c r="I41" s="6" t="s">
-        <v>176</v>
+        <v>198</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>177</v>
+        <v>199</v>
       </c>
       <c r="K41" s="8" t="s">
-        <v>178</v>
+        <v>200</v>
       </c>
       <c r="L41" s="6" t="s">
-        <v>179</v>
+        <v>201</v>
       </c>
       <c r="M41" s="6" t="s">
         <v>52</v>
@@ -2821,7 +2925,7 @@
       </c>
       <c r="D42" s="9"/>
       <c r="E42" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F42" s="9"/>
       <c r="G42" s="9"/>
@@ -2832,7 +2936,7 @@
       <c r="L42" s="9"/>
       <c r="M42" s="9"/>
       <c r="N42" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2847,7 +2951,7 @@
       </c>
       <c r="D43" s="9"/>
       <c r="E43" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F43" s="9"/>
       <c r="G43" s="9"/>
@@ -2858,7 +2962,7 @@
       <c r="L43" s="9"/>
       <c r="M43" s="9"/>
       <c r="N43" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2873,7 +2977,7 @@
       </c>
       <c r="D44" s="9"/>
       <c r="E44" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F44" s="9"/>
       <c r="G44" s="9"/>
@@ -2884,7 +2988,7 @@
       <c r="L44" s="9"/>
       <c r="M44" s="9"/>
       <c r="N44" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2899,7 +3003,7 @@
       </c>
       <c r="D45" s="9"/>
       <c r="E45" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F45" s="9"/>
       <c r="G45" s="9"/>
@@ -2910,7 +3014,7 @@
       <c r="L45" s="9"/>
       <c r="M45" s="9"/>
       <c r="N45" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2925,7 +3029,7 @@
       </c>
       <c r="D46" s="9"/>
       <c r="E46" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F46" s="9"/>
       <c r="G46" s="9"/>
@@ -2936,7 +3040,7 @@
       <c r="L46" s="9"/>
       <c r="M46" s="9"/>
       <c r="N46" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2951,7 +3055,7 @@
       </c>
       <c r="D47" s="9"/>
       <c r="E47" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F47" s="9"/>
       <c r="G47" s="9"/>
@@ -2962,7 +3066,7 @@
       <c r="L47" s="9"/>
       <c r="M47" s="9"/>
       <c r="N47" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2977,7 +3081,7 @@
       </c>
       <c r="D48" s="9"/>
       <c r="E48" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F48" s="9"/>
       <c r="G48" s="9"/>
@@ -2988,7 +3092,7 @@
       <c r="L48" s="9"/>
       <c r="M48" s="9"/>
       <c r="N48" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3003,7 +3107,7 @@
       </c>
       <c r="D49" s="9"/>
       <c r="E49" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F49" s="9"/>
       <c r="G49" s="9"/>
@@ -3014,7 +3118,7 @@
       <c r="L49" s="9"/>
       <c r="M49" s="9"/>
       <c r="N49" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3029,7 +3133,7 @@
       </c>
       <c r="D50" s="9"/>
       <c r="E50" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F50" s="9"/>
       <c r="G50" s="9"/>
@@ -3040,7 +3144,7 @@
       <c r="L50" s="9"/>
       <c r="M50" s="9"/>
       <c r="N50" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3055,7 +3159,7 @@
       </c>
       <c r="D51" s="9"/>
       <c r="E51" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F51" s="9"/>
       <c r="G51" s="9"/>
@@ -3066,7 +3170,7 @@
       <c r="L51" s="9"/>
       <c r="M51" s="9"/>
       <c r="N51" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3080,34 +3184,34 @@
         <v>46348</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>180</v>
+        <v>202</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>181</v>
+        <v>203</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>182</v>
+        <v>204</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>183</v>
+        <v>205</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>184</v>
+        <v>206</v>
       </c>
       <c r="I52" s="6" t="s">
-        <v>185</v>
+        <v>207</v>
       </c>
       <c r="J52" s="6" t="s">
-        <v>186</v>
+        <v>208</v>
       </c>
       <c r="K52" s="8" t="s">
-        <v>187</v>
+        <v>209</v>
       </c>
       <c r="L52" s="6" t="s">
-        <v>188</v>
+        <v>210</v>
       </c>
       <c r="M52" s="6" t="s">
-        <v>189</v>
+        <v>211</v>
       </c>
       <c r="N52" s="6" t="s">
         <v>161</v>
@@ -3125,7 +3229,7 @@
       </c>
       <c r="D53" s="9"/>
       <c r="E53" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F53" s="9"/>
       <c r="G53" s="9"/>
@@ -3136,7 +3240,7 @@
       <c r="L53" s="9"/>
       <c r="M53" s="9"/>
       <c r="N53" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3151,7 +3255,7 @@
       </c>
       <c r="D54" s="9"/>
       <c r="E54" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F54" s="9"/>
       <c r="G54" s="9"/>
@@ -3162,7 +3266,7 @@
       <c r="L54" s="9"/>
       <c r="M54" s="9"/>
       <c r="N54" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3177,7 +3281,7 @@
       </c>
       <c r="D55" s="9"/>
       <c r="E55" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F55" s="9"/>
       <c r="G55" s="9"/>
@@ -3188,7 +3292,7 @@
       <c r="L55" s="9"/>
       <c r="M55" s="9"/>
       <c r="N55" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3203,7 +3307,7 @@
       </c>
       <c r="D56" s="9"/>
       <c r="E56" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F56" s="9"/>
       <c r="G56" s="9"/>
@@ -3214,7 +3318,7 @@
       <c r="L56" s="9"/>
       <c r="M56" s="9"/>
       <c r="N56" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3231,28 +3335,28 @@
         <v>53</v>
       </c>
       <c r="E57" s="11" t="s">
-        <v>190</v>
+        <v>212</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>191</v>
+        <v>213</v>
       </c>
       <c r="G57" s="11" t="s">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="H57" s="11" t="s">
-        <v>193</v>
+        <v>215</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>194</v>
+        <v>216</v>
       </c>
       <c r="J57" s="11" t="s">
-        <v>195</v>
+        <v>217</v>
       </c>
       <c r="K57" s="13" t="s">
-        <v>196</v>
+        <v>218</v>
       </c>
       <c r="L57" s="11" t="s">
-        <v>197</v>
+        <v>219</v>
       </c>
       <c r="M57" s="11" t="s">
         <v>135</v>
@@ -3273,7 +3377,7 @@
       </c>
       <c r="D58" s="9"/>
       <c r="E58" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F58" s="9"/>
       <c r="G58" s="9"/>
@@ -3284,7 +3388,7 @@
       <c r="L58" s="9"/>
       <c r="M58" s="9"/>
       <c r="N58" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3299,7 +3403,7 @@
       </c>
       <c r="D59" s="9"/>
       <c r="E59" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F59" s="9"/>
       <c r="G59" s="9"/>
@@ -3310,7 +3414,7 @@
       <c r="L59" s="9"/>
       <c r="M59" s="9"/>
       <c r="N59" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3325,7 +3429,7 @@
       </c>
       <c r="D60" s="9"/>
       <c r="E60" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F60" s="9"/>
       <c r="G60" s="9"/>
@@ -3336,7 +3440,7 @@
       <c r="L60" s="9"/>
       <c r="M60" s="9"/>
       <c r="N60" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3351,7 +3455,7 @@
       </c>
       <c r="D61" s="9"/>
       <c r="E61" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F61" s="9"/>
       <c r="G61" s="9"/>
@@ -3362,7 +3466,7 @@
       <c r="L61" s="9"/>
       <c r="M61" s="9"/>
       <c r="N61" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3377,7 +3481,7 @@
       </c>
       <c r="D62" s="9"/>
       <c r="E62" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F62" s="9"/>
       <c r="G62" s="9"/>
@@ -3388,7 +3492,7 @@
       <c r="L62" s="9"/>
       <c r="M62" s="9"/>
       <c r="N62" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3403,7 +3507,7 @@
       </c>
       <c r="D63" s="9"/>
       <c r="E63" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F63" s="9"/>
       <c r="G63" s="9"/>
@@ -3414,7 +3518,7 @@
       <c r="L63" s="9"/>
       <c r="M63" s="9"/>
       <c r="N63" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3429,7 +3533,7 @@
       </c>
       <c r="D64" s="9"/>
       <c r="E64" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F64" s="9"/>
       <c r="G64" s="9"/>
@@ -3440,7 +3544,7 @@
       <c r="L64" s="9"/>
       <c r="M64" s="9"/>
       <c r="N64" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3455,7 +3559,7 @@
       </c>
       <c r="D65" s="9"/>
       <c r="E65" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F65" s="9"/>
       <c r="G65" s="9"/>
@@ -3466,7 +3570,7 @@
       <c r="L65" s="9"/>
       <c r="M65" s="9"/>
       <c r="N65" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3481,7 +3585,7 @@
       </c>
       <c r="D66" s="9"/>
       <c r="E66" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F66" s="9"/>
       <c r="G66" s="9"/>
@@ -3492,7 +3596,7 @@
       <c r="L66" s="9"/>
       <c r="M66" s="9"/>
       <c r="N66" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3507,7 +3611,7 @@
       </c>
       <c r="D67" s="9"/>
       <c r="E67" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F67" s="9"/>
       <c r="G67" s="9"/>
@@ -3518,7 +3622,7 @@
       <c r="L67" s="9"/>
       <c r="M67" s="9"/>
       <c r="N67" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3533,7 +3637,7 @@
       </c>
       <c r="D68" s="9"/>
       <c r="E68" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F68" s="9"/>
       <c r="G68" s="9"/>
@@ -3544,7 +3648,7 @@
       <c r="L68" s="9"/>
       <c r="M68" s="9"/>
       <c r="N68" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3561,28 +3665,28 @@
         <v>111</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>198</v>
+        <v>220</v>
       </c>
       <c r="F69" s="6" t="s">
-        <v>199</v>
+        <v>221</v>
       </c>
       <c r="G69" s="6" t="s">
-        <v>200</v>
+        <v>222</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>201</v>
+        <v>223</v>
       </c>
       <c r="I69" s="6" t="s">
-        <v>202</v>
+        <v>224</v>
       </c>
       <c r="J69" s="6" t="s">
-        <v>203</v>
+        <v>225</v>
       </c>
       <c r="K69" s="8" t="s">
-        <v>204</v>
+        <v>226</v>
       </c>
       <c r="L69" s="6" t="s">
-        <v>205</v>
+        <v>227</v>
       </c>
       <c r="M69" s="6" t="s">
         <v>52</v>
@@ -3603,7 +3707,7 @@
       </c>
       <c r="D70" s="9"/>
       <c r="E70" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F70" s="9"/>
       <c r="G70" s="9"/>
@@ -3614,7 +3718,7 @@
       <c r="L70" s="9"/>
       <c r="M70" s="9"/>
       <c r="N70" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3629,7 +3733,7 @@
       </c>
       <c r="D71" s="9"/>
       <c r="E71" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F71" s="9"/>
       <c r="G71" s="9"/>
@@ -3640,7 +3744,7 @@
       <c r="L71" s="9"/>
       <c r="M71" s="9"/>
       <c r="N71" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3655,7 +3759,7 @@
       </c>
       <c r="D72" s="9"/>
       <c r="E72" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F72" s="9"/>
       <c r="G72" s="9"/>
@@ -3666,7 +3770,7 @@
       <c r="L72" s="9"/>
       <c r="M72" s="9"/>
       <c r="N72" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3681,7 +3785,7 @@
       </c>
       <c r="D73" s="9"/>
       <c r="E73" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F73" s="9"/>
       <c r="G73" s="9"/>
@@ -3692,7 +3796,7 @@
       <c r="L73" s="9"/>
       <c r="M73" s="9"/>
       <c r="N73" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3707,7 +3811,7 @@
       </c>
       <c r="D74" s="9"/>
       <c r="E74" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F74" s="9"/>
       <c r="G74" s="9"/>
@@ -3718,7 +3822,7 @@
       <c r="L74" s="9"/>
       <c r="M74" s="9"/>
       <c r="N74" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3733,7 +3837,7 @@
       </c>
       <c r="D75" s="9"/>
       <c r="E75" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F75" s="9"/>
       <c r="G75" s="9"/>
@@ -3744,7 +3848,7 @@
       <c r="L75" s="9"/>
       <c r="M75" s="9"/>
       <c r="N75" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3761,31 +3865,31 @@
         <v>111</v>
       </c>
       <c r="E76" s="11" t="s">
-        <v>206</v>
+        <v>228</v>
       </c>
       <c r="F76" s="11" t="s">
-        <v>207</v>
+        <v>229</v>
       </c>
       <c r="G76" s="11" t="s">
-        <v>208</v>
+        <v>230</v>
       </c>
       <c r="H76" s="11" t="s">
-        <v>209</v>
+        <v>231</v>
       </c>
       <c r="I76" s="11" t="s">
-        <v>210</v>
+        <v>232</v>
       </c>
       <c r="J76" s="11" t="s">
-        <v>211</v>
+        <v>233</v>
       </c>
       <c r="K76" s="13" t="s">
-        <v>212</v>
+        <v>234</v>
       </c>
       <c r="L76" s="11" t="s">
-        <v>213</v>
+        <v>235</v>
       </c>
       <c r="M76" s="11" t="s">
-        <v>214</v>
+        <v>236</v>
       </c>
       <c r="N76" s="11" t="s">
         <v>161</v>
@@ -3803,7 +3907,7 @@
       </c>
       <c r="D77" s="9"/>
       <c r="E77" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F77" s="9"/>
       <c r="G77" s="9"/>
@@ -3814,7 +3918,7 @@
       <c r="L77" s="9"/>
       <c r="M77" s="9"/>
       <c r="N77" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3829,7 +3933,7 @@
       </c>
       <c r="D78" s="9"/>
       <c r="E78" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F78" s="9"/>
       <c r="G78" s="9"/>
@@ -3840,7 +3944,7 @@
       <c r="L78" s="9"/>
       <c r="M78" s="9"/>
       <c r="N78" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3855,7 +3959,7 @@
       </c>
       <c r="D79" s="9"/>
       <c r="E79" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F79" s="9"/>
       <c r="G79" s="9"/>
@@ -3866,7 +3970,7 @@
       <c r="L79" s="9"/>
       <c r="M79" s="9"/>
       <c r="N79" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3881,7 +3985,7 @@
       </c>
       <c r="D80" s="9"/>
       <c r="E80" s="9" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F80" s="9"/>
       <c r="G80" s="9"/>
@@ -3892,7 +3996,7 @@
       <c r="L80" s="9"/>
       <c r="M80" s="9"/>
       <c r="N80" s="9" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -3928,15 +4032,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>215</v>
+        <v>237</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>216</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="B2" s="15" t="n">
         <f aca="false">COUNTA('Lịch đăng'!$A$2:$A$80)</f>
@@ -3954,20 +4058,20 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>218</v>
+        <v>240</v>
       </c>
       <c r="B4" s="15" t="n">
         <f aca="false">COUNTIF('Lịch đăng'!$N$2:$N$80,"Cần chủ đề")</f>
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>219</v>
+        <v>241</v>
       </c>
       <c r="B5" s="15" t="n">
         <f aca="false">B2-B3-B4</f>
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Video tuần 12 đến 18/10 đã xuất, đưa lên hub kèm ảnh bìa và bộ ảnh lướt 12/10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dpu4oyZ8FYSVLE8FrdnGTC
</commit_message>
<xml_diff>
--- a/video/plan/lich-noi-dung-tiktok.xlsx
+++ b/video/plan/lich-noi-dung-tiktok.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="241">
   <si>
     <t xml:space="preserve">Lịch nội dung TikTok Adtek</t>
   </si>
@@ -372,9 +372,6 @@
   </si>
   <si>
     <t xml:space="preserve">shopee mall; tiktok shop mall; bán hàng trên sàn 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đã viết kịch bản</t>
   </si>
   <si>
     <t xml:space="preserve">Thứ Ba</t>
@@ -1926,7 +1923,7 @@
         <v>52</v>
       </c>
       <c r="N11" s="9" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1934,7 +1931,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C12" s="10" t="n">
         <v>46308</v>
@@ -1943,34 +1940,34 @@
         <v>83</v>
       </c>
       <c r="E12" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="F12" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="G12" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="H12" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="H12" s="9" t="s">
+      <c r="I12" s="9" t="s">
         <v>107</v>
-      </c>
-      <c r="I12" s="9" t="s">
-        <v>108</v>
       </c>
       <c r="J12" s="9" t="s">
         <v>99</v>
       </c>
       <c r="K12" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="L12" s="9" t="s">
         <v>109</v>
-      </c>
-      <c r="L12" s="9" t="s">
-        <v>110</v>
       </c>
       <c r="M12" s="9" t="s">
         <v>52</v>
       </c>
       <c r="N12" s="9" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="135.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1984,37 +1981,37 @@
         <v>46309</v>
       </c>
       <c r="D13" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="E13" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="F13" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="G13" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="H13" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="H13" s="6" t="s">
+      <c r="I13" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="I13" s="6" t="s">
+      <c r="J13" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="J13" s="6" t="s">
+      <c r="K13" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="K13" s="8" t="s">
+      <c r="L13" s="6" t="s">
         <v>118</v>
-      </c>
-      <c r="L13" s="6" t="s">
-        <v>119</v>
       </c>
       <c r="M13" s="6" t="s">
         <v>52</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2031,34 +2028,34 @@
         <v>63</v>
       </c>
       <c r="E14" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="F14" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="G14" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="H14" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="H14" s="6" t="s">
+      <c r="I14" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="I14" s="6" t="s">
+      <c r="J14" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="K14" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="J14" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="K14" s="8" t="s">
+      <c r="L14" s="6" t="s">
         <v>125</v>
-      </c>
-      <c r="L14" s="6" t="s">
-        <v>126</v>
       </c>
       <c r="M14" s="6" t="s">
         <v>52</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2072,37 +2069,37 @@
         <v>46311</v>
       </c>
       <c r="D15" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="E15" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="F15" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="G15" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="G15" s="11" t="s">
+      <c r="H15" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="H15" s="11" t="s">
+      <c r="I15" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="I15" s="11" t="s">
+      <c r="J15" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="K15" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="J15" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="K15" s="13" t="s">
+      <c r="L15" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="L15" s="11" t="s">
+      <c r="M15" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="M15" s="11" t="s">
-        <v>135</v>
-      </c>
       <c r="N15" s="11" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2116,37 +2113,37 @@
         <v>46312</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E16" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="F16" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="G16" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="H16" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="H16" s="11" t="s">
+      <c r="I16" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="I16" s="11" t="s">
+      <c r="J16" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="K16" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="J16" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="K16" s="13" t="s">
+      <c r="L16" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="L16" s="11" t="s">
-        <v>142</v>
-      </c>
       <c r="M16" s="11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="N16" s="11" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2160,37 +2157,37 @@
         <v>46313</v>
       </c>
       <c r="D17" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="E17" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="F17" s="11" t="s">
         <v>144</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="G17" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="G17" s="11" t="s">
+      <c r="H17" s="11" t="s">
         <v>146</v>
       </c>
-      <c r="H17" s="11" t="s">
+      <c r="I17" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="I17" s="11" t="s">
+      <c r="J17" s="11" t="s">
         <v>148</v>
       </c>
-      <c r="J17" s="11" t="s">
+      <c r="K17" s="13" t="s">
         <v>149</v>
       </c>
-      <c r="K17" s="13" t="s">
+      <c r="L17" s="11" t="s">
         <v>150</v>
-      </c>
-      <c r="L17" s="11" t="s">
-        <v>151</v>
       </c>
       <c r="M17" s="11" t="s">
         <v>52</v>
       </c>
       <c r="N17" s="11" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2204,37 +2201,37 @@
         <v>46314</v>
       </c>
       <c r="D18" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="E18" s="11" t="s">
         <v>152</v>
       </c>
-      <c r="E18" s="11" t="s">
+      <c r="F18" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="F18" s="11" t="s">
+      <c r="G18" s="11" t="s">
         <v>154</v>
       </c>
-      <c r="G18" s="11" t="s">
+      <c r="H18" s="11" t="s">
         <v>155</v>
       </c>
-      <c r="H18" s="11" t="s">
+      <c r="I18" s="11" t="s">
         <v>156</v>
       </c>
-      <c r="I18" s="11" t="s">
+      <c r="J18" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="J18" s="11" t="s">
+      <c r="K18" s="13" t="s">
         <v>158</v>
       </c>
-      <c r="K18" s="13" t="s">
+      <c r="L18" s="11" t="s">
         <v>159</v>
-      </c>
-      <c r="L18" s="11" t="s">
-        <v>160</v>
       </c>
       <c r="M18" s="11" t="s">
         <v>52</v>
       </c>
       <c r="N18" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2242,40 +2239,40 @@
         <v>18</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C19" s="12" t="n">
         <v>46315</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E19" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="F19" s="11" t="s">
         <v>162</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="G19" s="11" t="s">
         <v>163</v>
       </c>
-      <c r="G19" s="11" t="s">
+      <c r="H19" s="11" t="s">
         <v>164</v>
       </c>
-      <c r="H19" s="11" t="s">
+      <c r="I19" s="11" t="s">
         <v>165</v>
       </c>
-      <c r="I19" s="11" t="s">
+      <c r="J19" s="11" t="s">
         <v>166</v>
       </c>
-      <c r="J19" s="11" t="s">
+      <c r="K19" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="K19" s="13" t="s">
+      <c r="L19" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="L19" s="11" t="s">
-        <v>169</v>
-      </c>
       <c r="M19" s="11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="N19" s="11" t="s">
         <v>72</v>
@@ -2292,28 +2289,28 @@
         <v>46316</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E20" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="F20" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="G20" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="G20" s="9" t="s">
+      <c r="H20" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="H20" s="9" t="s">
+      <c r="I20" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="I20" s="9" t="s">
+      <c r="J20" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="J20" s="9" t="s">
+      <c r="K20" s="9" t="s">
         <v>175</v>
-      </c>
-      <c r="K20" s="9" t="s">
-        <v>176</v>
       </c>
       <c r="L20" s="9"/>
       <c r="M20" s="9"/>
@@ -2332,28 +2329,28 @@
         <v>46317</v>
       </c>
       <c r="D21" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="E21" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="F21" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="F21" s="9" t="s">
+      <c r="G21" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="G21" s="9" t="s">
+      <c r="H21" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="H21" s="9" t="s">
+      <c r="I21" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="I21" s="9" t="s">
+      <c r="J21" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="J21" s="9" t="s">
+      <c r="K21" s="9" t="s">
         <v>183</v>
-      </c>
-      <c r="K21" s="9" t="s">
-        <v>184</v>
       </c>
       <c r="L21" s="9"/>
       <c r="M21" s="9"/>
@@ -2373,7 +2370,7 @@
       </c>
       <c r="D22" s="9"/>
       <c r="E22" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F22" s="9"/>
       <c r="G22" s="9"/>
@@ -2384,7 +2381,7 @@
       <c r="L22" s="9"/>
       <c r="M22" s="9"/>
       <c r="N22" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2399,7 +2396,7 @@
       </c>
       <c r="D23" s="9"/>
       <c r="E23" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F23" s="9"/>
       <c r="G23" s="9"/>
@@ -2410,7 +2407,7 @@
       <c r="L23" s="9"/>
       <c r="M23" s="9"/>
       <c r="N23" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2425,7 +2422,7 @@
       </c>
       <c r="D24" s="9"/>
       <c r="E24" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F24" s="9"/>
       <c r="G24" s="9"/>
@@ -2436,7 +2433,7 @@
       <c r="L24" s="9"/>
       <c r="M24" s="9"/>
       <c r="N24" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2451,7 +2448,7 @@
       </c>
       <c r="D25" s="9"/>
       <c r="E25" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
@@ -2462,7 +2459,7 @@
       <c r="L25" s="9"/>
       <c r="M25" s="9"/>
       <c r="N25" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2470,14 +2467,14 @@
         <v>25</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C26" s="10" t="n">
         <v>46322</v>
       </c>
       <c r="D26" s="9"/>
       <c r="E26" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F26" s="9"/>
       <c r="G26" s="9"/>
@@ -2488,7 +2485,7 @@
       <c r="L26" s="9"/>
       <c r="M26" s="9"/>
       <c r="N26" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2505,25 +2502,25 @@
         <v>63</v>
       </c>
       <c r="E27" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="F27" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="F27" s="9" t="s">
+      <c r="G27" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="G27" s="9" t="s">
+      <c r="H27" s="9" t="s">
         <v>189</v>
       </c>
-      <c r="H27" s="9" t="s">
+      <c r="I27" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="I27" s="9" t="s">
+      <c r="J27" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="J27" s="9" t="s">
+      <c r="K27" s="9" t="s">
         <v>192</v>
-      </c>
-      <c r="K27" s="9" t="s">
-        <v>193</v>
       </c>
       <c r="L27" s="9"/>
       <c r="M27" s="9"/>
@@ -2543,7 +2540,7 @@
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -2554,7 +2551,7 @@
       <c r="L28" s="9"/>
       <c r="M28" s="9"/>
       <c r="N28" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2569,7 +2566,7 @@
       </c>
       <c r="D29" s="9"/>
       <c r="E29" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F29" s="9"/>
       <c r="G29" s="9"/>
@@ -2580,7 +2577,7 @@
       <c r="L29" s="9"/>
       <c r="M29" s="9"/>
       <c r="N29" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2595,7 +2592,7 @@
       </c>
       <c r="D30" s="9"/>
       <c r="E30" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F30" s="9"/>
       <c r="G30" s="9"/>
@@ -2606,7 +2603,7 @@
       <c r="L30" s="9"/>
       <c r="M30" s="9"/>
       <c r="N30" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2621,7 +2618,7 @@
       </c>
       <c r="D31" s="9"/>
       <c r="E31" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F31" s="9"/>
       <c r="G31" s="9"/>
@@ -2632,7 +2629,7 @@
       <c r="L31" s="9"/>
       <c r="M31" s="9"/>
       <c r="N31" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2647,7 +2644,7 @@
       </c>
       <c r="D32" s="9"/>
       <c r="E32" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F32" s="9"/>
       <c r="G32" s="9"/>
@@ -2658,7 +2655,7 @@
       <c r="L32" s="9"/>
       <c r="M32" s="9"/>
       <c r="N32" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2666,14 +2663,14 @@
         <v>32</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C33" s="10" t="n">
         <v>46329</v>
       </c>
       <c r="D33" s="9"/>
       <c r="E33" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -2684,7 +2681,7 @@
       <c r="L33" s="9"/>
       <c r="M33" s="9"/>
       <c r="N33" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2699,7 +2696,7 @@
       </c>
       <c r="D34" s="9"/>
       <c r="E34" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -2710,7 +2707,7 @@
       <c r="L34" s="9"/>
       <c r="M34" s="9"/>
       <c r="N34" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2725,7 +2722,7 @@
       </c>
       <c r="D35" s="9"/>
       <c r="E35" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -2736,7 +2733,7 @@
       <c r="L35" s="9"/>
       <c r="M35" s="9"/>
       <c r="N35" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2751,7 +2748,7 @@
       </c>
       <c r="D36" s="9"/>
       <c r="E36" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -2762,7 +2759,7 @@
       <c r="L36" s="9"/>
       <c r="M36" s="9"/>
       <c r="N36" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2777,7 +2774,7 @@
       </c>
       <c r="D37" s="9"/>
       <c r="E37" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
@@ -2788,7 +2785,7 @@
       <c r="L37" s="9"/>
       <c r="M37" s="9"/>
       <c r="N37" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2803,7 +2800,7 @@
       </c>
       <c r="D38" s="9"/>
       <c r="E38" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F38" s="9"/>
       <c r="G38" s="9"/>
@@ -2814,7 +2811,7 @@
       <c r="L38" s="9"/>
       <c r="M38" s="9"/>
       <c r="N38" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2829,7 +2826,7 @@
       </c>
       <c r="D39" s="9"/>
       <c r="E39" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F39" s="9"/>
       <c r="G39" s="9"/>
@@ -2840,7 +2837,7 @@
       <c r="L39" s="9"/>
       <c r="M39" s="9"/>
       <c r="N39" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2848,14 +2845,14 @@
         <v>39</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C40" s="10" t="n">
         <v>46336</v>
       </c>
       <c r="D40" s="9"/>
       <c r="E40" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F40" s="9"/>
       <c r="G40" s="9"/>
@@ -2866,7 +2863,7 @@
       <c r="L40" s="9"/>
       <c r="M40" s="9"/>
       <c r="N40" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2880,37 +2877,37 @@
         <v>46337</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E41" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="F41" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="F41" s="6" t="s">
+      <c r="G41" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="G41" s="6" t="s">
+      <c r="H41" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="H41" s="6" t="s">
+      <c r="I41" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="I41" s="6" t="s">
+      <c r="J41" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="J41" s="6" t="s">
+      <c r="K41" s="8" t="s">
         <v>199</v>
       </c>
-      <c r="K41" s="8" t="s">
+      <c r="L41" s="6" t="s">
         <v>200</v>
-      </c>
-      <c r="L41" s="6" t="s">
-        <v>201</v>
       </c>
       <c r="M41" s="6" t="s">
         <v>52</v>
       </c>
       <c r="N41" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2925,7 +2922,7 @@
       </c>
       <c r="D42" s="9"/>
       <c r="E42" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F42" s="9"/>
       <c r="G42" s="9"/>
@@ -2936,7 +2933,7 @@
       <c r="L42" s="9"/>
       <c r="M42" s="9"/>
       <c r="N42" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2951,7 +2948,7 @@
       </c>
       <c r="D43" s="9"/>
       <c r="E43" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F43" s="9"/>
       <c r="G43" s="9"/>
@@ -2962,7 +2959,7 @@
       <c r="L43" s="9"/>
       <c r="M43" s="9"/>
       <c r="N43" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2977,7 +2974,7 @@
       </c>
       <c r="D44" s="9"/>
       <c r="E44" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F44" s="9"/>
       <c r="G44" s="9"/>
@@ -2988,7 +2985,7 @@
       <c r="L44" s="9"/>
       <c r="M44" s="9"/>
       <c r="N44" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3003,7 +3000,7 @@
       </c>
       <c r="D45" s="9"/>
       <c r="E45" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F45" s="9"/>
       <c r="G45" s="9"/>
@@ -3014,7 +3011,7 @@
       <c r="L45" s="9"/>
       <c r="M45" s="9"/>
       <c r="N45" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3029,7 +3026,7 @@
       </c>
       <c r="D46" s="9"/>
       <c r="E46" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F46" s="9"/>
       <c r="G46" s="9"/>
@@ -3040,7 +3037,7 @@
       <c r="L46" s="9"/>
       <c r="M46" s="9"/>
       <c r="N46" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3048,14 +3045,14 @@
         <v>46</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C47" s="10" t="n">
         <v>46343</v>
       </c>
       <c r="D47" s="9"/>
       <c r="E47" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F47" s="9"/>
       <c r="G47" s="9"/>
@@ -3066,7 +3063,7 @@
       <c r="L47" s="9"/>
       <c r="M47" s="9"/>
       <c r="N47" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3081,7 +3078,7 @@
       </c>
       <c r="D48" s="9"/>
       <c r="E48" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F48" s="9"/>
       <c r="G48" s="9"/>
@@ -3092,7 +3089,7 @@
       <c r="L48" s="9"/>
       <c r="M48" s="9"/>
       <c r="N48" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3107,7 +3104,7 @@
       </c>
       <c r="D49" s="9"/>
       <c r="E49" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F49" s="9"/>
       <c r="G49" s="9"/>
@@ -3118,7 +3115,7 @@
       <c r="L49" s="9"/>
       <c r="M49" s="9"/>
       <c r="N49" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3133,7 +3130,7 @@
       </c>
       <c r="D50" s="9"/>
       <c r="E50" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F50" s="9"/>
       <c r="G50" s="9"/>
@@ -3144,7 +3141,7 @@
       <c r="L50" s="9"/>
       <c r="M50" s="9"/>
       <c r="N50" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3159,7 +3156,7 @@
       </c>
       <c r="D51" s="9"/>
       <c r="E51" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F51" s="9"/>
       <c r="G51" s="9"/>
@@ -3170,7 +3167,7 @@
       <c r="L51" s="9"/>
       <c r="M51" s="9"/>
       <c r="N51" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3184,37 +3181,37 @@
         <v>46348</v>
       </c>
       <c r="D52" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="E52" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="E52" s="6" t="s">
+      <c r="F52" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="F52" s="6" t="s">
+      <c r="G52" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="G52" s="6" t="s">
+      <c r="H52" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="H52" s="6" t="s">
+      <c r="I52" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="I52" s="6" t="s">
+      <c r="J52" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="J52" s="6" t="s">
+      <c r="K52" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="K52" s="8" t="s">
+      <c r="L52" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="L52" s="6" t="s">
+      <c r="M52" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="M52" s="6" t="s">
-        <v>211</v>
-      </c>
       <c r="N52" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3229,7 +3226,7 @@
       </c>
       <c r="D53" s="9"/>
       <c r="E53" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F53" s="9"/>
       <c r="G53" s="9"/>
@@ -3240,7 +3237,7 @@
       <c r="L53" s="9"/>
       <c r="M53" s="9"/>
       <c r="N53" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3248,14 +3245,14 @@
         <v>53</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C54" s="10" t="n">
         <v>46350</v>
       </c>
       <c r="D54" s="9"/>
       <c r="E54" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F54" s="9"/>
       <c r="G54" s="9"/>
@@ -3266,7 +3263,7 @@
       <c r="L54" s="9"/>
       <c r="M54" s="9"/>
       <c r="N54" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3281,7 +3278,7 @@
       </c>
       <c r="D55" s="9"/>
       <c r="E55" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F55" s="9"/>
       <c r="G55" s="9"/>
@@ -3292,7 +3289,7 @@
       <c r="L55" s="9"/>
       <c r="M55" s="9"/>
       <c r="N55" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3307,7 +3304,7 @@
       </c>
       <c r="D56" s="9"/>
       <c r="E56" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F56" s="9"/>
       <c r="G56" s="9"/>
@@ -3318,7 +3315,7 @@
       <c r="L56" s="9"/>
       <c r="M56" s="9"/>
       <c r="N56" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3335,34 +3332,34 @@
         <v>53</v>
       </c>
       <c r="E57" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="F57" s="11" t="s">
         <v>212</v>
       </c>
-      <c r="F57" s="11" t="s">
+      <c r="G57" s="11" t="s">
         <v>213</v>
       </c>
-      <c r="G57" s="11" t="s">
+      <c r="H57" s="11" t="s">
         <v>214</v>
       </c>
-      <c r="H57" s="11" t="s">
+      <c r="I57" s="11" t="s">
         <v>215</v>
       </c>
-      <c r="I57" s="11" t="s">
+      <c r="J57" s="11" t="s">
         <v>216</v>
       </c>
-      <c r="J57" s="11" t="s">
+      <c r="K57" s="13" t="s">
         <v>217</v>
       </c>
-      <c r="K57" s="13" t="s">
+      <c r="L57" s="11" t="s">
         <v>218</v>
       </c>
-      <c r="L57" s="11" t="s">
-        <v>219</v>
-      </c>
       <c r="M57" s="11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="N57" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3377,7 +3374,7 @@
       </c>
       <c r="D58" s="9"/>
       <c r="E58" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F58" s="9"/>
       <c r="G58" s="9"/>
@@ -3388,7 +3385,7 @@
       <c r="L58" s="9"/>
       <c r="M58" s="9"/>
       <c r="N58" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3403,7 +3400,7 @@
       </c>
       <c r="D59" s="9"/>
       <c r="E59" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F59" s="9"/>
       <c r="G59" s="9"/>
@@ -3414,7 +3411,7 @@
       <c r="L59" s="9"/>
       <c r="M59" s="9"/>
       <c r="N59" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3429,7 +3426,7 @@
       </c>
       <c r="D60" s="9"/>
       <c r="E60" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F60" s="9"/>
       <c r="G60" s="9"/>
@@ -3440,7 +3437,7 @@
       <c r="L60" s="9"/>
       <c r="M60" s="9"/>
       <c r="N60" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3448,14 +3445,14 @@
         <v>60</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C61" s="10" t="n">
         <v>46357</v>
       </c>
       <c r="D61" s="9"/>
       <c r="E61" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F61" s="9"/>
       <c r="G61" s="9"/>
@@ -3466,7 +3463,7 @@
       <c r="L61" s="9"/>
       <c r="M61" s="9"/>
       <c r="N61" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3481,7 +3478,7 @@
       </c>
       <c r="D62" s="9"/>
       <c r="E62" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F62" s="9"/>
       <c r="G62" s="9"/>
@@ -3492,7 +3489,7 @@
       <c r="L62" s="9"/>
       <c r="M62" s="9"/>
       <c r="N62" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3507,7 +3504,7 @@
       </c>
       <c r="D63" s="9"/>
       <c r="E63" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F63" s="9"/>
       <c r="G63" s="9"/>
@@ -3518,7 +3515,7 @@
       <c r="L63" s="9"/>
       <c r="M63" s="9"/>
       <c r="N63" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3533,7 +3530,7 @@
       </c>
       <c r="D64" s="9"/>
       <c r="E64" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F64" s="9"/>
       <c r="G64" s="9"/>
@@ -3544,7 +3541,7 @@
       <c r="L64" s="9"/>
       <c r="M64" s="9"/>
       <c r="N64" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3559,7 +3556,7 @@
       </c>
       <c r="D65" s="9"/>
       <c r="E65" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F65" s="9"/>
       <c r="G65" s="9"/>
@@ -3570,7 +3567,7 @@
       <c r="L65" s="9"/>
       <c r="M65" s="9"/>
       <c r="N65" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3585,7 +3582,7 @@
       </c>
       <c r="D66" s="9"/>
       <c r="E66" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F66" s="9"/>
       <c r="G66" s="9"/>
@@ -3596,7 +3593,7 @@
       <c r="L66" s="9"/>
       <c r="M66" s="9"/>
       <c r="N66" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3611,7 +3608,7 @@
       </c>
       <c r="D67" s="9"/>
       <c r="E67" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F67" s="9"/>
       <c r="G67" s="9"/>
@@ -3622,7 +3619,7 @@
       <c r="L67" s="9"/>
       <c r="M67" s="9"/>
       <c r="N67" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3630,14 +3627,14 @@
         <v>67</v>
       </c>
       <c r="B68" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C68" s="10" t="n">
         <v>46364</v>
       </c>
       <c r="D68" s="9"/>
       <c r="E68" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F68" s="9"/>
       <c r="G68" s="9"/>
@@ -3648,7 +3645,7 @@
       <c r="L68" s="9"/>
       <c r="M68" s="9"/>
       <c r="N68" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3662,37 +3659,37 @@
         <v>46365</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E69" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="F69" s="6" t="s">
         <v>220</v>
       </c>
-      <c r="F69" s="6" t="s">
+      <c r="G69" s="6" t="s">
         <v>221</v>
       </c>
-      <c r="G69" s="6" t="s">
+      <c r="H69" s="6" t="s">
         <v>222</v>
       </c>
-      <c r="H69" s="6" t="s">
+      <c r="I69" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="I69" s="6" t="s">
+      <c r="J69" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="J69" s="6" t="s">
+      <c r="K69" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="K69" s="8" t="s">
+      <c r="L69" s="6" t="s">
         <v>226</v>
-      </c>
-      <c r="L69" s="6" t="s">
-        <v>227</v>
       </c>
       <c r="M69" s="6" t="s">
         <v>52</v>
       </c>
       <c r="N69" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3707,7 +3704,7 @@
       </c>
       <c r="D70" s="9"/>
       <c r="E70" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F70" s="9"/>
       <c r="G70" s="9"/>
@@ -3718,7 +3715,7 @@
       <c r="L70" s="9"/>
       <c r="M70" s="9"/>
       <c r="N70" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3733,7 +3730,7 @@
       </c>
       <c r="D71" s="9"/>
       <c r="E71" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F71" s="9"/>
       <c r="G71" s="9"/>
@@ -3744,7 +3741,7 @@
       <c r="L71" s="9"/>
       <c r="M71" s="9"/>
       <c r="N71" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3759,7 +3756,7 @@
       </c>
       <c r="D72" s="9"/>
       <c r="E72" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F72" s="9"/>
       <c r="G72" s="9"/>
@@ -3770,7 +3767,7 @@
       <c r="L72" s="9"/>
       <c r="M72" s="9"/>
       <c r="N72" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3785,7 +3782,7 @@
       </c>
       <c r="D73" s="9"/>
       <c r="E73" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F73" s="9"/>
       <c r="G73" s="9"/>
@@ -3796,7 +3793,7 @@
       <c r="L73" s="9"/>
       <c r="M73" s="9"/>
       <c r="N73" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3811,7 +3808,7 @@
       </c>
       <c r="D74" s="9"/>
       <c r="E74" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F74" s="9"/>
       <c r="G74" s="9"/>
@@ -3822,7 +3819,7 @@
       <c r="L74" s="9"/>
       <c r="M74" s="9"/>
       <c r="N74" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3830,14 +3827,14 @@
         <v>74</v>
       </c>
       <c r="B75" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C75" s="10" t="n">
         <v>46371</v>
       </c>
       <c r="D75" s="9"/>
       <c r="E75" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F75" s="9"/>
       <c r="G75" s="9"/>
@@ -3848,7 +3845,7 @@
       <c r="L75" s="9"/>
       <c r="M75" s="9"/>
       <c r="N75" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3862,37 +3859,37 @@
         <v>46372</v>
       </c>
       <c r="D76" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E76" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="F76" s="11" t="s">
         <v>228</v>
       </c>
-      <c r="F76" s="11" t="s">
+      <c r="G76" s="11" t="s">
         <v>229</v>
       </c>
-      <c r="G76" s="11" t="s">
+      <c r="H76" s="11" t="s">
         <v>230</v>
       </c>
-      <c r="H76" s="11" t="s">
+      <c r="I76" s="11" t="s">
         <v>231</v>
       </c>
-      <c r="I76" s="11" t="s">
+      <c r="J76" s="11" t="s">
         <v>232</v>
       </c>
-      <c r="J76" s="11" t="s">
+      <c r="K76" s="13" t="s">
         <v>233</v>
       </c>
-      <c r="K76" s="13" t="s">
+      <c r="L76" s="11" t="s">
         <v>234</v>
       </c>
-      <c r="L76" s="11" t="s">
+      <c r="M76" s="11" t="s">
         <v>235</v>
       </c>
-      <c r="M76" s="11" t="s">
-        <v>236</v>
-      </c>
       <c r="N76" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3907,7 +3904,7 @@
       </c>
       <c r="D77" s="9"/>
       <c r="E77" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F77" s="9"/>
       <c r="G77" s="9"/>
@@ -3918,7 +3915,7 @@
       <c r="L77" s="9"/>
       <c r="M77" s="9"/>
       <c r="N77" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3933,7 +3930,7 @@
       </c>
       <c r="D78" s="9"/>
       <c r="E78" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F78" s="9"/>
       <c r="G78" s="9"/>
@@ -3944,7 +3941,7 @@
       <c r="L78" s="9"/>
       <c r="M78" s="9"/>
       <c r="N78" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3959,7 +3956,7 @@
       </c>
       <c r="D79" s="9"/>
       <c r="E79" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F79" s="9"/>
       <c r="G79" s="9"/>
@@ -3970,7 +3967,7 @@
       <c r="L79" s="9"/>
       <c r="M79" s="9"/>
       <c r="N79" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3985,7 +3982,7 @@
       </c>
       <c r="D80" s="9"/>
       <c r="E80" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F80" s="9"/>
       <c r="G80" s="9"/>
@@ -3996,7 +3993,7 @@
       <c r="L80" s="9"/>
       <c r="M80" s="9"/>
       <c r="N80" s="9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -4032,15 +4029,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
+        <v>236</v>
+      </c>
+      <c r="B1" s="14" t="s">
         <v>237</v>
-      </c>
-      <c r="B1" s="14" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B2" s="15" t="n">
         <f aca="false">COUNTA('Lịch đăng'!$A$2:$A$80)</f>
@@ -4058,7 +4055,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B4" s="15" t="n">
         <f aca="false">COUNTIF('Lịch đăng'!$N$2:$N$80,"Cần chủ đề")</f>
@@ -4067,7 +4064,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B5" s="15" t="n">
         <f aca="false">B2-B3-B4</f>

</xml_diff>

<commit_message>
Đánh dấu video đã đăng (10, 11/10 và Advantage+ đăng sớm 11/10), dồn lịch từ 15/10 lên 1 ngày
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dpu4oyZ8FYSVLE8FrdnGTC
</commit_message>
<xml_diff>
--- a/video/plan/lich-noi-dung-tiktok.xlsx
+++ b/video/plan/lich-noi-dung-tiktok.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="234">
   <si>
     <t xml:space="preserve">Lịch nội dung TikTok Adtek</t>
   </si>
@@ -330,7 +330,8 @@
   <si>
     <t xml:space="preserve">• Kiểu phá hiểu lầm, đóng dấu SAI
 • Mẫu nhỏ (200 người, chỉ HN và HCM), phải ghi rõ trên video
-• Ngày phát hành ước tính cuối 09/2026 Đã nhắc</t>
+• Ngày phát hành ước tính cuối 09/2026 Đã nhắc
+• Ngày 11/10 đăng thêm video "Giá quảng cáo Meta +12%, có nên giao hết cho Advantage+?" (vốn xếp lịch 14/10)</t>
   </si>
   <si>
     <t xml:space="preserve">kol; review sản phẩm; đánh giá 5 sao; chốt đơn</t>
@@ -408,39 +409,6 @@
     <t xml:space="preserve">quảng cáo facebook hay tiktok; chạy quảng cáo youtube; zalo ads</t>
   </si>
   <si>
-    <t xml:space="preserve">Performance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Giá quảng cáo Meta +12%, có nên giao hết cho Advantage+?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quảng cáo Facebook đang đắt lên, có nên giao hết cho AI chạy?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Giá mỗi quảng cáo Meta +12%, lượt hiển thị +14% (quý 2/2026)
-• Advantage+ vượt 75 tỷ USD/năm, từ 60 tỷ (quý 3/2025)
-• Haus, 640 thử nghiệm: 58% thương hiệu hiệu quả hơn khi tự cài chiến dịch; sau khi tắt quảng cáo: tự cài +32%, Advantage+ +17%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Meta, kết quả quý 2/2026 (29/07/2026) và họp công bố quý 3/2025, quý 2/2026
-• Haus, The Meta report: 640 incrementality experiments, 07/2025
-• Việc làm ngay: Trung tâm trợ giúp Meta Business (A/B testing, Audience segments, giới hạn chi khách cũ, Incremental attribution)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://s21.q4cdn.com/399680738/files/doc_news/Meta-Reports-Second-Quarter-2026-Results-2026.pdf
-https://www.haus.io/blog/the-meta-report-lessons-from-640-haus-incrementality-experiments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Đã mở trang gốc (10/10/2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Toàn bộ là số liệu toàn cầu (không tìm được số Việt Nam kiểm chứng được), ghi rõ trên video
-• Số Advantage+ do Meta tự công bố; Haus phần lớn là thương hiệu lớn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">quảng cáo facebook 2026; advantage+; meta ads</t>
-  </si>
-  <si>
     <t xml:space="preserve">Livestream: chỉ 13% khách mua ngẫu hứng</t>
   </si>
   <si>
@@ -463,6 +431,9 @@
 https://services.google.com/fh/files/misc/e_conomy_sea_2025_report_combined.pdf</t>
   </si>
   <si>
+    <t xml:space="preserve">• Đã mở trang gốc (10/10/2026)</t>
+  </si>
+  <si>
     <t xml:space="preserve">• Nội dung pháp lý, nên nhờ luật sư duyệt câu chữ
 • Mẫu Q&amp;Me nhỏ, ghi rõ trên video</t>
   </si>
@@ -620,6 +591,9 @@
   </si>
   <si>
     <t xml:space="preserve">kinh tế số việt nam; digital 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Performance</t>
   </si>
   <si>
     <t xml:space="preserve">Chữ động: đừng chạy sale 11.11 nếu chưa biết 3 điều này</t>
@@ -1835,7 +1809,7 @@
         <v>52</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>72</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1879,7 +1853,7 @@
         <v>52</v>
       </c>
       <c r="N10" s="9" t="s">
-        <v>72</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1981,31 +1955,31 @@
         <v>46309</v>
       </c>
       <c r="D13" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E13" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="F13" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="G13" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="H13" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="H13" s="6" t="s">
+      <c r="I13" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="I13" s="6" t="s">
+      <c r="J13" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="J13" s="6" t="s">
+      <c r="K13" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="K13" s="8" t="s">
+      <c r="L13" s="6" t="s">
         <v>117</v>
-      </c>
-      <c r="L13" s="6" t="s">
-        <v>118</v>
       </c>
       <c r="M13" s="6" t="s">
         <v>52</v>
@@ -2025,7 +1999,7 @@
         <v>46310</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>63</v>
+        <v>118</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>119</v>
@@ -2043,7 +2017,7 @@
         <v>123</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="K14" s="8" t="s">
         <v>124</v>
@@ -2052,7 +2026,7 @@
         <v>125</v>
       </c>
       <c r="M14" s="6" t="s">
-        <v>52</v>
+        <v>126</v>
       </c>
       <c r="N14" s="6" t="s">
         <v>72</v>
@@ -2069,7 +2043,7 @@
         <v>46311</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="E15" s="11" t="s">
         <v>127</v>
@@ -2087,7 +2061,7 @@
         <v>131</v>
       </c>
       <c r="J15" s="11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="K15" s="13" t="s">
         <v>132</v>
@@ -2096,7 +2070,7 @@
         <v>133</v>
       </c>
       <c r="M15" s="11" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="N15" s="11" t="s">
         <v>72</v>
@@ -2113,7 +2087,7 @@
         <v>46312</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="E16" s="11" t="s">
         <v>135</v>
@@ -2131,16 +2105,16 @@
         <v>139</v>
       </c>
       <c r="J16" s="11" t="s">
-        <v>116</v>
+        <v>140</v>
       </c>
       <c r="K16" s="13" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="L16" s="11" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="M16" s="11" t="s">
-        <v>134</v>
+        <v>52</v>
       </c>
       <c r="N16" s="11" t="s">
         <v>72</v>
@@ -2157,37 +2131,37 @@
         <v>46313</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J17" s="11" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K17" s="13" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="L17" s="11" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="M17" s="11" t="s">
         <v>52</v>
       </c>
       <c r="N17" s="11" t="s">
-        <v>72</v>
+        <v>152</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2201,37 +2175,37 @@
         <v>46314</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I18" s="11" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J18" s="11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="K18" s="13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L18" s="11" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="M18" s="11" t="s">
-        <v>52</v>
+        <v>126</v>
       </c>
       <c r="N18" s="11" t="s">
-        <v>160</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2245,35 +2219,31 @@
         <v>46315</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="J19" s="11" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K19" s="13" t="s">
-        <v>167</v>
-      </c>
-      <c r="L19" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="M19" s="11" t="s">
-        <v>134</v>
-      </c>
+      <c r="L19" s="11"/>
+      <c r="M19" s="11"/>
       <c r="N19" s="11" t="s">
         <v>72</v>
       </c>
@@ -2289,28 +2259,28 @@
         <v>46316</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>110</v>
+        <v>169</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K20" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="L20" s="9"/>
       <c r="M20" s="9"/>
@@ -2328,34 +2298,20 @@
       <c r="C21" s="10" t="n">
         <v>46317</v>
       </c>
-      <c r="D21" s="9" t="s">
-        <v>176</v>
-      </c>
+      <c r="D21" s="9"/>
       <c r="E21" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="F21" s="9" t="s">
-        <v>178</v>
-      </c>
-      <c r="G21" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="H21" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="I21" s="9" t="s">
-        <v>181</v>
-      </c>
-      <c r="J21" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="K21" s="9" t="s">
-        <v>183</v>
-      </c>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="9"/>
       <c r="L21" s="9"/>
       <c r="M21" s="9"/>
       <c r="N21" s="9" t="s">
-        <v>72</v>
+        <v>178</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2370,7 +2326,7 @@
       </c>
       <c r="D22" s="9"/>
       <c r="E22" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F22" s="9"/>
       <c r="G22" s="9"/>
@@ -2381,7 +2337,7 @@
       <c r="L22" s="9"/>
       <c r="M22" s="9"/>
       <c r="N22" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2396,7 +2352,7 @@
       </c>
       <c r="D23" s="9"/>
       <c r="E23" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F23" s="9"/>
       <c r="G23" s="9"/>
@@ -2407,7 +2363,7 @@
       <c r="L23" s="9"/>
       <c r="M23" s="9"/>
       <c r="N23" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2422,7 +2378,7 @@
       </c>
       <c r="D24" s="9"/>
       <c r="E24" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F24" s="9"/>
       <c r="G24" s="9"/>
@@ -2433,7 +2389,7 @@
       <c r="L24" s="9"/>
       <c r="M24" s="9"/>
       <c r="N24" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2448,7 +2404,7 @@
       </c>
       <c r="D25" s="9"/>
       <c r="E25" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
@@ -2459,7 +2415,7 @@
       <c r="L25" s="9"/>
       <c r="M25" s="9"/>
       <c r="N25" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2472,20 +2428,34 @@
       <c r="C26" s="10" t="n">
         <v>46322</v>
       </c>
-      <c r="D26" s="9"/>
+      <c r="D26" s="9" t="s">
+        <v>63</v>
+      </c>
       <c r="E26" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="G26" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="H26" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="I26" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="J26" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9"/>
-      <c r="I26" s="9"/>
-      <c r="J26" s="9"/>
-      <c r="K26" s="9"/>
+      <c r="K26" s="9" t="s">
+        <v>185</v>
+      </c>
       <c r="L26" s="9"/>
       <c r="M26" s="9"/>
       <c r="N26" s="9" t="s">
-        <v>185</v>
+        <v>72</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2498,34 +2468,20 @@
       <c r="C27" s="10" t="n">
         <v>46323</v>
       </c>
-      <c r="D27" s="9" t="s">
-        <v>63</v>
-      </c>
+      <c r="D27" s="9"/>
       <c r="E27" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="F27" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="G27" s="9" t="s">
-        <v>188</v>
-      </c>
-      <c r="H27" s="9" t="s">
-        <v>189</v>
-      </c>
-      <c r="I27" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="J27" s="9" t="s">
-        <v>191</v>
-      </c>
-      <c r="K27" s="9" t="s">
-        <v>192</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+      <c r="I27" s="9"/>
+      <c r="J27" s="9"/>
+      <c r="K27" s="9"/>
       <c r="L27" s="9"/>
       <c r="M27" s="9"/>
       <c r="N27" s="9" t="s">
-        <v>72</v>
+        <v>178</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2540,7 +2496,7 @@
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -2551,7 +2507,7 @@
       <c r="L28" s="9"/>
       <c r="M28" s="9"/>
       <c r="N28" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2566,7 +2522,7 @@
       </c>
       <c r="D29" s="9"/>
       <c r="E29" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F29" s="9"/>
       <c r="G29" s="9"/>
@@ -2577,7 +2533,7 @@
       <c r="L29" s="9"/>
       <c r="M29" s="9"/>
       <c r="N29" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2592,7 +2548,7 @@
       </c>
       <c r="D30" s="9"/>
       <c r="E30" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F30" s="9"/>
       <c r="G30" s="9"/>
@@ -2603,7 +2559,7 @@
       <c r="L30" s="9"/>
       <c r="M30" s="9"/>
       <c r="N30" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2618,7 +2574,7 @@
       </c>
       <c r="D31" s="9"/>
       <c r="E31" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F31" s="9"/>
       <c r="G31" s="9"/>
@@ -2629,7 +2585,7 @@
       <c r="L31" s="9"/>
       <c r="M31" s="9"/>
       <c r="N31" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2644,7 +2600,7 @@
       </c>
       <c r="D32" s="9"/>
       <c r="E32" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F32" s="9"/>
       <c r="G32" s="9"/>
@@ -2655,7 +2611,7 @@
       <c r="L32" s="9"/>
       <c r="M32" s="9"/>
       <c r="N32" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2670,7 +2626,7 @@
       </c>
       <c r="D33" s="9"/>
       <c r="E33" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -2681,7 +2637,7 @@
       <c r="L33" s="9"/>
       <c r="M33" s="9"/>
       <c r="N33" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2696,7 +2652,7 @@
       </c>
       <c r="D34" s="9"/>
       <c r="E34" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -2707,7 +2663,7 @@
       <c r="L34" s="9"/>
       <c r="M34" s="9"/>
       <c r="N34" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2722,7 +2678,7 @@
       </c>
       <c r="D35" s="9"/>
       <c r="E35" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -2733,7 +2689,7 @@
       <c r="L35" s="9"/>
       <c r="M35" s="9"/>
       <c r="N35" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2748,7 +2704,7 @@
       </c>
       <c r="D36" s="9"/>
       <c r="E36" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -2759,7 +2715,7 @@
       <c r="L36" s="9"/>
       <c r="M36" s="9"/>
       <c r="N36" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2774,7 +2730,7 @@
       </c>
       <c r="D37" s="9"/>
       <c r="E37" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
@@ -2785,7 +2741,7 @@
       <c r="L37" s="9"/>
       <c r="M37" s="9"/>
       <c r="N37" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2800,7 +2756,7 @@
       </c>
       <c r="D38" s="9"/>
       <c r="E38" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F38" s="9"/>
       <c r="G38" s="9"/>
@@ -2811,7 +2767,7 @@
       <c r="L38" s="9"/>
       <c r="M38" s="9"/>
       <c r="N38" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2826,7 +2782,7 @@
       </c>
       <c r="D39" s="9"/>
       <c r="E39" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F39" s="9"/>
       <c r="G39" s="9"/>
@@ -2837,7 +2793,7 @@
       <c r="L39" s="9"/>
       <c r="M39" s="9"/>
       <c r="N39" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2850,20 +2806,38 @@
       <c r="C40" s="10" t="n">
         <v>46336</v>
       </c>
-      <c r="D40" s="9"/>
+      <c r="D40" s="9" t="s">
+        <v>161</v>
+      </c>
       <c r="E40" s="9" t="s">
-        <v>184</v>
-      </c>
-      <c r="F40" s="9"/>
-      <c r="G40" s="9"/>
-      <c r="H40" s="9"/>
-      <c r="I40" s="9"/>
-      <c r="J40" s="9"/>
-      <c r="K40" s="9"/>
-      <c r="L40" s="9"/>
-      <c r="M40" s="9"/>
+        <v>186</v>
+      </c>
+      <c r="F40" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="G40" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="H40" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="I40" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="J40" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="K40" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="L40" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="M40" s="9" t="s">
+        <v>52</v>
+      </c>
       <c r="N40" s="9" t="s">
-        <v>185</v>
+        <v>152</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2876,38 +2850,20 @@
       <c r="C41" s="7" t="n">
         <v>46337</v>
       </c>
-      <c r="D41" s="6" t="s">
-        <v>110</v>
-      </c>
+      <c r="D41" s="6"/>
       <c r="E41" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="F41" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="G41" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="H41" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="I41" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="J41" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="K41" s="8" t="s">
-        <v>199</v>
-      </c>
-      <c r="L41" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="M41" s="6" t="s">
-        <v>52</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="F41" s="6"/>
+      <c r="G41" s="6"/>
+      <c r="H41" s="6"/>
+      <c r="I41" s="6"/>
+      <c r="J41" s="6"/>
+      <c r="K41" s="8"/>
+      <c r="L41" s="6"/>
+      <c r="M41" s="6"/>
       <c r="N41" s="6" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2922,7 +2878,7 @@
       </c>
       <c r="D42" s="9"/>
       <c r="E42" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F42" s="9"/>
       <c r="G42" s="9"/>
@@ -2933,7 +2889,7 @@
       <c r="L42" s="9"/>
       <c r="M42" s="9"/>
       <c r="N42" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2948,7 +2904,7 @@
       </c>
       <c r="D43" s="9"/>
       <c r="E43" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F43" s="9"/>
       <c r="G43" s="9"/>
@@ -2959,7 +2915,7 @@
       <c r="L43" s="9"/>
       <c r="M43" s="9"/>
       <c r="N43" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2974,7 +2930,7 @@
       </c>
       <c r="D44" s="9"/>
       <c r="E44" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F44" s="9"/>
       <c r="G44" s="9"/>
@@ -2985,7 +2941,7 @@
       <c r="L44" s="9"/>
       <c r="M44" s="9"/>
       <c r="N44" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3000,7 +2956,7 @@
       </c>
       <c r="D45" s="9"/>
       <c r="E45" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F45" s="9"/>
       <c r="G45" s="9"/>
@@ -3011,7 +2967,7 @@
       <c r="L45" s="9"/>
       <c r="M45" s="9"/>
       <c r="N45" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3026,7 +2982,7 @@
       </c>
       <c r="D46" s="9"/>
       <c r="E46" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F46" s="9"/>
       <c r="G46" s="9"/>
@@ -3037,7 +2993,7 @@
       <c r="L46" s="9"/>
       <c r="M46" s="9"/>
       <c r="N46" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3052,7 +3008,7 @@
       </c>
       <c r="D47" s="9"/>
       <c r="E47" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F47" s="9"/>
       <c r="G47" s="9"/>
@@ -3063,7 +3019,7 @@
       <c r="L47" s="9"/>
       <c r="M47" s="9"/>
       <c r="N47" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3078,7 +3034,7 @@
       </c>
       <c r="D48" s="9"/>
       <c r="E48" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F48" s="9"/>
       <c r="G48" s="9"/>
@@ -3089,7 +3045,7 @@
       <c r="L48" s="9"/>
       <c r="M48" s="9"/>
       <c r="N48" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3104,7 +3060,7 @@
       </c>
       <c r="D49" s="9"/>
       <c r="E49" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F49" s="9"/>
       <c r="G49" s="9"/>
@@ -3115,7 +3071,7 @@
       <c r="L49" s="9"/>
       <c r="M49" s="9"/>
       <c r="N49" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3130,7 +3086,7 @@
       </c>
       <c r="D50" s="9"/>
       <c r="E50" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F50" s="9"/>
       <c r="G50" s="9"/>
@@ -3141,7 +3097,7 @@
       <c r="L50" s="9"/>
       <c r="M50" s="9"/>
       <c r="N50" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3154,20 +3110,38 @@
       <c r="C51" s="10" t="n">
         <v>46347</v>
       </c>
-      <c r="D51" s="9"/>
+      <c r="D51" s="9" t="s">
+        <v>194</v>
+      </c>
       <c r="E51" s="9" t="s">
-        <v>184</v>
-      </c>
-      <c r="F51" s="9"/>
-      <c r="G51" s="9"/>
-      <c r="H51" s="9"/>
-      <c r="I51" s="9"/>
-      <c r="J51" s="9"/>
-      <c r="K51" s="9"/>
-      <c r="L51" s="9"/>
-      <c r="M51" s="9"/>
+        <v>195</v>
+      </c>
+      <c r="F51" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="G51" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="H51" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="I51" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="J51" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="K51" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="L51" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="M51" s="9" t="s">
+        <v>203</v>
+      </c>
       <c r="N51" s="9" t="s">
-        <v>185</v>
+        <v>152</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3180,38 +3154,20 @@
       <c r="C52" s="7" t="n">
         <v>46348</v>
       </c>
-      <c r="D52" s="6" t="s">
-        <v>201</v>
-      </c>
+      <c r="D52" s="6"/>
       <c r="E52" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="F52" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="G52" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="H52" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="I52" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="J52" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="K52" s="8" t="s">
-        <v>208</v>
-      </c>
-      <c r="L52" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="M52" s="6" t="s">
-        <v>210</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="F52" s="6"/>
+      <c r="G52" s="6"/>
+      <c r="H52" s="6"/>
+      <c r="I52" s="6"/>
+      <c r="J52" s="6"/>
+      <c r="K52" s="8"/>
+      <c r="L52" s="6"/>
+      <c r="M52" s="6"/>
       <c r="N52" s="6" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3226,7 +3182,7 @@
       </c>
       <c r="D53" s="9"/>
       <c r="E53" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F53" s="9"/>
       <c r="G53" s="9"/>
@@ -3237,7 +3193,7 @@
       <c r="L53" s="9"/>
       <c r="M53" s="9"/>
       <c r="N53" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3252,7 +3208,7 @@
       </c>
       <c r="D54" s="9"/>
       <c r="E54" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F54" s="9"/>
       <c r="G54" s="9"/>
@@ -3263,7 +3219,7 @@
       <c r="L54" s="9"/>
       <c r="M54" s="9"/>
       <c r="N54" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3278,7 +3234,7 @@
       </c>
       <c r="D55" s="9"/>
       <c r="E55" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F55" s="9"/>
       <c r="G55" s="9"/>
@@ -3289,7 +3245,7 @@
       <c r="L55" s="9"/>
       <c r="M55" s="9"/>
       <c r="N55" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3302,20 +3258,38 @@
       <c r="C56" s="10" t="n">
         <v>46352</v>
       </c>
-      <c r="D56" s="9"/>
+      <c r="D56" s="9" t="s">
+        <v>53</v>
+      </c>
       <c r="E56" s="9" t="s">
-        <v>184</v>
-      </c>
-      <c r="F56" s="9"/>
-      <c r="G56" s="9"/>
-      <c r="H56" s="9"/>
-      <c r="I56" s="9"/>
-      <c r="J56" s="9"/>
-      <c r="K56" s="9"/>
-      <c r="L56" s="9"/>
-      <c r="M56" s="9"/>
+        <v>204</v>
+      </c>
+      <c r="F56" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="G56" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="H56" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="I56" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="J56" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="K56" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="L56" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="M56" s="9" t="s">
+        <v>126</v>
+      </c>
       <c r="N56" s="9" t="s">
-        <v>185</v>
+        <v>152</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3328,38 +3302,20 @@
       <c r="C57" s="12" t="n">
         <v>46353</v>
       </c>
-      <c r="D57" s="11" t="s">
-        <v>53</v>
-      </c>
+      <c r="D57" s="11"/>
       <c r="E57" s="11" t="s">
-        <v>211</v>
-      </c>
-      <c r="F57" s="11" t="s">
-        <v>212</v>
-      </c>
-      <c r="G57" s="11" t="s">
-        <v>213</v>
-      </c>
-      <c r="H57" s="11" t="s">
-        <v>214</v>
-      </c>
-      <c r="I57" s="11" t="s">
-        <v>215</v>
-      </c>
-      <c r="J57" s="11" t="s">
-        <v>216</v>
-      </c>
-      <c r="K57" s="13" t="s">
-        <v>217</v>
-      </c>
-      <c r="L57" s="11" t="s">
-        <v>218</v>
-      </c>
-      <c r="M57" s="11" t="s">
-        <v>134</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="F57" s="11"/>
+      <c r="G57" s="11"/>
+      <c r="H57" s="11"/>
+      <c r="I57" s="11"/>
+      <c r="J57" s="11"/>
+      <c r="K57" s="13"/>
+      <c r="L57" s="11"/>
+      <c r="M57" s="11"/>
       <c r="N57" s="11" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3374,7 +3330,7 @@
       </c>
       <c r="D58" s="9"/>
       <c r="E58" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F58" s="9"/>
       <c r="G58" s="9"/>
@@ -3385,7 +3341,7 @@
       <c r="L58" s="9"/>
       <c r="M58" s="9"/>
       <c r="N58" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3400,7 +3356,7 @@
       </c>
       <c r="D59" s="9"/>
       <c r="E59" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F59" s="9"/>
       <c r="G59" s="9"/>
@@ -3411,7 +3367,7 @@
       <c r="L59" s="9"/>
       <c r="M59" s="9"/>
       <c r="N59" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3426,7 +3382,7 @@
       </c>
       <c r="D60" s="9"/>
       <c r="E60" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F60" s="9"/>
       <c r="G60" s="9"/>
@@ -3437,7 +3393,7 @@
       <c r="L60" s="9"/>
       <c r="M60" s="9"/>
       <c r="N60" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3452,7 +3408,7 @@
       </c>
       <c r="D61" s="9"/>
       <c r="E61" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F61" s="9"/>
       <c r="G61" s="9"/>
@@ -3463,7 +3419,7 @@
       <c r="L61" s="9"/>
       <c r="M61" s="9"/>
       <c r="N61" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3478,7 +3434,7 @@
       </c>
       <c r="D62" s="9"/>
       <c r="E62" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F62" s="9"/>
       <c r="G62" s="9"/>
@@ -3489,7 +3445,7 @@
       <c r="L62" s="9"/>
       <c r="M62" s="9"/>
       <c r="N62" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3504,7 +3460,7 @@
       </c>
       <c r="D63" s="9"/>
       <c r="E63" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F63" s="9"/>
       <c r="G63" s="9"/>
@@ -3515,7 +3471,7 @@
       <c r="L63" s="9"/>
       <c r="M63" s="9"/>
       <c r="N63" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3530,7 +3486,7 @@
       </c>
       <c r="D64" s="9"/>
       <c r="E64" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F64" s="9"/>
       <c r="G64" s="9"/>
@@ -3541,7 +3497,7 @@
       <c r="L64" s="9"/>
       <c r="M64" s="9"/>
       <c r="N64" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3556,7 +3512,7 @@
       </c>
       <c r="D65" s="9"/>
       <c r="E65" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F65" s="9"/>
       <c r="G65" s="9"/>
@@ -3567,7 +3523,7 @@
       <c r="L65" s="9"/>
       <c r="M65" s="9"/>
       <c r="N65" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3582,7 +3538,7 @@
       </c>
       <c r="D66" s="9"/>
       <c r="E66" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F66" s="9"/>
       <c r="G66" s="9"/>
@@ -3593,7 +3549,7 @@
       <c r="L66" s="9"/>
       <c r="M66" s="9"/>
       <c r="N66" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3608,7 +3564,7 @@
       </c>
       <c r="D67" s="9"/>
       <c r="E67" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F67" s="9"/>
       <c r="G67" s="9"/>
@@ -3619,7 +3575,7 @@
       <c r="L67" s="9"/>
       <c r="M67" s="9"/>
       <c r="N67" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3632,20 +3588,38 @@
       <c r="C68" s="10" t="n">
         <v>46364</v>
       </c>
-      <c r="D68" s="9"/>
+      <c r="D68" s="9" t="s">
+        <v>161</v>
+      </c>
       <c r="E68" s="9" t="s">
-        <v>184</v>
-      </c>
-      <c r="F68" s="9"/>
-      <c r="G68" s="9"/>
-      <c r="H68" s="9"/>
-      <c r="I68" s="9"/>
-      <c r="J68" s="9"/>
-      <c r="K68" s="9"/>
-      <c r="L68" s="9"/>
-      <c r="M68" s="9"/>
+        <v>212</v>
+      </c>
+      <c r="F68" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="G68" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="H68" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="I68" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="J68" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="K68" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="L68" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="M68" s="9" t="s">
+        <v>52</v>
+      </c>
       <c r="N68" s="9" t="s">
-        <v>185</v>
+        <v>152</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3658,38 +3632,20 @@
       <c r="C69" s="7" t="n">
         <v>46365</v>
       </c>
-      <c r="D69" s="6" t="s">
-        <v>110</v>
-      </c>
+      <c r="D69" s="6"/>
       <c r="E69" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="F69" s="6" t="s">
-        <v>220</v>
-      </c>
-      <c r="G69" s="6" t="s">
-        <v>221</v>
-      </c>
-      <c r="H69" s="6" t="s">
-        <v>222</v>
-      </c>
-      <c r="I69" s="6" t="s">
-        <v>223</v>
-      </c>
-      <c r="J69" s="6" t="s">
-        <v>224</v>
-      </c>
-      <c r="K69" s="8" t="s">
-        <v>225</v>
-      </c>
-      <c r="L69" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="M69" s="6" t="s">
-        <v>52</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="F69" s="6"/>
+      <c r="G69" s="6"/>
+      <c r="H69" s="6"/>
+      <c r="I69" s="6"/>
+      <c r="J69" s="6"/>
+      <c r="K69" s="8"/>
+      <c r="L69" s="6"/>
+      <c r="M69" s="6"/>
       <c r="N69" s="6" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3704,7 +3660,7 @@
       </c>
       <c r="D70" s="9"/>
       <c r="E70" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F70" s="9"/>
       <c r="G70" s="9"/>
@@ -3715,7 +3671,7 @@
       <c r="L70" s="9"/>
       <c r="M70" s="9"/>
       <c r="N70" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3730,7 +3686,7 @@
       </c>
       <c r="D71" s="9"/>
       <c r="E71" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F71" s="9"/>
       <c r="G71" s="9"/>
@@ -3741,7 +3697,7 @@
       <c r="L71" s="9"/>
       <c r="M71" s="9"/>
       <c r="N71" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3756,7 +3712,7 @@
       </c>
       <c r="D72" s="9"/>
       <c r="E72" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F72" s="9"/>
       <c r="G72" s="9"/>
@@ -3767,7 +3723,7 @@
       <c r="L72" s="9"/>
       <c r="M72" s="9"/>
       <c r="N72" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3782,7 +3738,7 @@
       </c>
       <c r="D73" s="9"/>
       <c r="E73" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F73" s="9"/>
       <c r="G73" s="9"/>
@@ -3793,7 +3749,7 @@
       <c r="L73" s="9"/>
       <c r="M73" s="9"/>
       <c r="N73" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3808,7 +3764,7 @@
       </c>
       <c r="D74" s="9"/>
       <c r="E74" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F74" s="9"/>
       <c r="G74" s="9"/>
@@ -3819,7 +3775,7 @@
       <c r="L74" s="9"/>
       <c r="M74" s="9"/>
       <c r="N74" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3832,20 +3788,38 @@
       <c r="C75" s="10" t="n">
         <v>46371</v>
       </c>
-      <c r="D75" s="9"/>
+      <c r="D75" s="9" t="s">
+        <v>161</v>
+      </c>
       <c r="E75" s="9" t="s">
-        <v>184</v>
-      </c>
-      <c r="F75" s="9"/>
-      <c r="G75" s="9"/>
-      <c r="H75" s="9"/>
-      <c r="I75" s="9"/>
-      <c r="J75" s="9"/>
-      <c r="K75" s="9"/>
-      <c r="L75" s="9"/>
-      <c r="M75" s="9"/>
+        <v>220</v>
+      </c>
+      <c r="F75" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="G75" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="H75" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="I75" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="J75" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="K75" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="L75" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="M75" s="9" t="s">
+        <v>228</v>
+      </c>
       <c r="N75" s="9" t="s">
-        <v>185</v>
+        <v>152</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3858,38 +3832,20 @@
       <c r="C76" s="12" t="n">
         <v>46372</v>
       </c>
-      <c r="D76" s="11" t="s">
-        <v>110</v>
-      </c>
+      <c r="D76" s="11"/>
       <c r="E76" s="11" t="s">
-        <v>227</v>
-      </c>
-      <c r="F76" s="11" t="s">
-        <v>228</v>
-      </c>
-      <c r="G76" s="11" t="s">
-        <v>229</v>
-      </c>
-      <c r="H76" s="11" t="s">
-        <v>230</v>
-      </c>
-      <c r="I76" s="11" t="s">
-        <v>231</v>
-      </c>
-      <c r="J76" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="K76" s="13" t="s">
-        <v>233</v>
-      </c>
-      <c r="L76" s="11" t="s">
-        <v>234</v>
-      </c>
-      <c r="M76" s="11" t="s">
-        <v>235</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="F76" s="11"/>
+      <c r="G76" s="11"/>
+      <c r="H76" s="11"/>
+      <c r="I76" s="11"/>
+      <c r="J76" s="11"/>
+      <c r="K76" s="13"/>
+      <c r="L76" s="11"/>
+      <c r="M76" s="11"/>
       <c r="N76" s="11" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3904,7 +3860,7 @@
       </c>
       <c r="D77" s="9"/>
       <c r="E77" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F77" s="9"/>
       <c r="G77" s="9"/>
@@ -3915,7 +3871,7 @@
       <c r="L77" s="9"/>
       <c r="M77" s="9"/>
       <c r="N77" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3930,7 +3886,7 @@
       </c>
       <c r="D78" s="9"/>
       <c r="E78" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F78" s="9"/>
       <c r="G78" s="9"/>
@@ -3941,7 +3897,7 @@
       <c r="L78" s="9"/>
       <c r="M78" s="9"/>
       <c r="N78" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3956,7 +3912,7 @@
       </c>
       <c r="D79" s="9"/>
       <c r="E79" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F79" s="9"/>
       <c r="G79" s="9"/>
@@ -3967,7 +3923,7 @@
       <c r="L79" s="9"/>
       <c r="M79" s="9"/>
       <c r="N79" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3982,7 +3938,7 @@
       </c>
       <c r="D80" s="9"/>
       <c r="E80" s="9" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="F80" s="9"/>
       <c r="G80" s="9"/>
@@ -3993,7 +3949,7 @@
       <c r="L80" s="9"/>
       <c r="M80" s="9"/>
       <c r="N80" s="9" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -4029,15 +3985,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="B2" s="15" t="n">
         <f aca="false">COUNTA('Lịch đăng'!$A$2:$A$80)</f>
@@ -4050,25 +4006,25 @@
       </c>
       <c r="B3" s="15" t="n">
         <f aca="false">COUNTIF('Lịch đăng'!$N$2:$N$80,"Đã đăng")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="B4" s="15" t="n">
         <f aca="false">COUNTIF('Lịch đăng'!$N$2:$N$80,"Cần chủ đề")</f>
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="B5" s="15" t="n">
         <f aca="false">B2-B3-B4</f>
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Apply big-text opener to upcoming videos, add 30s short tests, move 22/10
- hook field on videos from 14/10 to 27/10 (kinetic 20/10 keeps its own opening)
- opener text wraps to two balanced lines only when long
- short 30-second variants for 14/10 and 15/10 (scripts/<slug>/2.json)
- messaging video moved from 09/10 to 22/10, sources rechecked and chart source lines corrected

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dpu4oyZ8FYSVLE8FrdnGTC
</commit_message>
<xml_diff>
--- a/video/plan/lich-noi-dung-tiktok.xlsx
+++ b/video/plan/lich-noi-dung-tiktok.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="236">
   <si>
     <t xml:space="preserve">Lịch nội dung TikTok Adtek</t>
   </si>
@@ -226,7 +226,394 @@
     <t xml:space="preserve">Thứ Sáu</t>
   </si>
   <si>
+    <t xml:space="preserve">Đã dời sang 22/10: Khách muốn nhắn tin trước khi mua</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dời lịch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Bảy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growth, Performance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khách so giá, chờ sale (đố số liệu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đoán thử: bao nhiêu % người Việt so giá ở nhiều nơi trước khi mua?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• 89.5% so giá nhiều nơi trước khi mua; 39.5% hoãn mua chờ khuyến mãi
+• 65% mua online mỗi tuần (Đông Nam Á 50%); lý do mua: giảm giá 64%, ship rẻ 55%, nhiều lựa chọn 52% (khu vực 47%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Vietnam Report, khảo sát người tiêu dùng ngành bán lẻ, 08/2026
+• Milieu Insight, 09/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://vietnamreport.net.vn/Top-10-Cong-ty-uy-tin-nganh-Ban-le-nam-2026-12576-1006.html
+https://www.mili.eu/vn/insights/vietnams-online-shoppers-demand-speed-and-reliability-in-2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Video mẫu kiểu đố số liệu (scripts/khach-so-gia-cho-sale/1.json)
+• Giọng v4 chưa huấn luyện; video trên trang hub
+• Đã nhắc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">so sánh giá; săn sale; khuyến mãi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chủ nhật</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Digital, Performance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thuê KOL nổi tiếng là khách sẽ tin? (phá hiểu lầm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Cứ thuê KOL nổi tiếng là khách sẽ tin và chốt đơn." Đúng hay sai?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• 54% tin đánh giá của người dùng thường hơn KOL, chỉ 13% nghiêng về người nổi tiếng
+• 78% bị đánh giá online ảnh hưởng mạnh tới lựa chọn (87% ở tuổi 20)
+• Đánh giá đáng tin: có ảnh/video 69%, nội dung chi tiết 60%, số sao 51%; dưới 3.6 sao bị loại; 74% cần từ 50 đánh giá
+• 67% tự tin nhận ra đánh giá giả</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Q&amp;Me, How Vietnamese consumers trust online reviews, khoảng 09/2026, 200 người 20-49 tuổi tại Hà Nội và TP.HCM
+• Việc làm ngay: Google Business Profile Help (xin đánh giá bằng link/QR, cấm tặng quà đổi đánh giá, trả lời đánh giá); TikTok Ads Help (Spark Ads dùng video của khách, nhà sáng tạo nhỏ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://qandme.net/en/report/how-vietnamese-consumers-trust-online-reviews.html
+https://support.google.com/business/answer/3474122
+https://support.google.com/business/answer/3474050
+https://ads.tiktok.com/help/article/spark-ads</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Đã mở trang gốc, khớp số liệu (09/10/2026). Báo cáo đầy đủ cần đăng ký, chỉ kiểm tra phần tóm tắt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Kiểu phá hiểu lầm, đóng dấu SAI
+• Mẫu nhỏ (200 người, chỉ HN và HCM), phải ghi rõ trên video
+• Ngày phát hành ước tính cuối 09/2026 Đã nhắc
+• Ngày 11/10 đăng thêm video "Giá quảng cáo Meta +12%, có nên giao hết cho Advantage+?" (vốn xếp lịch 14/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kol; review sản phẩm; đánh giá 5 sao; chốt đơn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Hai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Performance, Growth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chưa tới 3% gian hàng nắm 1/3 doanh số sàn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trên Shopee, TikTok Shop, Lazada, cứ 100 gian hàng thì chưa tới 3 shop Mall. Họ đang nắm bao nhiêu phần doanh số?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Shop Mall: 2.79% số gian hàng nhưng 34.2% doanh số (Shopee, Lazada, TikTok Shop, 6 tháng 2026); số shop Mall giảm 6%, doanh số tăng 54%
+• 4 sàn đạt 291.6 nghìn tỷ đồng, tăng 44.11%; 613.8 nghìn shop có đơn
+• Thị phần GMV: Shopee 54.5% (+15%), TikTok Shop 43.4% (+27%); TikTok Shop nắm 56.2% ngành thời trang
+• Hàng trên 1 triệu đồng chiếm 18.2% doanh số (+3.1 điểm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Metric, Báo cáo TMĐT Việt Nam 6 tháng đầu năm 2026, 29/07/2026
+• YouNet ECI, Toàn cảnh TMĐT Việt Nam nửa đầu năm 2026, 12/08/2026
+• Việc làm ngay: TikTok Shop Seller University (Mall, lịch 11.11 từ 03-12/11 và 12.12, Cộng tác mở); Shopee Help (tiếp thị liên kết trả theo đơn)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://metric.vn/insights/metric-bao-cao-thuong-mai-dien-tu-viet-nam-6-thang-dau-nam-2026/
+https://www.younetgroup.com/vi/bao-cao-toan-canh-tmdt-viet-nam-nua-dau-nam-2026
+https://seller-vn.tiktok.com/university/essay?knowledge_id=6210902215264001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Đã mở trang gốc, khớp số liệu (09/10/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Metric (doanh số, +44%) và YouNet (GMV, +19%) đo khác nhau: không đặt chung một biểu đồ
+• Tỷ lệ Mall tính trên 3 sàn, không phải 4
+• Đã nhắc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shopee mall; tiktok shop mall; bán hàng trên sàn 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đã có video</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Ba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quảng cáo nền tảng nào tiếp cận nhiều người Việt nhất? (đố số liệu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đoán thử: quảng cáo trên nền tảng nào tiếp cận nhiều người Việt nhất? A. TikTok, B. Facebook, C. YouTube</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Lượng người quảng cáo có thể tiếp cận: Facebook 79.0 triệu, TikTok 76.1 triệu (18+), YouTube 62.1 triệu, Messenger 57.8 triệu (cuối 2025)
+• Thời gian dùng mỗi ngày (Android, 08/2025): TikTok 1 giờ 56 phút, YouTube 1 giờ 21 phút, Facebook 1 giờ 11 phút
+• 84.9% người dùng internet tìm thông tin thương hiệu trên mạng xã hội
+• Zalo 81.3 triệu người dùng tháng (quý 2/2026, VNG): là số người dùng, không so trực tiếp với số tiếp cận quảng cáo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• DataReportal, Digital 2026: Vietnam (số liệu đến 10/2025)
+• VNG, Snapshot quý 2/2026
+• Việc làm ngay: TikTok Spark Ads; Google Ads Demand Gen (YouTube Shorts, Lookalike); Zalo Business Message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://datareportal.com/reports/digital-2026-vietnam
+https://cms-investor-cdn.vng.com.vn/VNG_Snapshot_Q2_2026_EN_8dc74b151d.pdf
+https://support.google.com/google-ads/answer/13695777
+https://zalo.solutions/business-message</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Kiểu đố số liệu, ảnh bìa không lộ đáp án
+• Số tiếp cận quảng cáo không phải số người dùng thật, có thể trùng; ghi rõ
+• Tránh lặp quảng cáo Click-to-Messenger (đã nói trong video nhắn tin 09/10)
+• Đã nhắc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">quảng cáo facebook hay tiktok; chạy quảng cáo youtube; zalo ads</t>
+  </si>
+  <si>
     <t xml:space="preserve">Performance, Digital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Livestream: chỉ 13% khách mua ngẫu hứng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Livestream sống nhờ khách mua ngẫu hứng?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Chỉ 13% mua ngẫu hứng; 47% đang cân nhắc; 40% định mua từ trước
+• 650,000 người bán và cửa hàng bán qua video (+60%), 1.3 tỷ giao dịch
+• 50% chủ yếu mua từ tài khoản chính thức của thương hiệu
+• Luật TMĐT 122/2025 (từ 01/07/2026): xác thực người live, lưu buổi live 1 năm; Nghị định 87/2026: người có ảnh hưởng giới thiệu hàng chưa dùng phạt 80-100 triệu, tổ chức gấp đôi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Q&amp;Me, Live commerce, 04/2026, 245 người (mẫu nhỏ)
+• e-Conomy SEA 2025, trang 144
+• Luật Thương mại điện tử 122/2025/QH15; Nghị định 87/2026/NĐ-CP (vanban.chinhphu.vn)
+• Việc làm ngay: TikTok Shop Seller University</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://qandme.net/vi/baibaocao/xu-huong-live-commerce-va-hanh-vi-nguoi-mua-viet-nam.html
+https://services.google.com/fh/files/misc/e_conomy_sea_2025_report_combined.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Đã mở trang gốc (10/10/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Nội dung pháp lý, nên nhờ luật sư duyệt câu chữ
+• Mẫu Q&amp;Me nhỏ, ghi rõ trên video</t>
+  </si>
+  <si>
+    <t xml:space="preserve">livestream bán hàng; luật livestream; kol bị phạt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App Marketing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thị trường app Việt Nam đã chạm đỉnh?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thị trường app Việt Nam đã chạm đỉnh? Tiền quảng cáo app nên đổ vào đâu?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Lượt cài +136% từ 2018, 2.17 tỷ năm 2024, giảm nhẹ 2025
+• iOS 22% lên 33% (2017-2025); app tài chính iOS 54.5%
+• Quý 2/2026 ngân sách kéo người dùng Android: tài chính +153%, giải trí +194%, game -46%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• AppsFlyer, State of App Marketing in Vietnam 2025, 11/2025
+• AppsFlyer, State of Marketing in APAC 2026, 09/2026
+• Việc làm ngay: Apple custom product pages, Play Console custom store listings, Google Ads App campaigns engagement, AppsFlyer Cohort</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.appsflyer.com/resources/reports/app-marketing-vietnam-report/
+https://www.appsflyer.com/resources/reports/state-of-marketing-apac-report/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Biểu đồ xu hướng dùng chỉ số quy đổi của AppsFlyer, đã ghi rõ
+• Số liệu là lượt cài AppsFlyer đo được, không phải toàn thị trường</t>
+  </si>
+  <si>
+    <t xml:space="preserve">thị trường app việt nam; quảng cáo app; iphone hay android</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trung bình</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bao nhiêu lượt cài app là gian lận? (đố số liệu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cứ 100 lượt cài app ở Việt Nam, bao nhiêu lượt là gian lận? A 5, B 20, C 50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Việt Nam 20% (quý 1/2026), từ 29%; Indonesia 17% xuống 13%
+• App tài chính Việt Nam 46% vs 22% châu Á Thái Bình Dương (2025)
+• Toàn cầu: 52% lượt cài gian lận nằm ở nguồn tự nhiên, affiliate gần 40%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• AppsFlyer, State of Fraud for Marketers 2026, 06/2026
+• AppsFlyer, State of Finance for Marketers APAC 2026
+• Việc làm ngay: AppsFlyer Protect360 và Validation Rules, Adjust Fraud Prevention, Apple AdAttributionKit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.appsflyer.com/resources/reports/state-fraud-marketers-report/
+https://www.appsflyer.com/resources/reports/apac-finance-marketing-report/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Kiểu đố số liệu, ảnh bìa không lộ đáp án
+• Tỷ lệ 20% là toàn thị trường, có thể chỉ Android; mức giảm một phần do một đường dây gian lận bị chặn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gian lận quảng cáo; cpi là gì; marketing app tài chính</t>
+  </si>
+  <si>
+    <t xml:space="preserve">App Marketing, Digital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Người Việt sống trong app 127 tỷ giờ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Một năm, người Việt dành bao nhiêu giờ trong app?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• 127 tỷ giờ dùng app năm 2025 (thế giới khoảng 3.6 giờ/người/ngày)
+• Mỗi lần mở app giải trí 24.46 phút (quý 1/2026), Đông Nam Á 14.28 phút
+• App giải trí quý 1/2026: lượt cài +32%, số lần mở +76%
+• Chỉ 8% quay lại ngày hôm sau, ngày 30 còn 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Adjust, Mobile app trends spotlight: Vietnam 2026 (PDF 26/05/2026)
+• Sensor Tower, State of Mobile 2026
+• Việc làm ngay: GA4 Cohort exploration, Firebase In-App Messaging, Google Ads App campaigns engagement, Apple In-App Events</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.adjust.com/blog/vietnam-app-trends-2026/
+https://sensortower.com/blog/state-of-mobile-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• adjust.com chặn truy cập tự động (lỗi 429); đã đọc file PDF gốc của Adjust qua bản đăng lại, khớp số liệu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Số liệu chỉ gồm app Adjust đo được</t>
+  </si>
+  <si>
+    <t xml:space="preserve">thời gian dùng điện thoại; tiktok việt nam; app ai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Digital, Growth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua data khách hàng để chạy quảng cáo: rủi ro tới đâu?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua một tệp data khách hàng để chạy quảng cáo, rủi ro lớn nhất là gì?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Luật 91/2025/QH15, hiệu lực 01/01/2026: mua bán dữ liệu phạt tới 10 lần khoản thu; chuyển dữ liệu ra nước ngoài trái quy định tới 5% doanh thu; vi phạm khác tới 3 tỷ đồng
+• 72% tin công ty ít hơn 1 năm trước; 65% thấy doanh nghiệp bất cẩn với dữ liệu; gần 75% muốn biết đang nói chuyện với AI hay người</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Quốc hội, Luật Bảo vệ dữ liệu cá nhân 91/2025/QH15; Nghị định 356/2025/NĐ-CP
+• Salesforce, State of the AI Connected Customer (bản 7), 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://thuvienphapluat.vn/van-ban/Bo-may-hanh-chinh/Luat-Bao-ve-du-lieu-ca-nhan-2025-so-91-2025-QH15-625628.aspx
+https://www.salesforce.com/resources/research-reports/state-of-the-connected-customer/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Chưa mở được trang gốc (mạng chặn), đối chiếu qua VnEconomy, Báo Đầu tư, PwC Việt Nam
+• Chưa mở được trang gốc (mạng chặn), đối chiếu qua salesforce.com/news</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Nội dung pháp lý, nên nhờ luật sư duyệt kịch bản
+• Khảo sát 2024. Hợp đăng cạnh video luật dữ liệu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">luật bảo vệ dữ liệu cá nhân; data khách hàng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ý tưởng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bản đồ: kinh tế số Việt Nam tăng 17%, nhanh thứ 2 Đông Nam Á</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kinh tế số Việt Nam tăng nhanh hay chậm so với láng giềng? Năm 2025, con số là 17%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tăng trưởng GMV kinh tế số 2025: Malaysia 19%, Việt Nam 17%, Thái Lan 16%, Philippines 16%, Indonesia 14%, Singapore 7%; Việt Nam 39 tỷ USD (2025, ước tính)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google, Temasek, Bain &amp; Company, e-Conomy SEA 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://services.google.com/fh/files/misc/e_conomy_sea_2025_report_combined.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đã mở báo cáo gốc (trang 84 đến 140)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Số 2025 là ước tính, quy đổi từ 6 tháng đầu năm. Dạng bản đồ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kinh tế số việt nam; digital 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Performance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chữ động: đừng chạy sale 11.11 nếu chưa biết 3 điều này</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chỉ còn 3 tuần nữa là 11.11, bạn định chạy sale mà chưa chuẩn bị gì sao?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.10.2025: 4 sàn bán 6,608 tỷ đồng, 376,000 gian hàng; khách thêm vào giỏ sớm 3 đến 5 ngày; Meta cần khoảng 50 kết quả trong 1 tuần; Google Ads điều chỉnh thời vụ cho sale 1 đến 7 ngày</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metric; Meta Business Help Center; Google Ads Help</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://metric.vn/insights/4-nhom-san-pham-ban-chay-nhat-tren-san-sau-ngay-doi-10-10/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đã mở trang gốc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'Gấp hơn 5 lần' và 'gần 29%' là phép tính từ số Metric. Dạng chữ động.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đếm ngược: top 5 từ khóa tăng mạnh nhất trên Google năm 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Năm 2025, người Việt tìm gì trên Google tăng mạnh nhất? Đoán thử hạng 1 rồi comment trước nhé.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xu hướng chung 2025: 5 Pixverse AI, 4 Gemini, 3 Phụ nữ trong các ngành STEM, 2 Chat GPT, 1 Deep Seek</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google Year in Search 2025 Việt Nam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://trends.withgoogle.com/year-in-search/2025/vn/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đã mở trang gốc và trang phương pháp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xếp theo mức tăng, không phải lượt tìm. Đăng trước khi có bản 2026 (đầu tháng 12). Dạng đếm ngược.</t>
   </si>
   <si>
     <t xml:space="preserve">Khách muốn nhắn tin trước khi mua</t>
@@ -239,16 +626,19 @@
 • 81.3 triệu người dùng hằng tháng (quý 2/2026); hơn 2.2 tỷ tin nhắn mỗi ngày; ~30,000 Official Account (+24%)</t>
   </si>
   <si>
-    <t xml:space="preserve">• Meta, nghiên cứu do Kantar và Ipsos thực hiện (khảo sát 11/2025)
-• VNG, kết quả kinh doanh quý 2/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.facebook.com/business/news
-https://vng.com.vn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Chưa có link bài cụ thể; Chưa mở được trang gốc (mạng chặn), đối chiếu qua Việt Nam News
-• Chưa có link bài cụ thể; Chưa mở được trang gốc (mạng chặn), đối chiếu qua VietnamPlus</t>
+    <t xml:space="preserve">• Meta: nghiên cứu Kantar (82.8%, 61.2%, 85.6%) và Holiday Shopping Study của Ipsos (85%, 66%, 44%; 11/2025, 14,473 người), công bố 25/09/2026
+• VNG, Snapshot và kết quả kinh doanh quý 2/2026 (81.3 triệu MAU, 2.2 tỷ tin nhắn/ngày, ~30,000 OA, +24%)
+• TikTok, SEA Apps Summit 29/10/2025 (70 triệu người dùng hằng tháng)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://vietnamnews.vn/economy/1800588/vietnamese-consumers-spread-shopping-across-multiple-peak-season-events.html
+https://cms-investor-cdn.vng.com.vn/VNG_Snapshot_Q2_2026_EN_8dc74b151d.pdf
+https://bizhub.vietnamnews.vn/tiktok-reaches-70-million-monthly-users-in-viet-nam-post389459.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Kiểm tra lại 13/10/2026: số liệu Meta khớp bài Vietnam News 25/09/2026 (Meta không đăng báo cáo Việt Nam công khai; báo cáo toàn cầu cần điền form)
+• VNG: đã mở PDF gốc, khớp 81.3 triệu và 2.2 tỷ; số OA theo công bố kết quả quý 2
+• Dòng nguồn trên biểu đồ đã sửa mốc thời gian Kantar và Ipsos</t>
   </si>
   <si>
     <t xml:space="preserve">• Chưa có URL trang gốc của Meta, cần tìm trước khi dựng
@@ -256,391 +646,11 @@
 • Giọng v4 chưa huấn luyện; video trên trang hub
 • Nằm trong Drafts của TikTok, dời sang 09/10
 • Xuất lại 09/10 theo hướng A và C
-• Đã nhắc</t>
+• Đã nhắc
+• Dời từ 09/10 (chưa đăng) sang 22/10 theo anh Tin duyệt 13/10/2026</t>
   </si>
   <si>
     <t xml:space="preserve">quảng cáo tin nhắn; zalo oa; chốt đơn inbox</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đã có video</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Bảy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Growth, Performance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Khách so giá, chờ sale (đố số liệu)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đoán thử: bao nhiêu % người Việt so giá ở nhiều nơi trước khi mua?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• 89.5% so giá nhiều nơi trước khi mua; 39.5% hoãn mua chờ khuyến mãi
-• 65% mua online mỗi tuần (Đông Nam Á 50%); lý do mua: giảm giá 64%, ship rẻ 55%, nhiều lựa chọn 52% (khu vực 47%)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Vietnam Report, khảo sát người tiêu dùng ngành bán lẻ, 08/2026
-• Milieu Insight, 09/2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://vietnamreport.net.vn/Top-10-Cong-ty-uy-tin-nganh-Ban-le-nam-2026-12576-1006.html
-https://www.mili.eu/vn/insights/vietnams-online-shoppers-demand-speed-and-reliability-in-2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Video mẫu kiểu đố số liệu (scripts/khach-so-gia-cho-sale/1.json)
-• Giọng v4 chưa huấn luyện; video trên trang hub
-• Đã nhắc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">so sánh giá; săn sale; khuyến mãi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chủ nhật</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Digital, Performance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thuê KOL nổi tiếng là khách sẽ tin? (phá hiểu lầm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"Cứ thuê KOL nổi tiếng là khách sẽ tin và chốt đơn." Đúng hay sai?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• 54% tin đánh giá của người dùng thường hơn KOL, chỉ 13% nghiêng về người nổi tiếng
-• 78% bị đánh giá online ảnh hưởng mạnh tới lựa chọn (87% ở tuổi 20)
-• Đánh giá đáng tin: có ảnh/video 69%, nội dung chi tiết 60%, số sao 51%; dưới 3.6 sao bị loại; 74% cần từ 50 đánh giá
-• 67% tự tin nhận ra đánh giá giả</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Q&amp;Me, How Vietnamese consumers trust online reviews, khoảng 09/2026, 200 người 20-49 tuổi tại Hà Nội và TP.HCM
-• Việc làm ngay: Google Business Profile Help (xin đánh giá bằng link/QR, cấm tặng quà đổi đánh giá, trả lời đánh giá); TikTok Ads Help (Spark Ads dùng video của khách, nhà sáng tạo nhỏ)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://qandme.net/en/report/how-vietnamese-consumers-trust-online-reviews.html
-https://support.google.com/business/answer/3474122
-https://support.google.com/business/answer/3474050
-https://ads.tiktok.com/help/article/spark-ads</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Đã mở trang gốc, khớp số liệu (09/10/2026). Báo cáo đầy đủ cần đăng ký, chỉ kiểm tra phần tóm tắt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Kiểu phá hiểu lầm, đóng dấu SAI
-• Mẫu nhỏ (200 người, chỉ HN và HCM), phải ghi rõ trên video
-• Ngày phát hành ước tính cuối 09/2026 Đã nhắc
-• Ngày 11/10 đăng thêm video "Giá quảng cáo Meta +12%, có nên giao hết cho Advantage+?" (vốn xếp lịch 14/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kol; review sản phẩm; đánh giá 5 sao; chốt đơn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Hai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Performance, Growth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chưa tới 3% gian hàng nắm 1/3 doanh số sàn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trên Shopee, TikTok Shop, Lazada, cứ 100 gian hàng thì chưa tới 3 shop Mall. Họ đang nắm bao nhiêu phần doanh số?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Shop Mall: 2.79% số gian hàng nhưng 34.2% doanh số (Shopee, Lazada, TikTok Shop, 6 tháng 2026); số shop Mall giảm 6%, doanh số tăng 54%
-• 4 sàn đạt 291.6 nghìn tỷ đồng, tăng 44.11%; 613.8 nghìn shop có đơn
-• Thị phần GMV: Shopee 54.5% (+15%), TikTok Shop 43.4% (+27%); TikTok Shop nắm 56.2% ngành thời trang
-• Hàng trên 1 triệu đồng chiếm 18.2% doanh số (+3.1 điểm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Metric, Báo cáo TMĐT Việt Nam 6 tháng đầu năm 2026, 29/07/2026
-• YouNet ECI, Toàn cảnh TMĐT Việt Nam nửa đầu năm 2026, 12/08/2026
-• Việc làm ngay: TikTok Shop Seller University (Mall, lịch 11.11 từ 03-12/11 và 12.12, Cộng tác mở); Shopee Help (tiếp thị liên kết trả theo đơn)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://metric.vn/insights/metric-bao-cao-thuong-mai-dien-tu-viet-nam-6-thang-dau-nam-2026/
-https://www.younetgroup.com/vi/bao-cao-toan-canh-tmdt-viet-nam-nua-dau-nam-2026
-https://seller-vn.tiktok.com/university/essay?knowledge_id=6210902215264001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Đã mở trang gốc, khớp số liệu (09/10/2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Metric (doanh số, +44%) và YouNet (GMV, +19%) đo khác nhau: không đặt chung một biểu đồ
-• Tỷ lệ Mall tính trên 3 sàn, không phải 4
-• Đã nhắc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">shopee mall; tiktok shop mall; bán hàng trên sàn 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Ba</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quảng cáo nền tảng nào tiếp cận nhiều người Việt nhất? (đố số liệu)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đoán thử: quảng cáo trên nền tảng nào tiếp cận nhiều người Việt nhất? A. TikTok, B. Facebook, C. YouTube</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Lượng người quảng cáo có thể tiếp cận: Facebook 79.0 triệu, TikTok 76.1 triệu (18+), YouTube 62.1 triệu, Messenger 57.8 triệu (cuối 2025)
-• Thời gian dùng mỗi ngày (Android, 08/2025): TikTok 1 giờ 56 phút, YouTube 1 giờ 21 phút, Facebook 1 giờ 11 phút
-• 84.9% người dùng internet tìm thông tin thương hiệu trên mạng xã hội
-• Zalo 81.3 triệu người dùng tháng (quý 2/2026, VNG): là số người dùng, không so trực tiếp với số tiếp cận quảng cáo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• DataReportal, Digital 2026: Vietnam (số liệu đến 10/2025)
-• VNG, Snapshot quý 2/2026
-• Việc làm ngay: TikTok Spark Ads; Google Ads Demand Gen (YouTube Shorts, Lookalike); Zalo Business Message</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://datareportal.com/reports/digital-2026-vietnam
-https://cms-investor-cdn.vng.com.vn/VNG_Snapshot_Q2_2026_EN_8dc74b151d.pdf
-https://support.google.com/google-ads/answer/13695777
-https://zalo.solutions/business-message</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Kiểu đố số liệu, ảnh bìa không lộ đáp án
-• Số tiếp cận quảng cáo không phải số người dùng thật, có thể trùng; ghi rõ
-• Tránh lặp quảng cáo Click-to-Messenger (đã nói trong video nhắn tin 09/10)
-• Đã nhắc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">quảng cáo facebook hay tiktok; chạy quảng cáo youtube; zalo ads</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Livestream: chỉ 13% khách mua ngẫu hứng</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Livestream sống nhờ khách mua ngẫu hứng?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Chỉ 13% mua ngẫu hứng; 47% đang cân nhắc; 40% định mua từ trước
-• 650,000 người bán và cửa hàng bán qua video (+60%), 1.3 tỷ giao dịch
-• 50% chủ yếu mua từ tài khoản chính thức của thương hiệu
-• Luật TMĐT 122/2025 (từ 01/07/2026): xác thực người live, lưu buổi live 1 năm; Nghị định 87/2026: người có ảnh hưởng giới thiệu hàng chưa dùng phạt 80-100 triệu, tổ chức gấp đôi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Q&amp;Me, Live commerce, 04/2026, 245 người (mẫu nhỏ)
-• e-Conomy SEA 2025, trang 144
-• Luật Thương mại điện tử 122/2025/QH15; Nghị định 87/2026/NĐ-CP (vanban.chinhphu.vn)
-• Việc làm ngay: TikTok Shop Seller University</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://qandme.net/vi/baibaocao/xu-huong-live-commerce-va-hanh-vi-nguoi-mua-viet-nam.html
-https://services.google.com/fh/files/misc/e_conomy_sea_2025_report_combined.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Đã mở trang gốc (10/10/2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Nội dung pháp lý, nên nhờ luật sư duyệt câu chữ
-• Mẫu Q&amp;Me nhỏ, ghi rõ trên video</t>
-  </si>
-  <si>
-    <t xml:space="preserve">livestream bán hàng; luật livestream; kol bị phạt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">App Marketing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thị trường app Việt Nam đã chạm đỉnh?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thị trường app Việt Nam đã chạm đỉnh? Tiền quảng cáo app nên đổ vào đâu?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Lượt cài +136% từ 2018, 2.17 tỷ năm 2024, giảm nhẹ 2025
-• iOS 22% lên 33% (2017-2025); app tài chính iOS 54.5%
-• Quý 2/2026 ngân sách kéo người dùng Android: tài chính +153%, giải trí +194%, game -46%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• AppsFlyer, State of App Marketing in Vietnam 2025, 11/2025
-• AppsFlyer, State of Marketing in APAC 2026, 09/2026
-• Việc làm ngay: Apple custom product pages, Play Console custom store listings, Google Ads App campaigns engagement, AppsFlyer Cohort</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.appsflyer.com/resources/reports/app-marketing-vietnam-report/
-https://www.appsflyer.com/resources/reports/state-of-marketing-apac-report/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Biểu đồ xu hướng dùng chỉ số quy đổi của AppsFlyer, đã ghi rõ
-• Số liệu là lượt cài AppsFlyer đo được, không phải toàn thị trường</t>
-  </si>
-  <si>
-    <t xml:space="preserve">thị trường app việt nam; quảng cáo app; iphone hay android</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trung bình</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bao nhiêu lượt cài app là gian lận? (đố số liệu)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cứ 100 lượt cài app ở Việt Nam, bao nhiêu lượt là gian lận? A 5, B 20, C 50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Việt Nam 20% (quý 1/2026), từ 29%; Indonesia 17% xuống 13%
-• App tài chính Việt Nam 46% vs 22% châu Á Thái Bình Dương (2025)
-• Toàn cầu: 52% lượt cài gian lận nằm ở nguồn tự nhiên, affiliate gần 40%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• AppsFlyer, State of Fraud for Marketers 2026, 06/2026
-• AppsFlyer, State of Finance for Marketers APAC 2026
-• Việc làm ngay: AppsFlyer Protect360 và Validation Rules, Adjust Fraud Prevention, Apple AdAttributionKit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.appsflyer.com/resources/reports/state-fraud-marketers-report/
-https://www.appsflyer.com/resources/reports/apac-finance-marketing-report/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Kiểu đố số liệu, ảnh bìa không lộ đáp án
-• Tỷ lệ 20% là toàn thị trường, có thể chỉ Android; mức giảm một phần do một đường dây gian lận bị chặn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gian lận quảng cáo; cpi là gì; marketing app tài chính</t>
-  </si>
-  <si>
-    <t xml:space="preserve">App Marketing, Digital</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Người Việt sống trong app 127 tỷ giờ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Một năm, người Việt dành bao nhiêu giờ trong app?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• 127 tỷ giờ dùng app năm 2025 (thế giới khoảng 3.6 giờ/người/ngày)
-• Mỗi lần mở app giải trí 24.46 phút (quý 1/2026), Đông Nam Á 14.28 phút
-• App giải trí quý 1/2026: lượt cài +32%, số lần mở +76%
-• Chỉ 8% quay lại ngày hôm sau, ngày 30 còn 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Adjust, Mobile app trends spotlight: Vietnam 2026 (PDF 26/05/2026)
-• Sensor Tower, State of Mobile 2026
-• Việc làm ngay: GA4 Cohort exploration, Firebase In-App Messaging, Google Ads App campaigns engagement, Apple In-App Events</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.adjust.com/blog/vietnam-app-trends-2026/
-https://sensortower.com/blog/state-of-mobile-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• adjust.com chặn truy cập tự động (lỗi 429); đã đọc file PDF gốc của Adjust qua bản đăng lại, khớp số liệu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Số liệu chỉ gồm app Adjust đo được</t>
-  </si>
-  <si>
-    <t xml:space="preserve">thời gian dùng điện thoại; tiktok việt nam; app ai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Digital, Growth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mua data khách hàng để chạy quảng cáo: rủi ro tới đâu?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mua một tệp data khách hàng để chạy quảng cáo, rủi ro lớn nhất là gì?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Luật 91/2025/QH15, hiệu lực 01/01/2026: mua bán dữ liệu phạt tới 10 lần khoản thu; chuyển dữ liệu ra nước ngoài trái quy định tới 5% doanh thu; vi phạm khác tới 3 tỷ đồng
-• 72% tin công ty ít hơn 1 năm trước; 65% thấy doanh nghiệp bất cẩn với dữ liệu; gần 75% muốn biết đang nói chuyện với AI hay người</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Quốc hội, Luật Bảo vệ dữ liệu cá nhân 91/2025/QH15; Nghị định 356/2025/NĐ-CP
-• Salesforce, State of the AI Connected Customer (bản 7), 2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://thuvienphapluat.vn/van-ban/Bo-may-hanh-chinh/Luat-Bao-ve-du-lieu-ca-nhan-2025-so-91-2025-QH15-625628.aspx
-https://www.salesforce.com/resources/research-reports/state-of-the-connected-customer/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Chưa mở được trang gốc (mạng chặn), đối chiếu qua VnEconomy, Báo Đầu tư, PwC Việt Nam
-• Chưa mở được trang gốc (mạng chặn), đối chiếu qua salesforce.com/news</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Nội dung pháp lý, nên nhờ luật sư duyệt kịch bản
-• Khảo sát 2024. Hợp đăng cạnh video luật dữ liệu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">luật bảo vệ dữ liệu cá nhân; data khách hàng</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ý tưởng</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bản đồ: kinh tế số Việt Nam tăng 17%, nhanh thứ 2 Đông Nam Á</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kinh tế số Việt Nam tăng nhanh hay chậm so với láng giềng? Năm 2025, con số là 17%.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tăng trưởng GMV kinh tế số 2025: Malaysia 19%, Việt Nam 17%, Thái Lan 16%, Philippines 16%, Indonesia 14%, Singapore 7%; Việt Nam 39 tỷ USD (2025, ước tính)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Google, Temasek, Bain &amp; Company, e-Conomy SEA 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://services.google.com/fh/files/misc/e_conomy_sea_2025_report_combined.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đã mở báo cáo gốc (trang 84 đến 140)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Số 2025 là ước tính, quy đổi từ 6 tháng đầu năm. Dạng bản đồ.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kinh tế số việt nam; digital 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Performance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chữ động: đừng chạy sale 11.11 nếu chưa biết 3 điều này</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chỉ còn 3 tuần nữa là 11.11, bạn định chạy sale mà chưa chuẩn bị gì sao?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10.10.2025: 4 sàn bán 6,608 tỷ đồng, 376,000 gian hàng; khách thêm vào giỏ sớm 3 đến 5 ngày; Meta cần khoảng 50 kết quả trong 1 tuần; Google Ads điều chỉnh thời vụ cho sale 1 đến 7 ngày</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Metric; Meta Business Help Center; Google Ads Help</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://metric.vn/insights/4-nhom-san-pham-ban-chay-nhat-tren-san-sau-ngay-doi-10-10/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đã mở trang gốc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'Gấp hơn 5 lần' và 'gần 29%' là phép tính từ số Metric. Dạng chữ động.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đếm ngược: top 5 từ khóa tăng mạnh nhất trên Google năm 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Năm 2025, người Việt tìm gì trên Google tăng mạnh nhất? Đoán thử hạng 1 rồi comment trước nhé.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Xu hướng chung 2025: 5 Pixverse AI, 4 Gemini, 3 Phụ nữ trong các ngành STEM, 2 Chat GPT, 1 Deep Seek</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Google Year in Search 2025 Việt Nam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://trends.withgoogle.com/year-in-search/2025/vn/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đã mở trang gốc và trang phương pháp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Xếp theo mức tăng, không phải lượt tìm. Đăng trước khi có bản 2026 (đầu tháng 12). Dạng đếm ngược.</t>
   </si>
   <si>
     <t xml:space="preserve">Slot trống: chủ đề trend Claude tự chọn khi viết kịch bản thứ Bảy</t>
@@ -1736,38 +1746,20 @@
       <c r="C8" s="7" t="n">
         <v>46304</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="6"/>
+      <c r="E8" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="6"/>
+      <c r="M8" s="6"/>
+      <c r="N8" s="6" t="s">
         <v>64</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="K8" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="L8" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="M8" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="N8" s="6" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1775,37 +1767,37 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="C9" s="7" t="n">
         <v>46305</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="J9" s="6" t="s">
         <v>59</v>
       </c>
       <c r="K9" s="8" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="M9" s="6" t="s">
         <v>52</v>
@@ -1819,37 +1811,37 @@
         <v>9</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="C10" s="10" t="n">
         <v>46306</v>
       </c>
       <c r="D10" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="J10" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="K10" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="L10" s="9" t="s">
         <v>83</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="G10" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="H10" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="I10" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="J10" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="K10" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="L10" s="9" t="s">
-        <v>91</v>
       </c>
       <c r="M10" s="9" t="s">
         <v>52</v>
@@ -1863,43 +1855,43 @@
         <v>10</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C11" s="10" t="n">
         <v>46307</v>
       </c>
       <c r="D11" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="I11" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="J11" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="K11" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="L11" s="9" t="s">
         <v>93</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="H11" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="I11" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="J11" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="K11" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="L11" s="9" t="s">
-        <v>101</v>
       </c>
       <c r="M11" s="9" t="s">
         <v>52</v>
       </c>
       <c r="N11" s="9" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1907,43 +1899,43 @@
         <v>11</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="C12" s="10" t="n">
         <v>46308</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="L12" s="9" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="M12" s="9" t="s">
         <v>52</v>
       </c>
       <c r="N12" s="9" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="135.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1957,37 +1949,37 @@
         <v>46309</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>63</v>
+        <v>103</v>
       </c>
       <c r="E13" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="K13" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="L13" s="6" t="s">
         <v>111</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="J13" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="K13" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="L13" s="6" t="s">
-        <v>117</v>
       </c>
       <c r="M13" s="6" t="s">
         <v>52</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2001,37 +1993,37 @@
         <v>46310</v>
       </c>
       <c r="D14" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="K14" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="L14" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="M14" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="G14" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="I14" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J14" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="K14" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="L14" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="M14" s="6" t="s">
-        <v>126</v>
-      </c>
       <c r="N14" s="6" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2045,37 +2037,37 @@
         <v>46311</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="E15" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="H15" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="J15" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="K15" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="L15" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="F15" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="G15" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="H15" s="11" t="s">
-        <v>130</v>
-      </c>
-      <c r="I15" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="J15" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="K15" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="L15" s="11" t="s">
-        <v>133</v>
-      </c>
       <c r="M15" s="11" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="N15" s="11" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2083,43 +2075,43 @@
         <v>15</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="C16" s="12" t="n">
         <v>46312</v>
       </c>
       <c r="D16" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="G16" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="H16" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="I16" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="J16" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="K16" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="L16" s="11" t="s">
         <v>136</v>
-      </c>
-      <c r="G16" s="11" t="s">
-        <v>137</v>
-      </c>
-      <c r="H16" s="11" t="s">
-        <v>138</v>
-      </c>
-      <c r="I16" s="11" t="s">
-        <v>139</v>
-      </c>
-      <c r="J16" s="11" t="s">
-        <v>140</v>
-      </c>
-      <c r="K16" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="L16" s="11" t="s">
-        <v>142</v>
       </c>
       <c r="M16" s="11" t="s">
         <v>52</v>
       </c>
       <c r="N16" s="11" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2127,43 +2119,43 @@
         <v>16</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="C17" s="12" t="n">
         <v>46313</v>
       </c>
       <c r="D17" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="H17" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="I17" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="J17" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="K17" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="L17" s="11" t="s">
         <v>145</v>
-      </c>
-      <c r="G17" s="11" t="s">
-        <v>146</v>
-      </c>
-      <c r="H17" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="I17" s="11" t="s">
-        <v>148</v>
-      </c>
-      <c r="J17" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="K17" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="L17" s="11" t="s">
-        <v>151</v>
       </c>
       <c r="M17" s="11" t="s">
         <v>52</v>
       </c>
       <c r="N17" s="11" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2171,43 +2163,43 @@
         <v>17</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C18" s="12" t="n">
         <v>46314</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="E18" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="G18" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="I18" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="J18" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="K18" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="F18" s="11" t="s">
+      <c r="L18" s="11" t="s">
         <v>154</v>
       </c>
-      <c r="G18" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="H18" s="11" t="s">
-        <v>156</v>
-      </c>
-      <c r="I18" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="J18" s="11" t="s">
-        <v>158</v>
-      </c>
-      <c r="K18" s="13" t="s">
-        <v>159</v>
-      </c>
-      <c r="L18" s="11" t="s">
-        <v>160</v>
-      </c>
       <c r="M18" s="11" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="N18" s="11" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2215,39 +2207,39 @@
         <v>18</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="C19" s="12" t="n">
         <v>46315</v>
       </c>
       <c r="D19" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="G19" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="H19" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="I19" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="J19" s="11" t="s">
         <v>161</v>
       </c>
-      <c r="E19" s="11" t="s">
+      <c r="K19" s="13" t="s">
         <v>162</v>
-      </c>
-      <c r="F19" s="11" t="s">
-        <v>163</v>
-      </c>
-      <c r="G19" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="H19" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="I19" s="11" t="s">
-        <v>166</v>
-      </c>
-      <c r="J19" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="K19" s="13" t="s">
-        <v>168</v>
       </c>
       <c r="L19" s="11"/>
       <c r="M19" s="11"/>
       <c r="N19" s="11" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2261,33 +2253,33 @@
         <v>46316</v>
       </c>
       <c r="D20" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="I20" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="J20" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="K20" s="9" t="s">
         <v>170</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>171</v>
-      </c>
-      <c r="G20" s="9" t="s">
-        <v>172</v>
-      </c>
-      <c r="H20" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="I20" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="J20" s="9" t="s">
-        <v>175</v>
-      </c>
-      <c r="K20" s="9" t="s">
-        <v>176</v>
       </c>
       <c r="L20" s="9"/>
       <c r="M20" s="9"/>
       <c r="N20" s="9" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2300,20 +2292,38 @@
       <c r="C21" s="10" t="n">
         <v>46317</v>
       </c>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9" t="s">
+      <c r="D21" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="K21" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="F21" s="9"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
-      <c r="J21" s="9"/>
-      <c r="K21" s="9"/>
-      <c r="L21" s="9"/>
-      <c r="M21" s="9"/>
-      <c r="N21" s="9" t="s">
+      <c r="L21" s="6" t="s">
         <v>178</v>
+      </c>
+      <c r="M21" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="N21" s="6" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2328,7 +2338,7 @@
       </c>
       <c r="D22" s="9"/>
       <c r="E22" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F22" s="9"/>
       <c r="G22" s="9"/>
@@ -2339,7 +2349,7 @@
       <c r="L22" s="9"/>
       <c r="M22" s="9"/>
       <c r="N22" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2347,14 +2357,14 @@
         <v>22</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="C23" s="10" t="n">
         <v>46319</v>
       </c>
       <c r="D23" s="9"/>
       <c r="E23" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F23" s="9"/>
       <c r="G23" s="9"/>
@@ -2365,7 +2375,7 @@
       <c r="L23" s="9"/>
       <c r="M23" s="9"/>
       <c r="N23" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2373,14 +2383,14 @@
         <v>23</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="C24" s="10" t="n">
         <v>46320</v>
       </c>
       <c r="D24" s="9"/>
       <c r="E24" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F24" s="9"/>
       <c r="G24" s="9"/>
@@ -2391,7 +2401,7 @@
       <c r="L24" s="9"/>
       <c r="M24" s="9"/>
       <c r="N24" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2399,14 +2409,14 @@
         <v>24</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C25" s="10" t="n">
         <v>46321</v>
       </c>
       <c r="D25" s="9"/>
       <c r="E25" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
@@ -2417,7 +2427,7 @@
       <c r="L25" s="9"/>
       <c r="M25" s="9"/>
       <c r="N25" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2425,39 +2435,39 @@
         <v>25</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="C26" s="10" t="n">
         <v>46322</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>63</v>
+        <v>103</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="I26" s="9" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="J26" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="L26" s="9"/>
       <c r="M26" s="9"/>
       <c r="N26" s="9" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2472,7 +2482,7 @@
       </c>
       <c r="D27" s="9"/>
       <c r="E27" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F27" s="9"/>
       <c r="G27" s="9"/>
@@ -2483,7 +2493,7 @@
       <c r="L27" s="9"/>
       <c r="M27" s="9"/>
       <c r="N27" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2498,7 +2508,7 @@
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -2509,7 +2519,7 @@
       <c r="L28" s="9"/>
       <c r="M28" s="9"/>
       <c r="N28" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2524,7 +2534,7 @@
       </c>
       <c r="D29" s="9"/>
       <c r="E29" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F29" s="9"/>
       <c r="G29" s="9"/>
@@ -2535,7 +2545,7 @@
       <c r="L29" s="9"/>
       <c r="M29" s="9"/>
       <c r="N29" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2543,14 +2553,14 @@
         <v>29</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="C30" s="10" t="n">
         <v>46326</v>
       </c>
       <c r="D30" s="9"/>
       <c r="E30" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F30" s="9"/>
       <c r="G30" s="9"/>
@@ -2561,7 +2571,7 @@
       <c r="L30" s="9"/>
       <c r="M30" s="9"/>
       <c r="N30" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2569,14 +2579,14 @@
         <v>30</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="C31" s="10" t="n">
         <v>46327</v>
       </c>
       <c r="D31" s="9"/>
       <c r="E31" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F31" s="9"/>
       <c r="G31" s="9"/>
@@ -2587,7 +2597,7 @@
       <c r="L31" s="9"/>
       <c r="M31" s="9"/>
       <c r="N31" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2595,14 +2605,14 @@
         <v>31</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C32" s="10" t="n">
         <v>46328</v>
       </c>
       <c r="D32" s="9"/>
       <c r="E32" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F32" s="9"/>
       <c r="G32" s="9"/>
@@ -2613,7 +2623,7 @@
       <c r="L32" s="9"/>
       <c r="M32" s="9"/>
       <c r="N32" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2621,14 +2631,14 @@
         <v>32</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="C33" s="10" t="n">
         <v>46329</v>
       </c>
       <c r="D33" s="9"/>
       <c r="E33" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -2639,7 +2649,7 @@
       <c r="L33" s="9"/>
       <c r="M33" s="9"/>
       <c r="N33" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2654,7 +2664,7 @@
       </c>
       <c r="D34" s="9"/>
       <c r="E34" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -2665,7 +2675,7 @@
       <c r="L34" s="9"/>
       <c r="M34" s="9"/>
       <c r="N34" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2680,7 +2690,7 @@
       </c>
       <c r="D35" s="9"/>
       <c r="E35" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -2691,7 +2701,7 @@
       <c r="L35" s="9"/>
       <c r="M35" s="9"/>
       <c r="N35" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2706,7 +2716,7 @@
       </c>
       <c r="D36" s="9"/>
       <c r="E36" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -2717,7 +2727,7 @@
       <c r="L36" s="9"/>
       <c r="M36" s="9"/>
       <c r="N36" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2725,14 +2735,14 @@
         <v>36</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="C37" s="10" t="n">
         <v>46333</v>
       </c>
       <c r="D37" s="9"/>
       <c r="E37" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
@@ -2743,7 +2753,7 @@
       <c r="L37" s="9"/>
       <c r="M37" s="9"/>
       <c r="N37" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2751,14 +2761,14 @@
         <v>37</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="C38" s="10" t="n">
         <v>46334</v>
       </c>
       <c r="D38" s="9"/>
       <c r="E38" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F38" s="9"/>
       <c r="G38" s="9"/>
@@ -2769,7 +2779,7 @@
       <c r="L38" s="9"/>
       <c r="M38" s="9"/>
       <c r="N38" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2777,14 +2787,14 @@
         <v>38</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C39" s="10" t="n">
         <v>46335</v>
       </c>
       <c r="D39" s="9"/>
       <c r="E39" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F39" s="9"/>
       <c r="G39" s="9"/>
@@ -2795,7 +2805,7 @@
       <c r="L39" s="9"/>
       <c r="M39" s="9"/>
       <c r="N39" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2803,43 +2813,43 @@
         <v>39</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="C40" s="10" t="n">
         <v>46336</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="I40" s="9" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="J40" s="9" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="K40" s="9" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="L40" s="9" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="M40" s="9" t="s">
         <v>52</v>
       </c>
       <c r="N40" s="9" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2854,7 +2864,7 @@
       </c>
       <c r="D41" s="6"/>
       <c r="E41" s="6" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F41" s="6"/>
       <c r="G41" s="6"/>
@@ -2865,7 +2875,7 @@
       <c r="L41" s="6"/>
       <c r="M41" s="6"/>
       <c r="N41" s="6" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2880,7 +2890,7 @@
       </c>
       <c r="D42" s="9"/>
       <c r="E42" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F42" s="9"/>
       <c r="G42" s="9"/>
@@ -2891,7 +2901,7 @@
       <c r="L42" s="9"/>
       <c r="M42" s="9"/>
       <c r="N42" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2906,7 +2916,7 @@
       </c>
       <c r="D43" s="9"/>
       <c r="E43" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F43" s="9"/>
       <c r="G43" s="9"/>
@@ -2917,7 +2927,7 @@
       <c r="L43" s="9"/>
       <c r="M43" s="9"/>
       <c r="N43" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2925,14 +2935,14 @@
         <v>43</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="C44" s="10" t="n">
         <v>46340</v>
       </c>
       <c r="D44" s="9"/>
       <c r="E44" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F44" s="9"/>
       <c r="G44" s="9"/>
@@ -2943,7 +2953,7 @@
       <c r="L44" s="9"/>
       <c r="M44" s="9"/>
       <c r="N44" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2951,14 +2961,14 @@
         <v>44</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="C45" s="10" t="n">
         <v>46341</v>
       </c>
       <c r="D45" s="9"/>
       <c r="E45" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F45" s="9"/>
       <c r="G45" s="9"/>
@@ -2969,7 +2979,7 @@
       <c r="L45" s="9"/>
       <c r="M45" s="9"/>
       <c r="N45" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2977,14 +2987,14 @@
         <v>45</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C46" s="10" t="n">
         <v>46342</v>
       </c>
       <c r="D46" s="9"/>
       <c r="E46" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F46" s="9"/>
       <c r="G46" s="9"/>
@@ -2995,7 +3005,7 @@
       <c r="L46" s="9"/>
       <c r="M46" s="9"/>
       <c r="N46" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3003,14 +3013,14 @@
         <v>46</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="C47" s="10" t="n">
         <v>46343</v>
       </c>
       <c r="D47" s="9"/>
       <c r="E47" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F47" s="9"/>
       <c r="G47" s="9"/>
@@ -3021,7 +3031,7 @@
       <c r="L47" s="9"/>
       <c r="M47" s="9"/>
       <c r="N47" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3036,7 +3046,7 @@
       </c>
       <c r="D48" s="9"/>
       <c r="E48" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F48" s="9"/>
       <c r="G48" s="9"/>
@@ -3047,7 +3057,7 @@
       <c r="L48" s="9"/>
       <c r="M48" s="9"/>
       <c r="N48" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3062,7 +3072,7 @@
       </c>
       <c r="D49" s="9"/>
       <c r="E49" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F49" s="9"/>
       <c r="G49" s="9"/>
@@ -3073,7 +3083,7 @@
       <c r="L49" s="9"/>
       <c r="M49" s="9"/>
       <c r="N49" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3088,7 +3098,7 @@
       </c>
       <c r="D50" s="9"/>
       <c r="E50" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F50" s="9"/>
       <c r="G50" s="9"/>
@@ -3099,7 +3109,7 @@
       <c r="L50" s="9"/>
       <c r="M50" s="9"/>
       <c r="N50" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3107,43 +3117,43 @@
         <v>50</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="C51" s="10" t="n">
         <v>46347</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="H51" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I51" s="9" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="J51" s="9" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="K51" s="9" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="L51" s="9" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="M51" s="9" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="N51" s="9" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3151,14 +3161,14 @@
         <v>51</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="C52" s="7" t="n">
         <v>46348</v>
       </c>
       <c r="D52" s="6"/>
       <c r="E52" s="6" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F52" s="6"/>
       <c r="G52" s="6"/>
@@ -3169,7 +3179,7 @@
       <c r="L52" s="6"/>
       <c r="M52" s="6"/>
       <c r="N52" s="6" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3177,14 +3187,14 @@
         <v>52</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C53" s="10" t="n">
         <v>46349</v>
       </c>
       <c r="D53" s="9"/>
       <c r="E53" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F53" s="9"/>
       <c r="G53" s="9"/>
@@ -3195,7 +3205,7 @@
       <c r="L53" s="9"/>
       <c r="M53" s="9"/>
       <c r="N53" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3203,14 +3213,14 @@
         <v>53</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="C54" s="10" t="n">
         <v>46350</v>
       </c>
       <c r="D54" s="9"/>
       <c r="E54" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F54" s="9"/>
       <c r="G54" s="9"/>
@@ -3221,7 +3231,7 @@
       <c r="L54" s="9"/>
       <c r="M54" s="9"/>
       <c r="N54" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3236,7 +3246,7 @@
       </c>
       <c r="D55" s="9"/>
       <c r="E55" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F55" s="9"/>
       <c r="G55" s="9"/>
@@ -3247,7 +3257,7 @@
       <c r="L55" s="9"/>
       <c r="M55" s="9"/>
       <c r="N55" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3264,34 +3274,34 @@
         <v>53</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="H56" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="I56" s="9" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="J56" s="9" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="K56" s="9" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="L56" s="9" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="M56" s="9" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="N56" s="9" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3306,7 +3316,7 @@
       </c>
       <c r="D57" s="11"/>
       <c r="E57" s="11" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F57" s="11"/>
       <c r="G57" s="11"/>
@@ -3317,7 +3327,7 @@
       <c r="L57" s="11"/>
       <c r="M57" s="11"/>
       <c r="N57" s="11" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3325,14 +3335,14 @@
         <v>57</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="C58" s="10" t="n">
         <v>46354</v>
       </c>
       <c r="D58" s="9"/>
       <c r="E58" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F58" s="9"/>
       <c r="G58" s="9"/>
@@ -3343,7 +3353,7 @@
       <c r="L58" s="9"/>
       <c r="M58" s="9"/>
       <c r="N58" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3351,14 +3361,14 @@
         <v>58</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="C59" s="10" t="n">
         <v>46355</v>
       </c>
       <c r="D59" s="9"/>
       <c r="E59" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F59" s="9"/>
       <c r="G59" s="9"/>
@@ -3369,7 +3379,7 @@
       <c r="L59" s="9"/>
       <c r="M59" s="9"/>
       <c r="N59" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3377,14 +3387,14 @@
         <v>59</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C60" s="10" t="n">
         <v>46356</v>
       </c>
       <c r="D60" s="9"/>
       <c r="E60" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F60" s="9"/>
       <c r="G60" s="9"/>
@@ -3395,7 +3405,7 @@
       <c r="L60" s="9"/>
       <c r="M60" s="9"/>
       <c r="N60" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3403,14 +3413,14 @@
         <v>60</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="C61" s="10" t="n">
         <v>46357</v>
       </c>
       <c r="D61" s="9"/>
       <c r="E61" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F61" s="9"/>
       <c r="G61" s="9"/>
@@ -3421,7 +3431,7 @@
       <c r="L61" s="9"/>
       <c r="M61" s="9"/>
       <c r="N61" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3436,7 +3446,7 @@
       </c>
       <c r="D62" s="9"/>
       <c r="E62" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F62" s="9"/>
       <c r="G62" s="9"/>
@@ -3447,7 +3457,7 @@
       <c r="L62" s="9"/>
       <c r="M62" s="9"/>
       <c r="N62" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3462,7 +3472,7 @@
       </c>
       <c r="D63" s="9"/>
       <c r="E63" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F63" s="9"/>
       <c r="G63" s="9"/>
@@ -3473,7 +3483,7 @@
       <c r="L63" s="9"/>
       <c r="M63" s="9"/>
       <c r="N63" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3488,7 +3498,7 @@
       </c>
       <c r="D64" s="9"/>
       <c r="E64" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F64" s="9"/>
       <c r="G64" s="9"/>
@@ -3499,7 +3509,7 @@
       <c r="L64" s="9"/>
       <c r="M64" s="9"/>
       <c r="N64" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3507,14 +3517,14 @@
         <v>64</v>
       </c>
       <c r="B65" s="9" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="C65" s="10" t="n">
         <v>46361</v>
       </c>
       <c r="D65" s="9"/>
       <c r="E65" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F65" s="9"/>
       <c r="G65" s="9"/>
@@ -3525,7 +3535,7 @@
       <c r="L65" s="9"/>
       <c r="M65" s="9"/>
       <c r="N65" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3533,14 +3543,14 @@
         <v>65</v>
       </c>
       <c r="B66" s="9" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="C66" s="10" t="n">
         <v>46362</v>
       </c>
       <c r="D66" s="9"/>
       <c r="E66" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F66" s="9"/>
       <c r="G66" s="9"/>
@@ -3551,7 +3561,7 @@
       <c r="L66" s="9"/>
       <c r="M66" s="9"/>
       <c r="N66" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3559,14 +3569,14 @@
         <v>66</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C67" s="10" t="n">
         <v>46363</v>
       </c>
       <c r="D67" s="9"/>
       <c r="E67" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F67" s="9"/>
       <c r="G67" s="9"/>
@@ -3577,7 +3587,7 @@
       <c r="L67" s="9"/>
       <c r="M67" s="9"/>
       <c r="N67" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3585,43 +3595,43 @@
         <v>67</v>
       </c>
       <c r="B68" s="9" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="C68" s="10" t="n">
         <v>46364</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="E68" s="9" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="G68" s="9" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="H68" s="9" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="I68" s="9" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="J68" s="9" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="K68" s="9" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="L68" s="9" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="M68" s="9" t="s">
         <v>52</v>
       </c>
       <c r="N68" s="9" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3636,7 +3646,7 @@
       </c>
       <c r="D69" s="6"/>
       <c r="E69" s="6" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F69" s="6"/>
       <c r="G69" s="6"/>
@@ -3647,7 +3657,7 @@
       <c r="L69" s="6"/>
       <c r="M69" s="6"/>
       <c r="N69" s="6" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3662,7 +3672,7 @@
       </c>
       <c r="D70" s="9"/>
       <c r="E70" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F70" s="9"/>
       <c r="G70" s="9"/>
@@ -3673,7 +3683,7 @@
       <c r="L70" s="9"/>
       <c r="M70" s="9"/>
       <c r="N70" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3688,7 +3698,7 @@
       </c>
       <c r="D71" s="9"/>
       <c r="E71" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F71" s="9"/>
       <c r="G71" s="9"/>
@@ -3699,7 +3709,7 @@
       <c r="L71" s="9"/>
       <c r="M71" s="9"/>
       <c r="N71" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3707,14 +3717,14 @@
         <v>71</v>
       </c>
       <c r="B72" s="9" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="C72" s="10" t="n">
         <v>46368</v>
       </c>
       <c r="D72" s="9"/>
       <c r="E72" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F72" s="9"/>
       <c r="G72" s="9"/>
@@ -3725,7 +3735,7 @@
       <c r="L72" s="9"/>
       <c r="M72" s="9"/>
       <c r="N72" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3733,14 +3743,14 @@
         <v>72</v>
       </c>
       <c r="B73" s="9" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="C73" s="10" t="n">
         <v>46369</v>
       </c>
       <c r="D73" s="9"/>
       <c r="E73" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F73" s="9"/>
       <c r="G73" s="9"/>
@@ -3751,7 +3761,7 @@
       <c r="L73" s="9"/>
       <c r="M73" s="9"/>
       <c r="N73" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3759,14 +3769,14 @@
         <v>73</v>
       </c>
       <c r="B74" s="9" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C74" s="10" t="n">
         <v>46370</v>
       </c>
       <c r="D74" s="9"/>
       <c r="E74" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F74" s="9"/>
       <c r="G74" s="9"/>
@@ -3777,7 +3787,7 @@
       <c r="L74" s="9"/>
       <c r="M74" s="9"/>
       <c r="N74" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3785,43 +3795,43 @@
         <v>74</v>
       </c>
       <c r="B75" s="9" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="C75" s="10" t="n">
         <v>46371</v>
       </c>
       <c r="D75" s="9" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="F75" s="9" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="H75" s="9" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="I75" s="9" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="J75" s="9" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="K75" s="9" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="L75" s="9" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="M75" s="9" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="N75" s="9" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3836,7 +3846,7 @@
       </c>
       <c r="D76" s="11"/>
       <c r="E76" s="11" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F76" s="11"/>
       <c r="G76" s="11"/>
@@ -3847,7 +3857,7 @@
       <c r="L76" s="11"/>
       <c r="M76" s="11"/>
       <c r="N76" s="11" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3862,7 +3872,7 @@
       </c>
       <c r="D77" s="9"/>
       <c r="E77" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F77" s="9"/>
       <c r="G77" s="9"/>
@@ -3873,7 +3883,7 @@
       <c r="L77" s="9"/>
       <c r="M77" s="9"/>
       <c r="N77" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3888,7 +3898,7 @@
       </c>
       <c r="D78" s="9"/>
       <c r="E78" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F78" s="9"/>
       <c r="G78" s="9"/>
@@ -3899,7 +3909,7 @@
       <c r="L78" s="9"/>
       <c r="M78" s="9"/>
       <c r="N78" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3907,14 +3917,14 @@
         <v>78</v>
       </c>
       <c r="B79" s="9" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="C79" s="10" t="n">
         <v>46375</v>
       </c>
       <c r="D79" s="9"/>
       <c r="E79" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F79" s="9"/>
       <c r="G79" s="9"/>
@@ -3925,7 +3935,7 @@
       <c r="L79" s="9"/>
       <c r="M79" s="9"/>
       <c r="N79" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3933,14 +3943,14 @@
         <v>79</v>
       </c>
       <c r="B80" s="9" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="C80" s="10" t="n">
         <v>46376</v>
       </c>
       <c r="D80" s="9"/>
       <c r="E80" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F80" s="9"/>
       <c r="G80" s="9"/>
@@ -3951,7 +3961,7 @@
       <c r="L80" s="9"/>
       <c r="M80" s="9"/>
       <c r="N80" s="9" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -3987,15 +3997,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B2" s="15" t="n">
         <f aca="false">COUNTA('Lịch đăng'!$A$2:$A$80)</f>
@@ -4013,20 +4023,20 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B4" s="15" t="n">
         <f aca="false">COUNTIF('Lịch đăng'!$N$2:$N$80,"Cần chủ đề")</f>
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B5" s="15" t="n">
         <f aca="false">B2-B3-B4</f>
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add TikTok scripts for 18, 23, 24, 25 Oct with voice
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WxJyQayTE17duXYsRamVW7
</commit_message>
<xml_diff>
--- a/video/plan/lich-noi-dung-tiktok.xlsx
+++ b/video/plan/lich-noi-dung-tiktok.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="262">
   <si>
     <t xml:space="preserve">Lịch nội dung TikTok Adtek</t>
   </si>
@@ -516,36 +516,41 @@
     <t xml:space="preserve">Digital, Growth</t>
   </si>
   <si>
-    <t xml:space="preserve">Mua data khách hàng để chạy quảng cáo: rủi ro tới đâu?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mua một tệp data khách hàng để chạy quảng cáo, rủi ro lớn nhất là gì?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Luật 91/2025/QH15, hiệu lực 01/01/2026: mua bán dữ liệu phạt tới 10 lần khoản thu; chuyển dữ liệu ra nước ngoài trái quy định tới 5% doanh thu; vi phạm khác tới 3 tỷ đồng
-• 72% tin công ty ít hơn 1 năm trước; 65% thấy doanh nghiệp bất cẩn với dữ liệu; gần 75% muốn biết đang nói chuyện với AI hay người</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Quốc hội, Luật Bảo vệ dữ liệu cá nhân 91/2025/QH15; Nghị định 356/2025/NĐ-CP
-• Salesforce, State of the AI Connected Customer (bản 7), 2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://thuvienphapluat.vn/van-ban/Bo-may-hanh-chinh/Luat-Bao-ve-du-lieu-ca-nhan-2025-so-91-2025-QH15-625628.aspx
-https://www.salesforce.com/resources/research-reports/state-of-the-connected-customer/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Chưa mở được trang gốc (mạng chặn), đối chiếu qua VnEconomy, Báo Đầu tư, PwC Việt Nam
-• Chưa mở được trang gốc (mạng chặn), đối chiếu qua salesforce.com/news</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Nội dung pháp lý, nên nhờ luật sư duyệt kịch bản
-• Khảo sát 2024. Hợp đăng cạnh video luật dữ liệu</t>
+    <t xml:space="preserve">Mua data khách hàng để chạy quảng cáo: rủi ro tới đâu? (phá hiểu lầm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mua data khách hàng, có thể bị phạt tới 10 lần?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Luật 91/2025/QH15 (hiệu lực 01/01/2026): cấm mua, bán dữ liệu cá nhân (Điều 7 khoản 6); phạt tối đa 10 lần khoản thu, không có khoản thu thì tới 3 tỷ đồng; cá nhân bằng một nửa (Điều 8)
+• Điều 28: quảng cáo dùng dữ liệu cá nhân phải có đồng ý, có cách từ chối
+• NCA 2024: 66.24% nói thông tin từng bị dùng trái phép; 95.54% bị cuộc gọi rác làm phiền; nghi bị lộ khi mua hàng online 73.99%, nhà hàng khách sạn siêu thị 67.00%, mạng xã hội 62.13%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Quốc hội, Luật Bảo vệ dữ liệu cá nhân 91/2025/QH15
+• Hiệp hội An ninh mạng quốc gia (NCA), khảo sát 2024
+• Việc làm ngay: Google Ads Help (Customer Match), Meta Business Help Center (Instant Form, Custom Audience terms)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://hethongphapluat.com/luat-bao-ve-du-lieu-ca-nhan-2025
+https://lsvn.vn/du-lieu-ca-nhan-cua-hon-66-nguoi-dung-internet-bi-su-dung-trai-phep-trong-nam-2024-a151492.html
+https://support.google.com/adspolicy/answer/6299717
+https://www.facebook.com/business/help/1247534515288168</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Đã đọc toàn văn Điều 7, 8, 28, 38 (bản đăng lại toàn văn; cổng chinhphu.vn, thuvienphapluat chặn truy cập tự động)
+• Số NCA đối chiếu qua Tạp chí Luật sư Việt Nam (lsvn.vn); trang nca.org.vn không đọc được tự động
+• Bỏ số Salesforce 2024 (toàn cầu, cũ) để dùng số Việt Nam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Nội dung pháp lý, nên nhờ luật sư duyệt câu chữ
+• Dạng phá hiểu lầm</t>
   </si>
   <si>
     <t xml:space="preserve">luật bảo vệ dữ liệu cá nhân; data khách hàng</t>
   </si>
   <si>
-    <t xml:space="preserve">Ý tưởng</t>
+    <t xml:space="preserve">Đã viết kịch bản</t>
   </si>
   <si>
     <t xml:space="preserve">Bản đồ: kinh tế số Việt Nam tăng 17%, nhanh thứ 2 Đông Nam Á</t>
@@ -657,6 +662,95 @@
     <t xml:space="preserve">quảng cáo tin nhắn; zalo oa; chốt đơn inbox</t>
   </si>
   <si>
+    <t xml:space="preserve">Khách chọn mua online vì điều gì nhất? (đố số liệu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khách chọn mua online vì điều gì nhất? A giá rẻ, B chất lượng, C khuyến mãi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• eCCI quý 3/2026: 141 điểm (quý 2: 122); 58% thấy thu nhập tích cực (quý 2: 45%)
+• Chất lượng sản phẩm 74% (quý 2: 53%), giá 67%; khuyến mãi giảm 7 điểm phần trăm về mức quan trọng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• YouNet ECI, Báo cáo Doanh thu và Tiêu dùng TMĐT Việt Nam quý 3/2026 (13/10/2026)
+• Việc làm ngay: Google Ads Help (conversions with cart data, COGS), Merchant Center Help (Product Ratings, tối thiểu 50 đánh giá)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://youneteci.com/vi/bao-cao-toan-canh-tmdt-viet-nam-q3-2026/
+https://support.google.com/google-ads/answer/9028254
+https://support.google.com/merchants/answer/14549080</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đã mở trang gốc YouNet ECI 17/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Không dùng số thị phần Shopee, TikTok Shop để tránh trùng video 27/10
+• Bản H1 ghi chất lượng quý 2 là 52%, bản quý 3 ghi 53%: dùng số bản quý 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mua sắm online; sale cuối năm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7/10 người Việt từng mua hàng giả (infographic)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 trên 10 người Việt từng mua hàng giả?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">69% người thành thị từng mua hàng giả, tuổi 20 là 84%; quần áo 87%, giày dép 69%, túi xách 45%; phân biệt bằng mã QR 69% và cửa hàng chính hãng 69%; giá rẻ bất thường là dấu hiệu nghi ngờ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Q&amp;Me, Counterfeit Products in Vietnam: Consumer Attitudes and Behavior (2026)
+• Việc làm ngay: Shopee Brand IP Portal, Google Merchant Center Help (GTIN)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://qandme.net/en/report/counterfeit-products-in-vietnam-consumer-attitudes-and-behavior.html
+https://brandipp.shopee.com
+https://support.google.com/merchants/answer/6324461</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đã mở trang gốc Q&amp;Me 17/10/2026; trang không ghi cơ số của tỷ lệ theo nhóm hàng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Mẫu nhỏ (200 người, Hà Nội và TP.HCM), đã ghi rõ trên video</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hàng giả; hàng chính hãng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEO, AIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viết bài bằng AI là bị Google phạt? (phá hiểu lầm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viết bài bằng AI là bị Google phạt?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• 86.5% trang top 20 Google có dùng AI, 4.6% hoàn toàn AI (Ahrefs, 600,000 trang, 07/2025)
+• Tỷ lệ lập chỉ mục: ít AI 49.28%, rất nhiều AI 40.35%; top 3: 82.2% trang dùng AI dưới 50%, 5.3% hoàn toàn AI (Ahrefs, 07/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Google Search Central: hướng dẫn nội dung AI (02/2023), chính sách spam (scaled content abuse), nội dung hữu ích
+• Ahrefs, 2 nghiên cứu 07/2025 và 07/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://developers.google.com/search/blog/2023/02/google-search-and-ai-content
+https://developers.google.com/search/docs/essentials/spam-policies
+https://ahrefs.com/blog/ai-generated-content-does-not-hurt-your-google-rankings/
+https://ahrefs.com/blog/google-doesnt-punish-ai-content/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đã mở trang gốc Google và Ahrefs 17/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Số liệu quốc tế, đã ghi rõ
+• Ahrefs bán công cụ dò AI dùng trong nghiên cứu; là tương quan, không phải nhân quả</t>
+  </si>
+  <si>
+    <t xml:space="preserve">seo ai; viết bài bằng ai</t>
+  </si>
+  <si>
     <t xml:space="preserve">Slot trống: chủ đề trend Claude tự chọn khi viết kịch bản thứ Bảy</t>
   </si>
   <si>
@@ -716,6 +810,9 @@
   </si>
   <si>
     <t xml:space="preserve">tiktok shop; shopee hay tiktok shop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ý tưởng</t>
   </si>
   <si>
     <t xml:space="preserve">AIO, Performance</t>
@@ -2340,20 +2437,38 @@
       <c r="C22" s="10" t="n">
         <v>46318</v>
       </c>
-      <c r="D22" s="9"/>
+      <c r="D22" s="9" t="s">
+        <v>85</v>
+      </c>
       <c r="E22" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="F22" s="9"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="9"/>
-      <c r="K22" s="9"/>
-      <c r="L22" s="9"/>
-      <c r="M22" s="9"/>
+      <c r="F22" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="G22" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="H22" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="I22" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="J22" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="K22" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="L22" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="M22" s="9" t="s">
+        <v>120</v>
+      </c>
       <c r="N22" s="9" t="s">
-        <v>180</v>
+        <v>146</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2366,20 +2481,38 @@
       <c r="C23" s="10" t="n">
         <v>46319</v>
       </c>
-      <c r="D23" s="9"/>
+      <c r="D23" s="9" t="s">
+        <v>66</v>
+      </c>
       <c r="E23" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="F23" s="9"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="9"/>
-      <c r="K23" s="9"/>
-      <c r="L23" s="9"/>
-      <c r="M23" s="9"/>
+        <v>187</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="G23" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="H23" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="I23" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="J23" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="K23" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="L23" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="M23" s="9" t="s">
+        <v>120</v>
+      </c>
       <c r="N23" s="9" t="s">
-        <v>180</v>
+        <v>146</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2392,20 +2525,38 @@
       <c r="C24" s="10" t="n">
         <v>46320</v>
       </c>
-      <c r="D24" s="9"/>
+      <c r="D24" s="9" t="s">
+        <v>195</v>
+      </c>
       <c r="E24" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
-      <c r="K24" s="9"/>
-      <c r="L24" s="9"/>
-      <c r="M24" s="9"/>
+        <v>196</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="G24" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="H24" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="I24" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="J24" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="K24" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="L24" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="M24" s="9" t="s">
+        <v>120</v>
+      </c>
       <c r="N24" s="9" t="s">
-        <v>180</v>
+        <v>146</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2420,7 +2571,7 @@
       </c>
       <c r="D25" s="9"/>
       <c r="E25" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
@@ -2431,7 +2582,7 @@
       <c r="L25" s="9"/>
       <c r="M25" s="9"/>
       <c r="N25" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2448,25 +2599,25 @@
         <v>103</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>181</v>
+        <v>206</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>182</v>
+        <v>207</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>183</v>
+        <v>208</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>184</v>
+        <v>209</v>
       </c>
       <c r="I26" s="9" t="s">
-        <v>185</v>
+        <v>210</v>
       </c>
       <c r="J26" s="9" t="s">
-        <v>186</v>
+        <v>211</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>187</v>
+        <v>212</v>
       </c>
       <c r="L26" s="9"/>
       <c r="M26" s="9"/>
@@ -2486,7 +2637,7 @@
       </c>
       <c r="D27" s="9"/>
       <c r="E27" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F27" s="9"/>
       <c r="G27" s="9"/>
@@ -2497,7 +2648,7 @@
       <c r="L27" s="9"/>
       <c r="M27" s="9"/>
       <c r="N27" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2512,7 +2663,7 @@
       </c>
       <c r="D28" s="9"/>
       <c r="E28" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -2523,7 +2674,7 @@
       <c r="L28" s="9"/>
       <c r="M28" s="9"/>
       <c r="N28" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2538,7 +2689,7 @@
       </c>
       <c r="D29" s="9"/>
       <c r="E29" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F29" s="9"/>
       <c r="G29" s="9"/>
@@ -2549,7 +2700,7 @@
       <c r="L29" s="9"/>
       <c r="M29" s="9"/>
       <c r="N29" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2564,7 +2715,7 @@
       </c>
       <c r="D30" s="9"/>
       <c r="E30" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F30" s="9"/>
       <c r="G30" s="9"/>
@@ -2575,7 +2726,7 @@
       <c r="L30" s="9"/>
       <c r="M30" s="9"/>
       <c r="N30" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2590,7 +2741,7 @@
       </c>
       <c r="D31" s="9"/>
       <c r="E31" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F31" s="9"/>
       <c r="G31" s="9"/>
@@ -2601,7 +2752,7 @@
       <c r="L31" s="9"/>
       <c r="M31" s="9"/>
       <c r="N31" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2616,7 +2767,7 @@
       </c>
       <c r="D32" s="9"/>
       <c r="E32" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F32" s="9"/>
       <c r="G32" s="9"/>
@@ -2627,7 +2778,7 @@
       <c r="L32" s="9"/>
       <c r="M32" s="9"/>
       <c r="N32" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2642,7 +2793,7 @@
       </c>
       <c r="D33" s="9"/>
       <c r="E33" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -2653,7 +2804,7 @@
       <c r="L33" s="9"/>
       <c r="M33" s="9"/>
       <c r="N33" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2668,7 +2819,7 @@
       </c>
       <c r="D34" s="9"/>
       <c r="E34" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -2679,7 +2830,7 @@
       <c r="L34" s="9"/>
       <c r="M34" s="9"/>
       <c r="N34" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2694,7 +2845,7 @@
       </c>
       <c r="D35" s="9"/>
       <c r="E35" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -2705,7 +2856,7 @@
       <c r="L35" s="9"/>
       <c r="M35" s="9"/>
       <c r="N35" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2720,7 +2871,7 @@
       </c>
       <c r="D36" s="9"/>
       <c r="E36" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -2731,7 +2882,7 @@
       <c r="L36" s="9"/>
       <c r="M36" s="9"/>
       <c r="N36" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2746,7 +2897,7 @@
       </c>
       <c r="D37" s="9"/>
       <c r="E37" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
@@ -2757,7 +2908,7 @@
       <c r="L37" s="9"/>
       <c r="M37" s="9"/>
       <c r="N37" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2772,7 +2923,7 @@
       </c>
       <c r="D38" s="9"/>
       <c r="E38" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F38" s="9"/>
       <c r="G38" s="9"/>
@@ -2783,7 +2934,7 @@
       <c r="L38" s="9"/>
       <c r="M38" s="9"/>
       <c r="N38" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2798,7 +2949,7 @@
       </c>
       <c r="D39" s="9"/>
       <c r="E39" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F39" s="9"/>
       <c r="G39" s="9"/>
@@ -2809,7 +2960,7 @@
       <c r="L39" s="9"/>
       <c r="M39" s="9"/>
       <c r="N39" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2826,34 +2977,34 @@
         <v>155</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>188</v>
+        <v>213</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>189</v>
+        <v>214</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>190</v>
+        <v>215</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>191</v>
+        <v>216</v>
       </c>
       <c r="I40" s="9" t="s">
-        <v>192</v>
+        <v>217</v>
       </c>
       <c r="J40" s="9" t="s">
-        <v>193</v>
+        <v>218</v>
       </c>
       <c r="K40" s="9" t="s">
-        <v>194</v>
+        <v>219</v>
       </c>
       <c r="L40" s="9" t="s">
-        <v>195</v>
+        <v>220</v>
       </c>
       <c r="M40" s="9" t="s">
         <v>52</v>
       </c>
       <c r="N40" s="9" t="s">
-        <v>146</v>
+        <v>221</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2868,7 +3019,7 @@
       </c>
       <c r="D41" s="6"/>
       <c r="E41" s="6" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F41" s="6"/>
       <c r="G41" s="6"/>
@@ -2879,7 +3030,7 @@
       <c r="L41" s="6"/>
       <c r="M41" s="6"/>
       <c r="N41" s="6" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2894,7 +3045,7 @@
       </c>
       <c r="D42" s="9"/>
       <c r="E42" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F42" s="9"/>
       <c r="G42" s="9"/>
@@ -2905,7 +3056,7 @@
       <c r="L42" s="9"/>
       <c r="M42" s="9"/>
       <c r="N42" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2920,7 +3071,7 @@
       </c>
       <c r="D43" s="9"/>
       <c r="E43" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F43" s="9"/>
       <c r="G43" s="9"/>
@@ -2931,7 +3082,7 @@
       <c r="L43" s="9"/>
       <c r="M43" s="9"/>
       <c r="N43" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2946,7 +3097,7 @@
       </c>
       <c r="D44" s="9"/>
       <c r="E44" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F44" s="9"/>
       <c r="G44" s="9"/>
@@ -2957,7 +3108,7 @@
       <c r="L44" s="9"/>
       <c r="M44" s="9"/>
       <c r="N44" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2972,7 +3123,7 @@
       </c>
       <c r="D45" s="9"/>
       <c r="E45" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F45" s="9"/>
       <c r="G45" s="9"/>
@@ -2983,7 +3134,7 @@
       <c r="L45" s="9"/>
       <c r="M45" s="9"/>
       <c r="N45" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2998,7 +3149,7 @@
       </c>
       <c r="D46" s="9"/>
       <c r="E46" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F46" s="9"/>
       <c r="G46" s="9"/>
@@ -3009,7 +3160,7 @@
       <c r="L46" s="9"/>
       <c r="M46" s="9"/>
       <c r="N46" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3024,7 +3175,7 @@
       </c>
       <c r="D47" s="9"/>
       <c r="E47" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F47" s="9"/>
       <c r="G47" s="9"/>
@@ -3035,7 +3186,7 @@
       <c r="L47" s="9"/>
       <c r="M47" s="9"/>
       <c r="N47" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3050,7 +3201,7 @@
       </c>
       <c r="D48" s="9"/>
       <c r="E48" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F48" s="9"/>
       <c r="G48" s="9"/>
@@ -3061,7 +3212,7 @@
       <c r="L48" s="9"/>
       <c r="M48" s="9"/>
       <c r="N48" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3076,7 +3227,7 @@
       </c>
       <c r="D49" s="9"/>
       <c r="E49" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F49" s="9"/>
       <c r="G49" s="9"/>
@@ -3087,7 +3238,7 @@
       <c r="L49" s="9"/>
       <c r="M49" s="9"/>
       <c r="N49" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3102,7 +3253,7 @@
       </c>
       <c r="D50" s="9"/>
       <c r="E50" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F50" s="9"/>
       <c r="G50" s="9"/>
@@ -3113,7 +3264,7 @@
       <c r="L50" s="9"/>
       <c r="M50" s="9"/>
       <c r="N50" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3127,37 +3278,37 @@
         <v>46347</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>196</v>
+        <v>222</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>197</v>
+        <v>223</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>199</v>
+        <v>225</v>
       </c>
       <c r="H51" s="9" t="s">
-        <v>200</v>
+        <v>226</v>
       </c>
       <c r="I51" s="9" t="s">
-        <v>201</v>
+        <v>227</v>
       </c>
       <c r="J51" s="9" t="s">
-        <v>202</v>
+        <v>228</v>
       </c>
       <c r="K51" s="9" t="s">
-        <v>203</v>
+        <v>229</v>
       </c>
       <c r="L51" s="9" t="s">
-        <v>204</v>
+        <v>230</v>
       </c>
       <c r="M51" s="9" t="s">
-        <v>205</v>
+        <v>231</v>
       </c>
       <c r="N51" s="9" t="s">
-        <v>146</v>
+        <v>221</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3172,7 +3323,7 @@
       </c>
       <c r="D52" s="6"/>
       <c r="E52" s="6" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F52" s="6"/>
       <c r="G52" s="6"/>
@@ -3183,7 +3334,7 @@
       <c r="L52" s="6"/>
       <c r="M52" s="6"/>
       <c r="N52" s="6" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3198,7 +3349,7 @@
       </c>
       <c r="D53" s="9"/>
       <c r="E53" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F53" s="9"/>
       <c r="G53" s="9"/>
@@ -3209,7 +3360,7 @@
       <c r="L53" s="9"/>
       <c r="M53" s="9"/>
       <c r="N53" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3224,7 +3375,7 @@
       </c>
       <c r="D54" s="9"/>
       <c r="E54" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F54" s="9"/>
       <c r="G54" s="9"/>
@@ -3235,7 +3386,7 @@
       <c r="L54" s="9"/>
       <c r="M54" s="9"/>
       <c r="N54" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3250,7 +3401,7 @@
       </c>
       <c r="D55" s="9"/>
       <c r="E55" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F55" s="9"/>
       <c r="G55" s="9"/>
@@ -3261,7 +3412,7 @@
       <c r="L55" s="9"/>
       <c r="M55" s="9"/>
       <c r="N55" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3278,34 +3429,34 @@
         <v>53</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>206</v>
+        <v>232</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>207</v>
+        <v>233</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>208</v>
+        <v>234</v>
       </c>
       <c r="H56" s="9" t="s">
-        <v>209</v>
+        <v>235</v>
       </c>
       <c r="I56" s="9" t="s">
-        <v>210</v>
+        <v>236</v>
       </c>
       <c r="J56" s="9" t="s">
-        <v>211</v>
+        <v>237</v>
       </c>
       <c r="K56" s="9" t="s">
-        <v>212</v>
+        <v>238</v>
       </c>
       <c r="L56" s="9" t="s">
-        <v>213</v>
+        <v>239</v>
       </c>
       <c r="M56" s="9" t="s">
         <v>120</v>
       </c>
       <c r="N56" s="9" t="s">
-        <v>146</v>
+        <v>221</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3320,7 +3471,7 @@
       </c>
       <c r="D57" s="11"/>
       <c r="E57" s="11" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F57" s="11"/>
       <c r="G57" s="11"/>
@@ -3331,7 +3482,7 @@
       <c r="L57" s="11"/>
       <c r="M57" s="11"/>
       <c r="N57" s="11" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3346,7 +3497,7 @@
       </c>
       <c r="D58" s="9"/>
       <c r="E58" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F58" s="9"/>
       <c r="G58" s="9"/>
@@ -3357,7 +3508,7 @@
       <c r="L58" s="9"/>
       <c r="M58" s="9"/>
       <c r="N58" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3372,7 +3523,7 @@
       </c>
       <c r="D59" s="9"/>
       <c r="E59" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F59" s="9"/>
       <c r="G59" s="9"/>
@@ -3383,7 +3534,7 @@
       <c r="L59" s="9"/>
       <c r="M59" s="9"/>
       <c r="N59" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3398,7 +3549,7 @@
       </c>
       <c r="D60" s="9"/>
       <c r="E60" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F60" s="9"/>
       <c r="G60" s="9"/>
@@ -3409,7 +3560,7 @@
       <c r="L60" s="9"/>
       <c r="M60" s="9"/>
       <c r="N60" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3424,7 +3575,7 @@
       </c>
       <c r="D61" s="9"/>
       <c r="E61" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F61" s="9"/>
       <c r="G61" s="9"/>
@@ -3435,7 +3586,7 @@
       <c r="L61" s="9"/>
       <c r="M61" s="9"/>
       <c r="N61" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3450,7 +3601,7 @@
       </c>
       <c r="D62" s="9"/>
       <c r="E62" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F62" s="9"/>
       <c r="G62" s="9"/>
@@ -3461,7 +3612,7 @@
       <c r="L62" s="9"/>
       <c r="M62" s="9"/>
       <c r="N62" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3476,7 +3627,7 @@
       </c>
       <c r="D63" s="9"/>
       <c r="E63" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F63" s="9"/>
       <c r="G63" s="9"/>
@@ -3487,7 +3638,7 @@
       <c r="L63" s="9"/>
       <c r="M63" s="9"/>
       <c r="N63" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3502,7 +3653,7 @@
       </c>
       <c r="D64" s="9"/>
       <c r="E64" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F64" s="9"/>
       <c r="G64" s="9"/>
@@ -3513,7 +3664,7 @@
       <c r="L64" s="9"/>
       <c r="M64" s="9"/>
       <c r="N64" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3528,7 +3679,7 @@
       </c>
       <c r="D65" s="9"/>
       <c r="E65" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F65" s="9"/>
       <c r="G65" s="9"/>
@@ -3539,7 +3690,7 @@
       <c r="L65" s="9"/>
       <c r="M65" s="9"/>
       <c r="N65" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3554,7 +3705,7 @@
       </c>
       <c r="D66" s="9"/>
       <c r="E66" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F66" s="9"/>
       <c r="G66" s="9"/>
@@ -3565,7 +3716,7 @@
       <c r="L66" s="9"/>
       <c r="M66" s="9"/>
       <c r="N66" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3580,7 +3731,7 @@
       </c>
       <c r="D67" s="9"/>
       <c r="E67" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F67" s="9"/>
       <c r="G67" s="9"/>
@@ -3591,7 +3742,7 @@
       <c r="L67" s="9"/>
       <c r="M67" s="9"/>
       <c r="N67" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3608,34 +3759,34 @@
         <v>155</v>
       </c>
       <c r="E68" s="9" t="s">
-        <v>214</v>
+        <v>240</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>215</v>
+        <v>241</v>
       </c>
       <c r="G68" s="9" t="s">
-        <v>216</v>
+        <v>242</v>
       </c>
       <c r="H68" s="9" t="s">
-        <v>217</v>
+        <v>243</v>
       </c>
       <c r="I68" s="9" t="s">
-        <v>218</v>
+        <v>244</v>
       </c>
       <c r="J68" s="9" t="s">
-        <v>219</v>
+        <v>245</v>
       </c>
       <c r="K68" s="9" t="s">
-        <v>220</v>
+        <v>246</v>
       </c>
       <c r="L68" s="9" t="s">
-        <v>221</v>
+        <v>247</v>
       </c>
       <c r="M68" s="9" t="s">
         <v>52</v>
       </c>
       <c r="N68" s="9" t="s">
-        <v>146</v>
+        <v>221</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3650,7 +3801,7 @@
       </c>
       <c r="D69" s="6"/>
       <c r="E69" s="6" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F69" s="6"/>
       <c r="G69" s="6"/>
@@ -3661,7 +3812,7 @@
       <c r="L69" s="6"/>
       <c r="M69" s="6"/>
       <c r="N69" s="6" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3676,7 +3827,7 @@
       </c>
       <c r="D70" s="9"/>
       <c r="E70" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F70" s="9"/>
       <c r="G70" s="9"/>
@@ -3687,7 +3838,7 @@
       <c r="L70" s="9"/>
       <c r="M70" s="9"/>
       <c r="N70" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3702,7 +3853,7 @@
       </c>
       <c r="D71" s="9"/>
       <c r="E71" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F71" s="9"/>
       <c r="G71" s="9"/>
@@ -3713,7 +3864,7 @@
       <c r="L71" s="9"/>
       <c r="M71" s="9"/>
       <c r="N71" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3728,7 +3879,7 @@
       </c>
       <c r="D72" s="9"/>
       <c r="E72" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F72" s="9"/>
       <c r="G72" s="9"/>
@@ -3739,7 +3890,7 @@
       <c r="L72" s="9"/>
       <c r="M72" s="9"/>
       <c r="N72" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3754,7 +3905,7 @@
       </c>
       <c r="D73" s="9"/>
       <c r="E73" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F73" s="9"/>
       <c r="G73" s="9"/>
@@ -3765,7 +3916,7 @@
       <c r="L73" s="9"/>
       <c r="M73" s="9"/>
       <c r="N73" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3780,7 +3931,7 @@
       </c>
       <c r="D74" s="9"/>
       <c r="E74" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F74" s="9"/>
       <c r="G74" s="9"/>
@@ -3791,7 +3942,7 @@
       <c r="L74" s="9"/>
       <c r="M74" s="9"/>
       <c r="N74" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3808,34 +3959,34 @@
         <v>155</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>222</v>
+        <v>248</v>
       </c>
       <c r="F75" s="9" t="s">
-        <v>223</v>
+        <v>249</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>224</v>
+        <v>250</v>
       </c>
       <c r="H75" s="9" t="s">
-        <v>225</v>
+        <v>251</v>
       </c>
       <c r="I75" s="9" t="s">
-        <v>226</v>
+        <v>252</v>
       </c>
       <c r="J75" s="9" t="s">
-        <v>227</v>
+        <v>253</v>
       </c>
       <c r="K75" s="9" t="s">
-        <v>228</v>
+        <v>254</v>
       </c>
       <c r="L75" s="9" t="s">
-        <v>229</v>
+        <v>255</v>
       </c>
       <c r="M75" s="9" t="s">
-        <v>230</v>
+        <v>256</v>
       </c>
       <c r="N75" s="9" t="s">
-        <v>146</v>
+        <v>221</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3850,7 +4001,7 @@
       </c>
       <c r="D76" s="11"/>
       <c r="E76" s="11" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F76" s="11"/>
       <c r="G76" s="11"/>
@@ -3861,7 +4012,7 @@
       <c r="L76" s="11"/>
       <c r="M76" s="11"/>
       <c r="N76" s="11" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3876,7 +4027,7 @@
       </c>
       <c r="D77" s="9"/>
       <c r="E77" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F77" s="9"/>
       <c r="G77" s="9"/>
@@ -3887,7 +4038,7 @@
       <c r="L77" s="9"/>
       <c r="M77" s="9"/>
       <c r="N77" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3902,7 +4053,7 @@
       </c>
       <c r="D78" s="9"/>
       <c r="E78" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F78" s="9"/>
       <c r="G78" s="9"/>
@@ -3913,7 +4064,7 @@
       <c r="L78" s="9"/>
       <c r="M78" s="9"/>
       <c r="N78" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3928,7 +4079,7 @@
       </c>
       <c r="D79" s="9"/>
       <c r="E79" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F79" s="9"/>
       <c r="G79" s="9"/>
@@ -3939,7 +4090,7 @@
       <c r="L79" s="9"/>
       <c r="M79" s="9"/>
       <c r="N79" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3954,7 +4105,7 @@
       </c>
       <c r="D80" s="9"/>
       <c r="E80" s="9" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="F80" s="9"/>
       <c r="G80" s="9"/>
@@ -3965,7 +4116,7 @@
       <c r="L80" s="9"/>
       <c r="M80" s="9"/>
       <c r="N80" s="9" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -4001,15 +4152,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>231</v>
+        <v>257</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>232</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>233</v>
+        <v>259</v>
       </c>
       <c r="B2" s="15" t="n">
         <f aca="false">COUNTA('Lịch đăng'!$A$2:$A$80)</f>
@@ -4027,20 +4178,20 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>234</v>
+        <v>260</v>
       </c>
       <c r="B4" s="15" t="n">
         <f aca="false">COUNTIF('Lịch đăng'!$N$2:$N$80,"Cần chủ đề")</f>
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>235</v>
+        <v>261</v>
       </c>
       <c r="B5" s="15" t="n">
         <f aca="false">B2-B3-B4</f>
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Schedule: topic ideas for 26 Oct and 28 Oct to 1 Nov
Six topics proposed by the Marketing session, approved by Tin on 17/10.
Status is "Ý tưởng"; sources still need checking at the original page in
the Saturday script run.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015wnXjaRHuK6RciQ3JeDviz
</commit_message>
<xml_diff>
--- a/video/plan/lich-noi-dung-tiktok.xlsx
+++ b/video/plan/lich-noi-dung-tiktok.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="297">
   <si>
     <t xml:space="preserve">Lịch nội dung TikTok Adtek</t>
   </si>
@@ -751,31 +751,159 @@
     <t xml:space="preserve">seo ai; viết bài bằng ai</t>
   </si>
   <si>
+    <t xml:space="preserve">AIO, Performance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quảng cáo trên ChatGPT đã chạy ở Việt Nam, ai nên thử? (tin nóng)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quảng cáo trên ChatGPT đã chạy ở Việt Nam từ 23/9, ngành của bạn nên thử hay nên chờ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• OpenAI mở ChatGPT Ads tại Việt Nam 23/9/2026, chỉ hiện với gói Free và Go
+• 81% người dùng AI tại Việt Nam dùng ChatGPT (Decision Lab 8/2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• OpenAI (9/2026)
+• Decision Lab (8/2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://openai.com/index/chatgpt-ads-expands-southeast-asia-taiwan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chưa kiểm tra. Đề xuất của phiên Marketing (17/10/2026, content/editorial/calendar.json, nhánh claude/brave-curie-2c6zbc). Lượt viết kịch bản thứ Bảy phải mở link gốc kiểm tra từng số, số không khớp thì bỏ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Số Decision Lab đã hơn 1 năm: tìm số mới hơn hoặc ghi rõ năm trên video
+• Cùng ngày với bài blog 33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ý tưởng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biểu đồ đua: Shopee và TikTok Shop, khoảng cách 22 điểm còn 11 điểm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shopee còn giữ ngôi số 1 được bao lâu? Năm 2024, Shopee chiếm 64% doanh số các sàn, TikTok Shop 29%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thị phần doanh số tháng 1 đến 9/2025: Shopee 59% xuống 54%, TikTok Shop 37% lên 43%; năm 2024: Shopee 64%, TikTok Shop 29%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://metric.vn/insights/metric-bao-cao-thi-truong-san-thuong-mai-dien-tu-viet-nam-quy-3-2025/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đã mở báo cáo và biểu đồ gốc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Không có lượt vượt mặt. Cách video shop Mall (12/10) hơn 2 tuần. Dạng biểu đồ đua.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giảm giá 30% ngày 11.11, mỗi đơn còn lãi bao nhiêu? (chữ động)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giảm giá 30% ngày 11.11, mỗi đơn còn lãi bao nhiêu?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Ví dụ serum 400,000 đồng: lãi 123,000 đồng/đơn
+• Giảm 30%: ROAS 8 còn 46,800 đồng, ROAS 5 còn 25,800 đồng; phải bán gấp 2.6 lần
+• Phí xử lý giao dịch 6% từ 5/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Bài blog Adtek: Kế hoạch 11.11 (phép tính ví dụ)
+• Phí 6%: cần nguồn chính thức của sàn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://adtek.agency/ke-hoach-11-11/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Phép tính là ví dụ, ghi rõ trên video
+• Phí giao dịch 6% phải lấy từ thông báo chính thức của sàn, không lấy từ blog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Performance, App Marketing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GMV Max: AI chạy quảng cáo thay bạn, bạn còn làm gì? (giải thích)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GMV Max: AI chạy quảng cáo thay bạn, bạn còn làm gì?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• GMV Max là loại chiến dịch duy nhất cho TikTok Shop Ads từ 7/2025
+• Người làm marketing kiểm soát creative, sản phẩm, ngân sách, ROI mục tiêu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• TikTok Ads Help Center
+• Bài blog 10 (đăng 19/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Cần link trang TikTok Ads Help Center gốc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quảng cáo dùng AI phải gắn nhãn từ khi nào? (luật mới)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quảng cáo dùng AI phải gắn nhãn từ khi nào?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Luật Trí tuệ nhân tạo 134/2025/QH15 hiệu lực 1/3/2026
+• Nghị định 142/2026 hiệu lực 1/5/2026, Điều 18: nội dung mô phỏng ngoại hình, giọng nói người thật phải gắn nhãn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Quốc hội, Luật Trí tuệ nhân tạo 134/2025/QH15
+• Chính phủ, Nghị định 142/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Nội dung pháp lý, nên nhờ luật sư duyệt
+• Liên quan trực tiếp tới kênh này (giọng nhân bản của anh Tin): kiểm tra video của kênh có cần dòng "Giọng đọc tạo bằng AI" không</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hàng tiêu dùng nhanh trên sàn tăng bao nhiêu % quý III? (đố số liệu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đoán thử: hàng tiêu dùng nhanh trên sàn tăng bao nhiêu % trong quý III? A 12%, B 26%, C 36%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• FMCG trên sàn quý III/2026 tăng 36% (đáp án C); 9 tháng tăng 26%
+• GMV 9 tháng 411,800 tỷ đồng (+22%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• YouNet ECI, báo cáo quý III/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Khác chỉ số dùng ở video 23/10, kiểm tra không trùng ý
+• Ảnh bìa, khung đầu, caption không lộ đáp án</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Performance, SEO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bật AI Max là mất quyền kiểm soát từ khóa? (phá hiểu lầm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bật AI Max là mất quyền kiểm soát từ khóa?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Vẫn giữ được loại trừ thương hiệu, loại trừ URL, từ khóa phủ định
+• Google nói AI Max tăng 14% chuyển đổi ở cùng CPA (số nội bộ Google)
+• Nên chạy Experiments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Google Ads (5/2025)
+• Bài blog 8 (đăng 30/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Số 14% là số nội bộ Google, ghi rõ trên video</t>
+  </si>
+  <si>
     <t xml:space="preserve">Slot trống: chủ đề trend Claude tự chọn khi viết kịch bản thứ Bảy</t>
   </si>
   <si>
     <t xml:space="preserve">Cần chủ đề</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Biểu đồ đua: Shopee và TikTok Shop, khoảng cách 22 điểm còn 11 điểm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shopee còn giữ ngôi số 1 được bao lâu? Năm 2024, Shopee chiếm 64% doanh số các sàn, TikTok Shop 29%.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thị phần doanh số tháng 1 đến 9/2025: Shopee 59% xuống 54%, TikTok Shop 37% lên 43%; năm 2024: Shopee 64%, TikTok Shop 29%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Metric</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://metric.vn/insights/metric-bao-cao-thi-truong-san-thuong-mai-dien-tu-viet-nam-quy-3-2025/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đã mở báo cáo và biểu đồ gốc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Không có lượt vượt mặt. Cách video shop Mall (12/10) hơn 2 tuần. Dạng biểu đồ đua.</t>
   </si>
   <si>
     <t xml:space="preserve">TikTok Shop hay Shopee?</t>
@@ -810,12 +938,6 @@
   </si>
   <si>
     <t xml:space="preserve">tiktok shop; shopee hay tiktok shop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ý tưởng</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AIO, Performance</t>
   </si>
   <si>
     <t xml:space="preserve">Khách đến từ AI mua nhiều hơn</t>
@@ -2569,20 +2691,34 @@
       <c r="C25" s="10" t="n">
         <v>46321</v>
       </c>
-      <c r="D25" s="9"/>
+      <c r="D25" s="9" t="s">
+        <v>204</v>
+      </c>
       <c r="E25" s="9" t="s">
-        <v>204</v>
-      </c>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="9"/>
-      <c r="J25" s="9"/>
-      <c r="K25" s="9"/>
+        <v>205</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="H25" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="I25" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="J25" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="K25" s="9" t="s">
+        <v>211</v>
+      </c>
       <c r="L25" s="9"/>
       <c r="M25" s="9"/>
       <c r="N25" s="9" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2599,25 +2735,25 @@
         <v>103</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="I26" s="9" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="J26" s="9" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="L26" s="9"/>
       <c r="M26" s="9"/>
@@ -2635,20 +2771,34 @@
       <c r="C27" s="10" t="n">
         <v>46323</v>
       </c>
-      <c r="D27" s="9"/>
+      <c r="D27" s="9" t="s">
+        <v>85</v>
+      </c>
       <c r="E27" s="9" t="s">
-        <v>204</v>
-      </c>
-      <c r="F27" s="9"/>
-      <c r="G27" s="9"/>
-      <c r="H27" s="9"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="9"/>
-      <c r="K27" s="9"/>
+        <v>220</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="G27" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="H27" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="I27" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="J27" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="K27" s="9" t="s">
+        <v>225</v>
+      </c>
       <c r="L27" s="9"/>
       <c r="M27" s="9"/>
       <c r="N27" s="9" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2661,20 +2811,32 @@
       <c r="C28" s="10" t="n">
         <v>46324</v>
       </c>
-      <c r="D28" s="9"/>
+      <c r="D28" s="9" t="s">
+        <v>226</v>
+      </c>
       <c r="E28" s="9" t="s">
-        <v>204</v>
-      </c>
-      <c r="F28" s="9"/>
-      <c r="G28" s="9"/>
-      <c r="H28" s="9"/>
+        <v>227</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="G28" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>230</v>
+      </c>
       <c r="I28" s="9"/>
-      <c r="J28" s="9"/>
-      <c r="K28" s="9"/>
+      <c r="J28" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="K28" s="9" t="s">
+        <v>231</v>
+      </c>
       <c r="L28" s="9"/>
       <c r="M28" s="9"/>
       <c r="N28" s="9" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2687,20 +2849,32 @@
       <c r="C29" s="10" t="n">
         <v>46325</v>
       </c>
-      <c r="D29" s="9"/>
+      <c r="D29" s="9" t="s">
+        <v>75</v>
+      </c>
       <c r="E29" s="9" t="s">
-        <v>204</v>
-      </c>
-      <c r="F29" s="9"/>
-      <c r="G29" s="9"/>
-      <c r="H29" s="9"/>
+        <v>232</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="G29" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="H29" s="9" t="s">
+        <v>235</v>
+      </c>
       <c r="I29" s="9"/>
-      <c r="J29" s="9"/>
-      <c r="K29" s="9"/>
+      <c r="J29" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="K29" s="9" t="s">
+        <v>236</v>
+      </c>
       <c r="L29" s="9"/>
       <c r="M29" s="9"/>
       <c r="N29" s="9" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2713,20 +2887,32 @@
       <c r="C30" s="10" t="n">
         <v>46326</v>
       </c>
-      <c r="D30" s="9"/>
+      <c r="D30" s="9" t="s">
+        <v>66</v>
+      </c>
       <c r="E30" s="9" t="s">
-        <v>204</v>
-      </c>
-      <c r="F30" s="9"/>
-      <c r="G30" s="9"/>
-      <c r="H30" s="9"/>
+        <v>237</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="G30" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="H30" s="9" t="s">
+        <v>240</v>
+      </c>
       <c r="I30" s="9"/>
-      <c r="J30" s="9"/>
-      <c r="K30" s="9"/>
+      <c r="J30" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="K30" s="9" t="s">
+        <v>241</v>
+      </c>
       <c r="L30" s="9"/>
       <c r="M30" s="9"/>
       <c r="N30" s="9" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2739,20 +2925,32 @@
       <c r="C31" s="10" t="n">
         <v>46327</v>
       </c>
-      <c r="D31" s="9"/>
+      <c r="D31" s="9" t="s">
+        <v>242</v>
+      </c>
       <c r="E31" s="9" t="s">
-        <v>204</v>
-      </c>
-      <c r="F31" s="9"/>
-      <c r="G31" s="9"/>
-      <c r="H31" s="9"/>
+        <v>243</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>246</v>
+      </c>
       <c r="I31" s="9"/>
-      <c r="J31" s="9"/>
-      <c r="K31" s="9"/>
+      <c r="J31" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="K31" s="9" t="s">
+        <v>247</v>
+      </c>
       <c r="L31" s="9"/>
       <c r="M31" s="9"/>
       <c r="N31" s="9" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2767,7 +2965,7 @@
       </c>
       <c r="D32" s="9"/>
       <c r="E32" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F32" s="9"/>
       <c r="G32" s="9"/>
@@ -2778,7 +2976,7 @@
       <c r="L32" s="9"/>
       <c r="M32" s="9"/>
       <c r="N32" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2793,7 +2991,7 @@
       </c>
       <c r="D33" s="9"/>
       <c r="E33" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F33" s="9"/>
       <c r="G33" s="9"/>
@@ -2804,7 +3002,7 @@
       <c r="L33" s="9"/>
       <c r="M33" s="9"/>
       <c r="N33" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2819,7 +3017,7 @@
       </c>
       <c r="D34" s="9"/>
       <c r="E34" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F34" s="9"/>
       <c r="G34" s="9"/>
@@ -2830,7 +3028,7 @@
       <c r="L34" s="9"/>
       <c r="M34" s="9"/>
       <c r="N34" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2845,7 +3043,7 @@
       </c>
       <c r="D35" s="9"/>
       <c r="E35" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F35" s="9"/>
       <c r="G35" s="9"/>
@@ -2856,7 +3054,7 @@
       <c r="L35" s="9"/>
       <c r="M35" s="9"/>
       <c r="N35" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2871,7 +3069,7 @@
       </c>
       <c r="D36" s="9"/>
       <c r="E36" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F36" s="9"/>
       <c r="G36" s="9"/>
@@ -2882,7 +3080,7 @@
       <c r="L36" s="9"/>
       <c r="M36" s="9"/>
       <c r="N36" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2897,7 +3095,7 @@
       </c>
       <c r="D37" s="9"/>
       <c r="E37" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F37" s="9"/>
       <c r="G37" s="9"/>
@@ -2908,7 +3106,7 @@
       <c r="L37" s="9"/>
       <c r="M37" s="9"/>
       <c r="N37" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2923,7 +3121,7 @@
       </c>
       <c r="D38" s="9"/>
       <c r="E38" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F38" s="9"/>
       <c r="G38" s="9"/>
@@ -2934,7 +3132,7 @@
       <c r="L38" s="9"/>
       <c r="M38" s="9"/>
       <c r="N38" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2949,7 +3147,7 @@
       </c>
       <c r="D39" s="9"/>
       <c r="E39" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F39" s="9"/>
       <c r="G39" s="9"/>
@@ -2960,7 +3158,7 @@
       <c r="L39" s="9"/>
       <c r="M39" s="9"/>
       <c r="N39" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2977,34 +3175,34 @@
         <v>155</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>213</v>
+        <v>250</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>214</v>
+        <v>251</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>215</v>
+        <v>252</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>216</v>
+        <v>253</v>
       </c>
       <c r="I40" s="9" t="s">
-        <v>217</v>
+        <v>254</v>
       </c>
       <c r="J40" s="9" t="s">
-        <v>218</v>
+        <v>255</v>
       </c>
       <c r="K40" s="9" t="s">
-        <v>219</v>
+        <v>256</v>
       </c>
       <c r="L40" s="9" t="s">
-        <v>220</v>
+        <v>257</v>
       </c>
       <c r="M40" s="9" t="s">
         <v>52</v>
       </c>
       <c r="N40" s="9" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3019,7 +3217,7 @@
       </c>
       <c r="D41" s="6"/>
       <c r="E41" s="6" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F41" s="6"/>
       <c r="G41" s="6"/>
@@ -3030,7 +3228,7 @@
       <c r="L41" s="6"/>
       <c r="M41" s="6"/>
       <c r="N41" s="6" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3045,7 +3243,7 @@
       </c>
       <c r="D42" s="9"/>
       <c r="E42" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F42" s="9"/>
       <c r="G42" s="9"/>
@@ -3056,7 +3254,7 @@
       <c r="L42" s="9"/>
       <c r="M42" s="9"/>
       <c r="N42" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3071,7 +3269,7 @@
       </c>
       <c r="D43" s="9"/>
       <c r="E43" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F43" s="9"/>
       <c r="G43" s="9"/>
@@ -3082,7 +3280,7 @@
       <c r="L43" s="9"/>
       <c r="M43" s="9"/>
       <c r="N43" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3097,7 +3295,7 @@
       </c>
       <c r="D44" s="9"/>
       <c r="E44" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F44" s="9"/>
       <c r="G44" s="9"/>
@@ -3108,7 +3306,7 @@
       <c r="L44" s="9"/>
       <c r="M44" s="9"/>
       <c r="N44" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3123,7 +3321,7 @@
       </c>
       <c r="D45" s="9"/>
       <c r="E45" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F45" s="9"/>
       <c r="G45" s="9"/>
@@ -3134,7 +3332,7 @@
       <c r="L45" s="9"/>
       <c r="M45" s="9"/>
       <c r="N45" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3149,7 +3347,7 @@
       </c>
       <c r="D46" s="9"/>
       <c r="E46" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F46" s="9"/>
       <c r="G46" s="9"/>
@@ -3160,7 +3358,7 @@
       <c r="L46" s="9"/>
       <c r="M46" s="9"/>
       <c r="N46" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3175,7 +3373,7 @@
       </c>
       <c r="D47" s="9"/>
       <c r="E47" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F47" s="9"/>
       <c r="G47" s="9"/>
@@ -3186,7 +3384,7 @@
       <c r="L47" s="9"/>
       <c r="M47" s="9"/>
       <c r="N47" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3201,7 +3399,7 @@
       </c>
       <c r="D48" s="9"/>
       <c r="E48" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F48" s="9"/>
       <c r="G48" s="9"/>
@@ -3212,7 +3410,7 @@
       <c r="L48" s="9"/>
       <c r="M48" s="9"/>
       <c r="N48" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3227,7 +3425,7 @@
       </c>
       <c r="D49" s="9"/>
       <c r="E49" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F49" s="9"/>
       <c r="G49" s="9"/>
@@ -3238,7 +3436,7 @@
       <c r="L49" s="9"/>
       <c r="M49" s="9"/>
       <c r="N49" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3253,7 +3451,7 @@
       </c>
       <c r="D50" s="9"/>
       <c r="E50" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F50" s="9"/>
       <c r="G50" s="9"/>
@@ -3264,7 +3462,7 @@
       <c r="L50" s="9"/>
       <c r="M50" s="9"/>
       <c r="N50" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3278,37 +3476,37 @@
         <v>46347</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>222</v>
+        <v>204</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>223</v>
+        <v>258</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>224</v>
+        <v>259</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>225</v>
+        <v>260</v>
       </c>
       <c r="H51" s="9" t="s">
-        <v>226</v>
+        <v>261</v>
       </c>
       <c r="I51" s="9" t="s">
-        <v>227</v>
+        <v>262</v>
       </c>
       <c r="J51" s="9" t="s">
-        <v>228</v>
+        <v>263</v>
       </c>
       <c r="K51" s="9" t="s">
-        <v>229</v>
+        <v>264</v>
       </c>
       <c r="L51" s="9" t="s">
-        <v>230</v>
+        <v>265</v>
       </c>
       <c r="M51" s="9" t="s">
-        <v>231</v>
+        <v>266</v>
       </c>
       <c r="N51" s="9" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3323,7 +3521,7 @@
       </c>
       <c r="D52" s="6"/>
       <c r="E52" s="6" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F52" s="6"/>
       <c r="G52" s="6"/>
@@ -3334,7 +3532,7 @@
       <c r="L52" s="6"/>
       <c r="M52" s="6"/>
       <c r="N52" s="6" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3349,7 +3547,7 @@
       </c>
       <c r="D53" s="9"/>
       <c r="E53" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F53" s="9"/>
       <c r="G53" s="9"/>
@@ -3360,7 +3558,7 @@
       <c r="L53" s="9"/>
       <c r="M53" s="9"/>
       <c r="N53" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3375,7 +3573,7 @@
       </c>
       <c r="D54" s="9"/>
       <c r="E54" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F54" s="9"/>
       <c r="G54" s="9"/>
@@ -3386,7 +3584,7 @@
       <c r="L54" s="9"/>
       <c r="M54" s="9"/>
       <c r="N54" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3401,7 +3599,7 @@
       </c>
       <c r="D55" s="9"/>
       <c r="E55" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F55" s="9"/>
       <c r="G55" s="9"/>
@@ -3412,7 +3610,7 @@
       <c r="L55" s="9"/>
       <c r="M55" s="9"/>
       <c r="N55" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3429,34 +3627,34 @@
         <v>53</v>
       </c>
       <c r="E56" s="9" t="s">
-        <v>232</v>
+        <v>267</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>233</v>
+        <v>268</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>234</v>
+        <v>269</v>
       </c>
       <c r="H56" s="9" t="s">
-        <v>235</v>
+        <v>270</v>
       </c>
       <c r="I56" s="9" t="s">
-        <v>236</v>
+        <v>271</v>
       </c>
       <c r="J56" s="9" t="s">
-        <v>237</v>
+        <v>272</v>
       </c>
       <c r="K56" s="9" t="s">
-        <v>238</v>
+        <v>273</v>
       </c>
       <c r="L56" s="9" t="s">
-        <v>239</v>
+        <v>274</v>
       </c>
       <c r="M56" s="9" t="s">
         <v>120</v>
       </c>
       <c r="N56" s="9" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3471,7 +3669,7 @@
       </c>
       <c r="D57" s="11"/>
       <c r="E57" s="11" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F57" s="11"/>
       <c r="G57" s="11"/>
@@ -3482,7 +3680,7 @@
       <c r="L57" s="11"/>
       <c r="M57" s="11"/>
       <c r="N57" s="11" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3497,7 +3695,7 @@
       </c>
       <c r="D58" s="9"/>
       <c r="E58" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F58" s="9"/>
       <c r="G58" s="9"/>
@@ -3508,7 +3706,7 @@
       <c r="L58" s="9"/>
       <c r="M58" s="9"/>
       <c r="N58" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3523,7 +3721,7 @@
       </c>
       <c r="D59" s="9"/>
       <c r="E59" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F59" s="9"/>
       <c r="G59" s="9"/>
@@ -3534,7 +3732,7 @@
       <c r="L59" s="9"/>
       <c r="M59" s="9"/>
       <c r="N59" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3549,7 +3747,7 @@
       </c>
       <c r="D60" s="9"/>
       <c r="E60" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F60" s="9"/>
       <c r="G60" s="9"/>
@@ -3560,7 +3758,7 @@
       <c r="L60" s="9"/>
       <c r="M60" s="9"/>
       <c r="N60" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3575,7 +3773,7 @@
       </c>
       <c r="D61" s="9"/>
       <c r="E61" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F61" s="9"/>
       <c r="G61" s="9"/>
@@ -3586,7 +3784,7 @@
       <c r="L61" s="9"/>
       <c r="M61" s="9"/>
       <c r="N61" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3601,7 +3799,7 @@
       </c>
       <c r="D62" s="9"/>
       <c r="E62" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F62" s="9"/>
       <c r="G62" s="9"/>
@@ -3612,7 +3810,7 @@
       <c r="L62" s="9"/>
       <c r="M62" s="9"/>
       <c r="N62" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3627,7 +3825,7 @@
       </c>
       <c r="D63" s="9"/>
       <c r="E63" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F63" s="9"/>
       <c r="G63" s="9"/>
@@ -3638,7 +3836,7 @@
       <c r="L63" s="9"/>
       <c r="M63" s="9"/>
       <c r="N63" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3653,7 +3851,7 @@
       </c>
       <c r="D64" s="9"/>
       <c r="E64" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F64" s="9"/>
       <c r="G64" s="9"/>
@@ -3664,7 +3862,7 @@
       <c r="L64" s="9"/>
       <c r="M64" s="9"/>
       <c r="N64" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3679,7 +3877,7 @@
       </c>
       <c r="D65" s="9"/>
       <c r="E65" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F65" s="9"/>
       <c r="G65" s="9"/>
@@ -3690,7 +3888,7 @@
       <c r="L65" s="9"/>
       <c r="M65" s="9"/>
       <c r="N65" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3705,7 +3903,7 @@
       </c>
       <c r="D66" s="9"/>
       <c r="E66" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F66" s="9"/>
       <c r="G66" s="9"/>
@@ -3716,7 +3914,7 @@
       <c r="L66" s="9"/>
       <c r="M66" s="9"/>
       <c r="N66" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3731,7 +3929,7 @@
       </c>
       <c r="D67" s="9"/>
       <c r="E67" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F67" s="9"/>
       <c r="G67" s="9"/>
@@ -3742,7 +3940,7 @@
       <c r="L67" s="9"/>
       <c r="M67" s="9"/>
       <c r="N67" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3759,34 +3957,34 @@
         <v>155</v>
       </c>
       <c r="E68" s="9" t="s">
-        <v>240</v>
+        <v>275</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>241</v>
+        <v>276</v>
       </c>
       <c r="G68" s="9" t="s">
-        <v>242</v>
+        <v>277</v>
       </c>
       <c r="H68" s="9" t="s">
-        <v>243</v>
+        <v>278</v>
       </c>
       <c r="I68" s="9" t="s">
-        <v>244</v>
+        <v>279</v>
       </c>
       <c r="J68" s="9" t="s">
-        <v>245</v>
+        <v>280</v>
       </c>
       <c r="K68" s="9" t="s">
-        <v>246</v>
+        <v>281</v>
       </c>
       <c r="L68" s="9" t="s">
-        <v>247</v>
+        <v>282</v>
       </c>
       <c r="M68" s="9" t="s">
         <v>52</v>
       </c>
       <c r="N68" s="9" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3801,7 +3999,7 @@
       </c>
       <c r="D69" s="6"/>
       <c r="E69" s="6" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F69" s="6"/>
       <c r="G69" s="6"/>
@@ -3812,7 +4010,7 @@
       <c r="L69" s="6"/>
       <c r="M69" s="6"/>
       <c r="N69" s="6" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3827,7 +4025,7 @@
       </c>
       <c r="D70" s="9"/>
       <c r="E70" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F70" s="9"/>
       <c r="G70" s="9"/>
@@ -3838,7 +4036,7 @@
       <c r="L70" s="9"/>
       <c r="M70" s="9"/>
       <c r="N70" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3853,7 +4051,7 @@
       </c>
       <c r="D71" s="9"/>
       <c r="E71" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F71" s="9"/>
       <c r="G71" s="9"/>
@@ -3864,7 +4062,7 @@
       <c r="L71" s="9"/>
       <c r="M71" s="9"/>
       <c r="N71" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3879,7 +4077,7 @@
       </c>
       <c r="D72" s="9"/>
       <c r="E72" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F72" s="9"/>
       <c r="G72" s="9"/>
@@ -3890,7 +4088,7 @@
       <c r="L72" s="9"/>
       <c r="M72" s="9"/>
       <c r="N72" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3905,7 +4103,7 @@
       </c>
       <c r="D73" s="9"/>
       <c r="E73" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F73" s="9"/>
       <c r="G73" s="9"/>
@@ -3916,7 +4114,7 @@
       <c r="L73" s="9"/>
       <c r="M73" s="9"/>
       <c r="N73" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3931,7 +4129,7 @@
       </c>
       <c r="D74" s="9"/>
       <c r="E74" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F74" s="9"/>
       <c r="G74" s="9"/>
@@ -3942,7 +4140,7 @@
       <c r="L74" s="9"/>
       <c r="M74" s="9"/>
       <c r="N74" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3959,34 +4157,34 @@
         <v>155</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>248</v>
+        <v>283</v>
       </c>
       <c r="F75" s="9" t="s">
-        <v>249</v>
+        <v>284</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>250</v>
+        <v>285</v>
       </c>
       <c r="H75" s="9" t="s">
-        <v>251</v>
+        <v>286</v>
       </c>
       <c r="I75" s="9" t="s">
-        <v>252</v>
+        <v>287</v>
       </c>
       <c r="J75" s="9" t="s">
-        <v>253</v>
+        <v>288</v>
       </c>
       <c r="K75" s="9" t="s">
-        <v>254</v>
+        <v>289</v>
       </c>
       <c r="L75" s="9" t="s">
-        <v>255</v>
+        <v>290</v>
       </c>
       <c r="M75" s="9" t="s">
-        <v>256</v>
+        <v>291</v>
       </c>
       <c r="N75" s="9" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4001,7 +4199,7 @@
       </c>
       <c r="D76" s="11"/>
       <c r="E76" s="11" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F76" s="11"/>
       <c r="G76" s="11"/>
@@ -4012,7 +4210,7 @@
       <c r="L76" s="11"/>
       <c r="M76" s="11"/>
       <c r="N76" s="11" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4027,7 +4225,7 @@
       </c>
       <c r="D77" s="9"/>
       <c r="E77" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F77" s="9"/>
       <c r="G77" s="9"/>
@@ -4038,7 +4236,7 @@
       <c r="L77" s="9"/>
       <c r="M77" s="9"/>
       <c r="N77" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4053,7 +4251,7 @@
       </c>
       <c r="D78" s="9"/>
       <c r="E78" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F78" s="9"/>
       <c r="G78" s="9"/>
@@ -4064,7 +4262,7 @@
       <c r="L78" s="9"/>
       <c r="M78" s="9"/>
       <c r="N78" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4079,7 +4277,7 @@
       </c>
       <c r="D79" s="9"/>
       <c r="E79" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F79" s="9"/>
       <c r="G79" s="9"/>
@@ -4090,7 +4288,7 @@
       <c r="L79" s="9"/>
       <c r="M79" s="9"/>
       <c r="N79" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4105,7 +4303,7 @@
       </c>
       <c r="D80" s="9"/>
       <c r="E80" s="9" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F80" s="9"/>
       <c r="G80" s="9"/>
@@ -4116,7 +4314,7 @@
       <c r="L80" s="9"/>
       <c r="M80" s="9"/>
       <c r="N80" s="9" t="s">
-        <v>205</v>
+        <v>249</v>
       </c>
     </row>
   </sheetData>
@@ -4152,15 +4350,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>257</v>
+        <v>292</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>258</v>
+        <v>293</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="15" t="s">
-        <v>259</v>
+        <v>294</v>
       </c>
       <c r="B2" s="15" t="n">
         <f aca="false">COUNTA('Lịch đăng'!$A$2:$A$80)</f>
@@ -4178,20 +4376,20 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>260</v>
+        <v>295</v>
       </c>
       <c r="B4" s="15" t="n">
         <f aca="false">COUNTIF('Lịch đăng'!$N$2:$N$80,"Cần chủ đề")</f>
-        <v>50</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>261</v>
+        <v>296</v>
       </c>
       <c r="B5" s="15" t="n">
         <f aca="false">B2-B3-B4</f>
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Schedule: 18 Oct video posted on 17 Oct via Zernio
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015wnXjaRHuK6RciQ3JeDviz
</commit_message>
<xml_diff>
--- a/video/plan/lich-noi-dung-tiktok.xlsx
+++ b/video/plan/lich-noi-dung-tiktok.xlsx
@@ -544,13 +544,11 @@
   </si>
   <si>
     <t xml:space="preserve">• Nội dung pháp lý, nên nhờ luật sư duyệt câu chữ
-• Dạng phá hiểu lầm</t>
+• Dạng phá hiểu lầm
+• Đã đăng 17/10/2026 lúc 15:38 qua Zernio (phiên Tiktok post): https://www.tiktok.com/@adtek.growth.marketing/video/7697551427345943860</t>
   </si>
   <si>
     <t xml:space="preserve">luật bảo vệ dữ liệu cá nhân; data khách hàng</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đã viết kịch bản</t>
   </si>
   <si>
     <t xml:space="preserve">Bản đồ: kinh tế số Việt Nam tăng 17%, nhanh thứ 2 Đông Nam Á</t>
@@ -689,6 +687,9 @@
   </si>
   <si>
     <t xml:space="preserve">mua sắm online; sale cuối năm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đã viết kịch bản</t>
   </si>
   <si>
     <t xml:space="preserve">7/10 người Việt từng mua hàng giả (infographic)</t>
@@ -2378,7 +2379,7 @@
         <v>52</v>
       </c>
       <c r="N17" s="11" t="s">
-        <v>146</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2395,28 +2396,28 @@
         <v>137</v>
       </c>
       <c r="E18" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="F18" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="F18" s="11" t="s">
+      <c r="G18" s="11" t="s">
         <v>148</v>
       </c>
-      <c r="G18" s="11" t="s">
+      <c r="H18" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="H18" s="11" t="s">
+      <c r="I18" s="11" t="s">
         <v>150</v>
       </c>
-      <c r="I18" s="11" t="s">
+      <c r="J18" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="J18" s="11" t="s">
+      <c r="K18" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="K18" s="13" t="s">
+      <c r="L18" s="11" t="s">
         <v>153</v>
-      </c>
-      <c r="L18" s="11" t="s">
-        <v>154</v>
       </c>
       <c r="M18" s="11" t="s">
         <v>120</v>
@@ -2436,28 +2437,28 @@
         <v>46315</v>
       </c>
       <c r="D19" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="E19" s="11" t="s">
         <v>155</v>
       </c>
-      <c r="E19" s="11" t="s">
+      <c r="F19" s="11" t="s">
         <v>156</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="G19" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="G19" s="11" t="s">
+      <c r="H19" s="11" t="s">
         <v>158</v>
       </c>
-      <c r="H19" s="11" t="s">
+      <c r="I19" s="11" t="s">
         <v>159</v>
       </c>
-      <c r="I19" s="11" t="s">
+      <c r="J19" s="11" t="s">
         <v>160</v>
       </c>
-      <c r="J19" s="11" t="s">
+      <c r="K19" s="13" t="s">
         <v>161</v>
-      </c>
-      <c r="K19" s="13" t="s">
-        <v>162</v>
       </c>
       <c r="L19" s="11"/>
       <c r="M19" s="11"/>
@@ -2476,28 +2477,28 @@
         <v>46316</v>
       </c>
       <c r="D20" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="E20" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="F20" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="G20" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="G20" s="9" t="s">
+      <c r="H20" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="H20" s="9" t="s">
+      <c r="I20" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="I20" s="9" t="s">
+      <c r="J20" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="J20" s="9" t="s">
+      <c r="K20" s="9" t="s">
         <v>169</v>
-      </c>
-      <c r="K20" s="9" t="s">
-        <v>170</v>
       </c>
       <c r="L20" s="9"/>
       <c r="M20" s="9"/>
@@ -2519,28 +2520,28 @@
         <v>103</v>
       </c>
       <c r="E21" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F21" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="G21" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="G21" s="6" t="s">
+      <c r="H21" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="H21" s="6" t="s">
+      <c r="I21" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="I21" s="6" t="s">
+      <c r="J21" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="J21" s="6" t="s">
+      <c r="K21" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="K21" s="8" t="s">
+      <c r="L21" s="6" t="s">
         <v>177</v>
-      </c>
-      <c r="L21" s="6" t="s">
-        <v>178</v>
       </c>
       <c r="M21" s="6" t="s">
         <v>52</v>
@@ -2563,34 +2564,34 @@
         <v>85</v>
       </c>
       <c r="E22" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="F22" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="F22" s="9" t="s">
+      <c r="G22" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="G22" s="9" t="s">
+      <c r="H22" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="H22" s="9" t="s">
+      <c r="I22" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="I22" s="9" t="s">
+      <c r="J22" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="J22" s="9" t="s">
+      <c r="K22" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="K22" s="9" t="s">
+      <c r="L22" s="9" t="s">
         <v>185</v>
-      </c>
-      <c r="L22" s="9" t="s">
-        <v>186</v>
       </c>
       <c r="M22" s="9" t="s">
         <v>120</v>
       </c>
       <c r="N22" s="9" t="s">
-        <v>146</v>
+        <v>186</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2634,7 +2635,7 @@
         <v>120</v>
       </c>
       <c r="N23" s="9" t="s">
-        <v>146</v>
+        <v>186</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2678,7 +2679,7 @@
         <v>120</v>
       </c>
       <c r="N24" s="9" t="s">
-        <v>146</v>
+        <v>186</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3172,7 +3173,7 @@
         <v>46336</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E40" s="9" t="s">
         <v>250</v>
@@ -3954,7 +3955,7 @@
         <v>46364</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E68" s="9" t="s">
         <v>275</v>
@@ -4154,7 +4155,7 @@
         <v>46371</v>
       </c>
       <c r="D75" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>283</v>
@@ -4371,7 +4372,7 @@
       </c>
       <c r="B3" s="15" t="n">
         <f aca="false">COUNTIF('Lịch đăng'!$N$2:$N$80,"Đã đăng")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4389,7 +4390,7 @@
       </c>
       <c r="B5" s="15" t="n">
         <f aca="false">B2-B3-B4</f>
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>